<commit_message>
Update song list to Mar 1, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J809"/>
+  <dimension ref="A1:J810"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,7 +499,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/1/23</t>
+          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/1/23，2026/3/1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -510,12 +510,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>BV1Z1u9z9E4q</t>
+          <t>BV1Z1u9z9E4q，BV15MPuzCEEd</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/1/15</t>
+          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/1/15，2026/3/1</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3390,10 +3390,14 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>BV1LPPuzjE9K</t>
+        </is>
+      </c>
       <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
@@ -6571,7 +6575,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6582,7 +6586,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8895,7 +8899,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10</t>
+          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1</t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -8906,10 +8910,14 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I219" t="inlineStr"/>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>BV1gEGSzqEtk</t>
+        </is>
+      </c>
       <c r="J219" t="inlineStr"/>
     </row>
     <row r="220">
@@ -10299,7 +10307,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10310,7 +10318,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -12539,7 +12547,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>2025/04/10，2025/05/19，2025/06/27，2025/08/21，2025/08/29，2025/09/17，2025/10/17，2025/10/30</t>
+          <t>2025/04/10，2025/05/19，2025/06/27，2025/08/21，2025/08/29，2025/09/17，2025/10/17，2025/10/30，2026/3/1</t>
         </is>
       </c>
       <c r="F316" t="inlineStr"/>
@@ -12550,10 +12558,14 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I316" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>BV1dPPuzLEnD</t>
+        </is>
+      </c>
       <c r="J316" t="inlineStr"/>
     </row>
     <row r="317">
@@ -13275,7 +13287,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13286,7 +13298,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -14643,7 +14655,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/9，2025/11/26，2025/12/5，2025/12/6，2026/1/1，2026/1/29</t>
+          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/9，2025/11/26，2025/12/5，2025/12/6，2026/1/1，2026/1/29，2026/3/1</t>
         </is>
       </c>
       <c r="F372" t="inlineStr"/>
@@ -14654,7 +14666,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
@@ -19019,7 +19031,7 @@
       </c>
       <c r="E490" t="inlineStr">
         <is>
-          <t>2025/06/01，2025/09/04</t>
+          <t>2025/06/01，2025/09/04，2026/3/1</t>
         </is>
       </c>
       <c r="F490" t="inlineStr"/>
@@ -19030,10 +19042,14 @@
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I490" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>BV1LTPuz5EKL</t>
+        </is>
+      </c>
       <c r="J490" t="inlineStr"/>
     </row>
     <row r="491">
@@ -20415,7 +20431,7 @@
       </c>
       <c r="E528" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/09/05，2025/11/17，2026/1/9</t>
+          <t>2025/06/19，2025/09/05，2025/11/17，2026/1/9，2026/3/1</t>
         </is>
       </c>
       <c r="F528" t="inlineStr"/>
@@ -20426,10 +20442,14 @@
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I528" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>BV19MPuzkEZX</t>
+        </is>
+      </c>
       <c r="J528" t="inlineStr"/>
     </row>
     <row r="529">
@@ -30335,7 +30355,7 @@
       </c>
       <c r="E795" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1</t>
         </is>
       </c>
       <c r="F795" t="inlineStr"/>
@@ -30346,7 +30366,7 @@
       </c>
       <c r="H795" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I795" t="inlineStr">
@@ -30815,7 +30835,7 @@
       </c>
       <c r="E808" t="inlineStr">
         <is>
-          <t>2026/2/25，2026/2/28</t>
+          <t>2026/2/25，2026/2/28，2026/3/1</t>
         </is>
       </c>
       <c r="F808" t="inlineStr"/>
@@ -30826,7 +30846,7 @@
       </c>
       <c r="H808" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I808" t="inlineStr">
@@ -30875,6 +30895,46 @@
         </is>
       </c>
       <c r="J809" t="inlineStr"/>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr"/>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>远航星的告别</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr"/>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/jixwang/Tarokiki/Emi Evans</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr"/>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>BV1n5PMzSEAz</t>
+        </is>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>鸣潮</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update song list to Mar 5, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -2251,7 +2251,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/7，2025/11/9，2025/12/2，2026/1/21</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/7，2025/11/9，2025/12/2，2026/1/21，2026/3/5</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/06/26，2025/08/04，2025/09/18，2025/10/25</t>
+          <t>2025/03/15，2025/06/26，2025/08/04，2025/09/18，2025/10/25，2026/3/5</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -5406,10 +5406,14 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>BV14gKfzGEvA</t>
+        </is>
+      </c>
       <c r="J125" t="inlineStr"/>
     </row>
     <row r="126">
@@ -6039,7 +6043,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19</t>
+          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -6050,7 +6054,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8227,7 +8231,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/07/24，2025/07/29，2025/07/31，2025/09/04，2025/09/24，2025/10/03，2025/10/16，2025/11/18，2025/11/21</t>
+          <t>2025/03/25，2025/07/24，2025/07/29，2025/07/31，2025/09/04，2025/09/24，2025/10/03，2025/10/16，2025/11/18，2025/11/21，2026/3/5</t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
@@ -8238,10 +8242,14 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="I200" t="inlineStr"/>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>BV1qgb1z5EKh</t>
+        </is>
+      </c>
       <c r="J200" t="inlineStr"/>
     </row>
     <row r="201">
@@ -11759,7 +11767,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/2/14</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/2/14，2026/3/5</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -11770,7 +11778,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -18715,7 +18723,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/07/13，2025/10/31</t>
+          <t>2025/05/30，2025/07/13，2025/10/31，2026/3/5</t>
         </is>
       </c>
       <c r="F479" t="inlineStr"/>
@@ -18726,10 +18734,14 @@
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I479" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>BV1xm1LBvE6P</t>
+        </is>
+      </c>
       <c r="J479" t="inlineStr"/>
     </row>
     <row r="480">
@@ -19431,7 +19443,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23</t>
+          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5</t>
         </is>
       </c>
       <c r="F498" t="inlineStr"/>
@@ -19442,7 +19454,7 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
@@ -19655,7 +19667,7 @@
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/10/20，2025/11/1</t>
+          <t>2025/06/02，2025/10/20，2025/11/1，2026/3/5</t>
         </is>
       </c>
       <c r="F504" t="inlineStr"/>
@@ -19666,10 +19678,14 @@
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I504" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>BV1WnWmzmENc</t>
+        </is>
+      </c>
       <c r="J504" t="inlineStr"/>
     </row>
     <row r="505">
@@ -19951,7 +19967,7 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>2025/06/09，2025/08/26，2025/09/17，2025/10/11，2026/2/12</t>
+          <t>2025/06/09，2025/08/26，2025/09/17，2025/10/11，2026/2/12，2026/3/5</t>
         </is>
       </c>
       <c r="F512" t="inlineStr"/>
@@ -19962,7 +19978,7 @@
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I512" t="inlineStr">
@@ -20691,7 +20707,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5</t>
         </is>
       </c>
       <c r="F532" t="inlineStr"/>
@@ -20702,7 +20718,7 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
@@ -25915,7 +25931,7 @@
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>2025/09/26，2025/12/12</t>
+          <t>2025/09/26，2025/12/12，2026/3/5</t>
         </is>
       </c>
       <c r="F672" t="inlineStr"/>
@@ -25926,7 +25942,7 @@
       </c>
       <c r="H672" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I672" t="inlineStr"/>
@@ -30459,7 +30475,7 @@
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5</t>
         </is>
       </c>
       <c r="F794" t="inlineStr"/>
@@ -30470,7 +30486,7 @@
       </c>
       <c r="H794" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I794" t="inlineStr">
@@ -31015,7 +31031,7 @@
       </c>
       <c r="E809" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5</t>
         </is>
       </c>
       <c r="F809" t="inlineStr"/>
@@ -31026,7 +31042,7 @@
       </c>
       <c r="H809" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I809" t="inlineStr">
@@ -31105,7 +31121,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I811" t="inlineStr"/>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>BV17uPizoEkm</t>
+        </is>
+      </c>
       <c r="J811" t="inlineStr"/>
     </row>
     <row r="812">
@@ -31141,7 +31161,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I812" t="inlineStr"/>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>BV1j3PizxEzc</t>
+        </is>
+      </c>
       <c r="J812" t="inlineStr"/>
     </row>
     <row r="813">

</xml_diff>

<commit_message>
chore: Update song list to Mar 6, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J814"/>
+  <dimension ref="A1:J813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -715,7 +715,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/1/21，2026/1/25，2026/2/10，2026/2/23</t>
+          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/1/21，2026/1/25，2026/2/10，2026/2/23，2026/3/6</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/11，2025/04/29，2025/08/01，2025/10/26，2026/2/19，2026/2/23</t>
+          <t>2025/03/07，2025/04/11，2025/04/29，2025/08/01，2025/10/26，2026/2/19，2026/2/23，2026/3/6</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/06/19，2025/07/10，2025/09/07，2025/09/21，2025/12/1，2026/2/14</t>
+          <t>2025/03/21，2025/06/19，2025/07/10，2025/09/07，2025/09/21，2025/12/1，2026/2/14，2026/3/6</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/7</t>
+          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/7，2026/3/6</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -5638,10 +5638,14 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr"/>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>BV1fgP4zNEYf</t>
+        </is>
+      </c>
       <c r="J131" t="inlineStr"/>
     </row>
     <row r="132">
@@ -7375,7 +7379,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7386,7 +7390,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -8691,7 +8695,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/22，2025/04/28，2025/06/30</t>
+          <t>2025/03/27，2025/04/22，2025/04/28，2025/06/30，2026/3/6</t>
         </is>
       </c>
       <c r="F212" t="inlineStr"/>
@@ -8702,10 +8706,14 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>BV1EgP4zKE1D</t>
+        </is>
+      </c>
       <c r="J212" t="inlineStr"/>
     </row>
     <row r="213">
@@ -12451,7 +12459,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/2/23</t>
+          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/2/23，2026/3/6</t>
         </is>
       </c>
       <c r="F312" t="inlineStr"/>
@@ -12462,7 +12470,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -14051,7 +14059,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/06/01，2025/08/18</t>
+          <t>2025/04/17，2025/06/01，2025/08/18，2026/3/6</t>
         </is>
       </c>
       <c r="F354" t="inlineStr"/>
@@ -14062,7 +14070,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
@@ -19483,7 +19491,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/07/03，2025/10/09，2026/1/16</t>
+          <t>2025/06/02，2025/07/03，2025/10/09，2026/1/16，2026/3/6</t>
         </is>
       </c>
       <c r="F499" t="inlineStr"/>
@@ -19494,7 +19502,7 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
@@ -22935,7 +22943,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19</t>
+          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6</t>
         </is>
       </c>
       <c r="F592" t="inlineStr"/>
@@ -22946,7 +22954,7 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
@@ -25945,7 +25953,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I672" t="inlineStr"/>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>BV1LeP2znE7t</t>
+        </is>
+      </c>
       <c r="J672" t="inlineStr"/>
     </row>
     <row r="673">
@@ -27539,79 +27551,83 @@
     <row r="716">
       <c r="A716" t="inlineStr">
         <is>
-          <t>717</t>
+          <t>718</t>
         </is>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>梦的光点</t>
-        </is>
-      </c>
-      <c r="C716" t="inlineStr"/>
+          <t>幽ノ楽園</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>幽幽乐园</t>
+        </is>
+      </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>S.H.E</t>
+          <t xml:space="preserve">Albemuth </t>
         </is>
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>2025/10/24</t>
+          <t>2025/10/25，2025/12/2，2026/2/23</t>
         </is>
       </c>
       <c r="F716" t="inlineStr"/>
       <c r="G716" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>日语</t>
         </is>
       </c>
       <c r="H716" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I716" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>BV1oV2iBGEn4</t>
+        </is>
+      </c>
       <c r="J716" t="inlineStr"/>
     </row>
     <row r="717">
       <c r="A717" t="inlineStr">
         <is>
-          <t>718</t>
+          <t>719</t>
         </is>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>幽ノ楽園</t>
-        </is>
-      </c>
-      <c r="C717" t="inlineStr">
-        <is>
-          <t>幽幽乐园</t>
-        </is>
-      </c>
+          <t>晚婚</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t xml:space="preserve">Albemuth </t>
+          <t>江蕙</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>2025/10/25，2025/12/2，2026/2/23</t>
+          <t>2025/10/28，2025/11/1，2025/11/12，2025/12/19，2026/2/8，2026/2/10</t>
         </is>
       </c>
       <c r="F717" t="inlineStr"/>
       <c r="G717" t="inlineStr">
         <is>
-          <t>日语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H717" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I717" t="inlineStr">
         <is>
-          <t>BV1oV2iBGEn4</t>
+          <t>BV1bscPz1EEj</t>
         </is>
       </c>
       <c r="J717" t="inlineStr"/>
@@ -27619,63 +27635,59 @@
     <row r="718">
       <c r="A718" t="inlineStr">
         <is>
-          <t>719</t>
+          <t>720</t>
         </is>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>晚婚</t>
+          <t>Unstoppable</t>
         </is>
       </c>
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>江蕙</t>
+          <t>Sia</t>
         </is>
       </c>
       <c r="E718" t="inlineStr">
         <is>
-          <t>2025/10/28，2025/11/1，2025/11/12，2025/12/19，2026/2/8，2026/2/10</t>
+          <t>2025/10/30</t>
         </is>
       </c>
       <c r="F718" t="inlineStr"/>
       <c r="G718" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H718" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I718" t="inlineStr">
-        <is>
-          <t>BV1bscPz1EEj</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr"/>
       <c r="J718" t="inlineStr"/>
     </row>
     <row r="719">
       <c r="A719" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>721</t>
         </is>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>Unstoppable</t>
+          <t>the cutest pair</t>
         </is>
       </c>
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Sia</t>
+          <t>Regina Song</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>2025/10/30</t>
+          <t>2025/10/30，2025/11/3，2025/11/7，2025/11/13，2025/11/22，2025/12/5，2026/1/2</t>
         </is>
       </c>
       <c r="F719" t="inlineStr"/>
@@ -27686,32 +27698,36 @@
       </c>
       <c r="H719" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I719" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>BV1tJ1vBxEFQ</t>
+        </is>
+      </c>
       <c r="J719" t="inlineStr"/>
     </row>
     <row r="720">
       <c r="A720" t="inlineStr">
         <is>
-          <t>721</t>
+          <t>722</t>
         </is>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>the cutest pair</t>
+          <t>We Are Never Ever Getting Back Together</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Regina Song</t>
+          <t>Taylor Swift</t>
         </is>
       </c>
       <c r="E720" t="inlineStr">
         <is>
-          <t>2025/10/30，2025/11/3，2025/11/7，2025/11/13，2025/11/22，2025/12/5，2026/1/2</t>
+          <t>2025/10/31，2025/11/12</t>
         </is>
       </c>
       <c r="F720" t="inlineStr"/>
@@ -27722,47 +27738,43 @@
       </c>
       <c r="H720" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I720" t="inlineStr">
-        <is>
-          <t>BV1tJ1vBxEFQ</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr"/>
       <c r="J720" t="inlineStr"/>
     </row>
     <row r="721">
       <c r="A721" t="inlineStr">
         <is>
-          <t>722</t>
+          <t>723</t>
         </is>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>We Are Never Ever Getting Back Together</t>
+          <t>雨天</t>
         </is>
       </c>
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Taylor Swift</t>
+          <t>孙燕姿</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>2025/10/31，2025/11/12</t>
+          <t>2025/11/3</t>
         </is>
       </c>
       <c r="F721" t="inlineStr"/>
       <c r="G721" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H721" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I721" t="inlineStr"/>
@@ -27771,18 +27783,22 @@
     <row r="722">
       <c r="A722" t="inlineStr">
         <is>
-          <t>723</t>
+          <t>724</t>
         </is>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>雨天</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr"/>
+          <t>ミラーチューン</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Mirror Tune</t>
+        </is>
+      </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>孙燕姿</t>
+          <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
@@ -27793,7 +27809,7 @@
       <c r="F722" t="inlineStr"/>
       <c r="G722" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>日语</t>
         </is>
       </c>
       <c r="H722" t="inlineStr">
@@ -27807,33 +27823,29 @@
     <row r="723">
       <c r="A723" t="inlineStr">
         <is>
-          <t>724</t>
+          <t>725</t>
         </is>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>ミラーチューン</t>
-        </is>
-      </c>
-      <c r="C723" t="inlineStr">
-        <is>
-          <t>Mirror Tune</t>
-        </is>
-      </c>
+          <t>God Is a Girl</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>ずっと真夜中でいいのに。</t>
+          <t>Groove Coverage</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>2025/11/3</t>
+          <t>2025/11/9</t>
         </is>
       </c>
       <c r="F723" t="inlineStr"/>
       <c r="G723" t="inlineStr">
         <is>
-          <t>日语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H723" t="inlineStr">
@@ -27847,18 +27859,18 @@
     <row r="724">
       <c r="A724" t="inlineStr">
         <is>
-          <t>725</t>
+          <t>726</t>
         </is>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>God Is a Girl</t>
+          <t>给未来的自己</t>
         </is>
       </c>
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Groove Coverage</t>
+          <t>梁静茹</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
@@ -27869,7 +27881,7 @@
       <c r="F724" t="inlineStr"/>
       <c r="G724" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H724" t="inlineStr">
@@ -27883,18 +27895,18 @@
     <row r="725">
       <c r="A725" t="inlineStr">
         <is>
-          <t>726</t>
+          <t>727</t>
         </is>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>给未来的自己</t>
+          <t>夜车</t>
         </is>
       </c>
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>梁静茹</t>
+          <t>曾轶可</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
@@ -27919,34 +27931,34 @@
     <row r="726">
       <c r="A726" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>728</t>
         </is>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>夜车</t>
+          <t>All About U</t>
         </is>
       </c>
       <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>曾轶可</t>
+          <t>G.E.M. 邓紫棋</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>2025/11/9</t>
+          <t>2025/11/9，2026/1/14</t>
         </is>
       </c>
       <c r="F726" t="inlineStr"/>
       <c r="G726" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>粤语</t>
         </is>
       </c>
       <c r="H726" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I726" t="inlineStr"/>
@@ -27955,34 +27967,34 @@
     <row r="727">
       <c r="A727" t="inlineStr">
         <is>
-          <t>728</t>
+          <t>729</t>
         </is>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>All About U</t>
+          <t>Love Fool</t>
         </is>
       </c>
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr">
         <is>
-          <t>G.E.M. 邓紫棋</t>
+          <t>EXO</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>2025/11/9，2026/1/14</t>
+          <t>2025/11/9</t>
         </is>
       </c>
       <c r="F727" t="inlineStr"/>
       <c r="G727" t="inlineStr">
         <is>
-          <t>粤语</t>
+          <t>韩语</t>
         </is>
       </c>
       <c r="H727" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I727" t="inlineStr"/>
@@ -27991,34 +28003,34 @@
     <row r="728">
       <c r="A728" t="inlineStr">
         <is>
-          <t>729</t>
+          <t>730</t>
         </is>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Love Fool</t>
+          <t>Try</t>
         </is>
       </c>
       <c r="C728" t="inlineStr"/>
       <c r="D728" t="inlineStr">
         <is>
-          <t>EXO</t>
+          <t>Colbie Caillat</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>2025/11/9</t>
+          <t>2025/11/9，2025/11/14</t>
         </is>
       </c>
       <c r="F728" t="inlineStr"/>
       <c r="G728" t="inlineStr">
         <is>
-          <t>韩语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H728" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I728" t="inlineStr"/>
@@ -28027,34 +28039,34 @@
     <row r="729">
       <c r="A729" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>731</t>
         </is>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>Try</t>
+          <t>Tabacco</t>
         </is>
       </c>
       <c r="C729" t="inlineStr"/>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Colbie Caillat</t>
+          <t>로쿠</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>2025/11/9，2025/11/14</t>
+          <t>2025/11/10，2025/11/19，2026/1/5</t>
         </is>
       </c>
       <c r="F729" t="inlineStr"/>
       <c r="G729" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>韩语</t>
         </is>
       </c>
       <c r="H729" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I729" t="inlineStr"/>
@@ -28063,23 +28075,27 @@
     <row r="730">
       <c r="A730" t="inlineStr">
         <is>
-          <t>731</t>
+          <t>732</t>
         </is>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Tabacco</t>
-        </is>
-      </c>
-      <c r="C730" t="inlineStr"/>
+          <t>밤편지</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>夜信</t>
+        </is>
+      </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>로쿠</t>
+          <t>IU</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
         <is>
-          <t>2025/11/10，2025/11/19，2026/1/5</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9</t>
         </is>
       </c>
       <c r="F730" t="inlineStr"/>
@@ -28090,76 +28106,72 @@
       </c>
       <c r="H730" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I730" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>BV1i1C3BYEKh</t>
+        </is>
+      </c>
       <c r="J730" t="inlineStr"/>
     </row>
     <row r="731">
       <c r="A731" t="inlineStr">
         <is>
-          <t>732</t>
+          <t>733</t>
         </is>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>밤편지</t>
-        </is>
-      </c>
-      <c r="C731" t="inlineStr">
-        <is>
-          <t>夜信</t>
-        </is>
-      </c>
+          <t>雪落下的声音</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr"/>
       <c r="D731" t="inlineStr">
         <is>
-          <t>IU</t>
+          <t>陆虎</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9</t>
+          <t>2025/11/14，2025/12/26</t>
         </is>
       </c>
       <c r="F731" t="inlineStr"/>
       <c r="G731" t="inlineStr">
         <is>
-          <t>韩语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H731" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="I731" t="inlineStr">
-        <is>
-          <t>BV1i1C3BYEKh</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr"/>
       <c r="J731" t="inlineStr"/>
     </row>
     <row r="732">
       <c r="A732" t="inlineStr">
         <is>
-          <t>733</t>
+          <t>734</t>
         </is>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>雪落下的声音</t>
+          <t>唯一</t>
         </is>
       </c>
       <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>陆虎</t>
+          <t>G.E.M. 邓紫棋</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
         <is>
-          <t>2025/11/14，2025/12/26</t>
+          <t>2025/11/14</t>
         </is>
       </c>
       <c r="F732" t="inlineStr"/>
@@ -28170,7 +28182,7 @@
       </c>
       <c r="H732" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I732" t="inlineStr"/>
@@ -28179,23 +28191,23 @@
     <row r="733">
       <c r="A733" t="inlineStr">
         <is>
-          <t>734</t>
+          <t>735</t>
         </is>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>唯一</t>
+          <t>绿色</t>
         </is>
       </c>
       <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>G.E.M. 邓紫棋</t>
+          <t>陈雪凝</t>
         </is>
       </c>
       <c r="E733" t="inlineStr">
         <is>
-          <t>2025/11/14</t>
+          <t>2025/11/14，2025/12/11</t>
         </is>
       </c>
       <c r="F733" t="inlineStr"/>
@@ -28206,7 +28218,7 @@
       </c>
       <c r="H733" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I733" t="inlineStr"/>
@@ -28215,34 +28227,34 @@
     <row r="734">
       <c r="A734" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>736</t>
         </is>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>绿色</t>
+          <t>Bright</t>
         </is>
       </c>
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>陈雪凝</t>
+          <t>Echosmith</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>2025/11/14，2025/12/11</t>
+          <t>2025/11/14</t>
         </is>
       </c>
       <c r="F734" t="inlineStr"/>
       <c r="G734" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H734" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I734" t="inlineStr"/>
@@ -28251,34 +28263,30 @@
     <row r="735">
       <c r="A735" t="inlineStr">
         <is>
-          <t>736</t>
+          <t>737</t>
         </is>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>Bright</t>
+          <t>Despacito</t>
         </is>
       </c>
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Echosmith</t>
+          <t>Luis Fonsi</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
         <is>
-          <t>2025/11/14</t>
+          <t>2025/11/18，2025/11/26</t>
         </is>
       </c>
       <c r="F735" t="inlineStr"/>
-      <c r="G735" t="inlineStr">
-        <is>
-          <t>英语</t>
-        </is>
-      </c>
+      <c r="G735" t="inlineStr"/>
       <c r="H735" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I735" t="inlineStr"/>
@@ -28287,30 +28295,34 @@
     <row r="736">
       <c r="A736" t="inlineStr">
         <is>
-          <t>737</t>
+          <t>738</t>
         </is>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Despacito</t>
+          <t>FEARLESS</t>
         </is>
       </c>
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Luis Fonsi</t>
+          <t>LE SSERAFIM</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>2025/11/18，2025/11/26</t>
+          <t>2025/11/18</t>
         </is>
       </c>
       <c r="F736" t="inlineStr"/>
-      <c r="G736" t="inlineStr"/>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>韩语</t>
+        </is>
+      </c>
       <c r="H736" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I736" t="inlineStr"/>
@@ -28319,18 +28331,18 @@
     <row r="737">
       <c r="A737" t="inlineStr">
         <is>
-          <t>738</t>
+          <t>739</t>
         </is>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>FEARLESS</t>
+          <t>Cake by the Ocean</t>
         </is>
       </c>
       <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>LE SSERAFIM</t>
+          <t>DNCE</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
@@ -28341,7 +28353,7 @@
       <c r="F737" t="inlineStr"/>
       <c r="G737" t="inlineStr">
         <is>
-          <t>韩语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H737" t="inlineStr">
@@ -28355,23 +28367,23 @@
     <row r="738">
       <c r="A738" t="inlineStr">
         <is>
-          <t>739</t>
+          <t>740</t>
         </is>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Cake by the Ocean</t>
+          <t>Frankenstein</t>
         </is>
       </c>
       <c r="C738" t="inlineStr"/>
       <c r="D738" t="inlineStr">
         <is>
-          <t>DNCE</t>
+          <t>Claire Rosinkranz</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>2025/11/18</t>
+          <t>2025/11/19，2025/12/26，2026/3/6</t>
         </is>
       </c>
       <c r="F738" t="inlineStr"/>
@@ -28382,32 +28394,36 @@
       </c>
       <c r="H738" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I738" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>BV1eEP4zfEmB</t>
+        </is>
+      </c>
       <c r="J738" t="inlineStr"/>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr">
         <is>
-          <t>740</t>
+          <t>741</t>
         </is>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>Frankenstein</t>
+          <t>All I Want For Christmas Is You</t>
         </is>
       </c>
       <c r="C739" t="inlineStr"/>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Claire Rosinkranz</t>
+          <t>Mariah Carey</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>2025/11/19，2025/12/26</t>
+          <t>2025/11/24，2025/12/24</t>
         </is>
       </c>
       <c r="F739" t="inlineStr"/>
@@ -28427,34 +28443,34 @@
     <row r="740">
       <c r="A740" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>742</t>
         </is>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>All I Want For Christmas Is You</t>
+          <t>麦乐鸡(Melody)</t>
         </is>
       </c>
       <c r="C740" t="inlineStr"/>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Mariah Carey</t>
+          <t>陶喆</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>2025/11/24，2025/12/24</t>
+          <t>2025/11/24</t>
         </is>
       </c>
       <c r="F740" t="inlineStr"/>
       <c r="G740" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H740" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I740" t="inlineStr"/>
@@ -28463,18 +28479,18 @@
     <row r="741">
       <c r="A741" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>743</t>
         </is>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>麦乐鸡(Melody)</t>
+          <t>哈雪大冒险</t>
         </is>
       </c>
       <c r="C741" t="inlineStr"/>
       <c r="D741" t="inlineStr">
         <is>
-          <t>陶喆</t>
+          <t>曼波</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
@@ -28499,18 +28515,18 @@
     <row r="742">
       <c r="A742" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>744</t>
         </is>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>哈雪大冒险</t>
+          <t>Desperado</t>
         </is>
       </c>
       <c r="C742" t="inlineStr"/>
       <c r="D742" t="inlineStr">
         <is>
-          <t>曼波</t>
+          <t>Eagles</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
@@ -28521,7 +28537,7 @@
       <c r="F742" t="inlineStr"/>
       <c r="G742" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H742" t="inlineStr">
@@ -28535,23 +28551,23 @@
     <row r="743">
       <c r="A743" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>745</t>
         </is>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>Desperado</t>
+          <t>My heart will go on</t>
         </is>
       </c>
       <c r="C743" t="inlineStr"/>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Eagles</t>
+          <t>Céline Dion</t>
         </is>
       </c>
       <c r="E743" t="inlineStr">
         <is>
-          <t>2025/11/24</t>
+          <t>2025/11/26</t>
         </is>
       </c>
       <c r="F743" t="inlineStr"/>
@@ -28571,18 +28587,22 @@
     <row r="744">
       <c r="A744" t="inlineStr">
         <is>
-          <t>745</t>
+          <t>746</t>
         </is>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>My heart will go on</t>
-        </is>
-      </c>
-      <c r="C744" t="inlineStr"/>
+          <t>잘자요 아가씨</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>晚安大小姐</t>
+        </is>
+      </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Céline Dion</t>
+          <t>ASMRZ</t>
         </is>
       </c>
       <c r="E744" t="inlineStr">
@@ -28593,7 +28613,7 @@
       <c r="F744" t="inlineStr"/>
       <c r="G744" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>韩语</t>
         </is>
       </c>
       <c r="H744" t="inlineStr">
@@ -28607,63 +28627,63 @@
     <row r="745">
       <c r="A745" t="inlineStr">
         <is>
-          <t>746</t>
+          <t>747</t>
         </is>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>잘자요 아가씨</t>
-        </is>
-      </c>
-      <c r="C745" t="inlineStr">
-        <is>
-          <t>晚安大小姐</t>
-        </is>
-      </c>
+          <t>恋人</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr"/>
       <c r="D745" t="inlineStr">
         <is>
-          <t>ASMRZ</t>
+          <t>李荣浩</t>
         </is>
       </c>
       <c r="E745" t="inlineStr">
         <is>
-          <t>2025/11/26</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14</t>
         </is>
       </c>
       <c r="F745" t="inlineStr"/>
       <c r="G745" t="inlineStr">
         <is>
-          <t>韩语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H745" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I745" t="inlineStr"/>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>BV181SyBPERE</t>
+        </is>
+      </c>
       <c r="J745" t="inlineStr"/>
     </row>
     <row r="746">
       <c r="A746" t="inlineStr">
         <is>
-          <t>747</t>
+          <t>748</t>
         </is>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>恋人</t>
+          <t>我不难过</t>
         </is>
       </c>
       <c r="C746" t="inlineStr"/>
       <c r="D746" t="inlineStr">
         <is>
-          <t>李荣浩</t>
+          <t>孙燕姿</t>
         </is>
       </c>
       <c r="E746" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14</t>
+          <t>2025/11/28</t>
         </is>
       </c>
       <c r="F746" t="inlineStr"/>
@@ -28674,31 +28694,27 @@
       </c>
       <c r="H746" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I746" t="inlineStr">
-        <is>
-          <t>BV181SyBPERE</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr"/>
       <c r="J746" t="inlineStr"/>
     </row>
     <row r="747">
       <c r="A747" t="inlineStr">
         <is>
-          <t>748</t>
+          <t>749</t>
         </is>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>我不难过</t>
+          <t>泪桥</t>
         </is>
       </c>
       <c r="C747" t="inlineStr"/>
       <c r="D747" t="inlineStr">
         <is>
-          <t>孙燕姿</t>
+          <t>伍佰</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
@@ -28723,18 +28739,18 @@
     <row r="748">
       <c r="A748" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>751</t>
         </is>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>泪桥</t>
+          <t>九张机</t>
         </is>
       </c>
       <c r="C748" t="inlineStr"/>
       <c r="D748" t="inlineStr">
         <is>
-          <t>伍佰</t>
+          <t>叶炫清</t>
         </is>
       </c>
       <c r="E748" t="inlineStr">
@@ -28759,29 +28775,29 @@
     <row r="749">
       <c r="A749" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>752</t>
         </is>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>九张机</t>
+          <t>Hey Jude</t>
         </is>
       </c>
       <c r="C749" t="inlineStr"/>
       <c r="D749" t="inlineStr">
         <is>
-          <t>叶炫清</t>
+          <t>The Beatles</t>
         </is>
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>2025/11/28</t>
+          <t>2025/12/2</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
       <c r="G749" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H749" t="inlineStr">
@@ -28795,23 +28811,23 @@
     <row r="750">
       <c r="A750" t="inlineStr">
         <is>
-          <t>752</t>
+          <t>753</t>
         </is>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>Hey Jude</t>
+          <t>Loves Me Not</t>
         </is>
       </c>
       <c r="C750" t="inlineStr"/>
       <c r="D750" t="inlineStr">
         <is>
-          <t>The Beatles</t>
+          <t>t.A.T.u.</t>
         </is>
       </c>
       <c r="E750" t="inlineStr">
         <is>
-          <t>2025/12/2</t>
+          <t>2025/12/4</t>
         </is>
       </c>
       <c r="F750" t="inlineStr"/>
@@ -28826,23 +28842,27 @@
         </is>
       </c>
       <c r="I750" t="inlineStr"/>
-      <c r="J750" t="inlineStr"/>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="751">
       <c r="A751" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>754</t>
         </is>
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>Loves Me Not</t>
+          <t>不怕不怕</t>
         </is>
       </c>
       <c r="C751" t="inlineStr"/>
       <c r="D751" t="inlineStr">
         <is>
-          <t>t.A.T.u.</t>
+          <t>美美jocie</t>
         </is>
       </c>
       <c r="E751" t="inlineStr">
@@ -28853,7 +28873,7 @@
       <c r="F751" t="inlineStr"/>
       <c r="G751" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H751" t="inlineStr">
@@ -28862,32 +28882,28 @@
         </is>
       </c>
       <c r="I751" t="inlineStr"/>
-      <c r="J751" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+      <c r="J751" t="inlineStr"/>
     </row>
     <row r="752">
       <c r="A752" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>755</t>
         </is>
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>不怕不怕</t>
+          <t>卜卦</t>
         </is>
       </c>
       <c r="C752" t="inlineStr"/>
       <c r="D752" t="inlineStr">
         <is>
-          <t>美美jocie</t>
+          <t>崔子格</t>
         </is>
       </c>
       <c r="E752" t="inlineStr">
         <is>
-          <t>2025/12/4</t>
+          <t>2025/12/5</t>
         </is>
       </c>
       <c r="F752" t="inlineStr"/>
@@ -28907,103 +28923,107 @@
     <row r="753">
       <c r="A753" t="inlineStr">
         <is>
-          <t>755</t>
+          <t>756</t>
         </is>
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>卜卦</t>
-        </is>
-      </c>
-      <c r="C753" t="inlineStr"/>
+          <t>届かない恋</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>无法传达的恋爱</t>
+        </is>
+      </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>崔子格</t>
+          <t>上原玲奈</t>
         </is>
       </c>
       <c r="E753" t="inlineStr">
         <is>
-          <t>2025/12/5</t>
+          <t>2025/12/9，2026/2/2</t>
         </is>
       </c>
       <c r="F753" t="inlineStr"/>
       <c r="G753" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>日语</t>
         </is>
       </c>
       <c r="H753" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I753" t="inlineStr"/>
-      <c r="J753" t="inlineStr"/>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="754">
       <c r="A754" t="inlineStr">
         <is>
-          <t>756</t>
+          <t>757</t>
         </is>
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>届かない恋</t>
-        </is>
-      </c>
-      <c r="C754" t="inlineStr">
-        <is>
-          <t>无法传达的恋爱</t>
-        </is>
-      </c>
+          <t>听见</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr"/>
       <c r="D754" t="inlineStr">
         <is>
-          <t>上原玲奈</t>
+          <t>方雅贤</t>
         </is>
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>2025/12/9，2026/2/2</t>
+          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25</t>
         </is>
       </c>
       <c r="F754" t="inlineStr"/>
       <c r="G754" t="inlineStr">
         <is>
-          <t>日语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H754" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I754" t="inlineStr"/>
-      <c r="J754" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>BV1cWmnB5Etm</t>
+        </is>
+      </c>
+      <c r="J754" t="inlineStr"/>
     </row>
     <row r="755">
       <c r="A755" t="inlineStr">
         <is>
-          <t>757</t>
+          <t>758</t>
         </is>
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>听见</t>
+          <t>神探</t>
         </is>
       </c>
       <c r="C755" t="inlineStr"/>
       <c r="D755" t="inlineStr">
         <is>
-          <t>方雅贤</t>
+          <t>丁世光</t>
         </is>
       </c>
       <c r="E755" t="inlineStr">
         <is>
-          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25</t>
+          <t>2025/12/11，2025/12/12，2025/12/17，2026/1/2，2026/1/5，2026/1/11，2026/1/17，2026/1/29，2026/2/9</t>
         </is>
       </c>
       <c r="F755" t="inlineStr"/>
@@ -29014,12 +29034,12 @@
       </c>
       <c r="H755" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I755" t="inlineStr">
         <is>
-          <t>BV1cWmnB5Etm</t>
+          <t>BV1FekxB5Etj</t>
         </is>
       </c>
       <c r="J755" t="inlineStr"/>
@@ -29027,23 +29047,23 @@
     <row r="756">
       <c r="A756" t="inlineStr">
         <is>
-          <t>758</t>
+          <t>759</t>
         </is>
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>神探</t>
+          <t>我的天坑</t>
         </is>
       </c>
       <c r="C756" t="inlineStr"/>
       <c r="D756" t="inlineStr">
         <is>
-          <t>丁世光</t>
+          <t>南征北战NZBZ</t>
         </is>
       </c>
       <c r="E756" t="inlineStr">
         <is>
-          <t>2025/12/11，2025/12/12，2025/12/17，2026/1/2，2026/1/5，2026/1/11，2026/1/17，2026/1/29，2026/2/9</t>
+          <t>2025/12/12</t>
         </is>
       </c>
       <c r="F756" t="inlineStr"/>
@@ -29054,31 +29074,27 @@
       </c>
       <c r="H756" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="I756" t="inlineStr">
-        <is>
-          <t>BV1FekxB5Etj</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr"/>
       <c r="J756" t="inlineStr"/>
     </row>
     <row r="757">
       <c r="A757" t="inlineStr">
         <is>
-          <t>759</t>
+          <t>760</t>
         </is>
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>我的天坑</t>
+          <t>同桌的你</t>
         </is>
       </c>
       <c r="C757" t="inlineStr"/>
       <c r="D757" t="inlineStr">
         <is>
-          <t>南征北战NZBZ</t>
+          <t>老狼</t>
         </is>
       </c>
       <c r="E757" t="inlineStr">
@@ -29103,18 +29119,18 @@
     <row r="758">
       <c r="A758" t="inlineStr">
         <is>
-          <t>760</t>
+          <t>761</t>
         </is>
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>同桌的你</t>
+          <t>北京东路的日子</t>
         </is>
       </c>
       <c r="C758" t="inlineStr"/>
       <c r="D758" t="inlineStr">
         <is>
-          <t>老狼</t>
+          <t>群星</t>
         </is>
       </c>
       <c r="E758" t="inlineStr">
@@ -29139,18 +29155,18 @@
     <row r="759">
       <c r="A759" t="inlineStr">
         <is>
-          <t>761</t>
+          <t>762</t>
         </is>
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>北京东路的日子</t>
+          <t>倔强</t>
         </is>
       </c>
       <c r="C759" t="inlineStr"/>
       <c r="D759" t="inlineStr">
         <is>
-          <t>群星</t>
+          <t>五月天</t>
         </is>
       </c>
       <c r="E759" t="inlineStr">
@@ -29175,18 +29191,18 @@
     <row r="760">
       <c r="A760" t="inlineStr">
         <is>
-          <t>762</t>
+          <t>763</t>
         </is>
       </c>
       <c r="B760" t="inlineStr">
         <is>
-          <t>倔强</t>
+          <t>Brand new me</t>
         </is>
       </c>
       <c r="C760" t="inlineStr"/>
       <c r="D760" t="inlineStr">
         <is>
-          <t>五月天</t>
+          <t>Alicia Keys</t>
         </is>
       </c>
       <c r="E760" t="inlineStr">
@@ -29197,7 +29213,7 @@
       <c r="F760" t="inlineStr"/>
       <c r="G760" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H760" t="inlineStr">
@@ -29211,29 +29227,29 @@
     <row r="761">
       <c r="A761" t="inlineStr">
         <is>
-          <t>763</t>
+          <t>764</t>
         </is>
       </c>
       <c r="B761" t="inlineStr">
         <is>
-          <t>Brand new me</t>
+          <t>太难唱了</t>
         </is>
       </c>
       <c r="C761" t="inlineStr"/>
       <c r="D761" t="inlineStr">
         <is>
-          <t>Alicia Keys</t>
+          <t>彭佳慧</t>
         </is>
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/12</t>
+          <t>2025/12/16</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
       <c r="G761" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H761" t="inlineStr">
@@ -29247,23 +29263,23 @@
     <row r="762">
       <c r="A762" t="inlineStr">
         <is>
-          <t>764</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B762" t="inlineStr">
         <is>
-          <t>太难唱了</t>
+          <t>他一定很爱你</t>
         </is>
       </c>
       <c r="C762" t="inlineStr"/>
       <c r="D762" t="inlineStr">
         <is>
-          <t>彭佳慧</t>
+          <t>阿杜</t>
         </is>
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/16</t>
+          <t>2025/12/17</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -29283,75 +29299,79 @@
     <row r="763">
       <c r="A763" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>766</t>
         </is>
       </c>
       <c r="B763" t="inlineStr">
         <is>
-          <t>他一定很爱你</t>
+          <t>Please Please Please</t>
         </is>
       </c>
       <c r="C763" t="inlineStr"/>
       <c r="D763" t="inlineStr">
         <is>
-          <t>阿杜</t>
+          <t>Sabrina Carpenter</t>
         </is>
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>2025/12/17</t>
+          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29</t>
         </is>
       </c>
       <c r="F763" t="inlineStr"/>
       <c r="G763" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H763" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I763" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>BV1K8isBiExx</t>
+        </is>
+      </c>
       <c r="J763" t="inlineStr"/>
     </row>
     <row r="764">
       <c r="A764" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>767</t>
         </is>
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>Please Please Please</t>
+          <t>流浪者之歌</t>
         </is>
       </c>
       <c r="C764" t="inlineStr"/>
       <c r="D764" t="inlineStr">
         <is>
-          <t>Sabrina Carpenter</t>
+          <t>F.I.R.飞儿乐团</t>
         </is>
       </c>
       <c r="E764" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29</t>
+          <t>2025/12/19，2026/2/8</t>
         </is>
       </c>
       <c r="F764" t="inlineStr"/>
       <c r="G764" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H764" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I764" t="inlineStr">
         <is>
-          <t>BV1K8isBiExx</t>
+          <t>BV1WVqrBLEc2</t>
         </is>
       </c>
       <c r="J764" t="inlineStr"/>
@@ -29359,23 +29379,23 @@
     <row r="765">
       <c r="A765" t="inlineStr">
         <is>
-          <t>767</t>
+          <t>768</t>
         </is>
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>流浪者之歌</t>
+          <t>气球</t>
         </is>
       </c>
       <c r="C765" t="inlineStr"/>
       <c r="D765" t="inlineStr">
         <is>
-          <t>F.I.R.飞儿乐团</t>
+          <t>许哲珮</t>
         </is>
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/19，2026/2/8</t>
+          <t>2025/12/19</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -29386,36 +29406,32 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I765" t="inlineStr">
-        <is>
-          <t>BV1WVqrBLEc2</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr"/>
       <c r="J765" t="inlineStr"/>
     </row>
     <row r="766">
       <c r="A766" t="inlineStr">
         <is>
-          <t>768</t>
+          <t>769</t>
         </is>
       </c>
       <c r="B766" t="inlineStr">
         <is>
-          <t>气球</t>
+          <t>一样的月光</t>
         </is>
       </c>
       <c r="C766" t="inlineStr"/>
       <c r="D766" t="inlineStr">
         <is>
-          <t>许哲珮</t>
+          <t>徐佳莹</t>
         </is>
       </c>
       <c r="E766" t="inlineStr">
         <is>
-          <t>2025/12/19</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23</t>
         </is>
       </c>
       <c r="F766" t="inlineStr"/>
@@ -29426,48 +29442,52 @@
       </c>
       <c r="H766" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I766" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>BV1oKiwBXE1L，BV1Csf6BeEYe</t>
+        </is>
+      </c>
       <c r="J766" t="inlineStr"/>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
         <is>
-          <t>769</t>
+          <t>770</t>
         </is>
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>一样的月光</t>
+          <t>BIRDS OF A FEATHER</t>
         </is>
       </c>
       <c r="C767" t="inlineStr"/>
       <c r="D767" t="inlineStr">
         <is>
-          <t>徐佳莹</t>
+          <t>Billie Eilish</t>
         </is>
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/1/2，2026/1/10</t>
         </is>
       </c>
       <c r="F767" t="inlineStr"/>
       <c r="G767" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
         <is>
-          <t>BV1oKiwBXE1L，BV1Csf6BeEYe</t>
+          <t>BV1GiicB5EFK</t>
         </is>
       </c>
       <c r="J767" t="inlineStr"/>
@@ -29475,23 +29495,23 @@
     <row r="768">
       <c r="A768" t="inlineStr">
         <is>
-          <t>770</t>
+          <t>771</t>
         </is>
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>BIRDS OF A FEATHER</t>
+          <t>Catch Me If You Can</t>
         </is>
       </c>
       <c r="C768" t="inlineStr"/>
       <c r="D768" t="inlineStr">
         <is>
-          <t>Billie Eilish</t>
+          <t>鸣潮先约电台</t>
         </is>
       </c>
       <c r="E768" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/1/2，2026/1/10</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25</t>
         </is>
       </c>
       <c r="F768" t="inlineStr"/>
@@ -29502,80 +29522,80 @@
       </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">
         <is>
-          <t>BV1GiicB5EFK</t>
-        </is>
-      </c>
-      <c r="J768" t="inlineStr"/>
+          <t>BV1pfzcBgERV，BV1aff2BvEZF</t>
+        </is>
+      </c>
+      <c r="J768" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="769">
       <c r="A769" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>772</t>
         </is>
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>Catch Me If You Can</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C769" t="inlineStr"/>
       <c r="D769" t="inlineStr">
         <is>
-          <t>鸣潮先约电台</t>
+          <t>队长/黄礼格</t>
         </is>
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25</t>
+          <t>2025/12/26，2026/1/19，2026/2/9</t>
         </is>
       </c>
       <c r="F769" t="inlineStr"/>
       <c r="G769" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H769" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I769" t="inlineStr">
         <is>
-          <t>BV1pfzcBgERV，BV1aff2BvEZF</t>
-        </is>
-      </c>
-      <c r="J769" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>BV1VUcuzvEaU</t>
+        </is>
+      </c>
+      <c r="J769" t="inlineStr"/>
     </row>
     <row r="770">
       <c r="A770" t="inlineStr">
         <is>
-          <t>772</t>
+          <t>773</t>
         </is>
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>鱼仔</t>
         </is>
       </c>
       <c r="C770" t="inlineStr"/>
       <c r="D770" t="inlineStr">
         <is>
-          <t>队长/黄礼格</t>
+          <t>卢广仲</t>
         </is>
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/19，2026/2/9</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23</t>
         </is>
       </c>
       <c r="F770" t="inlineStr"/>
@@ -29586,12 +29606,12 @@
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I770" t="inlineStr">
         <is>
-          <t>BV1VUcuzvEaU</t>
+          <t>BV1mNBfBBEkr</t>
         </is>
       </c>
       <c r="J770" t="inlineStr"/>
@@ -29599,23 +29619,23 @@
     <row r="771">
       <c r="A771" t="inlineStr">
         <is>
-          <t>773</t>
+          <t>774</t>
         </is>
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>鱼仔</t>
+          <t>Always Online</t>
         </is>
       </c>
       <c r="C771" t="inlineStr"/>
       <c r="D771" t="inlineStr">
         <is>
-          <t>卢广仲</t>
+          <t>林俊杰</t>
         </is>
       </c>
       <c r="E771" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23</t>
+          <t>2025/12/30</t>
         </is>
       </c>
       <c r="F771" t="inlineStr"/>
@@ -29626,36 +29646,32 @@
       </c>
       <c r="H771" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I771" t="inlineStr">
-        <is>
-          <t>BV1mNBfBBEkr</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr"/>
       <c r="J771" t="inlineStr"/>
     </row>
     <row r="772">
       <c r="A772" t="inlineStr">
         <is>
-          <t>774</t>
+          <t>775</t>
         </is>
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>Always Online</t>
+          <t>如愿</t>
         </is>
       </c>
       <c r="C772" t="inlineStr"/>
       <c r="D772" t="inlineStr">
         <is>
-          <t>林俊杰</t>
+          <t>王菲</t>
         </is>
       </c>
       <c r="E772" t="inlineStr">
         <is>
-          <t>2025/12/30</t>
+          <t>2026/1/5</t>
         </is>
       </c>
       <c r="F772" t="inlineStr"/>
@@ -29675,75 +29691,79 @@
     <row r="773">
       <c r="A773" t="inlineStr">
         <is>
-          <t>775</t>
+          <t>776</t>
         </is>
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>如愿</t>
+          <t>NOT CUTE ANYMORE</t>
         </is>
       </c>
       <c r="C773" t="inlineStr"/>
       <c r="D773" t="inlineStr">
         <is>
-          <t>王菲</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="E773" t="inlineStr">
         <is>
-          <t>2026/1/5</t>
+          <t>2025/12/27，2026/1/5，2026/1/6，2026/1/14，2026/1/23，2026/2/9</t>
         </is>
       </c>
       <c r="F773" t="inlineStr"/>
       <c r="G773" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>韩语</t>
         </is>
       </c>
       <c r="H773" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I773" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>BV1NrqABkEk4</t>
+        </is>
+      </c>
       <c r="J773" t="inlineStr"/>
     </row>
     <row r="774">
       <c r="A774" t="inlineStr">
         <is>
-          <t>776</t>
+          <t>777</t>
         </is>
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>NOT CUTE ANYMORE</t>
+          <t>莫名其妙爱上你</t>
         </is>
       </c>
       <c r="C774" t="inlineStr"/>
       <c r="D774" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>朱主爱</t>
         </is>
       </c>
       <c r="E774" t="inlineStr">
         <is>
-          <t>2025/12/27，2026/1/5，2026/1/6，2026/1/14，2026/1/23，2026/2/9</t>
+          <t>2026/1/14</t>
         </is>
       </c>
       <c r="F774" t="inlineStr"/>
       <c r="G774" t="inlineStr">
         <is>
-          <t>韩语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H774" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I774" t="inlineStr">
         <is>
-          <t>BV1NrqABkEk4</t>
+          <t>BV1c6rWBBEyT</t>
         </is>
       </c>
       <c r="J774" t="inlineStr"/>
@@ -29751,23 +29771,23 @@
     <row r="775">
       <c r="A775" t="inlineStr">
         <is>
-          <t>777</t>
+          <t>778</t>
         </is>
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>莫名其妙爱上你</t>
+          <t>三理之歌</t>
         </is>
       </c>
       <c r="C775" t="inlineStr"/>
       <c r="D775" t="inlineStr">
         <is>
-          <t>朱主爱</t>
+          <t>库里之歌</t>
         </is>
       </c>
       <c r="E775" t="inlineStr">
         <is>
-          <t>2026/1/14</t>
+          <t>2026/1/15，2026/1/29</t>
         </is>
       </c>
       <c r="F775" t="inlineStr"/>
@@ -29778,12 +29798,12 @@
       </c>
       <c r="H775" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I775" t="inlineStr">
         <is>
-          <t>BV1c6rWBBEyT</t>
+          <t>BV1kwkFBgEVE</t>
         </is>
       </c>
       <c r="J775" t="inlineStr"/>
@@ -29791,23 +29811,23 @@
     <row r="776">
       <c r="A776" t="inlineStr">
         <is>
-          <t>778</t>
+          <t>779</t>
         </is>
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>三理之歌</t>
+          <t>坏女孩</t>
         </is>
       </c>
       <c r="C776" t="inlineStr"/>
       <c r="D776" t="inlineStr">
         <is>
-          <t>库里之歌</t>
+          <t>徐良</t>
         </is>
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>2026/1/15，2026/1/29</t>
+          <t>2026/1/19</t>
         </is>
       </c>
       <c r="F776" t="inlineStr"/>
@@ -29818,36 +29838,32 @@
       </c>
       <c r="H776" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I776" t="inlineStr">
-        <is>
-          <t>BV1kwkFBgEVE</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr"/>
       <c r="J776" t="inlineStr"/>
     </row>
     <row r="777">
       <c r="A777" t="inlineStr">
         <is>
-          <t>779</t>
+          <t>780</t>
         </is>
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>坏女孩</t>
+          <t>分手快乐</t>
         </is>
       </c>
       <c r="C777" t="inlineStr"/>
       <c r="D777" t="inlineStr">
         <is>
-          <t>徐良</t>
+          <t>梁静茹</t>
         </is>
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>2026/1/19</t>
+          <t>2026/1/21</t>
         </is>
       </c>
       <c r="F777" t="inlineStr"/>
@@ -29867,23 +29883,23 @@
     <row r="778">
       <c r="A778" t="inlineStr">
         <is>
-          <t>780</t>
+          <t>781</t>
         </is>
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>分手快乐</t>
+          <t>我只在乎你</t>
         </is>
       </c>
       <c r="C778" t="inlineStr"/>
       <c r="D778" t="inlineStr">
         <is>
-          <t>梁静茹</t>
+          <t>邓丽君</t>
         </is>
       </c>
       <c r="E778" t="inlineStr">
         <is>
-          <t>2026/1/21</t>
+          <t>2026/1/23</t>
         </is>
       </c>
       <c r="F778" t="inlineStr"/>
@@ -29903,34 +29919,34 @@
     <row r="779">
       <c r="A779" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>782</t>
         </is>
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>我只在乎你</t>
+          <t>死别</t>
         </is>
       </c>
       <c r="C779" t="inlineStr"/>
       <c r="D779" t="inlineStr">
         <is>
-          <t>邓丽君</t>
+          <t>シャノン</t>
         </is>
       </c>
       <c r="E779" t="inlineStr">
         <is>
-          <t>2026/1/23</t>
+          <t>2026/1/23，2026/1/25，2026/2/5，2026/2/9</t>
         </is>
       </c>
       <c r="F779" t="inlineStr"/>
       <c r="G779" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>日语</t>
         </is>
       </c>
       <c r="H779" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I779" t="inlineStr"/>
@@ -29939,34 +29955,34 @@
     <row r="780">
       <c r="A780" t="inlineStr">
         <is>
-          <t>782</t>
+          <t>783</t>
         </is>
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>死别</t>
+          <t>情歌</t>
         </is>
       </c>
       <c r="C780" t="inlineStr"/>
       <c r="D780" t="inlineStr">
         <is>
-          <t>シャノン</t>
+          <t>梁静茹</t>
         </is>
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/1/23，2026/1/25，2026/2/5，2026/2/9</t>
+          <t>2026/1/23</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
       <c r="G780" t="inlineStr">
         <is>
-          <t>日语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I780" t="inlineStr"/>
@@ -29975,23 +29991,23 @@
     <row r="781">
       <c r="A781" t="inlineStr">
         <is>
-          <t>783</t>
+          <t>784</t>
         </is>
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>情歌</t>
+          <t>几分之几</t>
         </is>
       </c>
       <c r="C781" t="inlineStr"/>
       <c r="D781" t="inlineStr">
         <is>
-          <t>梁静茹</t>
+          <t>卢广仲</t>
         </is>
       </c>
       <c r="E781" t="inlineStr">
         <is>
-          <t>2026/1/23</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4</t>
         </is>
       </c>
       <c r="F781" t="inlineStr"/>
@@ -30002,32 +30018,36 @@
       </c>
       <c r="H781" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I781" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>BV1sEzxBCEua</t>
+        </is>
+      </c>
       <c r="J781" t="inlineStr"/>
     </row>
     <row r="782">
       <c r="A782" t="inlineStr">
         <is>
-          <t>784</t>
+          <t>785</t>
         </is>
       </c>
       <c r="B782" t="inlineStr">
         <is>
-          <t>几分之几</t>
+          <t>爱不单行</t>
         </is>
       </c>
       <c r="C782" t="inlineStr"/>
       <c r="D782" t="inlineStr">
         <is>
-          <t>卢广仲</t>
+          <t>罗志祥</t>
         </is>
       </c>
       <c r="E782" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4</t>
+          <t>2026/1/24，2026/2/8</t>
         </is>
       </c>
       <c r="F782" t="inlineStr"/>
@@ -30038,12 +30058,12 @@
       </c>
       <c r="H782" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I782" t="inlineStr">
         <is>
-          <t>BV1sEzxBCEua</t>
+          <t>BV1zPz1BRExW</t>
         </is>
       </c>
       <c r="J782" t="inlineStr"/>
@@ -30051,193 +30071,189 @@
     <row r="783">
       <c r="A783" t="inlineStr">
         <is>
-          <t>785</t>
+          <t>786</t>
         </is>
       </c>
       <c r="B783" t="inlineStr">
         <is>
-          <t>爱不单行</t>
-        </is>
-      </c>
-      <c r="C783" t="inlineStr"/>
+          <t>STAR WALKIN'</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>逐星</t>
+        </is>
+      </c>
       <c r="D783" t="inlineStr">
         <is>
-          <t>罗志祥</t>
+          <t>Lil Nas X</t>
         </is>
       </c>
       <c r="E783" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/2/8</t>
+          <t>2026/1/25</t>
         </is>
       </c>
       <c r="F783" t="inlineStr"/>
       <c r="G783" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H783" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I783" t="inlineStr">
-        <is>
-          <t>BV1zPz1BRExW</t>
-        </is>
-      </c>
-      <c r="J783" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr"/>
+      <c r="J783" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="784">
       <c r="A784" t="inlineStr">
         <is>
-          <t>786</t>
+          <t>787</t>
         </is>
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>STAR WALKIN'</t>
-        </is>
-      </c>
-      <c r="C784" t="inlineStr">
-        <is>
-          <t>逐星</t>
-        </is>
-      </c>
+          <t>阳光彩虹小白马</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr"/>
       <c r="D784" t="inlineStr">
         <is>
-          <t>Lil Nas X</t>
+          <t>大张伟</t>
         </is>
       </c>
       <c r="E784" t="inlineStr">
         <is>
-          <t>2026/1/25</t>
+          <t>2026/1/25，2026/2/10</t>
         </is>
       </c>
       <c r="F784" t="inlineStr"/>
       <c r="G784" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H784" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I784" t="inlineStr"/>
-      <c r="J784" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>BV1Gnc4zmEjA</t>
+        </is>
+      </c>
+      <c r="J784" t="inlineStr"/>
     </row>
     <row r="785">
       <c r="A785" t="inlineStr">
         <is>
-          <t>787</t>
+          <t>788</t>
         </is>
       </c>
       <c r="B785" t="inlineStr">
         <is>
-          <t>阳光彩虹小白马</t>
+          <t>Lulala! Lululala!</t>
         </is>
       </c>
       <c r="C785" t="inlineStr"/>
       <c r="D785" t="inlineStr">
         <is>
-          <t>大张伟</t>
+          <t>鸣潮先约电台</t>
         </is>
       </c>
       <c r="E785" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/2/10</t>
+          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25</t>
         </is>
       </c>
       <c r="F785" t="inlineStr"/>
       <c r="G785" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H785" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I785" t="inlineStr">
         <is>
-          <t>BV1Gnc4zmEjA</t>
-        </is>
-      </c>
-      <c r="J785" t="inlineStr"/>
+          <t>BV1Dv6qBsEXr</t>
+        </is>
+      </c>
+      <c r="J785" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="786">
-      <c r="A786" t="inlineStr">
-        <is>
-          <t>788</t>
-        </is>
-      </c>
+      <c r="A786" t="inlineStr"/>
       <c r="B786" t="inlineStr">
         <is>
-          <t>Lulala! Lululala!</t>
+          <t>爱要坦荡荡(R&amp;B版)</t>
         </is>
       </c>
       <c r="C786" t="inlineStr"/>
       <c r="D786" t="inlineStr">
         <is>
-          <t>鸣潮先约电台</t>
+          <t>顾叮当</t>
         </is>
       </c>
       <c r="E786" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25</t>
+          <t>2026/1/29</t>
         </is>
       </c>
       <c r="F786" t="inlineStr"/>
       <c r="G786" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H786" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I786" t="inlineStr">
         <is>
-          <t>BV1Dv6qBsEXr</t>
-        </is>
-      </c>
-      <c r="J786" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>BV1Xx6cBRE14</t>
+        </is>
+      </c>
+      <c r="J786" t="inlineStr"/>
     </row>
     <row r="787">
       <c r="A787" t="inlineStr"/>
       <c r="B787" t="inlineStr">
         <is>
-          <t>爱要坦荡荡(R&amp;B版)</t>
+          <t>Long Live</t>
         </is>
       </c>
       <c r="C787" t="inlineStr"/>
       <c r="D787" t="inlineStr">
         <is>
-          <t>顾叮当</t>
+          <t>Taylor Swift</t>
         </is>
       </c>
       <c r="E787" t="inlineStr">
         <is>
-          <t>2026/1/29</t>
+          <t>2026/1/30</t>
         </is>
       </c>
       <c r="F787" t="inlineStr"/>
       <c r="G787" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H787" t="inlineStr">
@@ -30245,61 +30261,61 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I787" t="inlineStr">
-        <is>
-          <t>BV1Xx6cBRE14</t>
-        </is>
-      </c>
+      <c r="I787" t="inlineStr"/>
       <c r="J787" t="inlineStr"/>
     </row>
     <row r="788">
       <c r="A788" t="inlineStr"/>
       <c r="B788" t="inlineStr">
         <is>
-          <t>Long Live</t>
+          <t>身不由己</t>
         </is>
       </c>
       <c r="C788" t="inlineStr"/>
       <c r="D788" t="inlineStr">
         <is>
-          <t>Taylor Swift</t>
+          <t>大都会乐团</t>
         </is>
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>2026/1/30</t>
+          <t>2026/2/2，2026/2/5，2026/2/9，2026/2/22</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
       <c r="G788" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H788" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I788" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>BV1fxFMzqEDd</t>
+        </is>
+      </c>
       <c r="J788" t="inlineStr"/>
     </row>
     <row r="789">
       <c r="A789" t="inlineStr"/>
       <c r="B789" t="inlineStr">
         <is>
-          <t>身不由己</t>
+          <t>乐鸣东方</t>
         </is>
       </c>
       <c r="C789" t="inlineStr"/>
       <c r="D789" t="inlineStr">
         <is>
-          <t>大都会乐团</t>
+          <t>洛天依</t>
         </is>
       </c>
       <c r="E789" t="inlineStr">
         <is>
-          <t>2026/2/2，2026/2/5，2026/2/9，2026/2/22</t>
+          <t>2026/2/7</t>
         </is>
       </c>
       <c r="F789" t="inlineStr"/>
@@ -30310,27 +30326,23 @@
       </c>
       <c r="H789" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I789" t="inlineStr">
-        <is>
-          <t>BV1fxFMzqEDd</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr"/>
       <c r="J789" t="inlineStr"/>
     </row>
     <row r="790">
       <c r="A790" t="inlineStr"/>
       <c r="B790" t="inlineStr">
         <is>
-          <t>乐鸣东方</t>
+          <t>爱的飞行日记</t>
         </is>
       </c>
       <c r="C790" t="inlineStr"/>
       <c r="D790" t="inlineStr">
         <is>
-          <t>洛天依</t>
+          <t>周杰伦</t>
         </is>
       </c>
       <c r="E790" t="inlineStr">
@@ -30349,25 +30361,29 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I790" t="inlineStr"/>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>BV1wGF4zFEBM</t>
+        </is>
+      </c>
       <c r="J790" t="inlineStr"/>
     </row>
     <row r="791">
       <c r="A791" t="inlineStr"/>
       <c r="B791" t="inlineStr">
         <is>
-          <t>爱的飞行日记</t>
+          <t>相亲相爱</t>
         </is>
       </c>
       <c r="C791" t="inlineStr"/>
       <c r="D791" t="inlineStr">
         <is>
-          <t>周杰伦</t>
+          <t>陈慧琳/张惠妹/孙楠/古淖文</t>
         </is>
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>2026/2/7</t>
+          <t>2026/2/8</t>
         </is>
       </c>
       <c r="F791" t="inlineStr"/>
@@ -30383,7 +30399,7 @@
       </c>
       <c r="I791" t="inlineStr">
         <is>
-          <t>BV1wGF4zFEBM</t>
+          <t>BV1U9cTzpEjm</t>
         </is>
       </c>
       <c r="J791" t="inlineStr"/>
@@ -30392,18 +30408,18 @@
       <c r="A792" t="inlineStr"/>
       <c r="B792" t="inlineStr">
         <is>
-          <t>相亲相爱</t>
+          <t>混入人类计划</t>
         </is>
       </c>
       <c r="C792" t="inlineStr"/>
       <c r="D792" t="inlineStr">
         <is>
-          <t>陈慧琳/张惠妹/孙楠/古淖文</t>
+          <t>ChiliChill</t>
         </is>
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>2026/2/8</t>
+          <t>2026/2/8，2026/2/9，2026/2/14，2026/2/20，2026/2/28</t>
         </is>
       </c>
       <c r="F792" t="inlineStr"/>
@@ -30414,12 +30430,12 @@
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
         <is>
-          <t>BV1U9cTzpEjm</t>
+          <t>BV1JncczQEuJ，BV1c6fGBDEG1</t>
         </is>
       </c>
       <c r="J792" t="inlineStr"/>
@@ -30428,94 +30444,94 @@
       <c r="A793" t="inlineStr"/>
       <c r="B793" t="inlineStr">
         <is>
-          <t>混入人类计划</t>
+          <t>纸飞机</t>
         </is>
       </c>
       <c r="C793" t="inlineStr"/>
       <c r="D793" t="inlineStr">
         <is>
-          <t>ChiliChill</t>
+          <t>鸣潮先约电台/飞行雪绒</t>
         </is>
       </c>
       <c r="E793" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/14，2026/2/20，2026/2/28</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5</t>
         </is>
       </c>
       <c r="F793" t="inlineStr"/>
       <c r="G793" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
         <is>
-          <t>BV1JncczQEuJ，BV1c6fGBDEG1</t>
-        </is>
-      </c>
-      <c r="J793" t="inlineStr"/>
+          <t>BV1W4cuzSE8Y，BV12Ef6BBE5C</t>
+        </is>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="794">
       <c r="A794" t="inlineStr"/>
       <c r="B794" t="inlineStr">
         <is>
-          <t>纸飞机</t>
+          <t>刻在我心底的名字</t>
         </is>
       </c>
       <c r="C794" t="inlineStr"/>
       <c r="D794" t="inlineStr">
         <is>
-          <t>鸣潮先约电台/飞行雪绒</t>
+          <t>卢广仲</t>
         </is>
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5</t>
+          <t>2026/2/9，2026/2/27</t>
         </is>
       </c>
       <c r="F794" t="inlineStr"/>
       <c r="G794" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H794" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I794" t="inlineStr">
         <is>
-          <t>BV1W4cuzSE8Y，BV12Ef6BBE5C</t>
-        </is>
-      </c>
-      <c r="J794" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>BV1EkcszREeP，BV11dAQz2ESx</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr"/>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr"/>
       <c r="B795" t="inlineStr">
         <is>
-          <t>刻在我心底的名字</t>
+          <t>词不达意</t>
         </is>
       </c>
       <c r="C795" t="inlineStr"/>
       <c r="D795" t="inlineStr">
         <is>
-          <t>卢广仲</t>
+          <t>林忆莲</t>
         </is>
       </c>
       <c r="E795" t="inlineStr">
         <is>
-          <t>2026/2/9，2026/2/27</t>
+          <t>2026/2/12</t>
         </is>
       </c>
       <c r="F795" t="inlineStr"/>
@@ -30526,12 +30542,12 @@
       </c>
       <c r="H795" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I795" t="inlineStr">
         <is>
-          <t>BV1EkcszREeP，BV11dAQz2ESx</t>
+          <t>BV1BNcBz4ECH</t>
         </is>
       </c>
       <c r="J795" t="inlineStr"/>
@@ -30540,64 +30556,68 @@
       <c r="A796" t="inlineStr"/>
       <c r="B796" t="inlineStr">
         <is>
-          <t>词不达意</t>
-        </is>
-      </c>
-      <c r="C796" t="inlineStr"/>
+          <t>RUNNING FOR YOUR LIFE</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>无所遁藏</t>
+        </is>
+      </c>
       <c r="D796" t="inlineStr">
         <is>
-          <t>林忆莲</t>
+          <t>鸣潮先约电台/Casey Lee Williams</t>
         </is>
       </c>
       <c r="E796" t="inlineStr">
         <is>
-          <t>2026/2/12</t>
+          <t>2026/2/14，2026/2/24</t>
         </is>
       </c>
       <c r="F796" t="inlineStr"/>
       <c r="G796" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H796" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I796" t="inlineStr">
         <is>
-          <t>BV1BNcBz4ECH</t>
-        </is>
-      </c>
-      <c r="J796" t="inlineStr"/>
+          <t>BV14GZEBgErZ</t>
+        </is>
+      </c>
+      <c r="J796" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr"/>
       <c r="B797" t="inlineStr">
         <is>
-          <t>RUNNING FOR YOUR LIFE</t>
-        </is>
-      </c>
-      <c r="C797" t="inlineStr">
-        <is>
-          <t>无所遁藏</t>
-        </is>
-      </c>
+          <t>发财发福中国年</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr"/>
       <c r="D797" t="inlineStr">
         <is>
-          <t>鸣潮先约电台/Casey Lee Williams</t>
+          <t>中国娃娃</t>
         </is>
       </c>
       <c r="E797" t="inlineStr">
         <is>
-          <t>2026/2/14，2026/2/24</t>
+          <t>2026/2/17，2026/2/19</t>
         </is>
       </c>
       <c r="F797" t="inlineStr"/>
       <c r="G797" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H797" t="inlineStr">
@@ -30607,31 +30627,27 @@
       </c>
       <c r="I797" t="inlineStr">
         <is>
-          <t>BV14GZEBgErZ</t>
-        </is>
-      </c>
-      <c r="J797" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>BV1EYZ1B6ECT</t>
+        </is>
+      </c>
+      <c r="J797" t="inlineStr"/>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr"/>
       <c r="B798" t="inlineStr">
         <is>
-          <t>发财发福中国年</t>
+          <t>恭喜发财</t>
         </is>
       </c>
       <c r="C798" t="inlineStr"/>
       <c r="D798" t="inlineStr">
         <is>
-          <t>中国娃娃</t>
+          <t>刘德华</t>
         </is>
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>2026/2/17，2026/2/19</t>
+          <t>2026/2/17</t>
         </is>
       </c>
       <c r="F798" t="inlineStr"/>
@@ -30642,38 +30658,34 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I798" t="inlineStr">
-        <is>
-          <t>BV1EYZ1B6ECT</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr"/>
       <c r="J798" t="inlineStr"/>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr"/>
       <c r="B799" t="inlineStr">
         <is>
-          <t>恭喜发财</t>
+          <t>迎春花</t>
         </is>
       </c>
       <c r="C799" t="inlineStr"/>
       <c r="D799" t="inlineStr">
         <is>
-          <t>刘德华</t>
+          <t>卓依婷</t>
         </is>
       </c>
       <c r="E799" t="inlineStr">
         <is>
-          <t>2026/2/17</t>
+          <t>2026/2/19</t>
         </is>
       </c>
       <c r="F799" t="inlineStr"/>
       <c r="G799" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>粤语</t>
         </is>
       </c>
       <c r="H799" t="inlineStr">
@@ -30681,20 +30693,24 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I799" t="inlineStr"/>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>BV1gnZBBiEmr</t>
+        </is>
+      </c>
       <c r="J799" t="inlineStr"/>
     </row>
     <row r="800">
       <c r="A800" t="inlineStr"/>
       <c r="B800" t="inlineStr">
         <is>
-          <t>迎春花</t>
+          <t>天堂</t>
         </is>
       </c>
       <c r="C800" t="inlineStr"/>
       <c r="D800" t="inlineStr">
         <is>
-          <t>卓依婷</t>
+          <t>腾格尔</t>
         </is>
       </c>
       <c r="E800" t="inlineStr">
@@ -30705,7 +30721,7 @@
       <c r="F800" t="inlineStr"/>
       <c r="G800" t="inlineStr">
         <is>
-          <t>粤语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H800" t="inlineStr">
@@ -30715,7 +30731,7 @@
       </c>
       <c r="I800" t="inlineStr">
         <is>
-          <t>BV1gnZBBiEmr</t>
+          <t>BV166ZBBQEWz</t>
         </is>
       </c>
       <c r="J800" t="inlineStr"/>
@@ -30724,18 +30740,18 @@
       <c r="A801" t="inlineStr"/>
       <c r="B801" t="inlineStr">
         <is>
-          <t>天堂</t>
+          <t>退后</t>
         </is>
       </c>
       <c r="C801" t="inlineStr"/>
       <c r="D801" t="inlineStr">
         <is>
-          <t>腾格尔</t>
+          <t>周杰伦</t>
         </is>
       </c>
       <c r="E801" t="inlineStr">
         <is>
-          <t>2026/2/19</t>
+          <t>2026/2/20</t>
         </is>
       </c>
       <c r="F801" t="inlineStr"/>
@@ -30751,7 +30767,7 @@
       </c>
       <c r="I801" t="inlineStr">
         <is>
-          <t>BV166ZBBQEWz</t>
+          <t>BV1zkfGBEELD</t>
         </is>
       </c>
       <c r="J801" t="inlineStr"/>
@@ -30760,13 +30776,13 @@
       <c r="A802" t="inlineStr"/>
       <c r="B802" t="inlineStr">
         <is>
-          <t>退后</t>
+          <t>最近还好吗</t>
         </is>
       </c>
       <c r="C802" t="inlineStr"/>
       <c r="D802" t="inlineStr">
         <is>
-          <t>周杰伦</t>
+          <t>S.H.E</t>
         </is>
       </c>
       <c r="E802" t="inlineStr">
@@ -30787,7 +30803,7 @@
       </c>
       <c r="I802" t="inlineStr">
         <is>
-          <t>BV1zkfGBEELD</t>
+          <t>BV14Tf3BWEef</t>
         </is>
       </c>
       <c r="J802" t="inlineStr"/>
@@ -30796,89 +30812,89 @@
       <c r="A803" t="inlineStr"/>
       <c r="B803" t="inlineStr">
         <is>
-          <t>最近还好吗</t>
+          <t>持续瞬间的永恒</t>
         </is>
       </c>
       <c r="C803" t="inlineStr"/>
       <c r="D803" t="inlineStr">
         <is>
-          <t>S.H.E</t>
+          <t>鸣潮先约电台/jixwang/markmilian/Sophia</t>
         </is>
       </c>
       <c r="E803" t="inlineStr">
         <is>
-          <t>2026/2/20</t>
+          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25</t>
         </is>
       </c>
       <c r="F803" t="inlineStr"/>
       <c r="G803" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H803" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I803" t="inlineStr">
         <is>
-          <t>BV14Tf3BWEef</t>
-        </is>
-      </c>
-      <c r="J803" t="inlineStr"/>
+          <t>BV1K7f6BgE9r</t>
+        </is>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr"/>
       <c r="B804" t="inlineStr">
         <is>
-          <t>持续瞬间的永恒</t>
+          <t>安静</t>
         </is>
       </c>
       <c r="C804" t="inlineStr"/>
       <c r="D804" t="inlineStr">
         <is>
-          <t>鸣潮先约电台/jixwang/markmilian/Sophia</t>
+          <t>周杰伦</t>
         </is>
       </c>
       <c r="E804" t="inlineStr">
         <is>
-          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25</t>
+          <t>2026/2/23</t>
         </is>
       </c>
       <c r="F804" t="inlineStr"/>
       <c r="G804" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H804" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I804" t="inlineStr">
         <is>
-          <t>BV1K7f6BgE9r</t>
-        </is>
-      </c>
-      <c r="J804" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>BV11nf6BTE4b</t>
+        </is>
+      </c>
+      <c r="J804" t="inlineStr"/>
     </row>
     <row r="805">
       <c r="A805" t="inlineStr"/>
       <c r="B805" t="inlineStr">
         <is>
-          <t>安静</t>
+          <t>可惜没如果</t>
         </is>
       </c>
       <c r="C805" t="inlineStr"/>
       <c r="D805" t="inlineStr">
         <is>
-          <t>周杰伦</t>
+          <t>林俊杰</t>
         </is>
       </c>
       <c r="E805" t="inlineStr">
@@ -30899,7 +30915,7 @@
       </c>
       <c r="I805" t="inlineStr">
         <is>
-          <t>BV11nf6BTE4b</t>
+          <t>BV1w1fzBwEhj</t>
         </is>
       </c>
       <c r="J805" t="inlineStr"/>
@@ -30908,94 +30924,94 @@
       <c r="A806" t="inlineStr"/>
       <c r="B806" t="inlineStr">
         <is>
-          <t>可惜没如果</t>
+          <t>星炬不熄</t>
         </is>
       </c>
       <c r="C806" t="inlineStr"/>
       <c r="D806" t="inlineStr">
         <is>
-          <t>林俊杰</t>
+          <t>鸣潮先约电台/飞行雪绒/星炬学院毕业生</t>
         </is>
       </c>
       <c r="E806" t="inlineStr">
         <is>
-          <t>2026/2/23</t>
+          <t>2026/2/25，2026/2/28，2026/3/1</t>
         </is>
       </c>
       <c r="F806" t="inlineStr"/>
       <c r="G806" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>华语，日语，英语，韩语</t>
         </is>
       </c>
       <c r="H806" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I806" t="inlineStr">
         <is>
-          <t>BV1w1fzBwEhj</t>
-        </is>
-      </c>
-      <c r="J806" t="inlineStr"/>
+          <t>BV1WDfaByEfD</t>
+        </is>
+      </c>
+      <c r="J806" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="807">
       <c r="A807" t="inlineStr"/>
       <c r="B807" t="inlineStr">
         <is>
-          <t>星炬不熄</t>
+          <t>Everglow</t>
         </is>
       </c>
       <c r="C807" t="inlineStr"/>
       <c r="D807" t="inlineStr">
         <is>
-          <t>鸣潮先约电台/飞行雪绒/星炬学院毕业生</t>
+          <t>Coldplay</t>
         </is>
       </c>
       <c r="E807" t="inlineStr">
         <is>
-          <t>2026/2/25，2026/2/28，2026/3/1</t>
+          <t>2026/2/27</t>
         </is>
       </c>
       <c r="F807" t="inlineStr"/>
       <c r="G807" t="inlineStr">
         <is>
-          <t>华语，日语，英语，韩语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H807" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I807" t="inlineStr">
         <is>
-          <t>BV1WDfaByEfD</t>
-        </is>
-      </c>
-      <c r="J807" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>BV1kcAXzVEXm</t>
+        </is>
+      </c>
+      <c r="J807" t="inlineStr"/>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr"/>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Everglow</t>
+          <t>远航星的告别</t>
         </is>
       </c>
       <c r="C808" t="inlineStr"/>
       <c r="D808" t="inlineStr">
         <is>
-          <t>Coldplay</t>
+          <t>鸣潮先约电台/jixwang/Tarokiki/Emi Evans</t>
         </is>
       </c>
       <c r="E808" t="inlineStr">
         <is>
-          <t>2026/2/27</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6</t>
         </is>
       </c>
       <c r="F808" t="inlineStr"/>
@@ -31006,71 +31022,67 @@
       </c>
       <c r="H808" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I808" t="inlineStr">
         <is>
-          <t>BV1kcAXzVEXm</t>
-        </is>
-      </c>
-      <c r="J808" t="inlineStr"/>
+          <t>BV1n5PMzSEAz</t>
+        </is>
+      </c>
+      <c r="J808" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr"/>
       <c r="B809" t="inlineStr">
         <is>
-          <t>远航星的告别</t>
-        </is>
-      </c>
-      <c r="C809" t="inlineStr"/>
+          <t>月迷風影</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>月迷风影</t>
+        </is>
+      </c>
       <c r="D809" t="inlineStr">
         <is>
-          <t>鸣潮先约电台/jixwang/Tarokiki/Emi Evans</t>
+          <t>有坂美香</t>
         </is>
       </c>
       <c r="E809" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5</t>
+          <t>2026/3/4</t>
         </is>
       </c>
       <c r="F809" t="inlineStr"/>
       <c r="G809" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>日语</t>
         </is>
       </c>
       <c r="H809" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I809" t="inlineStr">
-        <is>
-          <t>BV1n5PMzSEAz</t>
-        </is>
-      </c>
-      <c r="J809" t="inlineStr">
-        <is>
-          <t>游戏</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr"/>
+      <c r="J809" t="inlineStr"/>
     </row>
     <row r="810">
       <c r="A810" t="inlineStr"/>
       <c r="B810" t="inlineStr">
         <is>
-          <t>月迷風影</t>
-        </is>
-      </c>
-      <c r="C810" t="inlineStr">
-        <is>
-          <t>月迷风影</t>
-        </is>
-      </c>
+          <t>我还想她</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr"/>
       <c r="D810" t="inlineStr">
         <is>
-          <t>有坂美香</t>
+          <t>林俊杰</t>
         </is>
       </c>
       <c r="E810" t="inlineStr">
@@ -31081,7 +31093,7 @@
       <c r="F810" t="inlineStr"/>
       <c r="G810" t="inlineStr">
         <is>
-          <t>日语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H810" t="inlineStr">
@@ -31089,20 +31101,28 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I810" t="inlineStr"/>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>BV17uPizoEkm</t>
+        </is>
+      </c>
       <c r="J810" t="inlineStr"/>
     </row>
     <row r="811">
       <c r="A811" t="inlineStr"/>
       <c r="B811" t="inlineStr">
         <is>
-          <t>我还想她</t>
-        </is>
-      </c>
-      <c r="C811" t="inlineStr"/>
+          <t>未来へ</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>向着未来</t>
+        </is>
+      </c>
       <c r="D811" t="inlineStr">
         <is>
-          <t>林俊杰</t>
+          <t>Kiroro</t>
         </is>
       </c>
       <c r="E811" t="inlineStr">
@@ -31113,7 +31133,7 @@
       <c r="F811" t="inlineStr"/>
       <c r="G811" t="inlineStr">
         <is>
-          <t>华语</t>
+          <t>日语</t>
         </is>
       </c>
       <c r="H811" t="inlineStr">
@@ -31123,7 +31143,7 @@
       </c>
       <c r="I811" t="inlineStr">
         <is>
-          <t>BV17uPizoEkm</t>
+          <t>BV1j3PizxEzc</t>
         </is>
       </c>
       <c r="J811" t="inlineStr"/>
@@ -31132,38 +31152,34 @@
       <c r="A812" t="inlineStr"/>
       <c r="B812" t="inlineStr">
         <is>
-          <t>未来へ</t>
-        </is>
-      </c>
-      <c r="C812" t="inlineStr">
-        <is>
-          <t>向着未来</t>
-        </is>
-      </c>
+          <t>突然的陀螺</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr"/>
       <c r="D812" t="inlineStr">
         <is>
-          <t>Kiroro</t>
+          <t>蔚蓝边际</t>
         </is>
       </c>
       <c r="E812" t="inlineStr">
         <is>
-          <t>2026/3/4</t>
+          <t>2025/12/8，2026/1/9，2026/3/4</t>
         </is>
       </c>
       <c r="F812" t="inlineStr"/>
       <c r="G812" t="inlineStr">
         <is>
-          <t>日语</t>
+          <t>华语</t>
         </is>
       </c>
       <c r="H812" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I812" t="inlineStr">
         <is>
-          <t>BV1j3PizxEzc</t>
+          <t>BV13z2yBtEb1</t>
         </is>
       </c>
       <c r="J812" t="inlineStr"/>
@@ -31172,18 +31188,18 @@
       <c r="A813" t="inlineStr"/>
       <c r="B813" t="inlineStr">
         <is>
-          <t>突然的陀螺</t>
+          <t>不为谁而做的歌</t>
         </is>
       </c>
       <c r="C813" t="inlineStr"/>
       <c r="D813" t="inlineStr">
         <is>
-          <t>蔚蓝边际</t>
+          <t>林俊杰</t>
         </is>
       </c>
       <c r="E813" t="inlineStr">
         <is>
-          <t>2025/12/8，2026/1/9，2026/3/4</t>
+          <t>2025/12/8</t>
         </is>
       </c>
       <c r="F813" t="inlineStr"/>
@@ -31194,47 +31210,11 @@
       </c>
       <c r="H813" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I813" t="inlineStr">
-        <is>
-          <t>BV13z2yBtEb1</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr"/>
       <c r="J813" t="inlineStr"/>
-    </row>
-    <row r="814">
-      <c r="A814" t="inlineStr"/>
-      <c r="B814" t="inlineStr">
-        <is>
-          <t>不为谁而做的歌</t>
-        </is>
-      </c>
-      <c r="C814" t="inlineStr"/>
-      <c r="D814" t="inlineStr">
-        <is>
-          <t>林俊杰</t>
-        </is>
-      </c>
-      <c r="E814" t="inlineStr">
-        <is>
-          <t>2025/12/8</t>
-        </is>
-      </c>
-      <c r="F814" t="inlineStr"/>
-      <c r="G814" t="inlineStr">
-        <is>
-          <t>华语</t>
-        </is>
-      </c>
-      <c r="H814" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I814" t="inlineStr"/>
-      <c r="J814" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 6, 2026 v2
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -5587,7 +5587,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5598,7 +5598,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -20271,7 +20271,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6</t>
         </is>
       </c>
       <c r="F520" t="inlineStr"/>
@@ -20282,7 +20282,7 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I520" t="inlineStr">
@@ -21359,7 +21359,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9</t>
+          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -21374,7 +21374,7 @@
       </c>
       <c r="H549" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I549" t="inlineStr">
@@ -21382,7 +21382,11 @@
           <t>BV12MzyBAEbS</t>
         </is>
       </c>
-      <c r="J549" t="inlineStr"/>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>特殊</t>
+        </is>
+      </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -26723,7 +26727,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13</t>
+          <t>2025/10/13，2026/3/4</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -26738,11 +26742,19 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I693" t="inlineStr"/>
-      <c r="J693" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>BV1WKPKz7EBS</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>特殊</t>
+        </is>
+      </c>
     </row>
     <row r="694">
       <c r="A694" t="inlineStr">
@@ -29511,7 +29523,7 @@
       </c>
       <c r="E768" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6</t>
         </is>
       </c>
       <c r="F768" t="inlineStr"/>
@@ -29522,7 +29534,7 @@
       </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 7, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J813"/>
+  <dimension ref="A1:J815"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,7 +583,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19</t>
+          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -594,7 +594,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/19，2025/06/02，2025/06/17，2025/06/23，2025/07/20，2025/09/24，2025/10/09，2026/2/17</t>
+          <t>2025/03/07，2025/04/04，2025/04/19，2025/06/02，2025/06/17，2025/06/23，2025/07/20，2025/09/24，2025/10/09，2026/2/17，2026/3/7</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4</t>
+          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5598,7 +5598,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28</t>
+          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7</t>
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
@@ -9494,7 +9494,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -9607,18 +9607,18 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>英语，韩语</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/1/9</t>
+          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/1/9，2026/3/7</t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
@@ -9966,10 +9966,14 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I245" t="inlineStr"/>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>BV1jANPzvEDw</t>
+        </is>
+      </c>
       <c r="J245" t="inlineStr"/>
     </row>
     <row r="246">
@@ -21483,7 +21487,7 @@
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>2025/06/27</t>
+          <t>2025/06/27，2026/3/7</t>
         </is>
       </c>
       <c r="F552" t="inlineStr"/>
@@ -21494,7 +21498,7 @@
       </c>
       <c r="H552" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I552" t="inlineStr"/>
@@ -22503,7 +22507,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/1/9</t>
+          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/1/9，2026/3/7</t>
         </is>
       </c>
       <c r="F580" t="inlineStr"/>
@@ -22514,10 +22518,14 @@
       </c>
       <c r="H580" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I580" t="inlineStr"/>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>BV1PNNAzLEvL</t>
+        </is>
+      </c>
       <c r="J580" t="inlineStr"/>
     </row>
     <row r="581">
@@ -22835,7 +22843,7 @@
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>2025/07/15，2026/1/5，2026/1/10，2026/1/25，2026/2/10，2026/2/27</t>
+          <t>2025/07/15，2026/1/5，2026/1/10，2026/1/25，2026/2/10，2026/2/27，2026/3/7</t>
         </is>
       </c>
       <c r="F589" t="inlineStr"/>
@@ -22846,7 +22854,7 @@
       </c>
       <c r="H589" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I589" t="inlineStr">
@@ -26207,7 +26215,7 @@
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/6，2026/1/15，2026/1/19</t>
+          <t>2025/09/29，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/6，2026/1/15，2026/1/19，2026/3/7</t>
         </is>
       </c>
       <c r="F679" t="inlineStr"/>
@@ -26218,7 +26226,7 @@
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I679" t="inlineStr">
@@ -28619,7 +28627,7 @@
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>2025/11/26</t>
+          <t>2025/11/26，2026/3/7</t>
         </is>
       </c>
       <c r="F744" t="inlineStr"/>
@@ -28630,10 +28638,14 @@
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I744" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>BV1zDUzBaENk</t>
+        </is>
+      </c>
       <c r="J744" t="inlineStr"/>
     </row>
     <row r="745">
@@ -30583,7 +30595,7 @@
       </c>
       <c r="E796" t="inlineStr">
         <is>
-          <t>2026/2/14，2026/2/24</t>
+          <t>2026/2/14，2026/2/24，2026/3/7</t>
         </is>
       </c>
       <c r="F796" t="inlineStr"/>
@@ -30594,7 +30606,7 @@
       </c>
       <c r="H796" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I796" t="inlineStr">
@@ -31227,6 +31239,70 @@
       </c>
       <c r="I813" t="inlineStr"/>
       <c r="J813" t="inlineStr"/>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr"/>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>AS IF IT'S YOUR LAST</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr"/>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>BLACKPINK</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>2026/3/7</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr"/>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>韩语</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr"/>
+      <c r="J814" t="inlineStr"/>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr"/>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>天下</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr"/>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>张杰</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>2026/3/7</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr"/>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr"/>
+      <c r="J815" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 7, 2026 v2
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -9499,7 +9499,7 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>BV1crarzEEsn</t>
+          <t>BV1r3NAzgErm，BV1crarzEEsn</t>
         </is>
       </c>
       <c r="J233" t="inlineStr"/>
@@ -21501,7 +21501,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I552" t="inlineStr"/>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>BV163NAzgEyz</t>
+        </is>
+      </c>
       <c r="J552" t="inlineStr"/>
     </row>
     <row r="553">
@@ -31206,7 +31210,11 @@
           <t>BV13z2yBtEb1</t>
         </is>
       </c>
-      <c r="J812" t="inlineStr"/>
+      <c r="J812" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="813">
       <c r="A813" t="inlineStr"/>
@@ -31247,7 +31255,11 @@
           <t>AS IF IT'S YOUR LAST</t>
         </is>
       </c>
-      <c r="C814" t="inlineStr"/>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>像最后一样</t>
+        </is>
+      </c>
       <c r="D814" t="inlineStr">
         <is>
           <t>BLACKPINK</t>
@@ -31269,7 +31281,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I814" t="inlineStr"/>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>BV1q7NAzKES6</t>
+        </is>
+      </c>
       <c r="J814" t="inlineStr"/>
     </row>
     <row r="815">
@@ -31301,7 +31317,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I815" t="inlineStr"/>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>BV1zLNAzqEVL</t>
+        </is>
+      </c>
       <c r="J815" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: Update song list to Mar 8, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/21，2025/04/05，2025/04/14，2025/04/24，2025/05/20，2025/06/05，2025/06/17，2025/06/23，2025/06/26，2025/08/12，2025/08/21，2025/09/14，2025/09/24，2025/10/16，2025/10/24，2025/12/17，2026/2/14</t>
+          <t>2025/03/04，2025/03/21，2025/04/05，2025/04/14，2025/04/24，2025/05/20，2025/06/05，2025/06/17，2025/06/23，2025/06/26，2025/08/12，2025/08/21，2025/09/14，2025/09/24，2025/10/16，2025/10/24，2025/12/17，2026/2/14，2026/3/8</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2025/03/07</t>
+          <t>2025/03/07，2026/3/8</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23</t>
+          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>爱你</t>
+          <t>爱你（把我们衣服纽扣互扣）</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/06，2025/04/11，2025/04/29，2025/06/09，2025/09/26，2025/11/22</t>
+          <t>2025/03/14，2025/04/06，2025/04/11，2025/04/29，2025/06/09，2025/09/26，2025/11/22，2026/3/8</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -9043,7 +9043,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/25</t>
+          <t>2025/03/28，2025/05/25，2026/3/8</t>
         </is>
       </c>
       <c r="F221" t="inlineStr"/>
@@ -9054,10 +9054,14 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I221" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>BV11bKWzGEza</t>
+        </is>
+      </c>
       <c r="J221" t="inlineStr"/>
     </row>
     <row r="222">
@@ -10071,7 +10075,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/1/1，2026/1/25</t>
+          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/1/1，2026/1/25，2026/3/8</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
@@ -10082,7 +10086,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -10375,7 +10379,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10386,7 +10390,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -20495,7 +20499,7 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>2025/06/17，2025/09/12</t>
+          <t>2025/06/17，2025/09/12，2026/3/8</t>
         </is>
       </c>
       <c r="F526" t="inlineStr"/>
@@ -20506,10 +20510,14 @@
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I526" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>BV1HcN6zkEPV</t>
+        </is>
+      </c>
       <c r="J526" t="inlineStr"/>
     </row>
     <row r="527">
@@ -20611,7 +20619,7 @@
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/09/02</t>
+          <t>2025/06/19，2025/09/02，2026/3/8</t>
         </is>
       </c>
       <c r="F529" t="inlineStr"/>
@@ -20622,7 +20630,7 @@
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I529" t="inlineStr"/>
@@ -21327,7 +21335,7 @@
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28</t>
+          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/3/8</t>
         </is>
       </c>
       <c r="F548" t="inlineStr"/>
@@ -21338,10 +21346,14 @@
       </c>
       <c r="H548" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I548" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>BV1dgy9BnEVC</t>
+        </is>
+      </c>
       <c r="J548" t="inlineStr"/>
     </row>
     <row r="549">
@@ -22511,7 +22523,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/1/9，2026/3/7</t>
+          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/1/9，2026/3/7，2026/3/8</t>
         </is>
       </c>
       <c r="F580" t="inlineStr"/>
@@ -22522,7 +22534,7 @@
       </c>
       <c r="H580" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I580" t="inlineStr">
@@ -22735,7 +22747,7 @@
       </c>
       <c r="E586" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/09/05，2025/11/9</t>
+          <t>2025/07/14，2025/09/05，2025/11/9，2026/3/8</t>
         </is>
       </c>
       <c r="F586" t="inlineStr"/>
@@ -22746,10 +22758,14 @@
       </c>
       <c r="H586" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I586" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>BV1wJahzXEz4</t>
+        </is>
+      </c>
       <c r="J586" t="inlineStr"/>
     </row>
     <row r="587">
@@ -25543,7 +25559,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8</t>
         </is>
       </c>
       <c r="F661" t="inlineStr"/>
@@ -25554,7 +25570,7 @@
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
@@ -25583,7 +25599,7 @@
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>2025/09/22，2025/10/09，2025/12/5，2026/1/25</t>
+          <t>2025/09/22，2025/10/09，2025/12/5，2026/1/25，2026/3/8</t>
         </is>
       </c>
       <c r="F662" t="inlineStr"/>
@@ -25594,7 +25610,7 @@
       </c>
       <c r="H662" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I662" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 9, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J815"/>
+  <dimension ref="A1:J816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05</t>
+          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/3/9</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2561,7 +2561,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>BV1e1NVzoExD</t>
+        </is>
+      </c>
       <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2931,7 +2935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2942,7 +2946,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4475,7 +4479,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/9，2025/11/22</t>
+          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/9，2025/11/22，2026/3/9</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -4486,10 +4490,14 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>BV1qLpgzaEQ5，BV1k2T1zPEcd</t>
+        </is>
+      </c>
       <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
@@ -6823,7 +6831,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -6834,7 +6842,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7450,7 +7458,7 @@
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Sān-Z/HOYO-MiX</t>
+          <t>Sān-Z/HOYO-MiX/于梓贝</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -7470,7 +7478,11 @@
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" t="inlineStr"/>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7491,7 +7503,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7502,10 +7514,14 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr"/>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>BV17HP9zkE69</t>
+        </is>
+      </c>
       <c r="J180" t="inlineStr"/>
     </row>
     <row r="181">
@@ -8387,7 +8403,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/20，2025/06/01，2025/07/15，2025/09/27，2025/10/03</t>
+          <t>2025/03/25，2025/05/20，2025/06/01，2025/07/15，2025/09/27，2025/10/03，2026/3/9</t>
         </is>
       </c>
       <c r="F204" t="inlineStr"/>
@@ -8398,10 +8414,14 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I204" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>BV13dPXz8ELA</t>
+        </is>
+      </c>
       <c r="J204" t="inlineStr"/>
     </row>
     <row r="205">
@@ -8531,7 +8551,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/2/14，2026/2/23，2026/2/25</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/2/14，2026/2/23，2026/2/25，2026/3/9</t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
@@ -8542,7 +8562,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -9307,7 +9327,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/7，2025/11/24，2025/12/5，2026/1/23</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/7，2025/11/24，2025/12/5，2026/1/23，2026/3/9</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9318,10 +9338,14 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="I228" t="inlineStr"/>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>BV1GRPXzcE32，BV171egzwEks</t>
+        </is>
+      </c>
       <c r="J228" t="inlineStr"/>
     </row>
     <row r="229">
@@ -11040,10 +11064,14 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>나는 아픈 건 딱 질색이니까 (Fate)</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr"/>
+          <t>나는 아픈 건 딱 질색이니까</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Fate/因为我无法忍受痛苦</t>
+        </is>
+      </c>
       <c r="D274" t="inlineStr">
         <is>
           <t>(G)I-DLE</t>
@@ -11051,7 +11079,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11062,10 +11090,14 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I274" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>BV1ZnP9zGECv</t>
+        </is>
+      </c>
       <c r="J274" t="inlineStr"/>
     </row>
     <row r="275">
@@ -12123,7 +12155,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22</t>
+          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/3/9</t>
         </is>
       </c>
       <c r="F303" t="inlineStr"/>
@@ -12134,10 +12166,14 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I303" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>BV1CAVDz8EwC</t>
+        </is>
+      </c>
       <c r="J303" t="inlineStr"/>
     </row>
     <row r="304">
@@ -12891,7 +12927,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -12902,7 +12938,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -13371,7 +13407,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13382,7 +13418,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -15767,7 +15803,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/23，2025/10/09，2026/1/22</t>
+          <t>2025/04/25，2025/06/23，2025/10/09，2026/1/22，2026/3/9</t>
         </is>
       </c>
       <c r="F399" t="inlineStr"/>
@@ -15778,10 +15814,14 @@
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I399" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>BV1WbKhzxEhK</t>
+        </is>
+      </c>
       <c r="J399" t="inlineStr"/>
     </row>
     <row r="400">
@@ -17399,7 +17439,7 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/27，2025/07/10</t>
+          <t>2025/05/18，2025/06/27，2025/07/10，2026/3/9</t>
         </is>
       </c>
       <c r="F443" t="inlineStr"/>
@@ -17410,10 +17450,14 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I443" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>BV14JJVz1EKo</t>
+        </is>
+      </c>
       <c r="J443" t="inlineStr"/>
     </row>
     <row r="444">
@@ -20633,7 +20677,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I529" t="inlineStr"/>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>BV1eyNVztEz8</t>
+        </is>
+      </c>
       <c r="J529" t="inlineStr"/>
     </row>
     <row r="530">
@@ -20919,7 +20967,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -20930,7 +20978,7 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
@@ -22043,7 +22091,7 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25</t>
+          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9</t>
         </is>
       </c>
       <c r="F567" t="inlineStr"/>
@@ -22054,7 +22102,7 @@
       </c>
       <c r="H567" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I567" t="inlineStr">
@@ -22539,7 +22587,7 @@
       </c>
       <c r="I580" t="inlineStr">
         <is>
-          <t>BV1PNNAzLEvL</t>
+          <t>BV1PNNAzLEvL，BV1bRNVzDETM</t>
         </is>
       </c>
       <c r="J580" t="inlineStr"/>
@@ -26347,7 +26395,7 @@
       </c>
       <c r="E682" t="inlineStr">
         <is>
-          <t>2025/09/30，2025/10/16</t>
+          <t>2025/09/30，2025/10/16，2026/3/9</t>
         </is>
       </c>
       <c r="F682" t="inlineStr"/>
@@ -26358,10 +26406,14 @@
       </c>
       <c r="H682" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I682" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>BV1V6WizNEa5</t>
+        </is>
+      </c>
       <c r="J682" t="inlineStr"/>
     </row>
     <row r="683">
@@ -29639,7 +29691,7 @@
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9</t>
         </is>
       </c>
       <c r="F770" t="inlineStr"/>
@@ -29650,7 +29702,7 @@
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I770" t="inlineStr">
@@ -29791,7 +29843,7 @@
       </c>
       <c r="E774" t="inlineStr">
         <is>
-          <t>2026/1/14</t>
+          <t>2026/1/14，2026/3/9</t>
         </is>
       </c>
       <c r="F774" t="inlineStr"/>
@@ -29802,7 +29854,7 @@
       </c>
       <c r="H774" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I774" t="inlineStr">
@@ -30539,7 +30591,7 @@
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>2026/2/9，2026/2/27</t>
+          <t>2026/2/9，2026/2/27，2026/3/9</t>
         </is>
       </c>
       <c r="F794" t="inlineStr"/>
@@ -30550,7 +30602,7 @@
       </c>
       <c r="H794" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I794" t="inlineStr">
@@ -31339,6 +31391,42 @@
         </is>
       </c>
       <c r="J815" t="inlineStr"/>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr"/>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>多幸运</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr"/>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>韩安旭</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>2026/3/9</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr"/>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>BV1fEP9zCEL8</t>
+        </is>
+      </c>
+      <c r="J816" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 12, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -2079,7 +2079,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/04，2025/04/18，2025/04/25，2025/05/01，2025/05/25，2025/06/02，2025/06/06，2025/12/26，2026/1/21</t>
+          <t>2025/03/21，2025/04/04，2025/04/18，2025/04/25，2025/05/01，2025/05/25，2025/06/02，2025/06/06，2025/12/26，2026/1/21，2026/3/12</t>
         </is>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -7474,7 +7474,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1</t>
+          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12</t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -10995,7 +10995,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/1/23，2026/2/18</t>
+          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/1/23，2026/2/18，2026/3/12</t>
         </is>
       </c>
       <c r="F272" t="inlineStr"/>
@@ -11006,7 +11006,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -17410,7 +17410,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -29691,7 +29691,7 @@
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12</t>
         </is>
       </c>
       <c r="F770" t="inlineStr"/>
@@ -29702,7 +29702,7 @@
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I770" t="inlineStr">
@@ -30103,7 +30103,7 @@
       </c>
       <c r="E781" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12</t>
         </is>
       </c>
       <c r="F781" t="inlineStr"/>
@@ -30114,7 +30114,7 @@
       </c>
       <c r="H781" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I781" t="inlineStr">
@@ -30267,7 +30267,7 @@
       </c>
       <c r="E785" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25</t>
+          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12</t>
         </is>
       </c>
       <c r="F785" t="inlineStr"/>
@@ -30278,7 +30278,7 @@
       </c>
       <c r="H785" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I785" t="inlineStr">
@@ -30551,7 +30551,7 @@
       </c>
       <c r="E793" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12</t>
         </is>
       </c>
       <c r="F793" t="inlineStr"/>
@@ -30562,7 +30562,7 @@
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
@@ -31107,7 +31107,7 @@
       </c>
       <c r="E808" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12</t>
         </is>
       </c>
       <c r="F808" t="inlineStr"/>
@@ -31118,7 +31118,7 @@
       </c>
       <c r="H808" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I808" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 13, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J816"/>
+  <dimension ref="A1:J819"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,7 +963,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/4，2026/1/24，2026/1/24，2026/2/19，2026/2/25</t>
+          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/4，2026/1/24，2026/1/24，2026/2/19，2026/2/25，2026/3/13</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/03，2025/04/17，2025/05/22，2025/06/03，2025/07/24，2025/08/12，2025/09/03，2025/10/10，2025/11/9，2025/11/10</t>
+          <t>2025/03/04，2025/04/03，2025/04/17，2025/05/22，2025/06/03，2025/07/24，2025/08/12，2025/09/03，2025/10/10，2025/11/9，2025/11/10，2026/3/13</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/15，2025/06/30，2025/08/13，2025/10/25</t>
+          <t>2025/03/14，2025/05/15，2025/06/30，2025/08/13，2025/10/25，2026/3/13</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -4798,10 +4798,14 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>BV1RmEnz1ETY</t>
+        </is>
+      </c>
       <c r="J109" t="inlineStr"/>
     </row>
     <row r="110">
@@ -5939,7 +5943,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -5950,7 +5954,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6247,7 +6251,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6258,7 +6262,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6635,7 +6639,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6646,7 +6650,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -7387,7 +7391,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7398,7 +7402,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -7477,7 +7481,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I179" t="inlineStr"/>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>BV1jGjGzDE4g</t>
+        </is>
+      </c>
       <c r="J179" t="inlineStr">
         <is>
           <t>游戏</t>
@@ -9063,7 +9071,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/25，2026/3/8</t>
+          <t>2025/03/28，2025/05/25，2026/3/8，2026/3/13</t>
         </is>
       </c>
       <c r="F221" t="inlineStr"/>
@@ -9074,7 +9082,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -10403,7 +10411,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10414,7 +10422,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -11079,7 +11087,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11090,7 +11098,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -11527,7 +11535,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/06/26</t>
+          <t>2025/04/04，2025/06/26，2026/3/13</t>
         </is>
       </c>
       <c r="F286" t="inlineStr"/>
@@ -11538,10 +11546,14 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I286" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>BV1W7KfzqEwh</t>
+        </is>
+      </c>
       <c r="J286" t="inlineStr"/>
     </row>
     <row r="287">
@@ -12387,7 +12399,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12398,7 +12410,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -14027,7 +14039,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/21，2025/05/08，2025/06/10，2025/06/28，2025/07/08，2025/08/22，2025/09/11，2025/10/25</t>
+          <t>2025/04/17，2025/04/21，2025/05/08，2025/06/10，2025/06/28，2025/07/08，2025/08/22，2025/09/11，2025/10/25，2026/3/13</t>
         </is>
       </c>
       <c r="F352" t="inlineStr"/>
@@ -14038,10 +14050,14 @@
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="I352" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>BV1FdMgzNEUo</t>
+        </is>
+      </c>
       <c r="J352" t="inlineStr"/>
     </row>
     <row r="353">
@@ -15071,7 +15087,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>2025/04/22，2025/04/29，2025/05/03，2025/05/03，2025/06/03，2025/09/02，2025/10/10，2025/10/20，2025/10/31，2026/2/7</t>
+          <t>2025/04/22，2025/04/29，2025/05/03，2025/05/03，2025/06/03，2025/09/02，2025/10/10，2025/10/20，2025/10/31，2026/2/7，2026/3/13</t>
         </is>
       </c>
       <c r="F379" t="inlineStr"/>
@@ -15082,7 +15098,7 @@
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I379" t="inlineStr">
@@ -18563,7 +18579,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13</t>
         </is>
       </c>
       <c r="F473" t="inlineStr"/>
@@ -18574,7 +18590,7 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
@@ -23851,7 +23867,7 @@
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>2025/08/09</t>
+          <t>2025/08/09，2026/3/13</t>
         </is>
       </c>
       <c r="F614" t="inlineStr">
@@ -23866,10 +23882,14 @@
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I614" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>BV1BSt8zzESY</t>
+        </is>
+      </c>
       <c r="J614" t="inlineStr"/>
     </row>
     <row r="615">
@@ -24307,7 +24327,7 @@
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>2025/09/04</t>
+          <t>2025/09/04，2026/3/13</t>
         </is>
       </c>
       <c r="F626" t="inlineStr"/>
@@ -24318,10 +24338,14 @@
       </c>
       <c r="H626" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I626" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>BV1rqwJz2Ejp</t>
+        </is>
+      </c>
       <c r="J626" t="inlineStr"/>
     </row>
     <row r="627">
@@ -25123,7 +25147,7 @@
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/09/15，2025/09/22，2025/09/29，2025/09/29，2025/10/10，2025/10/28，2025/12/2，2026/1/5</t>
+          <t>2025/09/17，2025/09/15，2025/09/22，2025/09/29，2025/09/29，2025/10/10，2025/10/28，2025/12/2，2026/1/5，2026/3/13</t>
         </is>
       </c>
       <c r="F648" t="inlineStr"/>
@@ -25134,10 +25158,14 @@
       </c>
       <c r="H648" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="I648" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>BV1SFnwzXEzi</t>
+        </is>
+      </c>
       <c r="J648" t="inlineStr"/>
     </row>
     <row r="649">
@@ -25311,7 +25339,7 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>2025/09/15</t>
+          <t>2025/09/15，2026/3/13</t>
         </is>
       </c>
       <c r="F653" t="inlineStr"/>
@@ -25322,10 +25350,14 @@
       </c>
       <c r="H653" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I653" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>BV1xbpBz4E2N</t>
+        </is>
+      </c>
       <c r="J653" t="inlineStr"/>
     </row>
     <row r="654">
@@ -29567,7 +29599,7 @@
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/1/2，2026/1/10</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/1/2，2026/1/10，2026/3/13</t>
         </is>
       </c>
       <c r="F767" t="inlineStr"/>
@@ -29578,7 +29610,7 @@
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
@@ -30667,7 +30699,7 @@
       </c>
       <c r="E796" t="inlineStr">
         <is>
-          <t>2026/2/14，2026/2/24，2026/3/7</t>
+          <t>2026/2/14，2026/2/24，2026/3/7，2026/3/13</t>
         </is>
       </c>
       <c r="F796" t="inlineStr"/>
@@ -30678,7 +30710,7 @@
       </c>
       <c r="H796" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I796" t="inlineStr">
@@ -31427,6 +31459,110 @@
         </is>
       </c>
       <c r="J816" t="inlineStr"/>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr"/>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>靛青宇宙</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr"/>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/飞行雪绒</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>2026/3/13</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr"/>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr"/>
+      <c r="J817" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr"/>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>銀の龍の背に乗って</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>骑在银龙的背上</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>中岛美雪</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>2026/3/13</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr"/>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr"/>
+      <c r="J818" t="inlineStr"/>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr"/>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>啊！美丽卡洛</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr"/>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>ChiliChill</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>2026/3/13</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr"/>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr"/>
+      <c r="J819" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 13, 2026, v2
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -4991,7 +4991,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5002,12 +5002,12 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>BV1b1KmzUE9y</t>
+          <t>BV1b1KmzUE9y，BV1Qgw4z7ES1</t>
         </is>
       </c>
       <c r="J114" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 14, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J819"/>
+  <dimension ref="A1:J821"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/7，2025/12/24，2026/1/1，2026/1/16</t>
+          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/7，2025/12/24，2026/1/1，2026/1/16，2026/3/14</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/1/14，2026/2/19</t>
+          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/1/14，2026/2/19，2026/3/14</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7</t>
+          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7，2026/3/14</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13，2026/3/14</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7402,7 +7402,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -15163,7 +15163,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>2025/04/24，2025/05/12，2025/12/11，2026/1/24</t>
+          <t>2025/04/24，2025/05/12，2025/12/11，2026/1/24，2026/3/14</t>
         </is>
       </c>
       <c r="F381" t="inlineStr"/>
@@ -15174,10 +15174,14 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I381" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>BV1WdLzzGEtB</t>
+        </is>
+      </c>
       <c r="J381" t="inlineStr"/>
     </row>
     <row r="382">
@@ -19559,7 +19563,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/07/03，2025/10/09，2026/1/16，2026/3/6</t>
+          <t>2025/06/02，2025/07/03，2025/10/09，2026/1/16，2026/3/6，2026/3/14</t>
         </is>
       </c>
       <c r="F499" t="inlineStr"/>
@@ -19570,7 +19574,7 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
@@ -21355,7 +21359,7 @@
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13</t>
         </is>
       </c>
       <c r="F547" t="inlineStr"/>
@@ -21366,7 +21370,7 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -23679,7 +23683,7 @@
       </c>
       <c r="E609" t="inlineStr">
         <is>
-          <t>2025/08/02，2025/12/2</t>
+          <t>2025/08/02，2025/12/2，2026/3/14</t>
         </is>
       </c>
       <c r="F609" t="inlineStr"/>
@@ -23690,10 +23694,14 @@
       </c>
       <c r="H609" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I609" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>BV1NmSbBmEkm</t>
+        </is>
+      </c>
       <c r="J609" t="inlineStr"/>
     </row>
     <row r="610">
@@ -25899,7 +25907,7 @@
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/7，2025/11/26，2025/12/6，2025/12/12，2025/12/24，2026/1/5，2026/1/19，2026/2/18</t>
+          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/7，2025/11/26，2025/12/6，2025/12/12，2025/12/24，2026/1/5，2026/1/19，2026/2/18，2026/3/14</t>
         </is>
       </c>
       <c r="F668" t="inlineStr"/>
@@ -25910,7 +25918,7 @@
       </c>
       <c r="H668" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I668" t="inlineStr">
@@ -25939,7 +25947,7 @@
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/26</t>
+          <t>2025/09/24，2025/09/26，2026/3/14</t>
         </is>
       </c>
       <c r="F669" t="inlineStr"/>
@@ -25950,7 +25958,7 @@
       </c>
       <c r="H669" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I669" t="inlineStr"/>
@@ -27651,7 +27659,7 @@
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/1，2025/11/12，2025/11/26，2025/12/8，2026/1/2，2026/1/5，2026/1/9，2026/2/23</t>
+          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/1，2025/11/12，2025/11/26，2025/12/8，2026/1/2，2026/1/5，2026/1/9，2026/2/23，2026/3/14</t>
         </is>
       </c>
       <c r="F715" t="inlineStr"/>
@@ -27662,7 +27670,7 @@
       </c>
       <c r="H715" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I715" t="inlineStr">
@@ -28771,7 +28779,7 @@
       </c>
       <c r="E745" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14</t>
         </is>
       </c>
       <c r="F745" t="inlineStr"/>
@@ -28782,7 +28790,7 @@
       </c>
       <c r="H745" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I745" t="inlineStr">
@@ -29723,7 +29731,7 @@
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14</t>
         </is>
       </c>
       <c r="F770" t="inlineStr"/>
@@ -29734,7 +29742,7 @@
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I770" t="inlineStr">
@@ -30951,7 +30959,7 @@
       </c>
       <c r="E803" t="inlineStr">
         <is>
-          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25</t>
+          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25，2026/3/14</t>
         </is>
       </c>
       <c r="F803" t="inlineStr"/>
@@ -30962,7 +30970,7 @@
       </c>
       <c r="H803" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I803" t="inlineStr">
@@ -31547,7 +31555,7 @@
       </c>
       <c r="E819" t="inlineStr">
         <is>
-          <t>2026/3/13</t>
+          <t>2026/3/13，2026/3/14</t>
         </is>
       </c>
       <c r="F819" t="inlineStr"/>
@@ -31558,11 +31566,75 @@
       </c>
       <c r="H819" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I819" t="inlineStr"/>
       <c r="J819" t="inlineStr"/>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr"/>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>十年</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr"/>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>陈奕迅</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>2026/3/14</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr"/>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr"/>
+      <c r="J820" t="inlineStr"/>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr"/>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Yesterday Once More</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr"/>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Carpenters</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>2026/3/14</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr"/>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr"/>
+      <c r="J821" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 15, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J821"/>
+  <dimension ref="A1:J823"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,7 +583,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7</t>
+          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7，2026/3/15</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -594,7 +594,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28</t>
+          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/3/15</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/1/12，2026/2/7</t>
+          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/1/12，2026/2/7，2026/3/15</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -6599,7 +6599,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/22，2025/05/29，2025/06/03，2025/08/28，2025/09/11，2025/10/18，2025/10/30，2025/11/28，2025/12/28</t>
+          <t>2025/03/20，2025/05/22，2025/05/29，2025/06/03，2025/08/28，2025/09/11，2025/10/18，2025/10/30，2025/11/28，2025/12/28，2026/3/15</t>
         </is>
       </c>
       <c r="F156" t="inlineStr"/>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7326,12 +7326,12 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>BV1v84TzcEMv</t>
+          <t>BV1Rqw3zCEFo，BV1v84TzcEMv</t>
         </is>
       </c>
       <c r="J175" t="inlineStr"/>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/2/14，2026/2/23，2026/2/25，2026/3/9</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/2/14，2026/2/23，2026/2/25，2026/3/9，2026/3/15</t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
@@ -8570,7 +8570,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -9643,7 +9643,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -9654,12 +9654,12 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>BV1XWWNzyE2d</t>
+          <t>BV1Xkw3zgEHg，BV1XWWNzyE2d</t>
         </is>
       </c>
       <c r="J236" t="inlineStr"/>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/24，2025/05/15，2025/05/29，2025/09/21，2025/09/27，2025/10/24，2026/1/5，2026/2/9</t>
+          <t>2025/03/30，2025/04/24，2025/05/15，2025/05/29，2025/09/21，2025/09/27，2025/10/24，2026/1/5，2026/2/9，2026/3/15</t>
         </is>
       </c>
       <c r="F244" t="inlineStr"/>
@@ -9962,12 +9962,12 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>BV1a7E1zVEhr</t>
+          <t>BV1Q1w3zMEAZ，BV1a7E1zVEhr</t>
         </is>
       </c>
       <c r="J244" t="inlineStr"/>
@@ -20795,7 +20795,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15</t>
         </is>
       </c>
       <c r="F532" t="inlineStr"/>
@@ -20806,7 +20806,7 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
@@ -22931,7 +22931,7 @@
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>2025/07/15，2026/1/5，2026/1/10，2026/1/25，2026/2/10，2026/2/27，2026/3/7</t>
+          <t>2025/07/15，2026/1/5，2026/1/10，2026/1/25，2026/2/10，2026/2/27，2026/3/7，2026/3/15</t>
         </is>
       </c>
       <c r="F589" t="inlineStr"/>
@@ -22942,7 +22942,7 @@
       </c>
       <c r="H589" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I589" t="inlineStr">
@@ -26931,7 +26931,7 @@
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>2025/10/13，2025/10/18</t>
+          <t>2025/10/13，2025/10/18，2026/3/15</t>
         </is>
       </c>
       <c r="F695" t="inlineStr"/>
@@ -26942,10 +26942,14 @@
       </c>
       <c r="H695" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I695" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>BV1wiwMzUEKR</t>
+        </is>
+      </c>
       <c r="J695" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -31635,6 +31639,74 @@
       </c>
       <c r="I821" t="inlineStr"/>
       <c r="J821" t="inlineStr"/>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr"/>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>给你呀</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>for ya</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>蒋小呢</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>2026/3/15</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr"/>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr"/>
+      <c r="J822" t="inlineStr"/>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr"/>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Believer</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr"/>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Imagine Dragons</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>2026/3/15</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr"/>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr"/>
+      <c r="J823" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 17, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J823"/>
+  <dimension ref="A1:J828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -759,7 +759,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -770,7 +770,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7，2026/3/17</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7，2026/3/17</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7674,7 +7674,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -10523,7 +10523,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8</t>
+          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
@@ -10534,7 +10534,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -11087,7 +11087,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13，2026/3/17</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11098,7 +11098,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -13639,7 +13639,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/23，2025/06/06，2025/08/28，2025/09/05，2025/12/6</t>
+          <t>2025/04/13，2025/05/23，2025/06/06，2025/08/28，2025/09/05，2025/12/6，2026/3/17</t>
         </is>
       </c>
       <c r="F341" t="inlineStr"/>
@@ -13650,10 +13650,14 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I341" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>BV1QywoziEyC</t>
+        </is>
+      </c>
       <c r="J341" t="inlineStr"/>
     </row>
     <row r="342">
@@ -14119,7 +14123,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/06/01，2025/08/18，2026/3/6</t>
+          <t>2025/04/17，2025/06/01，2025/08/18，2026/3/6，2026/3/17</t>
         </is>
       </c>
       <c r="F354" t="inlineStr"/>
@@ -14130,7 +14134,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
@@ -17647,7 +17651,7 @@
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/1/2</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/1/2，2026/3/17</t>
         </is>
       </c>
       <c r="F448" t="inlineStr"/>
@@ -17658,7 +17662,7 @@
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I448" t="inlineStr">
@@ -18099,7 +18103,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2026/2/2</t>
+          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2026/2/2，2026/3/17</t>
         </is>
       </c>
       <c r="F460" t="inlineStr"/>
@@ -18110,7 +18114,7 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
@@ -19523,7 +19527,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5</t>
+          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5，2026/3/17</t>
         </is>
       </c>
       <c r="F498" t="inlineStr"/>
@@ -19534,7 +19538,7 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
@@ -20683,7 +20687,7 @@
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/09/02，2026/3/8</t>
+          <t>2025/06/19，2025/09/02，2026/3/8，2026/3/17</t>
         </is>
       </c>
       <c r="F529" t="inlineStr"/>
@@ -20694,7 +20698,7 @@
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
@@ -22631,7 +22635,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/09/30，2025/10/31，2025/12/4，2026/1/23，2026/2/12</t>
+          <t>2025/07/11，2025/09/30，2025/10/31，2025/12/4，2026/1/23，2026/2/12，2026/3/17</t>
         </is>
       </c>
       <c r="F581" t="inlineStr"/>
@@ -22642,7 +22646,7 @@
       </c>
       <c r="H581" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I581" t="inlineStr">
@@ -23995,7 +23999,7 @@
       </c>
       <c r="E617" t="inlineStr">
         <is>
-          <t>2025/08/21，2026/1/16，2026/2/2</t>
+          <t>2025/08/21，2026/1/16，2026/2/2，2026/3/17</t>
         </is>
       </c>
       <c r="F617" t="inlineStr"/>
@@ -24006,10 +24010,14 @@
       </c>
       <c r="H617" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I617" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>BV1QwwRz4E3D</t>
+        </is>
+      </c>
       <c r="J617" t="inlineStr"/>
     </row>
     <row r="618">
@@ -25195,7 +25203,7 @@
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/2/23</t>
+          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/2/23，2026/3/17</t>
         </is>
       </c>
       <c r="F649" t="inlineStr"/>
@@ -25206,7 +25214,7 @@
       </c>
       <c r="H649" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I649" t="inlineStr">
@@ -29735,7 +29743,7 @@
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17</t>
         </is>
       </c>
       <c r="F770" t="inlineStr"/>
@@ -29746,7 +29754,7 @@
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I770" t="inlineStr">
@@ -30595,7 +30603,7 @@
       </c>
       <c r="E793" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17</t>
         </is>
       </c>
       <c r="F793" t="inlineStr"/>
@@ -30606,7 +30614,7 @@
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
@@ -31591,7 +31599,7 @@
       </c>
       <c r="E820" t="inlineStr">
         <is>
-          <t>2026/3/14</t>
+          <t>2026/3/14，2026/3/17</t>
         </is>
       </c>
       <c r="F820" t="inlineStr"/>
@@ -31602,7 +31610,7 @@
       </c>
       <c r="H820" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I820" t="inlineStr"/>
@@ -31659,7 +31667,7 @@
       </c>
       <c r="E822" t="inlineStr">
         <is>
-          <t>2026/3/15</t>
+          <t>2026/3/15，2026/3/17</t>
         </is>
       </c>
       <c r="F822" t="inlineStr"/>
@@ -31670,11 +31678,15 @@
       </c>
       <c r="H822" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I822" t="inlineStr"/>
-      <c r="J822" t="inlineStr"/>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr"/>
@@ -31707,6 +31719,174 @@
       </c>
       <c r="I823" t="inlineStr"/>
       <c r="J823" t="inlineStr"/>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr"/>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>句号</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr"/>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>G.E.M. 邓紫棋</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>2026/3/17</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr"/>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr"/>
+      <c r="J824" t="inlineStr"/>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr"/>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>相思</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr"/>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>毛阿敏</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>2026/3/17</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr"/>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>BV1dXw9zYEn4</t>
+        </is>
+      </c>
+      <c r="J825" t="inlineStr"/>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr"/>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>若梦</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr"/>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>周深</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>2026/3/17</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr"/>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr"/>
+      <c r="J826" t="inlineStr"/>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr"/>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>唐·毒蛇</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr"/>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Bsh-1</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>2026/3/17</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr"/>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr"/>
+      <c r="J827" t="inlineStr"/>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr"/>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>小小奇迹</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr"/>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/jixwang/飞行雪绒</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>2026/3/17，2026/3/17</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr"/>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr"/>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 18, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -2017,7 +2017,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>BV1k7WpzkEsj，BV1xdGRz2E68</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2525,7 +2529,11 @@
           <t>16</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>BV1QWVzzjEmH，BV1BRSsBxEE7</t>
+        </is>
+      </c>
       <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2601,7 +2609,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>BV1B4j3zHEsq</t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2637,7 +2649,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>BV1UPWpzHE5C，BV1gAUfBKE3M</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
@@ -2713,7 +2729,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>BV1YHVDz7Ei4</t>
+        </is>
+      </c>
       <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2810,7 +2830,7 @@
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Kiss of Life/Mark Tuan</t>
+          <t>无畏契约/Kiss of Life/Mark Tuan</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2821,7 +2841,7 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>英语，韩语</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2829,8 +2849,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>BV1nAodYBEcN</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2935,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2946,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -2993,7 +3021,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>BV1PNMgzuEWm，BV1JdBCBEEPS</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
@@ -3153,7 +3185,11 @@
           <t>16</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>BV1GwX1Y9E9U，BV1b4Tuz3Eh1，BV1naVgzEEpG</t>
+        </is>
+      </c>
       <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -3229,7 +3265,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>BV1SrNtzdEsW，BV1hPJazzEeo</t>
+        </is>
+      </c>
       <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
@@ -3397,7 +3437,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>BV1WmT4zDE9V，BV11PLczYEDi</t>
+        </is>
+      </c>
       <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
@@ -3513,8 +3557,16 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>BV1fsnmzPEoD，BV1DDVQzjEMa</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3553,7 +3605,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>BV12pebzfEjf，BV1VjT8zzENA</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
@@ -3589,7 +3645,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>BV1JNVUzHEhw，BV1KttZztEWy，BV11qEPzEEP2</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
@@ -3625,7 +3685,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>BV19PGozFEg3，BV1GrkgBWEEt</t>
+        </is>
+      </c>
       <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
@@ -3957,7 +4021,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>BV14qQKYYEh8，BV1vbKozHEG3</t>
+        </is>
+      </c>
       <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
@@ -3993,7 +4061,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>BV1xv7rzHE88，BV1Roj2zmEn7，BV17oQKYSE76</t>
+        </is>
+      </c>
       <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
@@ -4149,7 +4221,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>BV1weQuYAEWL</t>
+        </is>
+      </c>
       <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
@@ -4185,7 +4261,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>BV1ryEPzCEag</t>
+        </is>
+      </c>
       <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
@@ -4327,7 +4407,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/2/10，2026/2/24</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/2/10，2026/2/24，2026/3/18</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4338,7 +4418,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -4421,7 +4501,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>BV1ynm3BsEbZ，BV1ZzQuYZEy2</t>
+        </is>
+      </c>
       <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
@@ -4457,7 +4541,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>BV14Bpgz2EkQ，BV18sTuzkEeX，BV1PtEnz8Edr</t>
+        </is>
+      </c>
       <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
@@ -4533,7 +4621,11 @@
           <t>13</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>BV1ujQuYyEDq，BV11WjQz1Etp</t>
+        </is>
+      </c>
       <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
@@ -4729,7 +4821,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>BV1XSobYHEvS，BV1ABKZzNETy</t>
+        </is>
+      </c>
       <c r="J107" t="inlineStr"/>
     </row>
     <row r="108">
@@ -4765,7 +4861,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>BV1SGCuB7EtQ</t>
+        </is>
+      </c>
       <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
@@ -4889,7 +4989,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>BV1uLQrYvEXC，BV1ZRCMBfEPY，BV1QtgozdEWF</t>
+        </is>
+      </c>
       <c r="J111" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -4969,7 +5073,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>BV1GMQrYgEZv，BV1F1JhzQEFY</t>
+        </is>
+      </c>
       <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
@@ -5045,7 +5153,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>BV1AtQrY4EzH，BV1fZyDBDEiJ</t>
+        </is>
+      </c>
       <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
@@ -5161,7 +5273,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
+        </is>
+      </c>
       <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
@@ -5197,7 +5313,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>BV1PHJizCEQj，BV1fTY4zMEw1，BV1HWrSBLE93</t>
+        </is>
+      </c>
       <c r="J119" t="inlineStr"/>
     </row>
     <row r="120">
@@ -5313,7 +5433,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>BV1aFjpzzEuJ</t>
+        </is>
+      </c>
       <c r="J122" t="inlineStr"/>
     </row>
     <row r="123">
@@ -5349,7 +5473,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>BV1fqQrYJEHd</t>
+        </is>
+      </c>
       <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
@@ -5385,7 +5513,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>BV1SwtfzPEQQ</t>
+        </is>
+      </c>
       <c r="J124" t="inlineStr"/>
     </row>
     <row r="125">
@@ -5461,7 +5593,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>BV1zTJHzdEvq，BV1ubQSYZEco</t>
+        </is>
+      </c>
       <c r="J126" t="inlineStr"/>
     </row>
     <row r="127">
@@ -5537,7 +5673,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>BV1f97Rz1EtK</t>
+        </is>
+      </c>
       <c r="J128" t="inlineStr"/>
     </row>
     <row r="129">
@@ -5693,7 +5833,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr"/>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>BV1NimyBWEr3，BV196X3YfEum</t>
+        </is>
+      </c>
       <c r="J132" t="inlineStr"/>
     </row>
     <row r="133">
@@ -5769,7 +5913,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>BV19SgWzYEEg，BV1NajHzfEyP</t>
+        </is>
+      </c>
       <c r="J134" t="inlineStr"/>
     </row>
     <row r="135">
@@ -5805,7 +5953,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>BV12DXuY5Ezm，BV1csJRzWE8o</t>
+        </is>
+      </c>
       <c r="J135" t="inlineStr"/>
     </row>
     <row r="136">
@@ -5881,7 +6033,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>BV1EAM4zyEh2，BV1QrXuYnEaL</t>
+        </is>
+      </c>
       <c r="J137" t="inlineStr"/>
     </row>
     <row r="138">
@@ -5997,7 +6153,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>BV1mJuKzKE7z，BV1quJJzmEe9</t>
+        </is>
+      </c>
       <c r="J140" t="inlineStr"/>
     </row>
     <row r="141">
@@ -6113,7 +6273,11 @@
           <t>13</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>BV1nnQdYtEur，BV18LNozTENV</t>
+        </is>
+      </c>
       <c r="J143" t="inlineStr"/>
     </row>
     <row r="144">
@@ -6149,7 +6313,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr"/>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>BV1n7QdY8Edw，BV18jM3zSE4Q</t>
+        </is>
+      </c>
       <c r="J144" t="inlineStr"/>
     </row>
     <row r="145">
@@ -6305,7 +6473,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>BV1mbHpz7Ern，BV1abpgzXEAM，BV1DbJGzSEQj</t>
+        </is>
+      </c>
       <c r="J148" t="inlineStr"/>
     </row>
     <row r="149">
@@ -6327,7 +6499,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/9</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6338,10 +6510,14 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr"/>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>BV19QnGzZE9f，BV1DZiFBgEhH，BV13rQZYQEem，BV1HD7VzqEQy，BV1UwSMBoE3e</t>
+        </is>
+      </c>
       <c r="J149" t="inlineStr"/>
     </row>
     <row r="150">
@@ -6377,7 +6553,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>BV1aApuzQEXg，BV136QZYpEx3</t>
+        </is>
+      </c>
       <c r="J150" t="inlineStr"/>
     </row>
     <row r="151">
@@ -6388,7 +6568,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>walkashame</t>
+          <t>Walkashame</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
@@ -6413,7 +6593,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>BV1PP7ez8EEn，BV1B8XCYoE5b</t>
+        </is>
+      </c>
       <c r="J151" t="inlineStr"/>
     </row>
     <row r="152">
@@ -6737,7 +6921,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="I159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>BV1N5EAzjEbT，BV1ePXiYhEsn</t>
+        </is>
+      </c>
       <c r="J159" t="inlineStr"/>
     </row>
     <row r="160">
@@ -6773,7 +6961,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr"/>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>BV18VXiYsEnd</t>
+        </is>
+      </c>
       <c r="J160" t="inlineStr"/>
     </row>
     <row r="161">
@@ -6889,7 +7081,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr"/>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>BV1xQKmzyEdm</t>
+        </is>
+      </c>
       <c r="J163" t="inlineStr"/>
     </row>
     <row r="164">
@@ -6925,7 +7121,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>BV1TWY1zgE8f，BV1b2MtzPEBw</t>
+        </is>
+      </c>
       <c r="J164" t="inlineStr"/>
     </row>
     <row r="165">
@@ -6961,7 +7161,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr"/>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>BV1iuXkYHEUG</t>
+        </is>
+      </c>
       <c r="J165" t="inlineStr"/>
     </row>
     <row r="166">
@@ -7073,7 +7277,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>BV1wKgRzPEp1</t>
+        </is>
+      </c>
       <c r="J168" t="inlineStr"/>
     </row>
     <row r="169">
@@ -7109,7 +7317,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>BV1jrrMBQEz7，BV1oTT8zyEX4，BV1bKXCYVExo</t>
+        </is>
+      </c>
       <c r="J169" t="inlineStr"/>
     </row>
     <row r="170">
@@ -7185,7 +7397,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>BV16XrTBsEcd，BV1hzyXBkETx，BV1o9TCzDE4H</t>
+        </is>
+      </c>
       <c r="J171" t="inlineStr"/>
     </row>
     <row r="172">
@@ -7221,7 +7437,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>BV1NaarzsEjk，BV1TT7Kz9ESB</t>
+        </is>
+      </c>
       <c r="J172" t="inlineStr"/>
     </row>
     <row r="173">
@@ -7293,7 +7513,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>BV1ChndzwE25</t>
+        </is>
+      </c>
       <c r="J174" t="inlineStr"/>
     </row>
     <row r="175">
@@ -7369,7 +7593,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>BV1f4KfzhEoC，BV1qVXyY4ELM</t>
+        </is>
+      </c>
       <c r="J176" t="inlineStr"/>
     </row>
     <row r="177">
@@ -7445,7 +7673,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>BV1NoYNzxEcc，BV1p9KpzTEvo</t>
+        </is>
+      </c>
       <c r="J178" t="inlineStr"/>
     </row>
     <row r="179">
@@ -7565,7 +7797,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I181" t="inlineStr"/>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>BV188spztEYf，BV1dbVfzyEzW</t>
+        </is>
+      </c>
       <c r="J181" t="inlineStr"/>
     </row>
     <row r="182">
@@ -7601,7 +7837,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>BV1M3SABjEb9，BV1UbEPz9Eyd，BV1i1wbzwEaz</t>
+        </is>
+      </c>
       <c r="J182" t="inlineStr"/>
     </row>
     <row r="183">
@@ -7717,7 +7957,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I185" t="inlineStr"/>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>BV11GKVzVEfL</t>
+        </is>
+      </c>
       <c r="J185" t="inlineStr"/>
     </row>
     <row r="186">
@@ -7753,7 +7997,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I186" t="inlineStr"/>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>BV1EMpQzEEJx，BV18ZiFBgEyW，BV1z4j1zJELw，BV1HvWhzPEe3</t>
+        </is>
+      </c>
       <c r="J186" t="inlineStr"/>
     </row>
     <row r="187">
@@ -7869,7 +8117,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I189" t="inlineStr"/>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>BV1CDSbByE47，BV1PKLczAEhW，BV1rEj3zoEfG</t>
+        </is>
+      </c>
       <c r="J189" t="inlineStr"/>
     </row>
     <row r="190">
@@ -7905,7 +8157,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I190" t="inlineStr"/>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>BV1ZHGzz9EoH，BV19qupzZEJQ</t>
+        </is>
+      </c>
       <c r="J190" t="inlineStr"/>
     </row>
     <row r="191">
@@ -7941,7 +8197,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr"/>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>BV1FBokYTETa，BV1bjNoziEuq，BV1PtGLzYEkK</t>
+        </is>
+      </c>
       <c r="J191" t="inlineStr"/>
     </row>
     <row r="192">
@@ -7958,7 +8218,7 @@
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
-          <t>小野来了</t>
+          <t>暗杠</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -7977,7 +8237,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I192" t="inlineStr"/>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>BV14A5QzVE3K，BV1wE7KzjEG2，BV1dKq6BcErY</t>
+        </is>
+      </c>
       <c r="J192" t="inlineStr"/>
     </row>
     <row r="193">
@@ -8013,7 +8277,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I193" t="inlineStr"/>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>BV1xRepzCEKq，BV1VqNXziE8q，BV1ytRrYTEZa</t>
+        </is>
+      </c>
       <c r="J193" t="inlineStr"/>
     </row>
     <row r="194">
@@ -8089,7 +8357,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr"/>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>BV1kSrTB4EPi，BV1eKKhz3EE3</t>
+        </is>
+      </c>
       <c r="J195" t="inlineStr"/>
     </row>
     <row r="196">
@@ -8125,7 +8397,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I196" t="inlineStr"/>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>BV1wuZwYZEmf，BV1rnj3zxE6a</t>
+        </is>
+      </c>
       <c r="J196" t="inlineStr"/>
     </row>
     <row r="197">
@@ -8201,7 +8477,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I198" t="inlineStr"/>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>BV19MmPBJEoW，BV1Jg37zfEct</t>
+        </is>
+      </c>
       <c r="J198" t="inlineStr"/>
     </row>
     <row r="199">
@@ -8237,7 +8517,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I199" t="inlineStr"/>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>BV1cPk3BBEjq，BV1MiEMziEA9，BV1TcoaYQEZV</t>
+        </is>
+      </c>
       <c r="J199" t="inlineStr"/>
     </row>
     <row r="200">
@@ -8275,7 +8559,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>BV1qgb1z5EKh</t>
+          <t>BV1qgb1z5EKh，BV1ieP2znEAT</t>
         </is>
       </c>
       <c r="J200" t="inlineStr"/>
@@ -8313,7 +8597,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I201" t="inlineStr"/>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>BV1FwEwzvEjt，BV1bAeazgE8Z</t>
+        </is>
+      </c>
       <c r="J201" t="inlineStr"/>
     </row>
     <row r="202">
@@ -8349,7 +8637,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I202" t="inlineStr"/>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>BV1t8J9zcEcz</t>
+        </is>
+      </c>
       <c r="J202" t="inlineStr"/>
     </row>
     <row r="203">
@@ -8427,7 +8719,7 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>BV13dPXz8ELA</t>
+          <t>BV13dPXz8ELA，BV1UTJaziECc</t>
         </is>
       </c>
       <c r="J204" t="inlineStr"/>
@@ -8465,7 +8757,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I205" t="inlineStr"/>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>BV1wiY1zwEKF，BV18j5EzsEtC</t>
+        </is>
+      </c>
       <c r="J205" t="inlineStr"/>
     </row>
     <row r="206">
@@ -8501,7 +8797,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I206" t="inlineStr"/>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>BV1USWVzfEuB，BV1L5ZnYTE6Q</t>
+        </is>
+      </c>
       <c r="J206" t="inlineStr"/>
     </row>
     <row r="207">
@@ -8537,7 +8837,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I207" t="inlineStr"/>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>BV1CkpMzKEPy，BV1RGjdzzE4G</t>
+        </is>
+      </c>
       <c r="J207" t="inlineStr"/>
     </row>
     <row r="208">
@@ -8613,7 +8917,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I209" t="inlineStr"/>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>BV1MAEHziEEN，BV1XkzWBJEcL</t>
+        </is>
+      </c>
       <c r="J209" t="inlineStr"/>
     </row>
     <row r="210">
@@ -8697,7 +9005,11 @@
           <t>13</t>
         </is>
       </c>
-      <c r="I211" t="inlineStr"/>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>BV1iQBjBKE9h</t>
+        </is>
+      </c>
       <c r="J211" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -8777,7 +9089,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I213" t="inlineStr"/>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>BV1pbVgznEsP，BV1rNZ3YHEFy，BV1o1STBBEJK</t>
+        </is>
+      </c>
       <c r="J213" t="inlineStr"/>
     </row>
     <row r="214">
@@ -8969,7 +9285,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I218" t="inlineStr"/>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>BV1bwoRYJEXg，BV1NVahzoELQ</t>
+        </is>
+      </c>
       <c r="J218" t="inlineStr"/>
     </row>
     <row r="219">
@@ -9125,7 +9445,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I222" t="inlineStr"/>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>BV138GZzwE7G，BV1xUyXBiEeR</t>
+        </is>
+      </c>
       <c r="J222" t="inlineStr"/>
     </row>
     <row r="223">
@@ -9389,7 +9713,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I229" t="inlineStr"/>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>BV13UVQzUEZY，BV14oqVBGEQf</t>
+        </is>
+      </c>
       <c r="J229" t="inlineStr"/>
     </row>
     <row r="230">
@@ -9497,7 +9825,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="I232" t="inlineStr"/>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>BV1ZrZAYREtV，BV1CDT4zUEQV</t>
+        </is>
+      </c>
       <c r="J232" t="inlineStr"/>
     </row>
     <row r="233">
@@ -11678,7 +12010,7 @@
       <c r="C290" t="inlineStr"/>
       <c r="D290" t="inlineStr">
         <is>
-          <t>夏天</t>
+          <t>夏天Alex</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -12297,7 +12629,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I306" t="inlineStr"/>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>BV1XoHnznEsh</t>
+        </is>
+      </c>
       <c r="J306" t="inlineStr"/>
     </row>
     <row r="307">
@@ -12801,7 +13137,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I319" t="inlineStr"/>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>BV1fjqjBKECu，BV1isG5z1EF6</t>
+        </is>
+      </c>
       <c r="J319" t="inlineStr"/>
     </row>
     <row r="320">
@@ -13101,7 +13441,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I327" t="inlineStr"/>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>BV1NeJhzFEeY，BV1xkEQznE35</t>
+        </is>
+      </c>
       <c r="J327" t="inlineStr"/>
     </row>
     <row r="328">
@@ -13137,7 +13481,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="I328" t="inlineStr"/>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>BV1DCzcBJETG</t>
+        </is>
+      </c>
       <c r="J328" t="inlineStr"/>
     </row>
     <row r="329">
@@ -21265,7 +21613,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I544" t="inlineStr"/>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>BV1KgKezKEwo，BV1gFW3zxEZa</t>
+        </is>
+      </c>
       <c r="J544" t="inlineStr"/>
     </row>
     <row r="545">
@@ -31849,7 +32201,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I827" t="inlineStr"/>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>BV12uwRzQEpw</t>
+        </is>
+      </c>
       <c r="J827" t="inlineStr"/>
     </row>
     <row r="828">

</xml_diff>

<commit_message>
chore: Update song list to Mar 19, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>53</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/13，2025/04/19，2025/05/06，2025/06/03，2025/08/28，2025/09/17，2025/10/10，2025/11/17，2025/11/22，2025/12/24，2026/1/15，2026/1/29</t>
+          <t>2025/03/13，2025/04/13，2025/04/19，2025/05/06，2025/06/03，2025/08/28，2025/09/17，2025/10/10，2025/11/17，2025/11/22，2025/12/24，2026/1/15，2026/1/29，2026/3/19</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4338,7 +4338,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/05/22，2025/06/10，2025/11/9，2025/11/14</t>
+          <t>2025/03/15，2025/05/22，2025/06/10，2025/11/9，2025/11/14，2026/3/19</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -9601,7 +9601,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I226" t="inlineStr"/>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>BV19Lh2zmEUD，BV13hZoYwEet，BV161UjBiEza</t>
+        </is>
+      </c>
       <c r="J226" t="inlineStr"/>
     </row>
     <row r="227">
@@ -9637,7 +9641,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I227" t="inlineStr"/>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>BV1ezGRztEYW，BV18Cj1zBEfP</t>
+        </is>
+      </c>
       <c r="J227" t="inlineStr"/>
     </row>
     <row r="228">
@@ -9753,7 +9761,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>BV1sG7SzgEvQ，BV1KUxdzEE7L，BV1CFJdzbErv</t>
+        </is>
+      </c>
       <c r="J230" t="inlineStr"/>
     </row>
     <row r="231">
@@ -9789,7 +9801,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>BV1sjMzzWEW2，BV1VhJNzKEcZ，BV18oZAYyEmJ</t>
+        </is>
+      </c>
       <c r="J231" t="inlineStr"/>
     </row>
     <row r="232">
@@ -10029,7 +10045,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I237" t="inlineStr"/>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>BV1aGndz5Ewo，BV1hFUfBMEoe，BV1ZoBCB2ERE</t>
+        </is>
+      </c>
       <c r="J237" t="inlineStr"/>
     </row>
     <row r="238">
@@ -10153,7 +10173,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I240" t="inlineStr"/>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>BV1fbWmz3E5N</t>
+        </is>
+      </c>
       <c r="J240" t="inlineStr"/>
     </row>
     <row r="241">
@@ -10189,7 +10213,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I241" t="inlineStr"/>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>BV1SfNizjEvd，BV1GYyXB2Ez5</t>
+        </is>
+      </c>
       <c r="J241" t="inlineStr"/>
     </row>
     <row r="242">
@@ -10225,7 +10253,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I242" t="inlineStr"/>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>BV1GPM8zrE7N，BV1VKUhB8EUR，BV1mpjQzjE5U</t>
+        </is>
+      </c>
       <c r="J242" t="inlineStr"/>
     </row>
     <row r="243">
@@ -10261,7 +10293,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I243" t="inlineStr"/>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>BV1EhNRzEEJE</t>
+        </is>
+      </c>
       <c r="J243" t="inlineStr"/>
     </row>
     <row r="244">
@@ -10377,7 +10413,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I246" t="inlineStr"/>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>BV1J3y5B7EnS，BV1cJ7Kz1EMG</t>
+        </is>
+      </c>
       <c r="J246" t="inlineStr"/>
     </row>
     <row r="247">
@@ -10569,7 +10609,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I251" t="inlineStr"/>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>BV16LR6Y4EF8</t>
+        </is>
+      </c>
       <c r="J251" t="inlineStr"/>
     </row>
     <row r="252">
@@ -10645,7 +10689,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I253" t="inlineStr"/>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>BV17LibBaEAF</t>
+        </is>
+      </c>
       <c r="J253" t="inlineStr"/>
     </row>
     <row r="254">
@@ -10681,7 +10729,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I254" t="inlineStr"/>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>BV1Wh3FzHEiy</t>
+        </is>
+      </c>
       <c r="J254" t="inlineStr"/>
     </row>
     <row r="255">
@@ -10797,7 +10849,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I257" t="inlineStr"/>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>BV1ET4gzkEE4</t>
+        </is>
+      </c>
       <c r="J257" t="inlineStr"/>
     </row>
     <row r="258">
@@ -10833,7 +10889,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I258" t="inlineStr"/>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>BV1iyaUzbE51</t>
+        </is>
+      </c>
       <c r="J258" t="inlineStr"/>
     </row>
     <row r="259">
@@ -10949,7 +11009,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I261" t="inlineStr"/>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>BV14QvKzvEdc</t>
+        </is>
+      </c>
       <c r="J261" t="inlineStr"/>
     </row>
     <row r="262">
@@ -10985,7 +11049,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I262" t="inlineStr"/>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>BV1gtWAzNEGE</t>
+        </is>
+      </c>
       <c r="J262" t="inlineStr"/>
     </row>
     <row r="263">
@@ -11021,7 +11089,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I263" t="inlineStr"/>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>BV1z95mzQEUi，BV1n3WzzQEE5</t>
+        </is>
+      </c>
       <c r="J263" t="inlineStr"/>
     </row>
     <row r="264">
@@ -11057,7 +11129,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I264" t="inlineStr"/>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>BV1gvpGztEps</t>
+        </is>
+      </c>
       <c r="J264" t="inlineStr"/>
     </row>
     <row r="265">
@@ -11093,7 +11169,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I265" t="inlineStr"/>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>BV1w1jZzdEMn</t>
+        </is>
+      </c>
       <c r="J265" t="inlineStr"/>
     </row>
     <row r="266">
@@ -11169,7 +11249,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I267" t="inlineStr"/>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>BV15LvXBdEwz，BV13zEcznEcV</t>
+        </is>
+      </c>
       <c r="J267" t="inlineStr"/>
     </row>
     <row r="268">
@@ -11205,7 +11289,11 @@
           <t>13</t>
         </is>
       </c>
-      <c r="I268" t="inlineStr"/>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>BV1BbT9zmEbe，BV115dzYwEED</t>
+        </is>
+      </c>
       <c r="J268" t="inlineStr"/>
     </row>
     <row r="269">
@@ -11241,7 +11329,11 @@
           <t>14</t>
         </is>
       </c>
-      <c r="I269" t="inlineStr"/>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>BV18qT4ztEam，BV1Uz5QzmE2k</t>
+        </is>
+      </c>
       <c r="J269" t="inlineStr"/>
     </row>
     <row r="270">
@@ -11277,7 +11369,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I270" t="inlineStr"/>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>BV19y8CzTEj5</t>
+        </is>
+      </c>
       <c r="J270" t="inlineStr"/>
     </row>
     <row r="271">
@@ -11313,7 +11409,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I271" t="inlineStr"/>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>BV1LYKfz4EUD，BV1Bp29BFEMn</t>
+        </is>
+      </c>
       <c r="J271" t="inlineStr"/>
     </row>
     <row r="272">
@@ -11513,7 +11613,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I276" t="inlineStr"/>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>BV1NhUvBfEpm</t>
+        </is>
+      </c>
       <c r="J276" t="inlineStr"/>
     </row>
     <row r="277">
@@ -11549,7 +11653,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I277" t="inlineStr"/>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>BV15honYaEYY，BV18T7kz8EAB</t>
+        </is>
+      </c>
       <c r="J277" t="inlineStr"/>
     </row>
     <row r="278">
@@ -11587,7 +11695,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>BV1Yj7DzxEm9</t>
+          <t>BV1Yj7DzxEm9，BV1fjcYzCEPz，BV1V37DzfEhn</t>
         </is>
       </c>
       <c r="J278" t="inlineStr"/>
@@ -11625,7 +11733,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I279" t="inlineStr"/>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>BV1BiJwzNEhh</t>
+        </is>
+      </c>
       <c r="J279" t="inlineStr"/>
     </row>
     <row r="280">
@@ -11661,7 +11773,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I280" t="inlineStr"/>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>BV1HBuJzhEgD</t>
+        </is>
+      </c>
       <c r="J280" t="inlineStr"/>
     </row>
     <row r="281">
@@ -11697,7 +11813,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I281" t="inlineStr"/>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>BV1bzYyzgEHM</t>
+        </is>
+      </c>
       <c r="J281" t="inlineStr"/>
     </row>
     <row r="282">
@@ -11773,7 +11893,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I283" t="inlineStr"/>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>BV1sfqeBhEVS，BV1YY7SzREBq</t>
+        </is>
+      </c>
       <c r="J283" t="inlineStr"/>
     </row>
     <row r="284">
@@ -11921,7 +12045,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I287" t="inlineStr"/>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>BV1jFp3zaE7u</t>
+        </is>
+      </c>
       <c r="J287" t="inlineStr"/>
     </row>
     <row r="288">
@@ -11957,7 +12085,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I288" t="inlineStr"/>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>BV17rVyzgE62，BV1NWZZYdEUN</t>
+        </is>
+      </c>
       <c r="J288" t="inlineStr"/>
     </row>
     <row r="289">
@@ -12029,7 +12161,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I290" t="inlineStr"/>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>BV1ufBZBkE5H</t>
+        </is>
+      </c>
       <c r="J290" t="inlineStr"/>
     </row>
     <row r="291">
@@ -12065,7 +12201,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr"/>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>BV1RpuUzPE1A，BV1mz1eBXE8L</t>
+        </is>
+      </c>
       <c r="J291" t="inlineStr"/>
     </row>
     <row r="292">
@@ -12175,7 +12315,7 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>BV1vpYkzVEVW</t>
+          <t>BV1vpYkzVEVW，BV1DdZsBPEuS</t>
         </is>
       </c>
       <c r="J294" t="inlineStr"/>
@@ -12253,7 +12393,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I296" t="inlineStr"/>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>BV1cJ3Az4EZq</t>
+        </is>
+      </c>
       <c r="J296" t="inlineStr"/>
     </row>
     <row r="297">
@@ -12289,7 +12433,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I297" t="inlineStr"/>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>BV15iWVzzEDs，BV1QnVAzkE3H</t>
+        </is>
+      </c>
       <c r="J297" t="inlineStr"/>
     </row>
     <row r="298">
@@ -12553,7 +12701,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I304" t="inlineStr"/>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>BV1Nu4TzyExF</t>
+        </is>
+      </c>
       <c r="J304" t="inlineStr"/>
     </row>
     <row r="305">
@@ -12591,7 +12743,7 @@
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>BV1ugBMBAEFM</t>
+          <t>BV1ugBMBAEFM，BV1TBCJB3EMp，BV1dscYzMEKG，BV1D8GdzWE7M</t>
         </is>
       </c>
       <c r="J305" t="inlineStr"/>
@@ -12751,7 +12903,7 @@
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>BV1aXvxB1EKh</t>
+          <t>BV1aXvxB1EKh，BV1uNSgBeEKj，BV1YBVfzBEpm</t>
         </is>
       </c>
       <c r="J309" t="inlineStr"/>
@@ -13597,7 +13749,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I331" t="inlineStr"/>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>BV186tVz6EuE</t>
+        </is>
+      </c>
       <c r="J331" t="inlineStr"/>
     </row>
     <row r="332">
@@ -13673,7 +13829,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I333" t="inlineStr"/>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>BV1nCJ9zHEhj</t>
+        </is>
+      </c>
       <c r="J333" t="inlineStr"/>
     </row>
     <row r="334">
@@ -13709,7 +13869,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I334" t="inlineStr"/>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>BV16iuKzsE7v</t>
+        </is>
+      </c>
       <c r="J334" t="inlineStr"/>
     </row>
     <row r="335">
@@ -13827,7 +13991,7 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>BV1gKuwz8E9Y</t>
+          <t>BV1gKuwz8E9Y，BV18t7nziEmf</t>
         </is>
       </c>
       <c r="J337" t="inlineStr">
@@ -13859,7 +14023,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24</t>
+          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -13870,7 +14034,7 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -14113,7 +14277,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I344" t="inlineStr"/>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>BV18JjhzZEVj，BV1zzoJYTEka</t>
+        </is>
+      </c>
       <c r="J344" t="inlineStr"/>
     </row>
     <row r="345">
@@ -14225,7 +14393,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I347" t="inlineStr"/>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>BV1b1NzzXEMp，BV1MRETzeETU</t>
+        </is>
+      </c>
       <c r="J347" t="inlineStr"/>
     </row>
     <row r="348">
@@ -14261,7 +14433,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I348" t="inlineStr"/>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>BV1WgnVz1EfK，BV1G2LnziE1H</t>
+        </is>
+      </c>
       <c r="J348" t="inlineStr"/>
     </row>
     <row r="349">
@@ -14297,7 +14473,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="I349" t="inlineStr"/>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>BV1uAVLzCELY</t>
+        </is>
+      </c>
       <c r="J349" t="inlineStr"/>
     </row>
     <row r="350">
@@ -14333,7 +14513,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I350" t="inlineStr"/>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>BV1BzKhzUEYG，BV1KFLczTECE</t>
+        </is>
+      </c>
       <c r="J350" t="inlineStr"/>
     </row>
     <row r="351">
@@ -14445,7 +14629,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I353" t="inlineStr"/>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>BV1x23MzVEFJ，BV16iWhzaELz</t>
+        </is>
+      </c>
       <c r="J353" t="inlineStr"/>
     </row>
     <row r="354">
@@ -14645,7 +14833,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I358" t="inlineStr"/>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>BV1ccHRzoEKY，BV1Q17gzVE5c</t>
+        </is>
+      </c>
       <c r="J358" t="inlineStr"/>
     </row>
     <row r="359">
@@ -14698,7 +14890,7 @@
       <c r="C360" t="inlineStr"/>
       <c r="D360" t="inlineStr">
         <is>
-          <t>落日飛車</t>
+          <t>任贤齐</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -14717,7 +14909,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I360" t="inlineStr"/>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>BV1ytebzxEKA，BV1ZzVyzrEC8</t>
+        </is>
+      </c>
       <c r="J360" t="inlineStr"/>
     </row>
     <row r="361">
@@ -14865,7 +15061,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I364" t="inlineStr"/>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>BV1cq6SBkEz4</t>
+        </is>
+      </c>
       <c r="J364" t="inlineStr"/>
     </row>
     <row r="365">
@@ -14985,7 +15185,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I367" t="inlineStr"/>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>BV1cRW8zhEjd，BV1whUhBVEE4</t>
+        </is>
+      </c>
       <c r="J367" t="inlineStr"/>
     </row>
     <row r="368">
@@ -15021,7 +15225,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I368" t="inlineStr"/>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>BV1bAunz5EVY</t>
+        </is>
+      </c>
       <c r="J368" t="inlineStr"/>
     </row>
     <row r="369">
@@ -15789,7 +15997,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I388" t="inlineStr"/>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>BV1MLp3zHEmo</t>
+        </is>
+      </c>
       <c r="J388" t="inlineStr"/>
     </row>
     <row r="389">
@@ -15825,7 +16037,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I389" t="inlineStr"/>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>BV1BNekzUEnz</t>
+        </is>
+      </c>
       <c r="J389" t="inlineStr"/>
     </row>
     <row r="390">
@@ -15861,7 +16077,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I390" t="inlineStr"/>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>BV1aEpBzPEEq，BV1AMLHzHEA7</t>
+        </is>
+      </c>
       <c r="J390" t="inlineStr"/>
     </row>
     <row r="391">
@@ -15973,7 +16193,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I393" t="inlineStr"/>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>BV1bD3jzkEhN</t>
+        </is>
+      </c>
       <c r="J393" t="inlineStr"/>
     </row>
     <row r="394">
@@ -16081,7 +16305,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I396" t="inlineStr"/>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>BV1r9NZzFErx，BV1gLtdzZEHp</t>
+        </is>
+      </c>
       <c r="J396" t="inlineStr"/>
     </row>
     <row r="397">
@@ -16269,7 +16497,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I401" t="inlineStr"/>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>BV1rkLBzAEhH</t>
+        </is>
+      </c>
       <c r="J401" t="inlineStr"/>
     </row>
     <row r="402">
@@ -20077,7 +20309,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I503" t="inlineStr"/>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>BV1Lj7XzPEsE</t>
+        </is>
+      </c>
       <c r="J503" t="inlineStr"/>
     </row>
     <row r="504">
@@ -20561,7 +20797,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I516" t="inlineStr"/>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>BV1ySRJYkEK1</t>
+        </is>
+      </c>
       <c r="J516" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -20601,7 +20841,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I517" t="inlineStr"/>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>BV1JWMNzDEdH</t>
+        </is>
+      </c>
       <c r="J517" t="inlineStr"/>
     </row>
     <row r="518">
@@ -21865,7 +22109,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I550" t="inlineStr"/>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>BV1YzYxztEuV</t>
+        </is>
+      </c>
       <c r="J550" t="inlineStr"/>
     </row>
     <row r="551">
@@ -22035,7 +22283,7 @@
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/12/16</t>
+          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16</t>
         </is>
       </c>
       <c r="F555" t="inlineStr"/>
@@ -22046,10 +22294,14 @@
       </c>
       <c r="H555" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I555" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>BV1rhS5BwE38</t>
+        </is>
+      </c>
       <c r="J555" t="inlineStr"/>
     </row>
     <row r="556">
@@ -22629,7 +22881,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I571" t="inlineStr"/>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>BV1TRqVBCEDC</t>
+        </is>
+      </c>
       <c r="J571" t="inlineStr"/>
     </row>
     <row r="572">
@@ -22853,7 +23109,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I577" t="inlineStr"/>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>BV1i5GHziEo8</t>
+        </is>
+      </c>
       <c r="J577" t="inlineStr"/>
     </row>
     <row r="578">
@@ -23149,7 +23409,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="I585" t="inlineStr"/>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>BV1Q9aUzpEov，BV1oQs8zxEjE</t>
+        </is>
+      </c>
       <c r="J585" t="inlineStr"/>
     </row>
     <row r="586">
@@ -23341,7 +23605,11 @@
           <t>10</t>
         </is>
       </c>
-      <c r="I590" t="inlineStr"/>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>BV19UbDzXE7H</t>
+        </is>
+      </c>
       <c r="J590" t="inlineStr"/>
     </row>
     <row r="591">
@@ -30955,7 +31223,7 @@
       </c>
       <c r="E793" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19</t>
         </is>
       </c>
       <c r="F793" t="inlineStr"/>
@@ -30966,7 +31234,7 @@
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 21, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/29，2025/05/20，2025/07/13，2025/07/25，2025/07/31，2025/10/09，2025/12/2，2026/1/9</t>
+          <t>2025/03/04，2025/04/29，2025/05/20，2025/07/13，2025/07/25，2025/07/31，2025/10/09，2025/12/2，2026/1/9，2026/3/21</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7，2026/3/17</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7，2026/3/17，2026/3/21</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7，2026/3/17</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7，2026/3/17，2026/3/21</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/20，2026/3/21</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/08/28，2025/09/18，2025/11/21，2025/12/4</t>
+          <t>2025/03/28，2025/04/04，2025/08/28，2025/09/18，2025/11/21，2025/12/4，2026/3/21</t>
         </is>
       </c>
       <c r="F226" t="inlineStr"/>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -12727,7 +12727,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/1/29</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/1/29，2026/3/20</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12738,7 +12738,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -16613,7 +16613,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I404" t="inlineStr"/>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>BV162h5zKEMs，BV1Jd7VzPEBH</t>
+        </is>
+      </c>
       <c r="J404" t="inlineStr"/>
     </row>
     <row r="405">
@@ -16809,7 +16813,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I409" t="inlineStr"/>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>BV12579zWEyS</t>
+        </is>
+      </c>
       <c r="J409" t="inlineStr"/>
     </row>
     <row r="410">
@@ -17353,7 +17361,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I424" t="inlineStr"/>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>BV1dgy9BnEKm</t>
+        </is>
+      </c>
       <c r="J424" t="inlineStr"/>
     </row>
     <row r="425">
@@ -17425,7 +17437,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I426" t="inlineStr"/>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>BV1oUSuB5EpY</t>
+        </is>
+      </c>
       <c r="J426" t="inlineStr"/>
     </row>
     <row r="427">
@@ -18737,7 +18753,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I461" t="inlineStr"/>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>BV1JQkwByEBf</t>
+        </is>
+      </c>
       <c r="J461" t="inlineStr"/>
     </row>
     <row r="462">
@@ -18813,7 +18833,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I463" t="inlineStr"/>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>BV1ULsWzoEEy，BV1qCjJzkEGz</t>
+        </is>
+      </c>
       <c r="J463" t="inlineStr"/>
     </row>
     <row r="464">
@@ -19167,7 +19191,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21</t>
         </is>
       </c>
       <c r="F473" t="inlineStr"/>
@@ -19178,7 +19202,7 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
@@ -19477,7 +19501,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I481" t="inlineStr"/>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>BV1akvKzrEM3</t>
+        </is>
+      </c>
       <c r="J481" t="inlineStr"/>
     </row>
     <row r="482">
@@ -21101,7 +21129,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I524" t="inlineStr"/>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>BV1t9yVBfEnU</t>
+        </is>
+      </c>
       <c r="J524" t="inlineStr"/>
     </row>
     <row r="525">
@@ -21781,7 +21813,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I542" t="inlineStr"/>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>BV1RpK8z6EDo</t>
+        </is>
+      </c>
       <c r="J542" t="inlineStr"/>
     </row>
     <row r="543">
@@ -27945,7 +27981,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I705" t="inlineStr"/>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>BV1UfsZzsEJb</t>
+        </is>
+      </c>
       <c r="J705" t="inlineStr"/>
     </row>
     <row r="706">
@@ -30753,7 +30793,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I780" t="inlineStr"/>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>BV1g7zuBgEkG</t>
+        </is>
+      </c>
       <c r="J780" t="inlineStr"/>
     </row>
     <row r="781">
@@ -31779,7 +31823,7 @@
       </c>
       <c r="E808" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21</t>
         </is>
       </c>
       <c r="F808" t="inlineStr"/>
@@ -31790,7 +31834,7 @@
       </c>
       <c r="H808" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I808" t="inlineStr">

</xml_diff>

<commit_message>
chore: Fixed an error in the song list
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -5099,7 +5099,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/20，2026/3/21</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/21</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -30239,7 +30239,7 @@
       </c>
       <c r="E766" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20</t>
         </is>
       </c>
       <c r="F766" t="inlineStr"/>
@@ -30250,7 +30250,7 @@
       </c>
       <c r="H766" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I766" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 22, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,52 +417,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -499,7 +487,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/1/23，2026/3/1</t>
+          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/1/23，2026/3/1，2026/3/22</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -510,7 +498,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1003,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1014,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1603,7 +1591,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/13，2025/05/06，2025/05/15，2025/05/25，2025/06/06，2025/06/23，2025/07/15，2025/07/26，2025/09/15，2025/09/24，2025/10/03，2025/11/26，2025/12/26，2026/1/10</t>
+          <t>2025/03/04，2025/04/13，2025/05/06，2025/05/15，2025/05/25，2025/06/06，2025/06/23，2025/07/15，2025/07/26，2025/09/15，2025/09/24，2025/10/03，2025/11/26，2025/12/26，2026/1/10，2026/3/22</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -1614,7 +1602,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1683,7 +1671,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,7 +1682,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2351,7 +2339,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/1/15，2026/2/14</t>
+          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/1/15，2026/2/14，2026/3/22</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2362,7 +2350,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2795,7 +2783,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2806,7 +2794,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2923,7 +2911,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/1/21，2026/1/25，2026/2/10，2026/2/23，2026/3/6</t>
+          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/1/21，2026/1/25，2026/2/10，2026/2/23，2026/3/6，2026/3/22</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2934,7 +2922,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -2963,7 +2951,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2962,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6419,7 +6407,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13，2026/3/22</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6430,7 +6418,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6499,7 +6487,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6510,7 +6498,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -7903,7 +7891,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7914,7 +7902,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -8947,7 +8935,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/28，2025/04/29，2025/05/12，2025/06/06，2025/06/16，2025/07/24，2025/08/01，2025/09/05，2025/09/26，2025/10/28，2025/12/5，2026/1/9，2026/2/19</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/28，2025/04/29，2025/05/12，2025/06/06，2025/06/16，2025/07/24，2025/08/01，2025/09/05，2025/09/26，2025/10/28，2025/12/5，2026/1/9，2026/2/19，2026/3/22</t>
         </is>
       </c>
       <c r="F210" t="inlineStr"/>
@@ -8958,7 +8946,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -9075,7 +9063,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/15，2025/05/08，2025/06/10，2025/07/07，2025/08/04，2025/09/04，2025/10/01，2025/11/26，2026/1/10</t>
+          <t>2025/03/27，2025/04/15，2025/05/08，2025/06/10，2025/07/07，2025/08/04，2025/09/04，2025/10/01，2025/11/26，2026/1/10，2026/3/22</t>
         </is>
       </c>
       <c r="F213" t="inlineStr"/>
@@ -9086,7 +9074,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -15211,7 +15199,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/1/10</t>
+          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/22</t>
         </is>
       </c>
       <c r="F368" t="inlineStr"/>
@@ -15222,7 +15210,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -18475,7 +18463,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/6</t>
+          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/6，2026/3/22</t>
         </is>
       </c>
       <c r="F454" t="inlineStr"/>
@@ -18486,7 +18474,7 @@
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I454" t="inlineStr"/>
@@ -22079,7 +22067,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6</t>
+          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -22094,7 +22082,7 @@
       </c>
       <c r="H549" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I549" t="inlineStr">
@@ -24495,7 +24483,7 @@
       </c>
       <c r="E613" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22</t>
         </is>
       </c>
       <c r="F613" t="inlineStr"/>
@@ -24506,7 +24494,7 @@
       </c>
       <c r="H613" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I613" t="inlineStr">
@@ -26311,7 +26299,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22</t>
         </is>
       </c>
       <c r="F661" t="inlineStr"/>
@@ -26322,7 +26310,7 @@
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
@@ -26947,7 +26935,7 @@
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7</t>
+          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22</t>
         </is>
       </c>
       <c r="F678" t="inlineStr"/>
@@ -26958,7 +26946,7 @@
       </c>
       <c r="H678" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I678" t="inlineStr">
@@ -30123,7 +30111,7 @@
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29</t>
+          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29，2026/3/22</t>
         </is>
       </c>
       <c r="F763" t="inlineStr"/>
@@ -30134,7 +30122,7 @@
       </c>
       <c r="H763" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I763" t="inlineStr">

</xml_diff>

<commit_message>
chore: Add more BVID
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,52 +429,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -11957,7 +11969,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I285" t="inlineStr"/>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>BV1XsM9z5E9B</t>
+        </is>
+      </c>
       <c r="J285" t="inlineStr"/>
     </row>
     <row r="286">
@@ -12537,7 +12553,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I300" t="inlineStr"/>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>BV1jbnmzhEFK，BV1Y1YXzMEbB</t>
+        </is>
+      </c>
       <c r="J300" t="inlineStr"/>
     </row>
     <row r="301">
@@ -14229,7 +14249,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I343" t="inlineStr"/>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>BV1V8yXBUEfU，BV1ryYKzpEvD</t>
+        </is>
+      </c>
       <c r="J343" t="inlineStr"/>
     </row>
     <row r="344">
@@ -14541,7 +14565,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr"/>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>BV1x1G5zwEL1</t>
+        </is>
+      </c>
       <c r="J351" t="inlineStr"/>
     </row>
     <row r="352">
@@ -16671,7 +16699,7 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/05/20，2025/06/08，2025/08/18，2025/09/11</t>
+          <t>2025/04/27，2025/05/20，2025/06/08，2025/08/18，2025/09/11，2025/11/03</t>
         </is>
       </c>
       <c r="F406" t="inlineStr"/>
@@ -16682,10 +16710,14 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I406" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>BV1xL1kBGEXu</t>
+        </is>
+      </c>
       <c r="J406" t="inlineStr"/>
     </row>
     <row r="407">
@@ -16985,7 +17017,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I414" t="inlineStr"/>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>BV1S6GzzrExR</t>
+        </is>
+      </c>
       <c r="J414" t="inlineStr"/>
     </row>
     <row r="415">
@@ -17097,7 +17133,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I417" t="inlineStr"/>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>BV1buhSzEER7，BV19ZmMBaESn</t>
+        </is>
+      </c>
       <c r="J417" t="inlineStr"/>
     </row>
     <row r="418">
@@ -17613,7 +17653,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I431" t="inlineStr"/>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>BV12gVfzoEr1，BV1vJM9zmE58</t>
+        </is>
+      </c>
       <c r="J431" t="inlineStr"/>
     </row>
     <row r="432">
@@ -17649,7 +17693,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I432" t="inlineStr"/>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>BV1ZgKxzAEDk</t>
+        </is>
+      </c>
       <c r="J432" t="inlineStr"/>
     </row>
     <row r="433">
@@ -17685,7 +17733,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I433" t="inlineStr"/>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>BV1YTYuzLEjW</t>
+        </is>
+      </c>
       <c r="J433" t="inlineStr"/>
     </row>
     <row r="434">
@@ -17721,7 +17773,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I434" t="inlineStr"/>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>BV1hQuPziEjH，BV1UUKmz2EjB</t>
+        </is>
+      </c>
       <c r="J434" t="inlineStr"/>
     </row>
     <row r="435">
@@ -17909,7 +17965,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I439" t="inlineStr"/>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>BV1FBEpzhEoM</t>
+        </is>
+      </c>
       <c r="J439" t="inlineStr"/>
     </row>
     <row r="440">
@@ -17985,7 +18045,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I441" t="inlineStr"/>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>BV1KyT4zXELa</t>
+        </is>
+      </c>
       <c r="J441" t="inlineStr"/>
     </row>
     <row r="442">
@@ -18441,7 +18505,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I453" t="inlineStr"/>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>BV1cRB1BoEnG</t>
+        </is>
+      </c>
       <c r="J453" t="inlineStr"/>
     </row>
     <row r="454">
@@ -18477,7 +18545,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I454" t="inlineStr"/>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>BV1famFB7EmL，BV19JJHzmEUB，BV1En7PzTEo3</t>
+        </is>
+      </c>
       <c r="J454" t="inlineStr"/>
     </row>
     <row r="455">
@@ -18513,7 +18585,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I455" t="inlineStr"/>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>BV11ZJpz6EBr</t>
+        </is>
+      </c>
       <c r="J455" t="inlineStr"/>
     </row>
     <row r="456">
@@ -18549,7 +18625,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I456" t="inlineStr"/>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>BV1bgAMzbEEW</t>
+        </is>
+      </c>
       <c r="J456" t="inlineStr"/>
     </row>
     <row r="457">
@@ -19453,7 +19533,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I480" t="inlineStr"/>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>BV1NBnzzpE7i</t>
+        </is>
+      </c>
       <c r="J480" t="inlineStr"/>
     </row>
     <row r="481">
@@ -19569,7 +19653,11 @@
           <t>6</t>
         </is>
       </c>
-      <c r="I483" t="inlineStr"/>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>BV1TA7PzUEw8</t>
+        </is>
+      </c>
       <c r="J483" t="inlineStr"/>
     </row>
     <row r="484">
@@ -21045,7 +21133,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I522" t="inlineStr"/>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>BV1q9NhzLECV</t>
+        </is>
+      </c>
       <c r="J522" t="inlineStr"/>
     </row>
     <row r="523">
@@ -24425,7 +24517,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I611" t="inlineStr"/>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>BV1KG3qzFEUQ</t>
+        </is>
+      </c>
       <c r="J611" t="inlineStr"/>
     </row>
     <row r="612">
@@ -27397,7 +27493,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I690" t="inlineStr"/>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>BV1omCiBMEYU</t>
+        </is>
+      </c>
       <c r="J690" t="inlineStr"/>
     </row>
     <row r="691">
@@ -27437,7 +27537,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I691" t="inlineStr"/>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>BV1UcnVzQES5</t>
+        </is>
+      </c>
       <c r="J691" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -27477,7 +27581,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I692" t="inlineStr"/>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>BV1jQSFBHEye</t>
+        </is>
+      </c>
       <c r="J692" t="inlineStr"/>
     </row>
     <row r="693">
@@ -27641,7 +27749,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I696" t="inlineStr"/>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>BV1cFiPBiERh，BV1Z3zsB8ERD</t>
+        </is>
+      </c>
       <c r="J696" t="inlineStr"/>
     </row>
     <row r="697">
@@ -27677,7 +27789,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="I697" t="inlineStr"/>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>BV1yM2HBJEgf，BV1fEigB2EVM</t>
+        </is>
+      </c>
       <c r="J697" t="inlineStr"/>
     </row>
     <row r="698">
@@ -30709,7 +30825,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I778" t="inlineStr"/>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>BV1RDzuB2EsP</t>
+        </is>
+      </c>
       <c r="J778" t="inlineStr"/>
     </row>
     <row r="779">

</xml_diff>

<commit_message>
chore: Update song list to Mar 24, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6823,7 +6823,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/9，2025/12/5，2025/12/19，2025/12/26，2026/1/10，2026/1/19，2026/2/10</t>
+          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/9，2025/12/5，2025/12/19，2025/12/26，2026/1/10，2026/1/19，2026/2/10，2026/3/24</t>
         </is>
       </c>
       <c r="F313" t="inlineStr"/>
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>2025/04/10，2025/04/24，2025/05/13，2025/06/13，2025/09/03，2025/09/19，2025/10/13，2025/11/21，2026/3/4</t>
+          <t>2025/04/10，2025/04/24，2025/05/13，2025/06/13，2025/09/03，2025/09/19，2025/10/13，2025/11/21，2026/3/4，2026/3/24</t>
         </is>
       </c>
       <c r="F315" t="inlineStr"/>
@@ -13138,7 +13138,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -13439,7 +13439,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -13450,7 +13450,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13950,7 +13950,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -14719,7 +14719,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/01，2025/05/26，2025/07/03，2025/07/27，2025/09/18，2025/10/17，2025/11/21，2026/1/12，2026/1/24，2026/2/19，2026/2/23</t>
+          <t>2025/04/17，2025/05/01，2025/05/26，2025/07/03，2025/07/27，2025/09/18，2025/10/17，2025/11/21，2026/1/12，2026/1/24，2026/2/19，2026/2/23，2026/3/24</t>
         </is>
       </c>
       <c r="F355" t="inlineStr"/>
@@ -14730,7 +14730,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
@@ -18665,7 +18665,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I457" t="inlineStr"/>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>BV1H6JJzxES5，BV1CJMzzHEMy</t>
+        </is>
+      </c>
       <c r="J457" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -26655,7 +26659,7 @@
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/7，2025/11/26，2025/12/6，2025/12/12，2025/12/24，2026/1/5，2026/1/19，2026/2/18，2026/3/14</t>
+          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/7，2025/11/26，2025/12/6，2025/12/12，2025/12/24，2026/1/5，2026/1/19，2026/2/18，2026/3/14，2026/3/24</t>
         </is>
       </c>
       <c r="F668" t="inlineStr"/>
@@ -26666,7 +26670,7 @@
       </c>
       <c r="H668" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I668" t="inlineStr">
@@ -27443,7 +27447,7 @@
       </c>
       <c r="E689" t="inlineStr">
         <is>
-          <t>2025/10/07，2025/10/12，2025/10/22</t>
+          <t>2025/10/07，2025/10/12，2025/10/22，2026/3/24</t>
         </is>
       </c>
       <c r="F689" t="inlineStr"/>
@@ -27454,10 +27458,14 @@
       </c>
       <c r="H689" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I689" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>BV1gZQkBNELE</t>
+        </is>
+      </c>
       <c r="J689" t="inlineStr"/>
     </row>
     <row r="690">
@@ -27607,7 +27615,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2026/3/4</t>
+          <t>2025/10/13，2026/3/4，2026/3/24</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -27622,7 +27630,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 25, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J828"/>
+  <dimension ref="A1:J830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23</t>
+          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/1/3</t>
+          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/1/3，2026/3/25</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/9</t>
+          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/9，2026/3/25</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/19，2025/06/13，2025/07/22，2025/07/23，2025/08/25，2025/09/12，2025/10/26，2025/12/17，2026/2/9，2026/3/4</t>
+          <t>2025/03/21，2025/05/19，2025/06/13，2025/07/22，2025/07/23，2025/08/25，2025/09/12，2025/10/26，2025/12/17，2026/2/9，2026/3/4，2026/3/25</t>
         </is>
       </c>
       <c r="F167" t="inlineStr"/>
@@ -7234,7 +7234,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/28，2025/05/13，2025/06/07，2025/06/21，2025/08/28，2025/09/29，2025/10/24，2025/11/14，2025/12/17</t>
+          <t>2025/03/21，2025/04/28，2025/05/13，2025/06/07，2025/06/21，2025/08/28，2025/09/29，2025/10/24，2025/11/14，2025/12/17，2026/3/25</t>
         </is>
       </c>
       <c r="F182" t="inlineStr"/>
@@ -7834,7 +7834,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -8063,7 +8063,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9</t>
+          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -8074,7 +8074,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/9，2026/1/1，2026/2/7</t>
+          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/9，2026/1/1，2026/2/7，2026/3/25</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -8434,7 +8434,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04</t>
+          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/3/25</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -8594,7 +8594,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19</t>
+          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -9126,12 +9126,12 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>BV11GypBUErS</t>
+          <t>BV11GypBUErS，BV1KLVSzYEbC，BV1PFZ3YdENc</t>
         </is>
       </c>
       <c r="J214" t="inlineStr"/>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/7，2025/11/24，2025/12/5，2026/1/23，2026/3/9</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/7，2025/11/24，2025/12/5，2026/1/23，2026/3/9，2026/3/25</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9678,7 +9678,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -10239,7 +10239,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/1/16</t>
+          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/1/16，2026/3/25</t>
         </is>
       </c>
       <c r="F242" t="inlineStr"/>
@@ -10250,7 +10250,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -10955,7 +10955,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/1/2，2026/1/5，2026/2/2，2026/2/9，2026/2/19</t>
+          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/1/2，2026/1/5，2026/2/2，2026/2/9，2026/2/19，2026/3/25</t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
@@ -10966,7 +10966,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/04，2025/05/20，2025/06/23，2025/07/24，2025/09/12，2025/10/17，2025/12/9，2026/2/14</t>
+          <t>2025/04/02，2025/05/04，2025/05/20，2025/06/23，2025/07/24，2025/09/12，2025/10/17，2025/12/9，2026/2/14，2026/3/25</t>
         </is>
       </c>
       <c r="F266" t="inlineStr"/>
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11690,7 +11690,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -12775,7 +12775,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/19，2025/10/01，2025/10/31，2026/1/5</t>
+          <t>2025/04/07，2025/05/19，2025/10/01，2025/10/31，2026/1/5，2026/3/25，2026/3/25</t>
         </is>
       </c>
       <c r="F306" t="inlineStr"/>
@@ -12786,7 +12786,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12906,7 +12906,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -14391,7 +14391,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/1/16</t>
+          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/1/16，2026/3/25</t>
         </is>
       </c>
       <c r="F347" t="inlineStr"/>
@@ -14402,7 +14402,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -19603,7 +19603,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/05/31，2025/05/31，2025/06/02，2025/06/03，2025/06/05，2025/06/19，2025/06/26，2025/07/03，2025/07/14，2025/08/02，2025/08/24，2025/09/03，2025/09/18，2025/10/07，2025/11/19，2025/12/11，2026/1/10，2026/1/22</t>
+          <t>2025/05/30，2025/05/31，2025/05/31，2025/06/02，2025/06/03，2025/06/05，2025/06/19，2025/06/26，2025/07/03，2025/07/14，2025/08/02，2025/08/24，2025/09/03，2025/09/18，2025/10/07，2025/11/19，2025/12/11，2026/1/10，2026/1/22，2026/3/25</t>
         </is>
       </c>
       <c r="F482" t="inlineStr"/>
@@ -19614,7 +19614,7 @@
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I482" t="inlineStr">
@@ -20703,7 +20703,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>2025/06/08，2025/06/13，2025/06/16，2025/06/28，2025/07/18，2025/07/29，2025/08/18，2025/09/03，2025/09/11，2025/09/30，2025/10/05，2025/10/30，2025/11/17，2025/12/24，2026/2/2</t>
+          <t>2025/06/08，2025/06/13，2025/06/16，2025/06/28，2025/07/18，2025/07/29，2025/08/18，2025/09/03，2025/09/11，2025/09/30，2025/10/05，2025/10/30，2025/11/17，2025/12/24，2026/2/2，2026/3/25</t>
         </is>
       </c>
       <c r="F511" t="inlineStr"/>
@@ -20714,7 +20714,7 @@
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I511" t="inlineStr">
@@ -25947,7 +25947,7 @@
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/2/23，2026/3/17</t>
+          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/2/23，2026/3/17，2026/3/25</t>
         </is>
       </c>
       <c r="F649" t="inlineStr"/>
@@ -25958,7 +25958,7 @@
       </c>
       <c r="H649" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I649" t="inlineStr">
@@ -27615,7 +27615,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2026/3/4，2026/3/24</t>
+          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -27630,7 +27630,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">
@@ -29011,7 +29011,7 @@
       </c>
       <c r="E730" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9，2026/3/25</t>
         </is>
       </c>
       <c r="F730" t="inlineStr"/>
@@ -29022,7 +29022,7 @@
       </c>
       <c r="H730" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I730" t="inlineStr">
@@ -30431,7 +30431,7 @@
       </c>
       <c r="E768" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25</t>
         </is>
       </c>
       <c r="F768" t="inlineStr"/>
@@ -30442,7 +30442,7 @@
       </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">
@@ -32275,7 +32275,7 @@
       </c>
       <c r="E817" t="inlineStr">
         <is>
-          <t>2026/3/13</t>
+          <t>2026/3/13，2026/3/25</t>
         </is>
       </c>
       <c r="F817" t="inlineStr"/>
@@ -32286,7 +32286,7 @@
       </c>
       <c r="H817" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I817" t="inlineStr"/>
@@ -32651,7 +32651,7 @@
       </c>
       <c r="E828" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17</t>
+          <t>2026/3/17，2026/3/17，2026/3/25</t>
         </is>
       </c>
       <c r="F828" t="inlineStr"/>
@@ -32662,15 +32662,95 @@
       </c>
       <c r="H828" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I828" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>BV1ugQSBnE8x</t>
+        </is>
+      </c>
       <c r="J828" t="inlineStr">
         <is>
           <t>游戏</t>
         </is>
       </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr"/>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Deadline Disco</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>极限迪斯科</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/飞行雪绒</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>2026/3/25</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr"/>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr"/>
+      <c r="J829" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr"/>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>シリウスの心臓</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>天狼星的心脏</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>ヰ世界情緒</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>2026/3/25</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr"/>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr"/>
+      <c r="J830" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 27, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/1/23，2026/3/1，2026/3/22</t>
+          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/1/23，2026/3/1，2026/3/22，2026/3/27</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -510,12 +510,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>BV1Z1u9z9E4q，BV15MPuzCEEd</t>
+          <t>BV1dmXNBgE3x，BV1Z1u9z9E4q，BV15MPuzCEEd</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -550,12 +550,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BV1mm7KzxEGj，BV12yM2z7EfT</t>
+          <t>BV1bPXMBTE14，BV1mm7KzxEGj，BV12yM2z7EfT</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>56</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27</t>
+          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/3/27</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>BV1fsnmzPEoD，BV1DDVQzjEMa</t>
+          <t>BV1fsnmzPEoD，BV1DDVQzjEMa，BV1rzXTBWEux</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -24623,7 +24623,7 @@
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>2025/08/09，2026/3/13</t>
+          <t>2025/08/09，2026/3/13，2026/3/27</t>
         </is>
       </c>
       <c r="F614" t="inlineStr">
@@ -24638,12 +24638,12 @@
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I614" t="inlineStr">
         <is>
-          <t>BV1BSt8zzESY</t>
+          <t>BV1wiXTB4Emi，BV1BSt8zzESY</t>
         </is>
       </c>
       <c r="J614" t="inlineStr"/>
@@ -30515,7 +30515,7 @@
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27</t>
         </is>
       </c>
       <c r="F770" t="inlineStr"/>
@@ -30526,12 +30526,12 @@
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I770" t="inlineStr">
         <is>
-          <t>BV1mNBfBBEkr</t>
+          <t>BV1XVXTB3E9c，BV1mNBfBBEkr</t>
         </is>
       </c>
       <c r="J770" t="inlineStr"/>
@@ -32651,7 +32651,7 @@
       </c>
       <c r="E828" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27</t>
         </is>
       </c>
       <c r="F828" t="inlineStr"/>
@@ -32662,7 +32662,7 @@
       </c>
       <c r="H828" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I828" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Mar 28, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J830"/>
+  <dimension ref="A1:J831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BV1kG7szAEYF，BV1dcjSzXEAu</t>
+          <t>BV1aaXLBwEto，BV1kG7szAEYF，BV1dcjSzXEAu</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/05，2025/05/15，2025/08/12</t>
+          <t>2025/03/15，2025/04/05，2025/05/15，2025/08/12，2026/3/28</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -5510,12 +5510,12 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>BV1SwtfzPEQQ</t>
+          <t>BV132XyB5Ev6，BV1SwtfzPEQQ</t>
         </is>
       </c>
       <c r="J124" t="inlineStr"/>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6834,12 +6834,12 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>BV15uzuB1ECd</t>
+          <t>BV18mXyBCEzT，BV15uzuB1ECd</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/1/16，2026/2/7</t>
+          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/1/16，2026/2/7，2026/3/28</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -6998,12 +6998,12 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>BV1MCGzz6E9p</t>
+          <t>BV145XyBKEtS，BV1MCGzz6E9p</t>
         </is>
       </c>
       <c r="J161" t="inlineStr"/>
@@ -7027,7 +7027,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7038,12 +7038,12 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>BV19spgzxEJp</t>
+          <t>BV1gmXyBCEEx，BV19spgzxEJp</t>
         </is>
       </c>
       <c r="J162" t="inlineStr"/>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7</t>
+          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7，2026/3/28</t>
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
@@ -9878,12 +9878,12 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>BV1r3NAzgErm，BV1crarzEEsn</t>
+          <t>BV1tzXLB4EDj，BV1r3NAzgErm，BV1crarzEEsn</t>
         </is>
       </c>
       <c r="J233" t="inlineStr"/>
@@ -14835,7 +14835,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/31，2025/06/03，2025/06/14，2025/09/10</t>
+          <t>2025/04/17，2025/05/31，2025/06/03，2025/06/14，2025/09/10，2026/3/28</t>
         </is>
       </c>
       <c r="F358" t="inlineStr"/>
@@ -14846,12 +14846,12 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>BV1ccHRzoEKY，BV1Q17gzVE5c</t>
+          <t>BV132XyB5ENR，BV1ccHRzoEKY，BV1Q17gzVE5c</t>
         </is>
       </c>
       <c r="J358" t="inlineStr"/>
@@ -22839,7 +22839,7 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9</t>
+          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9，2026/3/28</t>
         </is>
       </c>
       <c r="F567" t="inlineStr"/>
@@ -22850,12 +22850,12 @@
       </c>
       <c r="H567" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I567" t="inlineStr">
         <is>
-          <t>BV1ttmJBQETy</t>
+          <t>BV1GxX1BmEgs，BV1ttmJBQETy</t>
         </is>
       </c>
       <c r="J567" t="inlineStr"/>
@@ -23787,7 +23787,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6</t>
+          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6，2026/3/28</t>
         </is>
       </c>
       <c r="F592" t="inlineStr"/>
@@ -23798,12 +23798,12 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
         <is>
-          <t>BV1uhbPzSE6S</t>
+          <t>BV1GaXLBwEud，BV1uhbPzSE6S</t>
         </is>
       </c>
       <c r="J592" t="inlineStr"/>
@@ -28079,7 +28079,7 @@
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>2025/10/23，2025/10/25，2025/12/12，2026/1/19</t>
+          <t>2025/10/23，2025/10/25，2025/12/12，2026/1/19，2026/3/28</t>
         </is>
       </c>
       <c r="F705" t="inlineStr"/>
@@ -28090,12 +28090,12 @@
       </c>
       <c r="H705" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I705" t="inlineStr">
         <is>
-          <t>BV1UfsZzsEJb</t>
+          <t>BV132XyB5Esk，BV1UfsZzsEJb</t>
         </is>
       </c>
       <c r="J705" t="inlineStr"/>
@@ -29943,7 +29943,7 @@
       </c>
       <c r="E755" t="inlineStr">
         <is>
-          <t>2025/12/11，2025/12/12，2025/12/17，2026/1/2，2026/1/5，2026/1/11，2026/1/17，2026/1/29，2026/2/9</t>
+          <t>2025/12/11，2025/12/12，2025/12/17，2026/1/2，2026/1/5，2026/1/11，2026/1/17，2026/1/29，2026/2/9，2026/3/28</t>
         </is>
       </c>
       <c r="F755" t="inlineStr"/>
@@ -29954,12 +29954,12 @@
       </c>
       <c r="H755" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I755" t="inlineStr">
         <is>
-          <t>BV1FekxB5Etj</t>
+          <t>BV1UzXLBxEGd，BV1FekxB5Etj</t>
         </is>
       </c>
       <c r="J755" t="inlineStr"/>
@@ -31099,7 +31099,7 @@
       </c>
       <c r="E785" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12</t>
+          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28</t>
         </is>
       </c>
       <c r="F785" t="inlineStr"/>
@@ -31110,7 +31110,7 @@
       </c>
       <c r="H785" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I785" t="inlineStr">
@@ -32275,7 +32275,7 @@
       </c>
       <c r="E817" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/25</t>
+          <t>2026/3/13，2026/3/25，2026/3/28</t>
         </is>
       </c>
       <c r="F817" t="inlineStr"/>
@@ -32286,10 +32286,14 @@
       </c>
       <c r="H817" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I817" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>BV1snXyBwEzu，BV1m1X7BFE8d</t>
+        </is>
+      </c>
       <c r="J817" t="inlineStr">
         <is>
           <t>游戏</t>
@@ -32347,7 +32351,7 @@
       </c>
       <c r="E819" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/14</t>
+          <t>2026/3/13，2026/3/14，2026/3/28</t>
         </is>
       </c>
       <c r="F819" t="inlineStr"/>
@@ -32358,10 +32362,14 @@
       </c>
       <c r="H819" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I819" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>BV1UzXLBxErn</t>
+        </is>
+      </c>
       <c r="J819" t="inlineStr"/>
     </row>
     <row r="820">
@@ -32749,8 +32757,48 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I830" t="inlineStr"/>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>BV1XYX7BMEZn</t>
+        </is>
+      </c>
       <c r="J830" t="inlineStr"/>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr"/>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>又三郎</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr"/>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>ヨルシカ (Yorushika)</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>2026/3/28</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr"/>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>BV1m6XLBREbN</t>
+        </is>
+      </c>
+      <c r="J831" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Mar 31, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>58</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13，2026/3/14</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13，2026/3/14，2026/3/31</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -12935,7 +12935,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/9，2026/1/24</t>
+          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/9，2026/1/24，2026/3/31</t>
         </is>
       </c>
       <c r="F310" t="inlineStr"/>
@@ -12946,7 +12946,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/1/14，2026/1/23，2026/2/12</t>
+          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/1/14，2026/1/23，2026/2/12，2026/3/31</t>
         </is>
       </c>
       <c r="F337" t="inlineStr"/>
@@ -13994,7 +13994,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -15281,7 +15281,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I369" t="inlineStr"/>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>BV13nh2z5ErP，BV1C3NqzMEmt</t>
+        </is>
+      </c>
       <c r="J369" t="inlineStr"/>
     </row>
     <row r="370">
@@ -16083,7 +16087,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30</t>
+          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31</t>
         </is>
       </c>
       <c r="F390" t="inlineStr"/>
@@ -16094,7 +16098,7 @@
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I390" t="inlineStr">
@@ -16365,7 +16369,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I397" t="inlineStr"/>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>BV1xHJVz5EN6</t>
+        </is>
+      </c>
       <c r="J397" t="inlineStr"/>
     </row>
     <row r="398">
@@ -24867,7 +24875,7 @@
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>2025/08/24，2025/09/20，2025/10/07，2025/11/9，2025/11/21，2026/2/25</t>
+          <t>2025/08/24，2025/09/20，2025/10/07，2025/11/9，2025/11/21，2026/2/25，2026/3/31</t>
         </is>
       </c>
       <c r="F620" t="inlineStr"/>
@@ -24878,7 +24886,7 @@
       </c>
       <c r="H620" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I620" t="inlineStr">
@@ -24943,7 +24951,7 @@
       </c>
       <c r="E622" t="inlineStr">
         <is>
-          <t>2025/08/26，2025/08/16，2025/11/13，2025/12/9，2026/1/29，2026/2/19</t>
+          <t>2025/08/26，2025/08/16，2025/11/13，2025/12/9，2026/1/29，2026/2/19，2026/3/31</t>
         </is>
       </c>
       <c r="F622" t="inlineStr"/>
@@ -24954,7 +24962,7 @@
       </c>
       <c r="H622" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I622" t="inlineStr">
@@ -30903,7 +30911,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -30914,7 +30922,7 @@
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I780" t="inlineStr">
@@ -31383,7 +31391,7 @@
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31</t>
         </is>
       </c>
       <c r="F792" t="inlineStr"/>
@@ -31394,7 +31402,7 @@
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
@@ -31999,7 +32007,7 @@
       </c>
       <c r="E807" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31</t>
         </is>
       </c>
       <c r="F807" t="inlineStr"/>
@@ -32010,7 +32018,7 @@
       </c>
       <c r="H807" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I807" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Apr 1, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J831"/>
+  <dimension ref="A1:J834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/21，2025/04/19，2025/05/11，2025/06/03，2026/1/19，2026/1/25，2026/2/25</t>
+          <t>2025/03/06，2025/03/21，2025/04/19，2025/05/11，2025/06/03，2026/1/19，2026/1/25，2026/2/25，2026/4/1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/3/27</t>
+          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/3/27，2026/4/1</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/12，2025/05/23，2025/06/26，2025/07/08，2025/07/31，2025/08/22，2025/09/02，2025/09/15，2025/10/10，2025/11/3，2026/2/2</t>
+          <t>2025/03/14，2025/04/02，2025/05/12，2025/05/23，2025/06/26，2025/07/08，2025/07/31，2025/08/22，2025/09/02，2025/09/15，2025/10/10，2025/11/3，2026/2/2，2026/4/1</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/06/26，2025/10/24</t>
+          <t>2025/03/21，2025/06/26，2025/10/24，2026/4/1</t>
         </is>
       </c>
       <c r="F176" t="inlineStr"/>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12</t>
+          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12，2026/4/1</t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16315,7 +16315,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/3，2025/12/30，2026/1/9</t>
+          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/3，2025/12/30，2026/1/9，2026/4/1</t>
         </is>
       </c>
       <c r="F396" t="inlineStr"/>
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
@@ -18275,7 +18275,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/11/28</t>
+          <t>2025/05/18，2025/11/28，2026/4/1</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -18286,10 +18286,14 @@
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I447" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>BV18u9EBqE8e，BV1rSJGzKE5z</t>
+        </is>
+      </c>
       <c r="J447" t="inlineStr"/>
     </row>
     <row r="448">
@@ -20155,7 +20159,7 @@
       </c>
       <c r="E496" t="inlineStr">
         <is>
-          <t>2025/6/1</t>
+          <t>2025/6/1，2026/4/1</t>
         </is>
       </c>
       <c r="F496" t="inlineStr"/>
@@ -20166,10 +20170,14 @@
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I496" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>BV1Du9EBqE5T，BV1cz7Dz6EQU</t>
+        </is>
+      </c>
       <c r="J496" t="inlineStr"/>
     </row>
     <row r="497">
@@ -21519,7 +21527,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1</t>
         </is>
       </c>
       <c r="F532" t="inlineStr"/>
@@ -21530,7 +21538,7 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
@@ -24595,7 +24603,7 @@
       </c>
       <c r="E613" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1</t>
         </is>
       </c>
       <c r="F613" t="inlineStr"/>
@@ -24606,7 +24614,7 @@
       </c>
       <c r="H613" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I613" t="inlineStr">
@@ -27627,7 +27635,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25</t>
+          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25，2026/4/1</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -27642,7 +27650,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">
@@ -29539,7 +29547,7 @@
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1</t>
         </is>
       </c>
       <c r="F744" t="inlineStr"/>
@@ -29550,7 +29558,7 @@
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I744" t="inlineStr">
@@ -30911,7 +30919,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -30922,7 +30930,7 @@
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I780" t="inlineStr">
@@ -33003,6 +33011,122 @@
         </is>
       </c>
       <c r="J831" t="inlineStr"/>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>勇气大爆发</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr"/>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>贝乐虎儿歌/土豆王国小乐队</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>2025/12/24，2025/12/25，2026/4/1</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr"/>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>BV1B997BUEMa，BV1DjB2BrEiu，BV1FGBRB7EuH</t>
+        </is>
+      </c>
+      <c r="J832" t="inlineStr"/>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>832</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>吴哥窟</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr"/>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>吴雨霏</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>2026/4/1</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr"/>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>粤语</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr"/>
+      <c r="J833" t="inlineStr"/>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>833</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>L!!!!ght</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr"/>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/Meredith Bull</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>2026/4/1</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr"/>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr"/>
+      <c r="J834" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 2, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J834"/>
+  <dimension ref="A1:J835"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/7，2026/3/6</t>
+          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/7，2026/3/6，2026/4/2</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7534,12 +7534,12 @@
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
-          <t>林俊杰</t>
+          <t>郭静</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15，2026/4/2</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/04，2025/04/19，2025/05/26，2025/06/02，2025/07/27，2025/09/06，2025/09/08，2025/10/11</t>
+          <t>2025/03/21，2025/04/04，2025/04/19，2025/05/26，2025/06/02，2025/07/27，2025/09/06，2025/09/08，2025/10/11，2026/4/2</t>
         </is>
       </c>
       <c r="F178" t="inlineStr"/>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -12303,7 +12303,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/2/14，2026/3/5</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/2/14，2026/3/5，2026/4/2</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -12314,7 +12314,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -12935,7 +12935,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/9，2026/1/24，2026/3/31</t>
+          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/9，2026/1/24，2026/3/31，2026/4/2</t>
         </is>
       </c>
       <c r="F310" t="inlineStr"/>
@@ -12946,7 +12946,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -23731,7 +23731,7 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2</t>
         </is>
       </c>
       <c r="F590" t="inlineStr"/>
@@ -23742,7 +23742,7 @@
       </c>
       <c r="H590" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I590" t="inlineStr">
@@ -26043,7 +26043,7 @@
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>2025/09/02，2025/09/22</t>
+          <t>2025/09/02，2025/09/22，2026/4/2</t>
         </is>
       </c>
       <c r="F651" t="inlineStr"/>
@@ -26054,10 +26054,14 @@
       </c>
       <c r="H651" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I651" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>BV1YYnwzcEZS，BV18H9wBsEuF</t>
+        </is>
+      </c>
       <c r="J651" t="inlineStr"/>
     </row>
     <row r="652">
@@ -27467,7 +27471,7 @@
       </c>
       <c r="E689" t="inlineStr">
         <is>
-          <t>2025/10/07，2025/10/12，2025/10/22，2026/3/24</t>
+          <t>2025/10/07，2025/10/12，2025/10/22，2026/3/24，2026/4/2</t>
         </is>
       </c>
       <c r="F689" t="inlineStr"/>
@@ -27478,7 +27482,7 @@
       </c>
       <c r="H689" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I689" t="inlineStr">
@@ -28355,7 +28359,7 @@
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>2025/10/23，2025/10/28</t>
+          <t>2025/10/23，2025/10/28，2026/4/2</t>
         </is>
       </c>
       <c r="F712" t="inlineStr"/>
@@ -28366,7 +28370,7 @@
       </c>
       <c r="H712" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I712" t="inlineStr"/>
@@ -30335,7 +30339,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -30346,7 +30350,7 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -32819,7 +32823,7 @@
       </c>
       <c r="E827" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2</t>
         </is>
       </c>
       <c r="F827" t="inlineStr"/>
@@ -32830,7 +32834,7 @@
       </c>
       <c r="H827" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I827" t="inlineStr">
@@ -33085,7 +33089,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I833" t="inlineStr"/>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>BV18qXfB2Epc</t>
+        </is>
+      </c>
       <c r="J833" t="inlineStr"/>
     </row>
     <row r="834">
@@ -33121,12 +33129,52 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I834" t="inlineStr"/>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>BV1SqXfB2EWL</t>
+        </is>
+      </c>
       <c r="J834" t="inlineStr">
         <is>
           <t>游戏</t>
         </is>
       </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>834</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>假如爱有天意</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr"/>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>李健</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>2026/4/2</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr"/>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr"/>
+      <c r="J835" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 5, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -18083,7 +18083,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12，2026/4/5</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -18094,12 +18094,12 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t>BV1J67NzGEDg，BV173fNB4EZX</t>
+          <t>BV1J67NzGEDg，BV173fNB4EZX，BV137SXBxEPC</t>
         </is>
       </c>
       <c r="J442" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 8, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -963,7 +963,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/4，2026/1/24，2026/1/24，2026/2/19，2026/2/25，2026/3/13</t>
+          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/4，2026/1/24，2026/1/24，2026/2/19，2026/2/25，2026/3/13，2026/4/8</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>59</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/04，2025/04/28，2025/07/08，2025/07/21，2025/08/18，2026/2/9</t>
+          <t>2025/03/09，2025/04/04，2025/04/28，2025/07/08，2025/07/21，2025/08/18，2026/2/9，2026/4/8</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/30，2025/04/17，2025/04/21，2025/05/05，2025/05/13，2025/05/20，2025/06/06，2025/06/20，2025/06/27，2025/07/05，2025/07/31，2025/08/24，2025/08/29，2025/09/20，2025/09/30，2025/10/22，2025/11/26，2026/1/15，2026/2/14</t>
+          <t>2025/03/13，2025/03/30，2025/04/17，2025/04/21，2025/05/05，2025/05/13，2025/05/20，2025/06/06，2025/06/20，2025/06/27，2025/07/05，2025/07/31，2025/08/24，2025/08/29，2025/09/20，2025/09/30，2025/10/22，2025/11/26，2026/1/15，2026/2/14，2026/4/8</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4178,12 +4178,12 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>BV1DUQNYKE5T</t>
+          <t>BV1uNDEB8EDJ，BV1DUQNYKE5T</t>
         </is>
       </c>
       <c r="J91" t="inlineStr"/>
@@ -5019,7 +5019,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/11，2025/04/25，2025/06/05，2025/06/15，2025/07/07，2025/09/11，2025/10/10，2025/11/14，2025/12/9</t>
+          <t>2025/03/14，2025/04/11，2025/04/25，2025/06/05，2025/06/15，2025/07/07，2025/09/11，2025/10/10，2025/11/14，2025/12/9，2026/4/8</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/05/22，2025/07/10，2025/09/08，2025/10/09，2025/11/1，2026/1/15</t>
+          <t>2025/03/18，2025/03/25，2025/05/22，2025/07/10，2025/09/08，2025/10/09，2025/11/1，2026/1/15，2026/4/8</t>
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/06/28，2025/08/04，2026/1/19</t>
+          <t>2025/03/21，2025/06/28，2025/08/04，2026/1/19，2026/4/8</t>
         </is>
       </c>
       <c r="F163" t="inlineStr"/>
@@ -7078,7 +7078,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -8743,7 +8743,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/18，2025/04/24，2025/06/23，2025/09/29，2025/12/17</t>
+          <t>2025/03/25，2025/04/18，2025/04/24，2025/06/23，2025/09/29，2025/12/17，2026/4/8</t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
@@ -8754,7 +8754,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9962,7 +9962,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10846,7 +10846,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -11639,7 +11639,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/14，2025/04/24，2025/06/01，2025/07/06，2025/09/21，2025/11/3，2025/12/12，2025/12/26</t>
+          <t>2025/04/03，2025/04/14，2025/04/24，2025/06/01，2025/07/06，2025/09/21，2025/11/3，2025/12/12，2025/12/26，2026/4/8</t>
         </is>
       </c>
       <c r="F277" t="inlineStr"/>
@@ -11650,7 +11650,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25，2026/4/8</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12906,7 +12906,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -17887,7 +17887,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>2025/05/12，2025/05/22，2025/05/25，2025/07/20，2025/09/12，2026/1/15，2026/1/24，2026/1/30</t>
+          <t>2025/05/12，2025/05/22，2025/05/25，2025/07/20，2025/09/12，2026/1/15，2026/1/24，2026/1/30，2026/4/8</t>
         </is>
       </c>
       <c r="F437" t="inlineStr"/>
@@ -17898,7 +17898,7 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
@@ -19095,7 +19095,7 @@
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/1/28</t>
+          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/1/28，2026/4/8</t>
         </is>
       </c>
       <c r="F468" t="inlineStr"/>
@@ -19106,7 +19106,7 @@
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I468" t="inlineStr">
@@ -24335,7 +24335,7 @@
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14</t>
+          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8</t>
         </is>
       </c>
       <c r="F606" t="inlineStr"/>
@@ -24346,7 +24346,7 @@
       </c>
       <c r="H606" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I606" t="inlineStr">
@@ -24603,7 +24603,7 @@
       </c>
       <c r="E613" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1，2026/4/8</t>
         </is>
       </c>
       <c r="F613" t="inlineStr"/>
@@ -24614,12 +24614,12 @@
       </c>
       <c r="H613" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I613" t="inlineStr">
         <is>
-          <t>BV1u4bwzyEez</t>
+          <t>BV1SNDEBbEXQ，BV1u4bwzyEez</t>
         </is>
       </c>
       <c r="J613" t="inlineStr"/>
@@ -24763,7 +24763,7 @@
       </c>
       <c r="E617" t="inlineStr">
         <is>
-          <t>2025/08/21，2026/1/16，2026/2/2，2026/3/17</t>
+          <t>2025/08/21，2026/1/16，2026/2/2，2026/3/17，2026/4/8</t>
         </is>
       </c>
       <c r="F617" t="inlineStr"/>
@@ -24774,7 +24774,7 @@
       </c>
       <c r="H617" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I617" t="inlineStr">
@@ -26383,7 +26383,7 @@
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/1，2025/12/6，2025/12/12，2026/1/19</t>
+          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/1，2025/12/6，2025/12/12，2026/1/19，2026/4/8</t>
         </is>
       </c>
       <c r="F660" t="inlineStr"/>
@@ -26394,7 +26394,7 @@
       </c>
       <c r="H660" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I660" t="inlineStr">
@@ -29551,7 +29551,7 @@
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8</t>
         </is>
       </c>
       <c r="F744" t="inlineStr"/>
@@ -29562,7 +29562,7 @@
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I744" t="inlineStr">
@@ -29891,7 +29891,7 @@
       </c>
       <c r="E753" t="inlineStr">
         <is>
-          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25</t>
+          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25，2026/4/8</t>
         </is>
       </c>
       <c r="F753" t="inlineStr"/>
@@ -29902,7 +29902,7 @@
       </c>
       <c r="H753" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I753" t="inlineStr">
@@ -32823,7 +32823,7 @@
       </c>
       <c r="E827" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8</t>
         </is>
       </c>
       <c r="F827" t="inlineStr"/>
@@ -32834,12 +32834,12 @@
       </c>
       <c r="H827" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I827" t="inlineStr">
         <is>
-          <t>BV1ugQSBnE8x</t>
+          <t>BV1nCD7ByEXM，BV1ugQSBnE8x</t>
         </is>
       </c>
       <c r="J827" t="inlineStr">
@@ -33173,7 +33173,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I835" t="inlineStr"/>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>BV13x9KBME9P</t>
+        </is>
+      </c>
       <c r="J835" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: Update song list to Apr 9, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J835"/>
+  <dimension ref="A1:J842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/1/10，2026/1/24</t>
+          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/1/10，2026/1/24，2026/4/9</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1054,12 +1054,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>BV1FSjUzwEfm</t>
+          <t>BV1yYD4BGE48，BV1FSjUzwEfm</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/1/15，2026/2/14，2026/3/4</t>
+          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/1/15，2026/2/14，2026/3/4，2026/4/9</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/4/9</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3182,7 +3182,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4047,7 +4047,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/03，2025/05/26，2025/06/01，2025/06/06，2025/09/08，2025/09/12</t>
+          <t>2025/03/13，2025/04/03，2025/05/26，2025/06/01，2025/06/06，2025/09/08，2025/09/12，2026/4/9</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/9，2026/1/23，2026/2/18</t>
+          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/9，2026/1/23，2026/2/18，2026/4/9</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/19，2025/05/20，2025/07/26，2025/08/16，2025/12/11</t>
+          <t>2025/03/14，2025/05/19，2025/05/20，2025/07/26，2025/08/16，2025/12/11，2026/4/9</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4498,12 +4498,12 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>BV1ynm3BsEbZ，BV1ZzQuYZEy2</t>
+          <t>BV1SWD4BEEB7，BV1ynm3BsEbZ，BV1ZzQuYZEy2</t>
         </is>
       </c>
       <c r="J99" t="inlineStr"/>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/15，2025/06/06，2025/07/31，2025/09/12</t>
+          <t>2025/03/14，2025/05/15，2025/06/06，2025/07/31，2025/09/12，2026/4/9</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/17，2025/04/25，2025/06/23，2025/08/30，2025/09/12，2025/09/15，2025/11/19，2026/2/8</t>
+          <t>2025/03/14，2025/04/17，2025/04/25，2025/06/23，2025/08/30，2025/09/12，2025/09/15，2025/11/19，2026/2/8，2026/4/9</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -4738,7 +4738,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/1/2，2026/1/30</t>
+          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/1/2，2026/1/30，2026/4/9</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/23，2025/07/22</t>
+          <t>2025/03/14，2025/05/23，2025/07/22，2026/4/9</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5430,7 +5430,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5630,7 +5630,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/9，2025/12/4，2026/1/1，2026/1/29</t>
+          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/9，2025/12/4，2026/1/1，2026/1/29，2026/4/9</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5</t>
+          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5，2026/4/9</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/05/13，2025/06/10，2025/08/21，2025/11/19，2026/1/10</t>
+          <t>2025/03/19，2025/04/07，2025/05/13，2025/06/10，2025/08/21，2025/11/19，2026/1/10，2026/4/9</t>
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
@@ -6310,7 +6310,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -6499,7 +6499,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6510,12 +6510,12 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>BV19QnGzZE9f，BV1DZiFBgEhH，BV13rQZYQEem，BV1HD7VzqEQy，BV1UwSMBoE3e</t>
+          <t>BV1cADbBrESS，BV19QnGzZE9f，BV1DZiFBgEhH，BV13rQZYQEem，BV1HD7VzqEQy，BV1UwSMBoE3e</t>
         </is>
       </c>
       <c r="J149" t="inlineStr"/>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/02，2025/05/18，2025/06/19，2025/07/07，2025/09/04，2025/09/12，2026/1/19</t>
+          <t>2025/03/24，2025/04/02，2025/05/18，2025/06/19，2025/07/07，2025/09/04，2025/09/12，2026/1/19，2026/4/9</t>
         </is>
       </c>
       <c r="F191" t="inlineStr"/>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/7，2026/1/17，2026/2/14</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/7，2026/1/17，2026/2/14，2026/4/9</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8314,7 +8314,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/06/23，2026/1/9</t>
+          <t>2025/03/24，2025/06/23，2026/1/9，2026/4/9</t>
         </is>
       </c>
       <c r="F195" t="inlineStr"/>
@@ -8354,7 +8354,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/06，2025/05/01，2025/06/23，2025/07/09，2025/09/05，2025/09/15，2025/10/16，2025/11/19，2025/12/17</t>
+          <t>2025/03/25，2025/04/06，2025/05/01，2025/06/23，2025/07/09，2025/09/05，2025/09/15，2025/10/16，2025/11/19，2025/12/17，2026/4/9</t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
@@ -8834,7 +8834,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25</t>
+          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25，2026/4/9</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -9126,7 +9126,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -10439,7 +10439,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/04，2025/04/26，2025/05/06，2025/05/18，2025/06/10，2025/07/03，2025/07/10，2025/07/24，2025/08/16，2025/09/18，2025/10/03，2025/11/1，2026/2/14</t>
+          <t>2025/03/30，2025/04/04，2025/04/26，2025/05/06，2025/05/18，2025/06/10，2025/07/03，2025/07/10，2025/07/24，2025/08/16，2025/09/18，2025/10/03，2025/11/1，2026/2/14，2026/4/9</t>
         </is>
       </c>
       <c r="F247" t="inlineStr"/>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -11355,7 +11355,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/08，2025/05/04，2025/05/08，2025/07/31</t>
+          <t>2025/04/02，2025/04/08，2025/05/04，2025/05/08，2025/07/31，2026/4/9</t>
         </is>
       </c>
       <c r="F270" t="inlineStr"/>
@@ -11366,12 +11366,12 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>BV19y8CzTEj5</t>
+          <t>BV1U4D4BjE35，BV19y8CzTEj5</t>
         </is>
       </c>
       <c r="J270" t="inlineStr"/>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/1/25，2026/2/14</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/1/25，2026/2/14，2026/4/9</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11486,7 +11486,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -11839,7 +11839,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/05/12，2025/05/18，2025/06/20，2025/07/05，2025/07/14，2025/12/23，2026/1/30</t>
+          <t>2025/04/04，2025/05/12，2025/05/18，2025/06/20，2025/07/05，2025/07/14，2025/12/23，2026/1/30，2026/4/9</t>
         </is>
       </c>
       <c r="F282" t="inlineStr"/>
@@ -11850,12 +11850,12 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>BV1zgKNzkEV1</t>
+          <t>BV1TkDWBzEWp，BV1zgKNzkEV1</t>
         </is>
       </c>
       <c r="J282" t="inlineStr"/>
@@ -12075,7 +12075,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/04/18，2025/06/06，2025/07/07，2025/08/04，2025/08/12，2025/09/17</t>
+          <t>2025/04/04，2025/04/18，2025/06/06，2025/07/07，2025/08/04，2025/08/12，2025/09/17，2026/4/9</t>
         </is>
       </c>
       <c r="F288" t="inlineStr"/>
@@ -12086,7 +12086,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>2025/04/06，2025/04/10，2025/06/20，2025/12/23</t>
+          <t>2025/04/06，2025/04/10，2025/06/20，2025/12/23，2026/4/9</t>
         </is>
       </c>
       <c r="F296" t="inlineStr"/>
@@ -12394,7 +12394,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/08/04，2025/09/12，2025/09/12</t>
+          <t>2025/04/11，2025/08/04，2025/09/12，2025/09/12，2026/4/9</t>
         </is>
       </c>
       <c r="F331" t="inlineStr"/>
@@ -13754,12 +13754,12 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>BV186tVz6EuE</t>
+          <t>BV186tVz6EuE，BV1qQdQYsEtx</t>
         </is>
       </c>
       <c r="J331" t="inlineStr"/>
@@ -14431,7 +14431,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/25，2025/05/30，2025/06/17，2025/09/26，2025/10/03，2025/11/3，2025/12/23</t>
+          <t>2025/04/15，2025/04/25，2025/05/30，2025/06/17，2025/09/26，2025/10/03，2025/11/3，2025/12/23，2026/4/9</t>
         </is>
       </c>
       <c r="F348" t="inlineStr"/>
@@ -14442,12 +14442,12 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t>BV1WgnVz1EfK，BV1G2LnziE1H</t>
+          <t>BV18yDtB9Eua，BV1WgnVz1EfK，BV1G2LnziE1H</t>
         </is>
       </c>
       <c r="J348" t="inlineStr"/>
@@ -15387,7 +15387,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/9，2025/11/26，2025/12/5，2025/12/6，2026/1/1，2026/1/29，2026/3/1</t>
+          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/9，2025/11/26，2025/12/5，2025/12/6，2026/1/1，2026/1/29，2026/3/1，2026/4/9</t>
         </is>
       </c>
       <c r="F372" t="inlineStr"/>
@@ -15398,7 +15398,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/19，2025/07/25，2025/08/07，2025/09/15，2025/09/29，2026/1/5，2026/2/14</t>
+          <t>2025/04/21，2025/05/19，2025/07/25，2025/08/07，2025/09/15，2025/09/29，2026/1/5，2026/2/14，2026/4/9</t>
         </is>
       </c>
       <c r="F378" t="inlineStr"/>
@@ -15638,7 +15638,7 @@
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I378" t="inlineStr">
@@ -16163,7 +16163,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/23，2025/12/5，2026/2/14</t>
+          <t>2025/04/25，2025/06/23，2025/12/5，2026/2/14，2026/4/9</t>
         </is>
       </c>
       <c r="F392" t="inlineStr"/>
@@ -16174,7 +16174,7 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
@@ -16511,7 +16511,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/06/02，2025/06/09，2025/07/09，2025/07/14，2025/08/26，2025/11/21，2025/12/17，2026/1/9</t>
+          <t>2025/04/27，2025/06/02，2025/06/09，2025/07/09，2025/07/14，2025/08/26，2025/11/21，2025/12/17，2026/1/9，2026/4/9</t>
         </is>
       </c>
       <c r="F401" t="inlineStr"/>
@@ -16522,7 +16522,7 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
@@ -16551,7 +16551,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/05/04，2025/05/26，2025/06/08，2025/08/28，2025/10/18，2025/11/18，2025/12/24，2026/1/29，2026/2/27</t>
+          <t>2025/04/27，2025/05/04，2025/05/26，2025/06/08，2025/08/28，2025/10/18，2025/11/18，2025/12/24，2026/1/29，2026/2/27，2026/4/9</t>
         </is>
       </c>
       <c r="F402" t="inlineStr"/>
@@ -16562,7 +16562,7 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/05/29，2025/06/17，2025/07/11，2025/08/03，2025/09/22</t>
+          <t>2025/04/27，2025/05/29，2025/06/17，2025/07/11，2025/08/03，2025/09/22，2026/4/9</t>
         </is>
       </c>
       <c r="F404" t="inlineStr"/>
@@ -16638,7 +16638,7 @@
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I404" t="inlineStr">
@@ -16791,7 +16791,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/11/18，2026/2/14</t>
+          <t>2025/04/28，2025/11/18，2026/2/14，2026/4/9</t>
         </is>
       </c>
       <c r="F408" t="inlineStr"/>
@@ -16802,7 +16802,7 @@
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
@@ -17927,7 +17927,7 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>2025/05/15，2025/10/31</t>
+          <t>2025/05/15，2025/10/31，2026/4/9</t>
         </is>
       </c>
       <c r="F438" t="inlineStr"/>
@@ -17938,10 +17938,14 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I438" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>BV1FADbBrErN，BV1Rgy9BnEGr，BV1aRNSz4EFN</t>
+        </is>
+      </c>
       <c r="J438" t="inlineStr"/>
     </row>
     <row r="439">
@@ -18123,7 +18127,7 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/27，2025/07/10，2026/3/9</t>
+          <t>2025/05/18，2025/06/27，2025/07/10，2026/3/9，2026/4/9</t>
         </is>
       </c>
       <c r="F443" t="inlineStr"/>
@@ -18134,7 +18138,7 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I443" t="inlineStr">
@@ -18507,7 +18511,7 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/07/13，2025/10/30，2025/10/31，2025/12/24，2026/1/9</t>
+          <t>2025/05/19，2025/07/13，2025/10/30，2025/10/31，2025/12/24，2026/1/9，2026/4/9</t>
         </is>
       </c>
       <c r="F453" t="inlineStr"/>
@@ -18518,7 +18522,7 @@
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I453" t="inlineStr">
@@ -18627,7 +18631,7 @@
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/12，2025/09/02，2025/12/5</t>
+          <t>2025/05/22，2025/09/12，2025/09/02，2025/12/5，2026/4/9</t>
         </is>
       </c>
       <c r="F456" t="inlineStr"/>
@@ -18638,7 +18642,7 @@
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I456" t="inlineStr">
@@ -19369,7 +19373,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I475" t="inlineStr"/>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>BV1Ns7GziETH</t>
+        </is>
+      </c>
       <c r="J475" t="inlineStr"/>
     </row>
     <row r="476">
@@ -19579,7 +19587,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/08/13，2025/08/26，2025/08/26，2025/09/20，2025/09/26，2025/11/21</t>
+          <t>2025/05/30，2025/08/13，2025/08/26，2025/08/26，2025/09/20，2025/09/26，2025/11/21，2026/4/9</t>
         </is>
       </c>
       <c r="F481" t="inlineStr"/>
@@ -19590,12 +19598,12 @@
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I481" t="inlineStr">
         <is>
-          <t>BV1akvKzrEM3</t>
+          <t>BV1SzDWBrEuy，BV1akvKzrEM3</t>
         </is>
       </c>
       <c r="J481" t="inlineStr"/>
@@ -22935,7 +22943,7 @@
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>2025/07/06，2025/07/18，2025/12/31</t>
+          <t>2025/07/06，2025/07/18，2025/12/31，2026/4/9</t>
         </is>
       </c>
       <c r="F569" t="inlineStr"/>
@@ -22946,10 +22954,14 @@
       </c>
       <c r="H569" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I569" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>BV1hC32zfE4f，BV1jbuRzsE6i，BV1rWv9BgEYk</t>
+        </is>
+      </c>
       <c r="J569" t="inlineStr"/>
     </row>
     <row r="570">
@@ -22971,7 +22983,7 @@
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>2025/7/7</t>
+          <t>2025/7/7，2026/4/9</t>
         </is>
       </c>
       <c r="F570" t="inlineStr"/>
@@ -22982,10 +22994,14 @@
       </c>
       <c r="H570" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I570" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>BV1j4DtBKEfp，BV12LGpz9ERg</t>
+        </is>
+      </c>
       <c r="J570" t="inlineStr"/>
     </row>
     <row r="571">
@@ -23047,7 +23063,7 @@
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>2025/07/07，2025/09/30</t>
+          <t>2025/07/07，2025/09/30，2026/4/9</t>
         </is>
       </c>
       <c r="F572" t="inlineStr"/>
@@ -23058,10 +23074,14 @@
       </c>
       <c r="H572" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I572" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>BV1pdDxBBEpZ，BV1uEGLzzEUw</t>
+        </is>
+      </c>
       <c r="J572" t="inlineStr"/>
     </row>
     <row r="573">
@@ -23083,7 +23103,7 @@
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>2025/07/07，2025/07/31，2025/09/11，2025/10/11，2025/11/7，2025/11/12，2025/12/9，2026/1/14，2026/1/30</t>
+          <t>2025/07/07，2025/07/31，2025/09/11，2025/10/11，2025/11/7，2025/11/12，2025/12/9，2026/1/14，2026/1/30，2026/4/9</t>
         </is>
       </c>
       <c r="F573" t="inlineStr"/>
@@ -23094,7 +23114,7 @@
       </c>
       <c r="H573" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I573" t="inlineStr">
@@ -23387,7 +23407,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/09/30，2025/10/31，2025/12/4，2026/1/23，2026/2/12，2026/3/17</t>
+          <t>2025/07/11，2025/09/30，2025/10/31，2025/12/4，2026/1/23，2026/2/12，2026/3/17，2026/4/9</t>
         </is>
       </c>
       <c r="F581" t="inlineStr"/>
@@ -23398,7 +23418,7 @@
       </c>
       <c r="H581" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I581" t="inlineStr">
@@ -24027,7 +24047,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>2025/07/23，2025/12/12，2026/2/25</t>
+          <t>2025/07/23，2025/12/12，2026/2/25，2026/4/9</t>
         </is>
       </c>
       <c r="F598" t="inlineStr"/>
@@ -24038,7 +24058,7 @@
       </c>
       <c r="H598" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I598" t="inlineStr">
@@ -33179,6 +33199,278 @@
         </is>
       </c>
       <c r="J835" t="inlineStr"/>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Poker Face</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>扑克脸</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Lady Gaga</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr"/>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>BV1aYDWB1E8a</t>
+        </is>
+      </c>
+      <c r="J836" t="inlineStr"/>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>836</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>最炫民族风</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr"/>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>凤凰传奇</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr"/>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>BV1UsD4BmEbA</t>
+        </is>
+      </c>
+      <c r="J837" t="inlineStr"/>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>837</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>不得不爱</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr"/>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>潘玮柏/弦子</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr"/>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>BV1sXDxB6Ewz</t>
+        </is>
+      </c>
+      <c r="J838" t="inlineStr"/>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>838</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>怎么办</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr"/>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>S.H.E</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr"/>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>BV1HjDxBNENK</t>
+        </is>
+      </c>
+      <c r="J839" t="inlineStr"/>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>839</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>爱情买卖</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr"/>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>慕容晓晓</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr"/>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr"/>
+      <c r="J840" t="inlineStr"/>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>840</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Bad Romance</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr"/>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Lady Gaga</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr"/>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr"/>
+      <c r="J841" t="inlineStr"/>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>841</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>北京欢迎你</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr"/>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>华语群星</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>2026/4/9</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr"/>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr"/>
+      <c r="J842" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 10, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1339,7 +1339,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BV1MR5GzNEck</t>
+          <t>BV1k5QFBeE6C，BV1MR5GzNEck</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BV1aaXLBwEto，BV1kG7szAEYF，BV1dcjSzXEAu</t>
+          <t>BV1M1QFBVENx，BV1aaXLBwEto，BV1kG7szAEYF，BV1dcjSzXEAu</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/06，2025/04/13，2025/04/22，2025/05/08，2025/05/09，2025/05/30，2025/06/08，2025/08/04，2025/09/18，2025/10/12，2025/11/21，2026/1/24，2026/2/14，2026/2/25</t>
+          <t>2025/03/06，2025/04/06，2025/04/13，2025/04/22，2025/05/08，2025/05/09，2025/05/30，2025/06/08，2025/08/04，2025/09/18，2025/10/12，2025/11/21，2026/1/24，2026/2/14，2026/2/25，2026/4/10</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13，2026/4/10</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2766,7 +2766,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>BV1GwX1Y9E9U，BV1b4Tuz3Eh1，BV1naVgzEEpG</t>
+          <t>BV14NQFB6Eyn，BV1GwX1Y9E9U，BV1b4Tuz3Eh1，BV1naVgzEEpG</t>
         </is>
       </c>
       <c r="J67" t="inlineStr"/>
@@ -4063,7 +4063,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>BV1xv7rzHE88，BV1Roj2zmEn7，BV17oQKYSE76</t>
+          <t>BV142QFBkEm5，BV1xv7rzHE88，BV1Roj2zmEn7，BV17oQKYSE76</t>
         </is>
       </c>
       <c r="J88" t="inlineStr"/>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>BV14jZRBVEJU</t>
+          <t>BV1sgQFBTEnm，BV14jZRBVEJU</t>
         </is>
       </c>
       <c r="J94" t="inlineStr"/>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
+          <t>BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
         </is>
       </c>
       <c r="J118" t="inlineStr"/>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>BV1BN21BzEaJ</t>
+          <t>BV1ukQFBLE4p，BV1TAZxB8EPw，BV1BN21BzEaJ</t>
         </is>
       </c>
       <c r="J127" t="inlineStr"/>
@@ -8839,7 +8839,7 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>BV1CkpMzKEPy，BV1RGjdzzE4G</t>
+          <t>BV1WVQFBNEE4，BV1CkpMzKEPy，BV1RGjdzzE4G</t>
         </is>
       </c>
       <c r="J207" t="inlineStr"/>
@@ -9131,7 +9131,7 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>BV11GypBUErS，BV1KLVSzYEbC，BV1PFZ3YdENc</t>
+          <t>BV142QFBkEXy，BV11GypBUErS，BV1KLVSzYEbC，BV1PFZ3YdENc</t>
         </is>
       </c>
       <c r="J214" t="inlineStr"/>
@@ -10455,7 +10455,7 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>BV1euRDY3ENr</t>
+          <t>BV1T1QFBVEZU，BV1jCZsBVEtd，BV1euRDY3ENr</t>
         </is>
       </c>
       <c r="J247" t="inlineStr"/>
@@ -11491,7 +11491,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>BV189uPzNEzM</t>
+          <t>BV1yQQFBuE1r，BV189uPzNEzM</t>
         </is>
       </c>
       <c r="J273" t="inlineStr"/>
@@ -22959,7 +22959,7 @@
       </c>
       <c r="I569" t="inlineStr">
         <is>
-          <t>BV1hC32zfE4f，BV1jbuRzsE6i，BV1rWv9BgEYk</t>
+          <t>BV1A3QFBvEfU，BV1hC32zfE4f，BV1jbuRzsE6i，BV1rWv9BgEYk</t>
         </is>
       </c>
       <c r="J569" t="inlineStr"/>
@@ -23119,7 +23119,7 @@
       </c>
       <c r="I573" t="inlineStr">
         <is>
-          <t>BV1FCrWBiE7J</t>
+          <t>BV11gQFBTEKR，BV1FCrWBiE7J</t>
         </is>
       </c>
       <c r="J573" t="inlineStr"/>
@@ -23309,7 +23309,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I578" t="inlineStr"/>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>BV1srM9zYEgK</t>
+        </is>
+      </c>
       <c r="J578" t="inlineStr"/>
     </row>
     <row r="579">
@@ -23423,7 +23427,7 @@
       </c>
       <c r="I581" t="inlineStr">
         <is>
-          <t>BV16AcBzZE4S</t>
+          <t>BV1ukQFBLE6x，BV16AcBzZE4S</t>
         </is>
       </c>
       <c r="J581" t="inlineStr"/>
@@ -24063,7 +24067,7 @@
       </c>
       <c r="I598" t="inlineStr">
         <is>
-          <t>BV1opmUBmE8R</t>
+          <t>BV1CVQFBNEvH，BV1opmUBmE8R</t>
         </is>
       </c>
       <c r="J598" t="inlineStr"/>
@@ -24743,7 +24747,7 @@
       </c>
       <c r="E616" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10</t>
         </is>
       </c>
       <c r="F616" t="inlineStr"/>
@@ -24754,7 +24758,7 @@
       </c>
       <c r="H616" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I616" t="inlineStr">
@@ -26255,7 +26259,7 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>2025/09/19，2025/09/26，2025/10/16，2025/11/26，2026/2/12</t>
+          <t>2025/09/19，2025/09/26，2025/10/16，2025/11/26，2026/2/12，2026/4/10</t>
         </is>
       </c>
       <c r="F656" t="inlineStr"/>
@@ -26266,7 +26270,7 @@
       </c>
       <c r="H656" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I656" t="inlineStr">
@@ -33397,7 +33401,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I840" t="inlineStr"/>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>BV12TQFBuEhn</t>
+        </is>
+      </c>
       <c r="J840" t="inlineStr"/>
     </row>
     <row r="841">
@@ -33433,7 +33441,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I841" t="inlineStr"/>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>BV14NQFB6EHA</t>
+        </is>
+      </c>
       <c r="J841" t="inlineStr"/>
     </row>
     <row r="842">
@@ -33469,7 +33481,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I842" t="inlineStr"/>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>BV14NQFB6E2U</t>
+        </is>
+      </c>
       <c r="J842" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: Update song list to Apr 11, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22</t>
+          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22，2026/4/11</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -22206,7 +22206,7 @@
       </c>
       <c r="H549" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I549" t="inlineStr">
@@ -30443,7 +30443,7 @@
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11</t>
         </is>
       </c>
       <c r="F767" t="inlineStr"/>
@@ -30454,7 +30454,7 @@
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
@@ -32415,7 +32415,7 @@
       </c>
       <c r="E816" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/25，2026/3/28</t>
+          <t>2026/3/13，2026/3/25，2026/3/28，2026/4/11</t>
         </is>
       </c>
       <c r="F816" t="inlineStr"/>
@@ -32426,7 +32426,7 @@
       </c>
       <c r="H816" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I816" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Apr 12, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -930,7 +930,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>咬碎秒针</t>
+          <t>噬咬秒针</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -22107,7 +22107,7 @@
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13，2026/4/12</t>
         </is>
       </c>
       <c r="F547" t="inlineStr"/>
@@ -22118,7 +22118,7 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -31111,7 +31111,7 @@
       </c>
       <c r="E784" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28</t>
+          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28，2026/4/12</t>
         </is>
       </c>
       <c r="F784" t="inlineStr"/>
@@ -31122,7 +31122,7 @@
       </c>
       <c r="H784" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I784" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Apr 13, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -11275,7 +11275,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/9，2025/12/6，2025/12/24</t>
+          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/9，2025/12/6，2025/12/24，2026/4/13</t>
         </is>
       </c>
       <c r="F268" t="inlineStr"/>
@@ -11286,7 +11286,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Apr 14, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J842"/>
+  <dimension ref="A1:J847"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1，2026/4/14</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BV1M1QFBVENx，BV1aaXLBwEto，BV1kG7szAEYF，BV1dcjSzXEAu</t>
+          <t>BV1n6QGBNEYY，BV1M1QFBVENx，BV1aaXLBwEto，BV1kG7szAEYF，BV1dcjSzXEAu</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8</t>
+          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,12 +2974,12 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>60</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>BV1BFXUBwEDj，BV191NVzoEZ7，BV1TzrrBAEpz，BV1L5fUB5Ebn，BV1g9M3zsE7c</t>
+          <t>BV1C9Q3BiE8m，BV1BFXUBwEDj，BV191NVzoEZ7，BV1TzrrBAEpz，BV1L5fUB5Ebn，BV1g9M3zsE7c</t>
         </is>
       </c>
       <c r="J62" t="inlineStr"/>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/2/2，2026/2/12</t>
+          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/2/2，2026/2/12，2026/4/14</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/2/19</t>
+          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/2/19，2026/4/14</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>BV1way6BfE6d</t>
+          <t>BV1LVQGB9E3r，BV1way6BfE6d</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/9，2025/11/22，2026/3/9</t>
+          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/9，2025/11/22，2026/3/9，2026/4/14</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -4578,12 +4578,12 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>BV1qLpgzaEQ5，BV1k2T1zPEcd</t>
+          <t>BV1vVQGBXELQ，BV1qLpgzaEQ5，BV1k2T1zPEcd</t>
         </is>
       </c>
       <c r="J101" t="inlineStr"/>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5190,12 +5190,12 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>BV1kcAXzVEWt，BV1QhgpzdEb7</t>
+          <t>BV1GBQ3BmEBA，BV1kcAXzVEWt，BV1QhgpzdEb7</t>
         </is>
       </c>
       <c r="J116" t="inlineStr"/>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9，2026/4/14</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5270,12 +5270,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
+          <t>BV1DrQ3ByECZ，BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
         </is>
       </c>
       <c r="J118" t="inlineStr"/>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11，2026/4/14</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5750,12 +5750,12 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>BV1A1fzBwEjQ，BV19KmPBDERd，BV1B1fGBjEtL</t>
+          <t>BV1pXD2BcECv，BV1A1fzBwEjQ，BV19KmPBDERd，BV1B1fGBjEtL</t>
         </is>
       </c>
       <c r="J130" t="inlineStr"/>
@@ -6419,7 +6419,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13，2026/3/22</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13，2026/3/22，2026/4/14</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/06/26</t>
+          <t>2025/03/20，2025/06/26，2026/4/14</t>
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/09/24，2025/11/27</t>
+          <t>2025/03/25，2025/09/24，2025/11/27，2026/4/14</t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
@@ -8634,12 +8634,12 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>BV1t8J9zcEcz</t>
+          <t>BV1qgQGBREWE，BV1t8J9zcEcz</t>
         </is>
       </c>
       <c r="J202" t="inlineStr"/>
@@ -11291,7 +11291,7 @@
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>BV1BbT9zmEbe，BV115dzYwEED</t>
+          <t>BV1iJQ8BkEkJ，BV1BbT9zmEbe，BV115dzYwEED</t>
         </is>
       </c>
       <c r="J268" t="inlineStr"/>
@@ -17351,7 +17351,7 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/10/31</t>
+          <t>2025/05/03，2025/10/31，2026/4/14</t>
         </is>
       </c>
       <c r="F423" t="inlineStr"/>
@@ -17362,10 +17362,14 @@
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I423" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>BV1hiyXByExY，BV1sCGZzpEZj</t>
+        </is>
+      </c>
       <c r="J423" t="inlineStr"/>
     </row>
     <row r="424">
@@ -17771,7 +17775,7 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>2025/05/12，2025/06/27，2025/07/11，2025/07/11，2025/07/13，2025/08/08，2025/09/06</t>
+          <t>2025/05/12，2025/06/27，2025/07/11，2025/07/11，2025/07/13，2025/08/08，2025/09/06，2026/4/14</t>
         </is>
       </c>
       <c r="F434" t="inlineStr"/>
@@ -17782,7 +17786,7 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
@@ -18715,7 +18719,7 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/07/21</t>
+          <t>2025/05/22，2025/07/21，2026/4/14</t>
         </is>
       </c>
       <c r="F458" t="inlineStr"/>
@@ -18726,10 +18730,14 @@
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I458" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>BV1ogQGBREtD，BV1bCgLzvEbT，BV148JJzAE88</t>
+        </is>
+      </c>
       <c r="J458" t="inlineStr"/>
     </row>
     <row r="459">
@@ -20471,7 +20479,7 @@
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/10/20，2025/11/1，2026/3/5</t>
+          <t>2025/06/02，2025/10/20，2025/11/1，2026/3/5，2026/4/14</t>
         </is>
       </c>
       <c r="F504" t="inlineStr"/>
@@ -20482,12 +20490,12 @@
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I504" t="inlineStr">
         <is>
-          <t>BV1WnWmzmENc</t>
+          <t>BV1m2Q3B3EeU，BV1WnWmzmENc</t>
         </is>
       </c>
       <c r="J504" t="inlineStr"/>
@@ -21423,7 +21431,7 @@
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/09/02，2026/3/8，2026/3/17</t>
+          <t>2025/06/19，2025/09/02，2026/3/8，2026/3/17，2026/4/14</t>
         </is>
       </c>
       <c r="F529" t="inlineStr"/>
@@ -21434,7 +21442,7 @@
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
@@ -24051,7 +24059,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>2025/07/23，2025/12/12，2026/2/25，2026/4/9</t>
+          <t>2025/07/23，2025/12/12，2026/2/25，2026/4/9，2026/4/14</t>
         </is>
       </c>
       <c r="F598" t="inlineStr"/>
@@ -24062,7 +24070,7 @@
       </c>
       <c r="H598" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I598" t="inlineStr">
@@ -29387,7 +29395,7 @@
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>2025/11/24</t>
+          <t>2025/11/24，2026/4/14</t>
         </is>
       </c>
       <c r="F739" t="inlineStr"/>
@@ -29398,10 +29406,14 @@
       </c>
       <c r="H739" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I739" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>BV1yxUkBLEcB</t>
+        </is>
+      </c>
       <c r="J739" t="inlineStr"/>
     </row>
     <row r="740">
@@ -29875,7 +29887,7 @@
       </c>
       <c r="E752" t="inlineStr">
         <is>
-          <t>2025/12/9，2026/2/2</t>
+          <t>2025/12/9，2026/2/2，2026/4/14</t>
         </is>
       </c>
       <c r="F752" t="inlineStr"/>
@@ -29886,7 +29898,7 @@
       </c>
       <c r="H752" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I752" t="inlineStr"/>
@@ -30947,7 +30959,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -30958,12 +30970,12 @@
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I780" t="inlineStr">
         <is>
-          <t>BV1sEzxBCEua</t>
+          <t>BV1mE9nBuEk1，BV1V89GBfE6h，BV1sEzxBCEua</t>
         </is>
       </c>
       <c r="J780" t="inlineStr"/>
@@ -31471,7 +31483,7 @@
       </c>
       <c r="E793" t="inlineStr">
         <is>
-          <t>2026/2/9，2026/2/27，2026/3/9</t>
+          <t>2026/2/9，2026/2/27，2026/3/9，2026/4/14</t>
         </is>
       </c>
       <c r="F793" t="inlineStr"/>
@@ -31482,7 +31494,7 @@
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
@@ -32939,7 +32951,7 @@
       </c>
       <c r="E829" t="inlineStr">
         <is>
-          <t>2026/3/25</t>
+          <t>2026/3/25，2026/4/14</t>
         </is>
       </c>
       <c r="F829" t="inlineStr"/>
@@ -32950,7 +32962,7 @@
       </c>
       <c r="H829" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I829" t="inlineStr">
@@ -32979,7 +32991,7 @@
       </c>
       <c r="E830" t="inlineStr">
         <is>
-          <t>2026/3/28</t>
+          <t>2026/3/28，2026/4/14</t>
         </is>
       </c>
       <c r="F830" t="inlineStr"/>
@@ -32990,7 +33002,7 @@
       </c>
       <c r="H830" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I830" t="inlineStr">
@@ -33487,6 +33499,190 @@
         </is>
       </c>
       <c r="J842" t="inlineStr"/>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>842</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>一千零一夜</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr"/>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>刘美麟</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>2026/4/14</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr"/>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>BV1kdQ3BNEUr</t>
+        </is>
+      </c>
+      <c r="J843" t="inlineStr"/>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Take Me Hand</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr"/>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>DAISHI DANCE/Cécile Corbel</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>2026/4/14</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr"/>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr"/>
+      <c r="J844" t="inlineStr"/>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>爱人错过</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr"/>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>告五人</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>2026/4/14</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr"/>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr"/>
+      <c r="J845" t="inlineStr"/>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>845</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>小小</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr"/>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>容祖儿</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>2026/4/14</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr"/>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr"/>
+      <c r="J846" t="inlineStr"/>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>想去海边</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr"/>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>夏日入侵企画</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>2026/4/14，2026/4/14</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr"/>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr"/>
+      <c r="J847" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 16, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J847"/>
+  <dimension ref="A1:J848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,7 +631,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4</t>
+          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -642,12 +642,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BV1EVGdzNEe7</t>
+          <t>BV1o7daBxEbp，BV1EVGdzNEe7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25</t>
+          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25，2026/4/16</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1374,12 +1374,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BV1jHT4zBEBW</t>
+          <t>BV1aGdvB4EV1，BV1jHT4zBEBW</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/05/09，2025/06/13，2025/06/19，2025/06/27，2025/07/10，2025/09/10，2025/09/19，2025/11/14，2025/12/31，2026/2/23</t>
+          <t>2025/03/04，2025/04/14，2025/05/09，2025/06/13，2025/06/19，2025/06/27，2025/07/10，2025/09/10，2025/09/19，2025/11/14，2025/12/31，2026/2/23，2026/4/16</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -1414,12 +1414,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BV1r4oLYfEjE，BV1Asf6BvEo3</t>
+          <t>BV1eudvBbE7C，BV1r4oLYfEjE，BV1Asf6BvEo3</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11，2026/4/16</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BV1PzPizTEty，BV1cG9pYkE8m，BV1B1fGBjEvg</t>
+          <t>BV1tBdeBDEfp，BV1PzPizTEty，BV1cG9pYkE8m，BV1B1fGBjEvg</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/1/14，2026/2/19，2026/3/14</t>
+          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/1/14，2026/2/19，2026/3/14，2026/4/16</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2134,12 +2134,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>BV14fsGzZESX</t>
+          <t>BV1zodeBqEpk，BV14fsGzZESX</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/7，2025/11/9，2025/12/2，2026/1/21，2026/3/5</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/7，2025/11/9，2025/12/2，2026/1/21，2026/3/5，2026/4/16</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2266,12 +2266,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>BV1n7SbBMEKD</t>
+          <t>BV1vMdvBFEcL，BV1n7SbBMEKD</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21，2026/4/16</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3350,12 +3350,12 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>BV1bVqVBkEJz</t>
+          <t>BV1XgdvBZEQ3，BV1bVqVBkEJz</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/13，2025/05/30，2025/06/06，2025/07/08，2025/08/07，2025/08/22，2025/09/30，2025/11/9，2025/11/13，2025/12/31</t>
+          <t>2025/03/20，2025/04/17，2025/05/13，2025/05/30，2025/06/06，2025/07/08，2025/08/07，2025/08/22，2025/09/30，2025/11/9，2025/11/13，2025/12/31，2026/4/16</t>
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -6918,12 +6918,12 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>BV1N5EAzjEbT，BV1ePXiYhEsn</t>
+          <t>BV1gLdvBxELz，BV1N5EAzjEbT，BV1ePXiYhEsn</t>
         </is>
       </c>
       <c r="J159" t="inlineStr"/>
@@ -7423,7 +7423,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/03/29，2025/04/25，2025/05/30，2025/06/22，2025/07/18，2025/09/03，2025/09/13</t>
+          <t>2025/03/21，2025/03/29，2025/04/25，2025/05/30，2025/06/22，2025/07/18，2025/09/03，2025/09/13，2026/4/16</t>
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -7434,12 +7434,12 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>BV1NaarzsEjk，BV1TT7Kz9ESB</t>
+          <t>BV1bEdvBpEBc，BV1NaarzsEjk，BV1TT7Kz9ESB</t>
         </is>
       </c>
       <c r="J172" t="inlineStr"/>
@@ -8947,7 +8947,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/28，2025/04/29，2025/05/12，2025/06/06，2025/06/16，2025/07/24，2025/08/01，2025/09/05，2025/09/26，2025/10/28，2025/12/5，2026/1/9，2026/2/19，2026/3/22</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/28，2025/04/29，2025/05/12，2025/06/06，2025/06/16，2025/07/24，2025/08/01，2025/09/05，2025/09/26，2025/10/28，2025/12/5，2026/1/9，2026/2/19，2026/3/22，2026/4/16</t>
         </is>
       </c>
       <c r="F210" t="inlineStr"/>
@@ -8958,12 +8958,12 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>BV1FCa8zEEue</t>
+          <t>BV1jEdaBdEwT，BV1FCa8zEEue</t>
         </is>
       </c>
       <c r="J210" t="inlineStr"/>
@@ -10635,7 +10635,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/2/12</t>
+          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/2/12，2026/4/16</t>
         </is>
       </c>
       <c r="F252" t="inlineStr"/>
@@ -10646,12 +10646,12 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>BV19G5TztEGW</t>
+          <t>BV1RndaBWEDB，BV19G5TztEGW</t>
         </is>
       </c>
       <c r="J252" t="inlineStr"/>
@@ -12855,7 +12855,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/2/4，2026/2/14</t>
+          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/2/4，2026/2/14，2026/4/15</t>
         </is>
       </c>
       <c r="F308" t="inlineStr"/>
@@ -12866,12 +12866,12 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>BV1BYyVBVELL</t>
+          <t>BV1KHQJBhEDw，BV1BYyVBVELL</t>
         </is>
       </c>
       <c r="J308" t="inlineStr"/>
@@ -17869,7 +17869,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I436" t="inlineStr"/>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>BV1nznZzeEgo</t>
+        </is>
+      </c>
       <c r="J436" t="inlineStr"/>
     </row>
     <row r="437">
@@ -21735,7 +21739,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -21746,12 +21750,12 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
         <is>
-          <t>BV1MosGzFEMe</t>
+          <t>BV1zodeBqEhq，BV1MosGzFEMe</t>
         </is>
       </c>
       <c r="J537" t="inlineStr"/>
@@ -25673,7 +25677,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I640" t="inlineStr"/>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>BV1k2pgz3E2X</t>
+        </is>
+      </c>
       <c r="J640" t="inlineStr"/>
     </row>
     <row r="641">
@@ -25785,7 +25793,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I643" t="inlineStr"/>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>BV1qApVzMEC3</t>
+        </is>
+      </c>
       <c r="J643" t="inlineStr"/>
     </row>
     <row r="644">
@@ -28659,7 +28671,7 @@
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>2025/10/30，2025/11/3，2025/11/7，2025/11/13，2025/11/22，2025/12/5，2026/1/2</t>
+          <t>2025/10/30，2025/11/3，2025/11/7，2025/11/13，2025/11/22，2025/12/5，2026/1/2，2026/4/15</t>
         </is>
       </c>
       <c r="F719" t="inlineStr"/>
@@ -28670,12 +28682,12 @@
       </c>
       <c r="H719" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I719" t="inlineStr">
         <is>
-          <t>BV1tJ1vBxEFQ</t>
+          <t>BV14WQJBFEw6，BV1tJ1vBxEFQ</t>
         </is>
       </c>
       <c r="J719" t="inlineStr"/>
@@ -30375,7 +30387,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -30386,12 +30398,12 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
         <is>
-          <t>BV1oKiwBXE1L，BV1Csf6BeEYe</t>
+          <t>BV1qAdvBYEKf，BV1oKiwBXE1L，BV1Csf6BeEYe</t>
         </is>
       </c>
       <c r="J765" t="inlineStr"/>
@@ -32859,7 +32871,7 @@
       </c>
       <c r="E827" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16</t>
         </is>
       </c>
       <c r="F827" t="inlineStr"/>
@@ -32870,12 +32882,12 @@
       </c>
       <c r="H827" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I827" t="inlineStr">
         <is>
-          <t>BV1nCD7ByEXM，BV1ugQSBnE8x</t>
+          <t>BV1vKdvBhE88，BV1nCD7ByEXM，BV1ugQSBnE8x</t>
         </is>
       </c>
       <c r="J827" t="inlineStr">
@@ -33573,7 +33585,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I844" t="inlineStr"/>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>BV1mQQVB1EBB</t>
+        </is>
+      </c>
       <c r="J844" t="inlineStr"/>
     </row>
     <row r="845">
@@ -33609,7 +33625,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I845" t="inlineStr"/>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>BV1UDQVBjEGt</t>
+        </is>
+      </c>
       <c r="J845" t="inlineStr"/>
     </row>
     <row r="846">
@@ -33681,8 +33701,52 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I847" t="inlineStr"/>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>BV1RWdaBHEsQ</t>
+        </is>
+      </c>
       <c r="J847" t="inlineStr"/>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>847</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>착하다는 말이 제일 싫어</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr"/>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>YENA</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>2026/4/16</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr"/>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>韩语</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>BV1XsdaBDEAD</t>
+        </is>
+      </c>
+      <c r="J848" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 17, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J848"/>
+  <dimension ref="A1:J849"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14</t>
+          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1974,12 +1974,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>BV1VxNdzrEGV</t>
+          <t>BV16ndLBJEJf，BV1VxNdzrEGV</t>
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/12，2025/05/20，2025/05/30，2025/06/27，2025/08/13，2025/09/11，2025/10/28，2025/12/20，2026/1/16</t>
+          <t>2025/03/14，2025/04/12，2025/05/20，2025/05/30，2025/06/27，2025/08/13，2025/09/11，2025/10/28，2025/12/20，2026/1/16，2026/4/17</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5310,12 +5310,12 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>BV1PHJizCEQj，BV1fTY4zMEw1，BV1HWrSBLE93</t>
+          <t>BV1rEdLBDEMF，BV1PHJizCEQj，BV1fTY4zMEw1，BV1HWrSBLE93</t>
         </is>
       </c>
       <c r="J119" t="inlineStr"/>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/06/08，2025/07/13，2025/07/21，2025/07/24，2025/07/28，2025/08/01，2025/08/16，2025/09/26，2025/10/28，2025/11/10，2025/11/17，2025/12/23</t>
+          <t>2025/03/27，2025/06/08，2025/07/13，2025/07/21，2025/07/24，2025/07/28，2025/08/01，2025/08/16，2025/09/26，2025/10/28，2025/11/10，2025/11/17，2025/12/23，2026/4/17</t>
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
@@ -9002,12 +9002,12 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>BV1iQBjBKE9h</t>
+          <t>BV1nndLBnE6F，BV1iQBjBKE9h</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9202,12 +9202,12 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>BV1yYMVz2E5E</t>
+          <t>BV1rEdLBDEFV，BV1yYMVz2E5E</t>
         </is>
       </c>
       <c r="J216" t="inlineStr"/>
@@ -12579,7 +12579,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>2025/04/06，2025/04/19，2025/05/03，2025/08/01，2025/10/31，2025/12/15，2026/2/22，2026/2/23</t>
+          <t>2025/04/06，2025/04/19，2025/05/03，2025/08/01，2025/10/31，2025/12/15，2026/2/22，2026/2/23，2026/4/17</t>
         </is>
       </c>
       <c r="F301" t="inlineStr"/>
@@ -12590,12 +12590,12 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>BV1SuqVB5EoV</t>
+          <t>BV1FndLBnEXN，BV1SuqVB5EoV</t>
         </is>
       </c>
       <c r="J301" t="inlineStr"/>
@@ -13939,7 +13939,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13950,12 +13950,12 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>BV1jEBuB1EAY</t>
+          <t>BV1rEdLBDEHv，BV1jEBuB1EAY</t>
         </is>
       </c>
       <c r="J336" t="inlineStr"/>
@@ -14471,7 +14471,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/04/20，2025/05/18，2025/05/20，2025/05/25，2025/06/28，2025/06/30，2025/08/24，2025/09/26，2026/1/9</t>
+          <t>2025/04/15，2025/04/18，2025/04/20，2025/05/18，2025/05/20，2025/05/25，2025/06/28，2025/06/30，2025/08/24，2025/09/26，2026/1/9，2026/4/17</t>
         </is>
       </c>
       <c r="F349" t="inlineStr"/>
@@ -14482,12 +14482,12 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>BV1uAVLzCELY</t>
+          <t>BV1rEdLBDEWK，BV1uAVLzCELY</t>
         </is>
       </c>
       <c r="J349" t="inlineStr"/>
@@ -20931,7 +20931,7 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>2025/06/12，2025/07/13，2025/07/18，2025/09/28，2025/10/20，2026/1/19</t>
+          <t>2025/06/12，2025/07/13，2025/07/18，2025/09/28，2025/10/20，2026/1/19，2026/4/17</t>
         </is>
       </c>
       <c r="F516" t="inlineStr"/>
@@ -20942,12 +20942,12 @@
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I516" t="inlineStr">
         <is>
-          <t>BV1ySRJYkEK1</t>
+          <t>BV1rEdLBDEsD，BV1ySRJYkEK1</t>
         </is>
       </c>
       <c r="J516" t="inlineStr">
@@ -29913,7 +29913,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I752" t="inlineStr"/>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>BV1QrQVBpEzs</t>
+        </is>
+      </c>
       <c r="J752" t="inlineStr">
         <is>
           <t>游戏</t>
@@ -33747,6 +33751,50 @@
         </is>
       </c>
       <c r="J848" t="inlineStr"/>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>848</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>星辉抵达之日</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr"/>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/baitian/waka</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>2026/4/17</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr"/>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>BV1mKdLBfEPD</t>
+        </is>
+      </c>
+      <c r="J849" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 18, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1003,7 +1003,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1014,12 +1014,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>BV1BvqVB4EFv</t>
+          <t>BV1B6dWBBE4v，BV1BvqVB4EFv</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/3/9</t>
+          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/3/9，2026/4/18</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27</t>
+          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/3，2025/12/12，2026/2/4</t>
+          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/3，2025/12/12，2026/2/4，2026/4/18</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>61</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/8，2026/1/12，2026/1/30，2026/2/7</t>
+          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/8，2026/1/12，2026/1/30，2026/2/7，2026/4/18</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/19，2025/05/20，2025/07/26，2025/08/16，2025/12/11，2026/4/9</t>
+          <t>2025/03/14，2025/05/19，2025/05/20，2025/07/26，2025/08/16，2025/12/11，2026/4/9，2026/4/18</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4498,12 +4498,12 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>BV1SWD4BEEB7，BV1ynm3BsEbZ，BV1ZzQuYZEy2</t>
+          <t>BV14AdsBXEZc，BV1SWD4BEEB7，BV1ynm3BsEbZ，BV1ZzQuYZEy2</t>
         </is>
       </c>
       <c r="J99" t="inlineStr"/>
@@ -5139,7 +5139,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/1/19</t>
+          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/1/19，2026/4/18</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5150,12 +5150,12 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>BV1AtQrY4EzH，BV1fZyDBDEiJ</t>
+          <t>BV1nRdpBgEYi，BV1AtQrY4EzH，BV1fZyDBDEiJ</t>
         </is>
       </c>
       <c r="J115" t="inlineStr"/>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7754,12 +7754,12 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>BV17HP9zkE69</t>
+          <t>BV13GdWBZEqB，BV17HP9zkE69</t>
         </is>
       </c>
       <c r="J180" t="inlineStr"/>
@@ -10119,7 +10119,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/08/12，2025/10/20，2025/11/14，2025/12/2，2026/1/10，2026/2/9</t>
+          <t>2025/03/29，2025/08/12，2025/10/20，2025/11/14，2025/12/2，2026/1/10，2026/2/9，2026/4/18</t>
         </is>
       </c>
       <c r="F239" t="inlineStr"/>
@@ -10130,7 +10130,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/9，2025/12/5，2025/12/19，2025/12/26，2026/1/10，2026/1/19，2026/2/10，2026/3/24</t>
+          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/9，2025/12/5，2025/12/19，2025/12/26，2026/1/10，2026/1/19，2026/2/10，2026/3/24，2026/4/18</t>
         </is>
       </c>
       <c r="F313" t="inlineStr"/>
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -14351,7 +14351,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/1/1，2026/1/9，2026/2/20</t>
+          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/1/1，2026/1/9，2026/2/20，2026/4/18</t>
         </is>
       </c>
       <c r="F346" t="inlineStr"/>
@@ -14362,7 +14362,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -14580,18 +14580,18 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>真夜中のドア/Stay With Me</t>
+          <t>真夜中のドア - Stay With Me</t>
         </is>
       </c>
       <c r="C352" t="inlineStr"/>
       <c r="D352" t="inlineStr">
         <is>
-          <t>松原美紀</t>
+          <t>松原みき</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/21，2025/05/08，2025/06/10，2025/06/28，2025/07/08，2025/08/22，2025/09/11，2025/10/25，2026/3/13</t>
+          <t>2025/04/17，2025/04/21，2025/05/08，2025/06/10，2025/06/28，2025/07/08，2025/08/22，2025/09/11，2025/10/25，2026/3/13，2026/4/18</t>
         </is>
       </c>
       <c r="F352" t="inlineStr"/>
@@ -14602,12 +14602,12 @@
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>BV1FdMgzNEUo</t>
+          <t>BV1kYdWBVEAN，BV1FdMgzNEUo</t>
         </is>
       </c>
       <c r="J352" t="inlineStr"/>
@@ -19295,7 +19295,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18</t>
         </is>
       </c>
       <c r="F473" t="inlineStr"/>
@@ -19306,12 +19306,12 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>BV1oQBjBKExX</t>
+          <t>BV1ZcdWBNE5r，BV1oQBjBKExX</t>
         </is>
       </c>
       <c r="J473" t="inlineStr"/>
@@ -26467,7 +26467,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18</t>
         </is>
       </c>
       <c r="F661" t="inlineStr"/>
@@ -26478,12 +26478,12 @@
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
         <is>
-          <t>BV1UAnwzQE3E</t>
+          <t>BV1mndWBHEQG，BV1UAnwzQE3E</t>
         </is>
       </c>
       <c r="J661" t="inlineStr"/>
@@ -30975,7 +30975,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -30986,7 +30986,7 @@
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I780" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Apr 19, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J849"/>
+  <dimension ref="A1:J850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -675,7 +675,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/9，2025/12/11，2026/1/15，2026/2/12</t>
+          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/9，2025/12/11，2026/1/15，2026/2/12，2026/4/19</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -686,12 +686,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BV1a67QzZENo</t>
+          <t>BV1p5dfBVE37，BV1a67QzZENo</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -759,7 +759,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17，2026/4/19</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -770,12 +770,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BV1UDXCYGEWL</t>
+          <t>BV1JndfBuExn，BV1UDXCYGEWL</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/1/12，2026/2/7，2026/3/15</t>
+          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/1/12，2026/2/7，2026/3/15，2026/4/19</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/19，2025/07/21，2025/10/20，2026/1/14，2026/2/19</t>
+          <t>2025/03/14，2025/05/19，2025/07/21，2025/10/20，2026/1/14，2026/2/19，2026/4/19</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/08，2025/04/18，2025/05/12，2025/05/23，2025/06/27，2025/07/24，2025/08/28，2025/10/11，2025/10/31，2025/11/24，2025/12/19，2026/2/2</t>
+          <t>2025/03/19，2025/04/08，2025/04/18，2025/05/12，2025/05/23，2025/06/27，2025/07/24，2025/08/28，2025/10/11，2025/10/31，2025/11/24，2025/12/19，2026/2/2，2026/4/19</t>
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
@@ -6350,12 +6350,12 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>BV1GTK6zaEPD</t>
+          <t>BV1AddfBjEtH，BV1GTK6zaEPD</t>
         </is>
       </c>
       <c r="J145" t="inlineStr"/>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>BV1RukTBmEp8</t>
+          <t>BV1U1QVBSEzo，BV1RukTBmEp8</t>
         </is>
       </c>
       <c r="J147" t="inlineStr"/>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>BV1gHpBzAEnJ</t>
+          <t>BV1eqDEBqEQp，BV1gHpBzAEnJ</t>
         </is>
       </c>
       <c r="J153" t="inlineStr"/>
@@ -7903,7 +7903,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22，2026/4/19</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7914,12 +7914,12 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>BV1Xr2xBVEqN，BV1Csf6BeE7B</t>
+          <t>BV1NDdfBUEL9，BV1Xr2xBVEqN，BV1Csf6BeE7B</t>
         </is>
       </c>
       <c r="J184" t="inlineStr"/>
@@ -8063,7 +8063,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25</t>
+          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25，2026/4/19</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -8074,12 +8074,12 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>BV1Q6E2zjE2b</t>
+          <t>BV1JwoFB3E6c，BV1Q6E2zjE2b</t>
         </is>
       </c>
       <c r="J188" t="inlineStr"/>
@@ -9547,7 +9547,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/05，2025/05/08，2025/05/15，2025/05/30，2025/06/13，2025/06/23，2025/07/10，2025/07/24，2025/08/04，2025/09/03，2025/09/21，2025/11/9，2025/11/26，2026/1/16，2026/1/29</t>
+          <t>2025/03/28，2025/05/05，2025/05/08，2025/05/15，2025/05/30，2025/06/13，2025/06/23，2025/07/10，2025/07/24，2025/08/04，2025/09/03，2025/09/21，2025/11/9，2025/11/26，2026/1/16，2026/1/29，2026/4/19</t>
         </is>
       </c>
       <c r="F225" t="inlineStr"/>
@@ -9558,12 +9558,12 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>BV1ZtE2zsEfw</t>
+          <t>BV1JEdfB6EZN，BV1ZtE2zsEfw</t>
         </is>
       </c>
       <c r="J225" t="inlineStr"/>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7，2026/3/28</t>
+          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7，2026/3/28，2026/4/19</t>
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
@@ -9878,12 +9878,12 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>BV1tzXLB4EDj，BV1r3NAzgErm，BV1crarzEEsn</t>
+          <t>BV1JHdfBBEgk，BV1tzXLB4EDj，BV1r3NAzgErm，BV1crarzEEsn</t>
         </is>
       </c>
       <c r="J233" t="inlineStr"/>
@@ -10359,7 +10359,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/1/9，2026/3/7</t>
+          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/1/9，2026/3/7，2026/4/19</t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
@@ -10370,12 +10370,12 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>BV1jANPzvEDw</t>
+          <t>BV1urdfBRE5i，BV1jANPzvEDw</t>
         </is>
       </c>
       <c r="J245" t="inlineStr"/>
@@ -13283,7 +13283,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/18，2025/06/09，2025/07/07，2025/08/26，2025/09/03，2025/09/13，2025/10/17，2025/10/30，2025/11/21，2025/12/17</t>
+          <t>2025/04/11，2025/05/18，2025/06/09，2025/07/07，2025/08/26，2025/09/03，2025/09/13，2025/10/17，2025/10/30，2025/11/21，2025/12/17，2026/4/19</t>
         </is>
       </c>
       <c r="F319" t="inlineStr"/>
@@ -13294,12 +13294,12 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>BV1fjqjBKECu，BV1isG5z1EF6</t>
+          <t>BV1HLdfBkEWj，BV1fjqjBKECu，BV1isG5z1EF6</t>
         </is>
       </c>
       <c r="J319" t="inlineStr"/>
@@ -13439,7 +13439,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24，2026/4/19</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -13450,12 +13450,12 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>BV1TP7LzmEnU</t>
+          <t>BV1SxowBaEyy，BV1TP7LzmEnU</t>
         </is>
       </c>
       <c r="J323" t="inlineStr"/>
@@ -13703,7 +13703,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/18，2025/09/08，2025/12/5，2026/1/28</t>
+          <t>2025/04/11，2025/05/18，2025/09/08，2025/12/5，2026/1/28，2026/4/19</t>
         </is>
       </c>
       <c r="F330" t="inlineStr"/>
@@ -13714,7 +13714,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -14511,7 +14511,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/26，2025/06/23，2025/09/29</t>
+          <t>2025/04/17，2025/05/26，2025/06/23，2025/09/29，2026/4/19</t>
         </is>
       </c>
       <c r="F350" t="inlineStr"/>
@@ -14522,12 +14522,12 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>BV1BzKhzUEYG，BV1KFLczTECE</t>
+          <t>BV1EWdfBTET2，BV1BzKhzUEYG，BV1KFLczTECE</t>
         </is>
       </c>
       <c r="J350" t="inlineStr"/>
@@ -23651,7 +23651,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/3，2025/11/22，2026/1/5，2026/2/18，2026/2/23</t>
+          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/3，2025/11/22，2026/1/5，2026/2/18，2026/2/23，2026/4/19</t>
         </is>
       </c>
       <c r="F587" t="inlineStr"/>
@@ -23662,12 +23662,12 @@
       </c>
       <c r="H587" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I587" t="inlineStr">
         <is>
-          <t>BV1JbaYzsEF3</t>
+          <t>BV1CXdfB7EkG，BV1JbaYzsEF3</t>
         </is>
       </c>
       <c r="J587" t="inlineStr"/>
@@ -23843,7 +23843,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6，2026/3/28</t>
+          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6，2026/3/28，2026/4/19</t>
         </is>
       </c>
       <c r="F592" t="inlineStr"/>
@@ -23854,7 +23854,7 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8</t>
+          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8，2026/4/19</t>
         </is>
       </c>
       <c r="F606" t="inlineStr"/>
@@ -24382,12 +24382,12 @@
       </c>
       <c r="H606" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I606" t="inlineStr">
         <is>
-          <t>BV1kfcqzhEv6</t>
+          <t>BV1n7dfB3EGS，BV1kfcqzhEv6</t>
         </is>
       </c>
       <c r="J606" t="inlineStr"/>
@@ -25895,7 +25895,7 @@
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/3，2025/11/13，2025/11/24，2025/12/5，2025/12/12，2025/12/17，2026/1/6，2026/1/15，2026/1/24，2026/2/27</t>
+          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/3，2025/11/13，2025/11/24，2025/12/5，2025/12/12，2025/12/17，2026/1/6，2026/1/15，2026/1/24，2026/2/27，2026/4/19</t>
         </is>
       </c>
       <c r="F646" t="inlineStr"/>
@@ -25906,12 +25906,12 @@
       </c>
       <c r="H646" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I646" t="inlineStr">
         <is>
-          <t>BV1p2p9zcELR</t>
+          <t>BV1FfdfBVEQL，BV1p2p9zcELR</t>
         </is>
       </c>
       <c r="J646" t="inlineStr"/>
@@ -26127,7 +26127,7 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>2025/09/15，2025/10/19，2025/10/20，2025/10/26，2025/11/1，2025/11/14，2026/1/15，2026/1/23</t>
+          <t>2025/09/15，2025/10/19，2025/10/20，2025/10/26，2025/11/1，2025/11/14，2026/1/15，2026/1/23，2026/4/19</t>
         </is>
       </c>
       <c r="F652" t="inlineStr"/>
@@ -26138,7 +26138,7 @@
       </c>
       <c r="H652" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I652" t="inlineStr">
@@ -31299,7 +31299,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>2026/2/7</t>
+          <t>2026/2/7，2026/4/19</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
@@ -31310,10 +31310,14 @@
       </c>
       <c r="H788" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I788" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>BV1A7dfBGEKE</t>
+        </is>
+      </c>
       <c r="J788" t="inlineStr"/>
     </row>
     <row r="789">
@@ -33791,6 +33795,46 @@
         </is>
       </c>
       <c r="J849" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Daisy Crown</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr"/>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/Empty old City</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>2026/4/19</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr"/>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr"/>
+      <c r="J850" t="inlineStr">
         <is>
           <t>游戏</t>
         </is>

</xml_diff>

<commit_message>
chore: Update song list to Apr 20, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J850"/>
+  <dimension ref="A1:J852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -715,7 +715,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1，2026/4/20</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -726,12 +726,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BV1df7RzGEDY</t>
+          <t>BV1K5d6BhEPj，BV1df7RzGEDY</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>BV1N8UvB8ExW</t>
+          <t>BV17uQABvEkz，BV1N8UvB8ExW</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>BV1BWGzzWEEP</t>
+          <t>BV1pJocBUEN7，BV1BWGzzWEEP</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>BV1UtzsBmE9n</t>
+          <t>BV1JpocB1EJS，BV1UtzsBmE9n</t>
         </is>
       </c>
       <c r="J106" t="inlineStr"/>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>BV1eqzWBXE55</t>
+          <t>BV1nJocBmES3，BV1eqzWBXE55</t>
         </is>
       </c>
       <c r="J110" t="inlineStr"/>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31，2026/4/20</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6190,12 +6190,12 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>BV17NkTBHEYN</t>
+          <t>BV1AEd6BZE99，BV17NkTBHEYN</t>
         </is>
       </c>
       <c r="J141" t="inlineStr"/>
@@ -6459,7 +6459,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/05/18，2025/06/13，2025/09/12，2025/10/01</t>
+          <t>2025/03/19，2025/04/07，2025/05/18，2025/06/13，2025/09/12，2025/10/01，2026/4/20</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -6470,12 +6470,12 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>BV1mbHpz7Ern，BV1abpgzXEAM，BV1DbJGzSEQj</t>
+          <t>BV1aJdUBFEHA，BV1mbHpz7Ern，BV1abpgzXEAM，BV1DbJGzSEQj</t>
         </is>
       </c>
       <c r="J148" t="inlineStr"/>
@@ -6499,7 +6499,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6510,12 +6510,12 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>BV1cADbBrESS，BV19QnGzZE9f，BV1DZiFBgEhH，BV13rQZYQEem，BV1HD7VzqEQy，BV1UwSMBoE3e</t>
+          <t>BV13JdUBFEQh，BV1cADbBrESS，BV19QnGzZE9f，BV1DZiFBgEhH，BV13rQZYQEem，BV1HD7VzqEQy，BV1UwSMBoE3e</t>
         </is>
       </c>
       <c r="J149" t="inlineStr"/>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>BV1Rqw3zCEFo，BV1v84TzcEMv</t>
+          <t>BV1wB9PBHEQp，BV1Rqw3zCEFo，BV1v84TzcEMv</t>
         </is>
       </c>
       <c r="J175" t="inlineStr"/>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7754,7 +7754,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11115,7 +11115,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/22，2025/08/22，2025/09/12</t>
+          <t>2025/04/02，2025/05/22，2025/08/22，2025/09/12，2026/4/20</t>
         </is>
       </c>
       <c r="F264" t="inlineStr"/>
@@ -11126,12 +11126,12 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>BV1gvpGztEps</t>
+          <t>BV1aJdUBFEBX，BV1gvpGztEps</t>
         </is>
       </c>
       <c r="J264" t="inlineStr"/>
@@ -12267,7 +12267,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>2025/4/4</t>
+          <t>2025/4/4，2026/4/20</t>
         </is>
       </c>
       <c r="F293" t="inlineStr"/>
@@ -12278,10 +12278,14 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I293" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>BV1modkBzEfh</t>
+        </is>
+      </c>
       <c r="J293" t="inlineStr"/>
     </row>
     <row r="294">
@@ -13719,7 +13723,7 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>BV1zYaZzZEYj</t>
+          <t>BV1pEocBEEML，BV1zYaZzZEYj</t>
         </is>
       </c>
       <c r="J330" t="inlineStr"/>
@@ -16355,7 +16359,7 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/05/18</t>
+          <t>2025/04/25，2025/05/18，2026/4/20</t>
         </is>
       </c>
       <c r="F397" t="inlineStr"/>
@@ -16366,12 +16370,12 @@
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>BV1xHJVz5EN6</t>
+          <t>BV13JdUBFEB1，BV1xHJVz5EN6</t>
         </is>
       </c>
       <c r="J397" t="inlineStr"/>
@@ -16551,7 +16555,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/05/04，2025/05/26，2025/06/08，2025/08/28，2025/10/18，2025/11/18，2025/12/24，2026/1/29，2026/2/27，2026/4/9</t>
+          <t>2025/04/27，2025/05/04，2025/05/26，2025/06/08，2025/08/28，2025/10/18，2025/11/18，2025/12/24，2026/1/29，2026/2/27，2026/4/9，2026/4/20</t>
         </is>
       </c>
       <c r="F402" t="inlineStr"/>
@@ -16562,12 +16566,12 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t>BV196BQBhEf1</t>
+          <t>BV1aJdUBFE8M，BV196BQBhEf1</t>
         </is>
       </c>
       <c r="J402" t="inlineStr"/>
@@ -16943,7 +16947,7 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>2025/04/29，2025/05/03</t>
+          <t>2025/04/29，2025/05/03，2026/4/20</t>
         </is>
       </c>
       <c r="F412" t="inlineStr"/>
@@ -16954,10 +16958,14 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I412" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>BV1UodkBzE3o，BV1UQGRzJE5b</t>
+        </is>
+      </c>
       <c r="J412" t="inlineStr"/>
     </row>
     <row r="413">
@@ -17185,7 +17193,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I418" t="inlineStr"/>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>BV1FpuRzbECp</t>
+        </is>
+      </c>
       <c r="J418" t="inlineStr"/>
     </row>
     <row r="419">
@@ -17221,7 +17233,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I419" t="inlineStr"/>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>BV1tCRhYjEgs</t>
+        </is>
+      </c>
       <c r="J419" t="inlineStr"/>
     </row>
     <row r="420">
@@ -17445,7 +17461,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I425" t="inlineStr"/>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>BV1awVSzGEYr</t>
+        </is>
+      </c>
       <c r="J425" t="inlineStr"/>
     </row>
     <row r="426">
@@ -17467,7 +17487,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26</t>
+          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/4/20</t>
         </is>
       </c>
       <c r="F426" t="inlineStr"/>
@@ -17478,12 +17498,12 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t>BV1oUSuB5EpY</t>
+          <t>BV1GJdUBFEgM，BV1oUSuB5EpY</t>
         </is>
       </c>
       <c r="J426" t="inlineStr"/>
@@ -17975,7 +17995,7 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>2025/05/15，2025/09/03，2025/09/13</t>
+          <t>2025/05/15，2025/09/03，2025/09/13，2026/4/20</t>
         </is>
       </c>
       <c r="F439" t="inlineStr"/>
@@ -17986,12 +18006,12 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t>BV1FBEpzhEoM</t>
+          <t>BV1TXd6BvEHP，BV1FBEpzhEoM</t>
         </is>
       </c>
       <c r="J439" t="inlineStr"/>
@@ -19559,7 +19579,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/09/03，2025/09/11，2025/09/29，2025/11/9，2026/1/1</t>
+          <t>2025/05/30，2025/09/03，2025/09/11，2025/09/29，2025/11/9，2026/1/1，2026/4/20</t>
         </is>
       </c>
       <c r="F480" t="inlineStr"/>
@@ -19570,12 +19590,12 @@
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I480" t="inlineStr">
         <is>
-          <t>BV1NBnzzpE7i</t>
+          <t>BV1XJdUBFEhy，BV1NBnzzpE7i</t>
         </is>
       </c>
       <c r="J480" t="inlineStr"/>
@@ -20295,7 +20315,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/07/03，2025/10/09，2026/1/16，2026/3/6，2026/3/14</t>
+          <t>2025/06/02，2025/07/03，2025/10/09，2026/1/16，2026/3/6，2026/3/14，2026/4/20</t>
         </is>
       </c>
       <c r="F499" t="inlineStr"/>
@@ -20306,12 +20326,12 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
         <is>
-          <t>BV1W97Sz3E5m</t>
+          <t>BV162drBtE6U，BV1W97Sz3E5m</t>
         </is>
       </c>
       <c r="J499" t="inlineStr"/>
@@ -20859,7 +20879,7 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>2025/06/09，2025/09/21</t>
+          <t>2025/06/09，2025/09/21，2026/4/20</t>
         </is>
       </c>
       <c r="F514" t="inlineStr"/>
@@ -20870,10 +20890,14 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I514" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>BV1aJdUBFEHK，BV1ykgozjEdD</t>
+        </is>
+      </c>
       <c r="J514" t="inlineStr"/>
     </row>
     <row r="515">
@@ -25071,7 +25095,7 @@
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>2025/9/3</t>
+          <t>2025/9/3，2026/4/20</t>
         </is>
       </c>
       <c r="F624" t="inlineStr"/>
@@ -25082,10 +25106,14 @@
       </c>
       <c r="H624" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I624" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>BV1CFdrBfELv</t>
+        </is>
+      </c>
       <c r="J624" t="inlineStr"/>
     </row>
     <row r="625">
@@ -26143,7 +26171,7 @@
       </c>
       <c r="I652" t="inlineStr">
         <is>
-          <t>BV1TzrrBAEq9</t>
+          <t>BV1HJocBmEnK，BV1TzrrBAEq9</t>
         </is>
       </c>
       <c r="J652" t="inlineStr"/>
@@ -29747,7 +29775,7 @@
       </c>
       <c r="E748" t="inlineStr">
         <is>
-          <t>2025/12/2</t>
+          <t>2025/12/2，2026/4/20</t>
         </is>
       </c>
       <c r="F748" t="inlineStr"/>
@@ -29758,10 +29786,14 @@
       </c>
       <c r="H748" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I748" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>BV1modkBzE44，BV1rdSbB3Eor</t>
+        </is>
+      </c>
       <c r="J748" t="inlineStr"/>
     </row>
     <row r="749">
@@ -30471,7 +30503,7 @@
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11，2026/4/20</t>
         </is>
       </c>
       <c r="F767" t="inlineStr"/>
@@ -30482,12 +30514,12 @@
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
         <is>
-          <t>BV1pfzcBgERV，BV1aff2BvEZF</t>
+          <t>BV1UodkBzEgD，BV1pfzcBgERV，BV1aff2BvEZF</t>
         </is>
       </c>
       <c r="J767" t="inlineStr">
@@ -31139,7 +31171,7 @@
       </c>
       <c r="E784" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28，2026/4/12</t>
+          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28，2026/4/12，2026/4/20</t>
         </is>
       </c>
       <c r="F784" t="inlineStr"/>
@@ -31150,12 +31182,12 @@
       </c>
       <c r="H784" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I784" t="inlineStr">
         <is>
-          <t>BV1Dv6qBsEXr</t>
+          <t>BV1zPDSBhEqa，BV1Dv6qBsEXr</t>
         </is>
       </c>
       <c r="J784" t="inlineStr">
@@ -31459,7 +31491,7 @@
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20</t>
         </is>
       </c>
       <c r="F792" t="inlineStr"/>
@@ -31470,12 +31502,12 @@
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
         <is>
-          <t>BV1W4cuzSE8Y，BV12Ef6BBE5C</t>
+          <t>BV1HW9jBJEUE，BV1W4cuzSE8Y，BV12Ef6BBE5C</t>
         </is>
       </c>
       <c r="J792" t="inlineStr">
@@ -31867,7 +31899,7 @@
       </c>
       <c r="E802" t="inlineStr">
         <is>
-          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25，2026/3/14</t>
+          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25，2026/3/14，2026/4/20</t>
         </is>
       </c>
       <c r="F802" t="inlineStr"/>
@@ -31878,12 +31910,12 @@
       </c>
       <c r="H802" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I802" t="inlineStr">
         <is>
-          <t>BV1K7f6BgE9r</t>
+          <t>BV1modkBzEQ9，BV1K7f6BgE9r</t>
         </is>
       </c>
       <c r="J802" t="inlineStr">
@@ -31991,7 +32023,7 @@
       </c>
       <c r="E805" t="inlineStr">
         <is>
-          <t>2026/2/25，2026/2/28，2026/3/1</t>
+          <t>2026/2/25，2026/2/28，2026/3/1，2026/4/20</t>
         </is>
       </c>
       <c r="F805" t="inlineStr"/>
@@ -32002,12 +32034,12 @@
       </c>
       <c r="H805" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I805" t="inlineStr">
         <is>
-          <t>BV1WDfaByEfD</t>
+          <t>BV1bodkB6EMm，BV1WDfaByEfD</t>
         </is>
       </c>
       <c r="J805" t="inlineStr">
@@ -32075,7 +32107,7 @@
       </c>
       <c r="E807" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20</t>
         </is>
       </c>
       <c r="F807" t="inlineStr"/>
@@ -32086,12 +32118,12 @@
       </c>
       <c r="H807" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I807" t="inlineStr">
         <is>
-          <t>BV1n5PMzSEAz</t>
+          <t>BV1ea9GBtE8q，BV1n5PMzSEAz</t>
         </is>
       </c>
       <c r="J807" t="inlineStr">
@@ -32447,7 +32479,7 @@
       </c>
       <c r="E816" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/25，2026/3/28，2026/4/11</t>
+          <t>2026/3/13，2026/3/25，2026/3/28，2026/4/11，2026/4/20</t>
         </is>
       </c>
       <c r="F816" t="inlineStr"/>
@@ -32458,7 +32490,7 @@
       </c>
       <c r="H816" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I816" t="inlineStr">
@@ -32879,7 +32911,7 @@
       </c>
       <c r="E827" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20</t>
         </is>
       </c>
       <c r="F827" t="inlineStr"/>
@@ -32890,7 +32922,7 @@
       </c>
       <c r="H827" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I827" t="inlineStr">
@@ -33839,6 +33871,54 @@
           <t>游戏</t>
         </is>
       </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr"/>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>最初的梦想</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr"/>
+      <c r="D851" t="inlineStr"/>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>2026/4/20</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr"/>
+      <c r="G851" t="inlineStr"/>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr"/>
+      <c r="J851" t="inlineStr"/>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr"/>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>勿听</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr"/>
+      <c r="D852" t="inlineStr"/>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>2026/4/20</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr"/>
+      <c r="G852" t="inlineStr"/>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr"/>
+      <c r="J852" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 24, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J852"/>
+  <dimension ref="A1:J855"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1，2026/4/14</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1，2026/4/14，2026/4/24</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11，2026/4/16</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11，2026/4/16，2026/4/23</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BV1tBdeBDEfp，BV1PzPizTEty，BV1cG9pYkE8m，BV1B1fGBjEvg</t>
+          <t>BV1yKo7BhEaJ，BV1tBdeBDEfp，BV1PzPizTEty，BV1cG9pYkE8m，BV1B1fGBjEvg</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BV1wUojYeEon</t>
+          <t>BV1hYobBkEum，BV1wUojYeEon</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/1/21，2026/1/25，2026/2/10，2026/2/23，2026/3/6，2026/3/22</t>
+          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/1/21，2026/1/25，2026/2/10，2026/2/23，2026/3/6，2026/3/22，2026/4/24</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2934,12 +2934,12 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>BV1ZEigB2ED4</t>
+          <t>BV1JQQDB3EDr，BV1ZEigB2ED4</t>
         </is>
       </c>
       <c r="J61" t="inlineStr"/>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/2/2，2026/2/12，2026/4/14</t>
+          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/2/2，2026/2/12，2026/4/14，2026/4/22</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3222,12 +3222,12 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>BV1Qky3BbEbV</t>
+          <t>BV1GrQVBWE3y，BV1Qky3BbEbV</t>
         </is>
       </c>
       <c r="J68" t="inlineStr"/>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14，2026/4/22</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5190,12 +5190,12 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>BV1GBQ3BmEBA，BV1kcAXzVEWt，BV1QhgpzdEb7</t>
+          <t>BV1GbobBLEDi，BV1GBQ3BmEBA，BV1kcAXzVEWt，BV1QhgpzdEb7</t>
         </is>
       </c>
       <c r="J116" t="inlineStr"/>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9，2026/4/14</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9，2026/4/14，2026/4/24</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5270,12 +5270,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>BV1DrQ3ByECZ，BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
+          <t>BV1jPoEBQEPw，BV1DrQ3ByECZ，BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
         </is>
       </c>
       <c r="J118" t="inlineStr"/>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25，2026/4/24</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/8，2025/12/24，2026/1/28</t>
+          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/8，2025/12/24，2026/1/28，2026/4/22</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -6634,12 +6634,12 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>BV143MzzoEpV</t>
+          <t>BV1bBobBuETA，BV143MzzoEpV</t>
         </is>
       </c>
       <c r="J152" t="inlineStr"/>
@@ -6867,7 +6867,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/11，2025/04/22，2025/05/08，2025/06/12，2025/08/22，2025/08/29，2025/09/05，2025/11/19，2025/12/31，2026/2/14</t>
+          <t>2025/03/20，2025/04/11，2025/04/22，2025/05/08，2025/06/12，2025/08/22，2025/08/29，2025/09/05，2025/11/19，2025/12/31，2026/2/14，2026/4/24</t>
         </is>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -6878,12 +6878,12 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>BV1BPvDBxEPY</t>
+          <t>BV1iKoEBnEnK，BV1BPvDBxEPY</t>
         </is>
       </c>
       <c r="J158" t="inlineStr"/>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/12，2025/12/7</t>
+          <t>2025/03/21，2025/05/12，2025/12/7，2026/4/24</t>
         </is>
       </c>
       <c r="F164" t="inlineStr"/>
@@ -7118,12 +7118,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>BV1TWY1zgE8f，BV1b2MtzPEBw</t>
+          <t>BV1YGoEBjE8F，BV1TWY1zgE8f，BV1b2MtzPEBw</t>
         </is>
       </c>
       <c r="J164" t="inlineStr"/>
@@ -7303,7 +7303,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/24，2025/06/05，2025/07/26，2025/09/21，2025/10/16，2025/10/30，2025/11/9，2026/1/9</t>
+          <t>2025/03/21，2025/04/24，2025/06/05，2025/07/26，2025/09/21，2025/10/16，2025/10/30，2025/11/9，2026/1/9，2026/4/24</t>
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
@@ -7314,12 +7314,12 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>BV1jrrMBQEz7，BV1oTT8zyEX4，BV1bKXCYVExo</t>
+          <t>BV17yoEBsEVA，BV1jrrMBQEz7，BV1oTT8zyEX4，BV1bKXCYVExo</t>
         </is>
       </c>
       <c r="J169" t="inlineStr"/>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8，2026/4/24</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9962,12 +9962,12 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>BV1aPjfzkEww</t>
+          <t>BV15uoEBEELW，BV1aPjfzkEww</t>
         </is>
       </c>
       <c r="J235" t="inlineStr"/>
@@ -9991,7 +9991,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15，2026/4/24</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -10002,12 +10002,12 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>BV1Xkw3zgEHg，BV1XWWNzyE2d</t>
+          <t>BV1paoEBYEs3，BV1Xkw3zgEHg，BV1XWWNzyE2d</t>
         </is>
       </c>
       <c r="J236" t="inlineStr"/>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18</t>
+          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/4/22</t>
         </is>
       </c>
       <c r="F246" t="inlineStr"/>
@@ -10410,12 +10410,12 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>BV1J3y5B7EnS，BV1cJ7Kz1EMG</t>
+          <t>BV1G8obByELW，BV1J3y5B7EnS，BV1cJ7Kz1EMG</t>
         </is>
       </c>
       <c r="J246" t="inlineStr"/>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25，2026/4/24</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11690,12 +11690,12 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>BV1Yj7DzxEm9，BV1fjcYzCEPz，BV1V37DzfEhn</t>
+          <t>BV1qAoEBpEEZ，BV1Yj7DzxEm9，BV1fjcYzCEPz，BV1V37DzfEhn</t>
         </is>
       </c>
       <c r="J278" t="inlineStr"/>
@@ -12739,7 +12739,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/1/29，2026/3/20</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/1/29，2026/3/20，2026/4/22</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12750,12 +12750,12 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>BV1ugBMBAEFM，BV1TBCJB3EMp，BV1dscYzMEKG，BV1D8GdzWE7M</t>
+          <t>BV1GbobBLEBY，BV1ugBMBAEFM，BV1TBCJB3EMp，BV1dscYzMEKG，BV1D8GdzWE7M</t>
         </is>
       </c>
       <c r="J305" t="inlineStr"/>
@@ -13015,7 +13015,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/2/23，2026/3/6</t>
+          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/2/23，2026/3/6，2026/4/22</t>
         </is>
       </c>
       <c r="F312" t="inlineStr"/>
@@ -13026,12 +13026,12 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>BV1cnWpzrEtD，BV1FSfzBbEpH</t>
+          <t>BV1GbobBLEza，BV1cnWpzrEtD，BV1FSfzBbEpH</t>
         </is>
       </c>
       <c r="J312" t="inlineStr"/>
@@ -13827,7 +13827,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>2025/04/12，2025/07/14，2025/09/24，2025/09/28，2025/11/9</t>
+          <t>2025/04/12，2025/07/14，2025/09/24，2025/09/28，2025/11/9，2026/4/24</t>
         </is>
       </c>
       <c r="F333" t="inlineStr"/>
@@ -13838,7 +13838,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/1/16，2026/3/25</t>
+          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/1/16，2026/3/25，2026/4/24</t>
         </is>
       </c>
       <c r="F347" t="inlineStr"/>
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -15231,7 +15231,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/22</t>
+          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/22，2026/4/24</t>
         </is>
       </c>
       <c r="F368" t="inlineStr"/>
@@ -15242,7 +15242,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -15863,7 +15863,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>2025/04/24，2025/05/25，2025/12/2，2025/12/31</t>
+          <t>2025/04/24，2025/05/25，2025/12/2，2025/12/31，2026/4/24</t>
         </is>
       </c>
       <c r="F384" t="inlineStr"/>
@@ -15874,12 +15874,12 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">
         <is>
-          <t>BV1L5jGzJEY5</t>
+          <t>BV1waoEBYEZa，BV1L5jGzJEY5</t>
         </is>
       </c>
       <c r="J384" t="inlineStr"/>
@@ -16091,7 +16091,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31</t>
+          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31，2026/4/24</t>
         </is>
       </c>
       <c r="F390" t="inlineStr"/>
@@ -16102,12 +16102,12 @@
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>BV1aEpBzPEEq，BV1AMLHzHEA7</t>
+          <t>BV1zzoEBZEQn，BV1aEpBzPEEq，BV1AMLHzHEA7</t>
         </is>
       </c>
       <c r="J390" t="inlineStr"/>
@@ -16167,7 +16167,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/23，2025/12/5，2026/2/14，2026/4/9</t>
+          <t>2025/04/25，2025/06/23，2025/12/5，2026/2/14，2026/4/9，2026/4/24</t>
         </is>
       </c>
       <c r="F392" t="inlineStr"/>
@@ -16178,12 +16178,12 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t>BV1M72EB2EvZ</t>
+          <t>BV1BroEB4E98，BV1M72EB2EvZ</t>
         </is>
       </c>
       <c r="J392" t="inlineStr"/>
@@ -18907,7 +18907,7 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/06/17，2025/07/21，2025/08/16，2025/10/16，2025/12/2</t>
+          <t>2025/05/22，2025/06/17，2025/07/21，2025/08/16，2025/10/16，2025/12/2，2026/4/22</t>
         </is>
       </c>
       <c r="F462" t="inlineStr"/>
@@ -18918,10 +18918,14 @@
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="I462" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>BV138obByE21</t>
+        </is>
+      </c>
       <c r="J462" t="inlineStr"/>
     </row>
     <row r="463">
@@ -19055,7 +19059,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>2025/05/23，2025/06/26，2025/07/21，2025/08/12，2025/09/10，2025/09/19，2025/11/1，2025/12/9，2025/12/13，2026/2/14</t>
+          <t>2025/05/23，2025/06/26，2025/07/21，2025/08/12，2025/09/10，2025/09/19，2025/11/1，2025/12/9，2025/12/13，2026/2/14，2026/4/24</t>
         </is>
       </c>
       <c r="F466" t="inlineStr"/>
@@ -19066,12 +19070,12 @@
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I466" t="inlineStr">
         <is>
-          <t>BV1K1yXBBEQ6</t>
+          <t>BV1Bjo7B9E31，BV1K1yXBBEQ6</t>
         </is>
       </c>
       <c r="J466" t="inlineStr"/>
@@ -20275,7 +20279,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5，2026/3/17</t>
+          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5，2026/3/17，2026/4/24</t>
         </is>
       </c>
       <c r="F498" t="inlineStr"/>
@@ -20286,7 +20290,7 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
@@ -21111,7 +21115,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22</t>
         </is>
       </c>
       <c r="F520" t="inlineStr"/>
@@ -21122,12 +21126,12 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I520" t="inlineStr">
         <is>
-          <t>BV1dgmMBeEF4</t>
+          <t>BV1g9ojB6Esh，BV1dgmMBeEF4</t>
         </is>
       </c>
       <c r="J520" t="inlineStr"/>
@@ -21763,7 +21767,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -21774,7 +21778,7 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
@@ -23791,7 +23795,7 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24</t>
         </is>
       </c>
       <c r="F590" t="inlineStr"/>
@@ -23802,12 +23806,12 @@
       </c>
       <c r="H590" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I590" t="inlineStr">
         <is>
-          <t>BV19UbDzXE7H</t>
+          <t>BV1xxoEBqE8N，BV19UbDzXE7H</t>
         </is>
       </c>
       <c r="J590" t="inlineStr"/>
@@ -24783,7 +24787,7 @@
       </c>
       <c r="E616" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10，2026/4/23</t>
         </is>
       </c>
       <c r="F616" t="inlineStr"/>
@@ -24794,12 +24798,12 @@
       </c>
       <c r="H616" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I616" t="inlineStr">
         <is>
-          <t>BV1RUSTBiEa5</t>
+          <t>BV1NNo7BAEid，BV1RUSTBiEa5</t>
         </is>
       </c>
       <c r="J616" t="inlineStr"/>
@@ -25475,7 +25479,7 @@
       </c>
       <c r="E634" t="inlineStr">
         <is>
-          <t>2025/9/12</t>
+          <t>2025/9/12，2026/4/24</t>
         </is>
       </c>
       <c r="F634" t="inlineStr"/>
@@ -25486,10 +25490,14 @@
       </c>
       <c r="H634" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I634" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>BV19UoEBDEHt，BV1AYHrztEi4</t>
+        </is>
+      </c>
       <c r="J634" t="inlineStr"/>
     </row>
     <row r="635">
@@ -26155,7 +26163,7 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>2025/09/15，2025/10/19，2025/10/20，2025/10/26，2025/11/1，2025/11/14，2026/1/15，2026/1/23，2026/4/19</t>
+          <t>2025/09/15，2025/10/19，2025/10/20，2025/10/26，2025/11/1，2025/11/14，2026/1/15，2026/1/23，2026/4/19，2026/4/24</t>
         </is>
       </c>
       <c r="F652" t="inlineStr"/>
@@ -26166,12 +26174,12 @@
       </c>
       <c r="H652" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I652" t="inlineStr">
         <is>
-          <t>BV1HJocBmEnK，BV1TzrrBAEq9</t>
+          <t>BV17koEBdEfu，BV1HJocBmEnK，BV1TzrrBAEq9</t>
         </is>
       </c>
       <c r="J652" t="inlineStr"/>
@@ -28539,7 +28547,7 @@
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/1，2025/11/12，2025/11/26，2025/12/8，2026/1/2，2026/1/5，2026/1/9，2026/2/23，2026/3/14，2026/3/29</t>
+          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/1，2025/11/12，2025/11/26，2025/12/8，2026/1/2，2026/1/5，2026/1/9，2026/2/23，2026/3/14，2026/3/29，2026/4/24</t>
         </is>
       </c>
       <c r="F715" t="inlineStr"/>
@@ -28550,12 +28558,12 @@
       </c>
       <c r="H715" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I715" t="inlineStr">
         <is>
-          <t>BV1TBihBsEo5，BV1ksf6BeE2k</t>
+          <t>BV1VgoEBmEpE，BV1TBihBsEo5，BV1ksf6BeE2k</t>
         </is>
       </c>
       <c r="J715" t="inlineStr"/>
@@ -28775,7 +28783,7 @@
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>2025/11/3</t>
+          <t>2025/11/3，2026/4/24</t>
         </is>
       </c>
       <c r="F721" t="inlineStr"/>
@@ -28786,10 +28794,14 @@
       </c>
       <c r="H721" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I721" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>BV1ZroEBxEAc</t>
+        </is>
+      </c>
       <c r="J721" t="inlineStr"/>
     </row>
     <row r="722">
@@ -30587,7 +30599,7 @@
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27，2026/4/24</t>
         </is>
       </c>
       <c r="F769" t="inlineStr"/>
@@ -30598,7 +30610,7 @@
       </c>
       <c r="H769" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I769" t="inlineStr">
@@ -33873,21 +33885,33 @@
       </c>
     </row>
     <row r="851">
-      <c r="A851" t="inlineStr"/>
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
       <c r="B851" t="inlineStr">
         <is>
           <t>最初的梦想</t>
         </is>
       </c>
       <c r="C851" t="inlineStr"/>
-      <c r="D851" t="inlineStr"/>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>范玮琪</t>
+        </is>
+      </c>
       <c r="E851" t="inlineStr">
         <is>
           <t>2026/4/20</t>
         </is>
       </c>
       <c r="F851" t="inlineStr"/>
-      <c r="G851" t="inlineStr"/>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
       <c r="H851" t="inlineStr">
         <is>
           <t>1</t>
@@ -33897,28 +33921,156 @@
       <c r="J851" t="inlineStr"/>
     </row>
     <row r="852">
-      <c r="A852" t="inlineStr"/>
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>851</t>
+        </is>
+      </c>
       <c r="B852" t="inlineStr">
         <is>
           <t>勿听</t>
         </is>
       </c>
       <c r="C852" t="inlineStr"/>
-      <c r="D852" t="inlineStr"/>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>张紫宁/赵紫骅/游戏科学</t>
+        </is>
+      </c>
       <c r="E852" t="inlineStr">
         <is>
           <t>2026/4/20</t>
         </is>
       </c>
       <c r="F852" t="inlineStr"/>
-      <c r="G852" t="inlineStr"/>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
       <c r="H852" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="I852" t="inlineStr"/>
-      <c r="J852" t="inlineStr"/>
+      <c r="J852" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>852</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Everywhere we go</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr"/>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>陈冠希/MC仁/厨房仔/应采儿</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>2026/4/24</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr"/>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>粤语</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr"/>
+      <c r="J853" t="inlineStr"/>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>853</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Komm,susser Tod</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr"/>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>ARIANNE</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>2026/4/24</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr"/>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr"/>
+      <c r="J854" t="inlineStr">
+        <is>
+          <t>动漫</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>854</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>突然好想你</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr"/>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>五月天</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>2026/4/24</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr"/>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr"/>
+      <c r="J855" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 26, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/04，2025/04/14，2025/04/20，2025/04/24，2025/05/09，2025/05/18，2025/05/29，2025/06/06，2025/08/01，2025/09/21，2025/10/10，2025/11/28，2025/12/8，2025/12/30</t>
+          <t>2025/03/03，2025/04/04，2025/04/14，2025/04/20，2025/04/24，2025/05/09，2025/05/18，2025/05/29，2025/06/06，2025/08/01，2025/09/21，2025/10/10，2025/11/28，2025/12/8，2025/12/30，2026/4/26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/21，2025/04/05，2025/04/14，2025/04/24，2025/05/20，2025/06/05，2025/06/17，2025/06/23，2025/06/26，2025/08/12，2025/08/21，2025/09/14，2025/09/24，2025/10/16，2025/10/24，2025/12/17，2026/2/14，2026/3/8</t>
+          <t>2025/03/04，2025/03/21，2025/04/05，2025/04/14，2025/04/24，2025/05/20，2025/06/05，2025/06/17，2025/06/23，2025/06/26，2025/08/12，2025/08/21，2025/09/14，2025/09/24，2025/10/16，2025/10/24，2025/12/17，2026/2/14，2026/3/8，2026/4/25</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1894,12 +1894,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>BV1QWZJBDEJf</t>
+          <t>BV1KgodBVELy，BV1QWZJBDEJf</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21，2026/4/26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2094,12 +2094,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>BV1rXkLBnEfb</t>
+          <t>BV1ryoeBzEFq，BV1rXkLBnEfb</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/06，2025/04/13，2025/04/22，2025/05/08，2025/05/09，2025/05/30，2025/06/08，2025/08/04，2025/09/18，2025/10/12，2025/11/21，2026/1/24，2026/2/14，2026/2/25，2026/4/10</t>
+          <t>2025/03/06，2025/04/06，2025/04/13，2025/04/22，2025/05/08，2025/05/09，2025/05/30，2025/06/08，2025/08/04，2025/09/18，2025/10/12，2025/11/21，2026/1/24，2026/2/14，2026/2/25，2026/4/10，2026/4/25</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2402,12 +2402,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>BV1vazyB2Emo</t>
+          <t>BV1TModByEji，BV1vazyB2Emo</t>
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,12 +2974,12 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>BV1C9Q3BiE8m，BV1BFXUBwEDj，BV191NVzoEZ7，BV1TzrrBAEpz，BV1L5fUB5Ebn，BV1g9M3zsE7c</t>
+          <t>BV1wCoeB3EVt，BV1C9Q3BiE8m，BV1BFXUBwEDj，BV191NVzoEZ7，BV1TzrrBAEpz，BV1L5fUB5Ebn，BV1g9M3zsE7c</t>
         </is>
       </c>
       <c r="J62" t="inlineStr"/>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22</t>
+          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/4/26</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/9，2026/3/25</t>
+          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/9，2026/3/25，2026/4/26</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/17，2025/05/13，2025/05/23，2025/07/21，2025/07/29，2025/08/07，2025/09/30，2025/10/31，2025/12/9，2026/1/12</t>
+          <t>2025/03/17，2025/04/17，2025/05/13，2025/05/23，2025/07/21，2025/07/29，2025/08/07，2025/09/30，2025/10/31，2025/12/9，2026/1/12，2026/4/26</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/9</t>
+          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/9，2026/4/26</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24</t>
+          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/4/26</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -6550,7 +6550,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24，2026/4/26</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/07，2025/04/18，2025/05/08，2025/10/24，2025/12/12</t>
+          <t>2025/03/21，2025/04/07，2025/04/18，2025/05/08，2025/10/24，2025/12/12，2026/4/26</t>
         </is>
       </c>
       <c r="F181" t="inlineStr"/>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/9，2026/1/1，2026/2/7，2026/3/25</t>
+          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/9，2026/1/1，2026/2/7，2026/3/25，2026/4/26</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -8434,7 +8434,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -10715,7 +10715,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/06/19</t>
+          <t>2025/04/01，2025/06/19，2026/4/25</t>
         </is>
       </c>
       <c r="F254" t="inlineStr"/>
@@ -10726,7 +10726,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/13，2025/05/10，2025/05/26，2025/06/02，2025/06/05，2025/06/17，2025/08/04，2025/09/10，2025/09/30，2025/10/16，2025/11/17，2025/12/6，2025/12/31</t>
+          <t>2025/04/02，2025/04/13，2025/05/10，2025/05/26，2025/06/02，2025/06/05，2025/06/17，2025/08/04，2025/09/10，2025/09/30，2025/10/16，2025/11/17，2025/12/6，2025/12/31，2026/4/26</t>
         </is>
       </c>
       <c r="F269" t="inlineStr"/>
@@ -11326,7 +11326,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -11599,7 +11599,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/05/17，2025/05/29，2025/06/16，2025/07/10，2025/08/24，2025/10/16，2025/11/26</t>
+          <t>2025/04/03，2025/05/17，2025/05/29，2025/06/16，2025/07/10，2025/08/24，2025/10/16，2025/11/26，2026/4/26</t>
         </is>
       </c>
       <c r="F276" t="inlineStr"/>
@@ -11610,7 +11610,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -17063,7 +17063,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>2025/05/02，2025/05/15，2025/06/14，2026/2/19</t>
+          <t>2025/05/02，2025/05/15，2025/06/14，2026/2/19，2026/4/26</t>
         </is>
       </c>
       <c r="F415" t="inlineStr"/>
@@ -17074,7 +17074,7 @@
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
@@ -17219,7 +17219,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/06/13，2025/09/08</t>
+          <t>2025/05/03，2025/06/13，2025/09/08，2026/4/25</t>
         </is>
       </c>
       <c r="F419" t="inlineStr"/>
@@ -17230,12 +17230,12 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t>BV1tCRhYjEgs</t>
+          <t>BV12ModBCE8W，BV1tCRhYjEgs</t>
         </is>
       </c>
       <c r="J419" t="inlineStr"/>
@@ -27719,7 +27719,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25，2026/4/1</t>
+          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25，2026/4/1，2026/4/25</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -27734,7 +27734,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Apr 27, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -930,12 +930,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>BV192j6zcEWE，BV1Sr7SzJEij</t>
+          <t>BV1Pfo2BUEHM，BV192j6zcEWE，BV1Sr7SzJEij</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28，2026/3/29</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28，2026/3/29，2026/4/27</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6834,12 +6834,12 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>BV18mXyBCEzT，BV15uzuB1ECd</t>
+          <t>BV1t4o1BDEdb，BV18mXyBCEzT，BV15uzuB1ECd</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/1/1，2026/1/25，2026/3/8</t>
+          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/1/1，2026/1/25，2026/3/8，2026/4/27</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
@@ -10490,12 +10490,12 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>BV11fVSzAEHq</t>
+          <t>BV1Cfo2BmED3，BV11fVSzAEHq</t>
         </is>
       </c>
       <c r="J248" t="inlineStr"/>
@@ -27139,7 +27139,7 @@
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22</t>
+          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22，2026/4/27</t>
         </is>
       </c>
       <c r="F678" t="inlineStr"/>
@@ -27150,12 +27150,12 @@
       </c>
       <c r="H678" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I678" t="inlineStr">
         <is>
-          <t>BV126rrBhEun</t>
+          <t>BV1yfo2BmEuU，BV126rrBhEun</t>
         </is>
       </c>
       <c r="J678" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: Update song list to Apr 29, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/20，2025/06/16，2025/06/27，2025/07/31，2025/10/05，2025/11/7，2025/12/4，2026/1/28</t>
+          <t>2025/03/03，2025/04/20，2025/06/16，2025/06/27，2025/07/31，2025/10/05，2025/11/7，2025/12/4，2026/1/28，2026/4/29</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -810,12 +810,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BV1pbEuzFEaX</t>
+          <t>BV1yd9xBEEC8，BV1pbEuzFEaX</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3934,12 +3934,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>BV1L2StBbEWk</t>
+          <t>BV1VC9jBiEcL，BV133Vdz8Eyi</t>
         </is>
       </c>
       <c r="J85" t="inlineStr"/>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/05/12，2025/05/22，2025/06/16，2025/06/30，2025/08/01，2025/08/16，2025/09/19，2025/10/05，2025/11/18，2025/12/23，2026/1/9，2026/2/27</t>
+          <t>2025/03/13，2025/05/12，2025/05/22，2025/06/16，2025/06/30，2025/08/01，2025/08/16，2025/09/19，2025/10/05，2025/11/18，2025/12/23，2026/1/9，2026/2/27，2026/4/29</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>BV1cRB1BoENX</t>
+          <t>BV1Jh9DBkE1q，BV1cRB1BoENX</t>
         </is>
       </c>
       <c r="J98" t="inlineStr"/>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11，2026/4/14</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11，2026/4/14，2026/4/29</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>2025/04/18，2025/05/29，2025/06/23，2025/09/21，2025/10/07，2026/1/10</t>
+          <t>2025/04/18，2025/05/29，2025/06/23，2025/09/21，2025/10/07，2026/1/10，2026/4/29</t>
         </is>
       </c>
       <c r="F364" t="inlineStr"/>
@@ -15078,7 +15078,7 @@
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I364" t="inlineStr">
@@ -17755,7 +17755,7 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05</t>
+          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/4/29</t>
         </is>
       </c>
       <c r="F433" t="inlineStr"/>
@@ -17766,7 +17766,7 @@
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I433" t="inlineStr">
@@ -18347,7 +18347,7 @@
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/1/2，2026/3/17</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/1/2，2026/3/17，2026/4/29</t>
         </is>
       </c>
       <c r="F448" t="inlineStr"/>
@@ -18358,7 +18358,7 @@
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I448" t="inlineStr">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/12，2025/10/03，2025/10/11，2026/1/15</t>
+          <t>2025/05/22，2025/09/12，2025/10/03，2025/10/11，2026/1/15，2026/4/29</t>
         </is>
       </c>
       <c r="F461" t="inlineStr"/>
@@ -18874,7 +18874,7 @@
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I461" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>2025/05/23，2025/05/29，2025/09/17，2025/09/02，2025/09/26，2025/10/09，2025/10/24</t>
+          <t>2025/05/23，2025/05/29，2025/09/17，2025/09/02，2025/09/26，2025/10/09，2025/10/24，2026/4/29</t>
         </is>
       </c>
       <c r="F463" t="inlineStr"/>
@@ -18958,7 +18958,7 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
@@ -30027,7 +30027,7 @@
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>2025/12/11，2025/12/12，2025/12/17，2026/1/2，2026/1/5，2026/1/11，2026/1/17，2026/1/29，2026/2/9，2026/3/28</t>
+          <t>2025/12/11，2025/12/12，2025/12/17，2026/1/2，2026/1/5，2026/1/11，2026/1/17，2026/1/29，2026/2/9，2026/3/28，2026/4/29</t>
         </is>
       </c>
       <c r="F754" t="inlineStr"/>
@@ -30038,7 +30038,7 @@
       </c>
       <c r="H754" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I754" t="inlineStr">
@@ -30319,7 +30319,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29，2026/3/22</t>
+          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29，2026/3/22，2026/4/29</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30330,7 +30330,7 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -30435,7 +30435,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -30446,7 +30446,7 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -32575,7 +32575,7 @@
       </c>
       <c r="E818" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/14，2026/3/28</t>
+          <t>2026/3/13，2026/3/14，2026/3/28，2026/4/29</t>
         </is>
       </c>
       <c r="F818" t="inlineStr"/>
@@ -32586,7 +32586,7 @@
       </c>
       <c r="H818" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I818" t="inlineStr">
@@ -33779,7 +33779,7 @@
       </c>
       <c r="E848" t="inlineStr">
         <is>
-          <t>2026/4/16</t>
+          <t>2026/4/16，2026/4/29</t>
         </is>
       </c>
       <c r="F848" t="inlineStr"/>
@@ -33790,7 +33790,7 @@
       </c>
       <c r="H848" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I848" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to May 1, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J855"/>
+  <dimension ref="A1:J860"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,7 +919,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27，2026/5/1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -930,7 +930,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15，2026/5/1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7，2026/3/17，2026/3/21</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/9，2025/12/16，2026/2/14，2026/3/7，2026/3/17，2026/3/21，2026/5/1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/7，2025/12/24，2026/1/1，2026/1/16，2026/3/14</t>
+          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/7，2025/12/24，2026/1/1，2026/1/16，2026/3/14，2026/5/1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17</t>
+          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17，2026/5/1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19，2026/5/1</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>63</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/1/19，2026/4/18</t>
+          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/1/19，2026/4/18，2026/5/1</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31，2026/4/20</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31，2026/4/20，2026/5/1</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15，2026/4/2</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15，2026/4/2，2026/5/1</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13，2026/3/14，2026/3/31</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/8，2026/2/18，2026/3/6，2026/3/13，2026/3/14，2026/3/31，2026/5/1</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12，2026/4/1</t>
+          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12，2026/4/1，2026/5/1</t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/24，2025/05/15，2025/05/29，2025/09/21，2025/09/27，2025/10/24，2026/1/5，2026/2/9，2026/3/15</t>
+          <t>2025/03/30，2025/04/24，2025/05/15，2025/05/29，2025/09/21，2025/09/27，2025/10/24，2026/1/5，2026/2/9，2026/3/15，2026/5/1</t>
         </is>
       </c>
       <c r="F244" t="inlineStr"/>
@@ -10330,7 +10330,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -10715,7 +10715,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/06/19，2026/4/25</t>
+          <t>2025/04/01，2025/06/19，2026/4/25，2026/5/1</t>
         </is>
       </c>
       <c r="F254" t="inlineStr"/>
@@ -10726,7 +10726,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8，2026/5/1</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10846,7 +10846,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -11519,7 +11519,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13，2026/3/17</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13，2026/3/17，2026/5/1</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11530,7 +11530,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -13943,7 +13943,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13954,7 +13954,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -14035,7 +14035,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19</t>
+          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19，2026/5/1</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -14046,7 +14046,7 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/18，2025/08/28，2026/1/16</t>
+          <t>2025/04/13，2025/04/18，2025/08/28，2026/1/16，2026/5/1</t>
         </is>
       </c>
       <c r="F339" t="inlineStr"/>
@@ -14090,7 +14090,7 @@
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
@@ -17179,7 +17179,7 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/07/18，2025/08/02，2025/10/16</t>
+          <t>2025/05/03，2025/07/18，2025/08/02，2025/10/16，2026/5/1</t>
         </is>
       </c>
       <c r="F418" t="inlineStr"/>
@@ -17190,7 +17190,7 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
@@ -18579,7 +18579,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/6，2026/3/22</t>
+          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/6，2026/3/22，2026/5/1</t>
         </is>
       </c>
       <c r="F454" t="inlineStr"/>
@@ -18590,7 +18590,7 @@
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I454" t="inlineStr">
@@ -20847,7 +20847,7 @@
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>2025/06/09，2025/09/26，2025/10/17，2025/10/25</t>
+          <t>2025/06/09，2025/09/26，2025/10/17，2025/10/25，2026/5/1</t>
         </is>
       </c>
       <c r="F513" t="inlineStr"/>
@@ -20858,10 +20858,14 @@
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="I513" t="inlineStr"/>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>BV1mzgozEEKv</t>
+        </is>
+      </c>
       <c r="J513" t="inlineStr"/>
     </row>
     <row r="514">
@@ -22191,7 +22195,7 @@
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/3/8</t>
+          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/3/8，2026/5/1</t>
         </is>
       </c>
       <c r="F548" t="inlineStr"/>
@@ -22202,7 +22206,7 @@
       </c>
       <c r="H548" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I548" t="inlineStr">
@@ -22231,7 +22235,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22，2026/4/11</t>
+          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22，2026/4/11，2026/4/30</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -26503,7 +26507,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1</t>
         </is>
       </c>
       <c r="F661" t="inlineStr"/>
@@ -26514,7 +26518,7 @@
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
@@ -29083,7 +29087,7 @@
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9，2026/3/25</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9，2026/3/25，2026/5/1</t>
         </is>
       </c>
       <c r="F729" t="inlineStr"/>
@@ -29094,7 +29098,7 @@
       </c>
       <c r="H729" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I729" t="inlineStr">
@@ -29639,7 +29643,7 @@
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1</t>
         </is>
       </c>
       <c r="F744" t="inlineStr"/>
@@ -29650,7 +29654,7 @@
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I744" t="inlineStr">
@@ -29987,7 +29991,7 @@
       </c>
       <c r="E753" t="inlineStr">
         <is>
-          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25，2026/4/8</t>
+          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25，2026/4/8，2026/5/1</t>
         </is>
       </c>
       <c r="F753" t="inlineStr"/>
@@ -29998,7 +30002,7 @@
       </c>
       <c r="H753" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I753" t="inlineStr">
@@ -30359,7 +30363,7 @@
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>2025/12/19，2026/2/8</t>
+          <t>2025/12/19，2026/2/8，2026/5/1</t>
         </is>
       </c>
       <c r="F763" t="inlineStr"/>
@@ -30370,7 +30374,7 @@
       </c>
       <c r="H763" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I763" t="inlineStr">
@@ -30599,7 +30603,7 @@
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27，2026/4/24</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27，2026/4/24，2026/5/1</t>
         </is>
       </c>
       <c r="F769" t="inlineStr"/>
@@ -30610,7 +30614,7 @@
       </c>
       <c r="H769" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I769" t="inlineStr">
@@ -32539,7 +32543,7 @@
       </c>
       <c r="E817" t="inlineStr">
         <is>
-          <t>2026/3/13</t>
+          <t>2026/3/13，2026/5/1</t>
         </is>
       </c>
       <c r="F817" t="inlineStr"/>
@@ -32550,7 +32554,7 @@
       </c>
       <c r="H817" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I817" t="inlineStr"/>
@@ -34055,7 +34059,7 @@
       </c>
       <c r="E855" t="inlineStr">
         <is>
-          <t>2026/4/24</t>
+          <t>2026/4/24，2026/5/1</t>
         </is>
       </c>
       <c r="F855" t="inlineStr"/>
@@ -34066,11 +34070,207 @@
       </c>
       <c r="H855" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>BV169oSBUEmT</t>
+        </is>
+      </c>
+      <c r="J855" t="inlineStr"/>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>855</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>连名带姓</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr"/>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>张惠妹</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>2026/5/1</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr"/>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I855" t="inlineStr"/>
-      <c r="J855" t="inlineStr"/>
+      <c r="I856" t="inlineStr"/>
+      <c r="J856" t="inlineStr"/>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>856</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>大香蕉</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr"/>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>龙智祥/吴非华</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>2026/5/1</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr"/>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>BV1aBRuBSEj2</t>
+        </is>
+      </c>
+      <c r="J857" t="inlineStr"/>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>857</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>大眠</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr"/>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>王心凌</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>2026/5/1</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr"/>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr"/>
+      <c r="J858" t="inlineStr"/>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>858</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Welcome To New York</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr"/>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>2026/5/1</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr"/>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr"/>
+      <c r="J859" t="inlineStr"/>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>859</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>ふわふわ時間</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>轻飘飘时间</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>樱高轻音部</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>2026/5/1</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr"/>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr"/>
+      <c r="J860" t="inlineStr">
+        <is>
+          <t>动漫</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to May 2, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -6823,7 +6823,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28，2026/3/29，2026/4/27</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28，2026/3/29，2026/4/27，2026/5/2</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -31551,7 +31551,7 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20，2026/5/2</t>
         </is>
       </c>
       <c r="F791" t="inlineStr"/>
@@ -31562,7 +31562,7 @@
       </c>
       <c r="H791" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I791" t="inlineStr">
@@ -32167,7 +32167,7 @@
       </c>
       <c r="E806" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2</t>
         </is>
       </c>
       <c r="F806" t="inlineStr"/>
@@ -32178,7 +32178,7 @@
       </c>
       <c r="H806" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I806" t="inlineStr">
@@ -32975,7 +32975,7 @@
       </c>
       <c r="E826" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20，2026/5/2</t>
         </is>
       </c>
       <c r="F826" t="inlineStr"/>
@@ -32986,7 +32986,7 @@
       </c>
       <c r="H826" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to May 5, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,52 +417,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -2883,7 +2871,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14</t>
+          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14，2026/5/4</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2894,7 +2882,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3007,7 +2995,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/14，2025/05/05，2025/05/19，2025/05/23，2025/06/13，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/12/2，2025/12/26</t>
+          <t>2025/03/07，2025/04/14，2025/05/05，2025/05/19，2025/05/23，2025/06/13，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/12/2，2025/12/26，2026/5/4</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -3018,7 +3006,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3131,7 +3119,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2025/03/08，2025/04/06，2025/05/15，2025/05/26，2025/07/22，2025/09/17，2025/12/30，2026/2/14</t>
+          <t>2025/03/08，2025/04/06，2025/05/15，2025/05/26，2025/07/22，2025/09/17，2025/12/30，2026/2/14，2026/5/4</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -3142,7 +3130,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3463,7 +3451,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/1/15，2026/3/1</t>
+          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/1/15，2026/3/1，2026/5/5</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3474,7 +3462,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5659,7 +5647,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/05/12，2025/06/23，2025/09/04，2025/12/23</t>
+          <t>2025/03/15，2025/05/12，2025/06/23，2025/09/04，2025/12/23，2026/5/5</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -5670,7 +5658,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -6623,7 +6611,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/8，2025/12/24，2026/1/28，2026/4/22</t>
+          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/8，2025/12/24，2026/1/28，2026/4/22，2026/5/5</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -6634,7 +6622,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -7027,7 +7015,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26，2026/5/5</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7038,7 +7026,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7343,7 +7331,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24，2026/4/26</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24，2026/4/26，2026/5/4</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7354,7 +7342,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -7383,7 +7371,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/14，2025/05/12，2025/06/07，2025/07/06，2025/07/21，2025/09/14，2025/10/31，2025/11/9，2026/1/9</t>
+          <t>2025/03/21，2025/04/14，2025/05/12，2025/06/07，2025/07/06，2025/07/21，2025/09/14，2025/10/31，2025/11/9，2026/1/9，2026/5/4</t>
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
@@ -7394,7 +7382,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -9707,7 +9695,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/09，2025/06/07，2025/07/31，2025/08/13，2025/08/21，2025/12/16，2026/1/19</t>
+          <t>2025/03/28，2025/05/09，2025/06/07，2025/07/31，2025/08/13，2025/08/21，2025/12/16，2026/1/19，2026/5/4</t>
         </is>
       </c>
       <c r="F229" t="inlineStr"/>
@@ -9718,7 +9706,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -10915,7 +10903,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17</t>
+          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17，2026/5/5</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
@@ -10926,7 +10914,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -10995,7 +10983,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/12，2025/05/26，2025/08/26，2025/08/16，2025/10/05</t>
+          <t>2025/04/02，2025/05/12，2025/05/26，2025/08/26，2025/08/16，2025/10/05，2026/5/4</t>
         </is>
       </c>
       <c r="F261" t="inlineStr"/>
@@ -11006,7 +10994,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -11235,7 +11223,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/13，2025/05/29，2025/09/04，2025/09/21，2025/10/22，2026/1/1，2026/1/15</t>
+          <t>2025/04/02，2025/05/13，2025/05/29，2025/09/04，2025/09/21，2025/10/22，2026/1/1，2026/1/15，2026/5/5</t>
         </is>
       </c>
       <c r="F267" t="inlineStr"/>
@@ -11246,7 +11234,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -11275,7 +11263,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/9，2025/12/6，2025/12/24，2026/4/13</t>
+          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/9，2025/12/6，2025/12/24，2026/4/13，2026/5/4</t>
         </is>
       </c>
       <c r="F268" t="inlineStr"/>
@@ -11286,7 +11274,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -14731,7 +14719,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/01，2025/05/26，2025/07/03，2025/07/27，2025/09/18，2025/10/17，2025/11/21，2026/1/12，2026/1/24，2026/2/19，2026/2/23，2026/3/24</t>
+          <t>2025/04/17，2025/05/01，2025/05/26，2025/07/03，2025/07/27，2025/09/18，2025/10/17，2025/11/21，2026/1/12，2026/1/24，2026/2/19，2026/2/23，2026/3/24，2026/5/4</t>
         </is>
       </c>
       <c r="F355" t="inlineStr"/>
@@ -14742,7 +14730,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
@@ -17931,7 +17919,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>2025/05/12，2025/05/22，2025/05/25，2025/07/20，2025/09/12，2026/1/15，2026/1/24，2026/1/30，2026/4/8</t>
+          <t>2025/05/12，2025/05/22，2025/05/25，2025/07/20，2025/09/12，2026/1/15，2026/1/24，2026/1/30，2026/4/8，2026/5/4</t>
         </is>
       </c>
       <c r="F437" t="inlineStr"/>
@@ -17942,7 +17930,7 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
@@ -18051,7 +18039,7 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>2025/05/15，2025/06/13，2025/06/23，2025/07/18，2025/08/02，2025/09/04，2025/09/15，2025/10/03，2025/10/28，2025/11/9，2025/11/14，2025/12/5，2026/2/2</t>
+          <t>2025/05/15，2025/06/13，2025/06/23，2025/07/18，2025/08/02，2025/09/04，2025/09/15，2025/10/03，2025/10/28，2025/11/9，2025/11/14，2025/12/5，2026/2/2，2026/5/4</t>
         </is>
       </c>
       <c r="F440" t="inlineStr"/>
@@ -18062,7 +18050,7 @@
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I440" t="inlineStr">
@@ -18131,7 +18119,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12，2026/4/5</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12，2026/4/5，2026/5/3</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -18142,7 +18130,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -18647,7 +18635,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/06/17，2025/06/23，2025/07/06，2025/07/15，2025/09/10，2025/10/18，2025/11/13</t>
+          <t>2025/05/22，2025/06/17，2025/06/23，2025/07/06，2025/07/15，2025/09/10，2025/10/18，2025/11/13，2026/5/4</t>
         </is>
       </c>
       <c r="F455" t="inlineStr"/>
@@ -18658,7 +18646,7 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
@@ -19347,7 +19335,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4</t>
         </is>
       </c>
       <c r="F473" t="inlineStr"/>
@@ -19358,7 +19346,7 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
@@ -21083,7 +21071,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>2025/06/13，2025/07/25</t>
+          <t>2025/06/13，2025/07/25，2026/5/5</t>
         </is>
       </c>
       <c r="F518" t="inlineStr"/>
@@ -21094,7 +21082,7 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I518" t="inlineStr"/>
@@ -21615,7 +21603,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1，2026/5/4</t>
         </is>
       </c>
       <c r="F532" t="inlineStr"/>
@@ -21626,7 +21614,7 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
@@ -25407,7 +25395,7 @@
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>2025/09/10，2025/09/22，2025/09/24，2025/10/23，2025/12/6，2026/1/24，2026/2/5，2026/2/23</t>
+          <t>2025/09/10，2025/09/22，2025/09/24，2025/10/23，2025/12/6，2026/1/24，2026/2/5，2026/2/23，2026/5/5</t>
         </is>
       </c>
       <c r="F630" t="inlineStr"/>
@@ -25418,7 +25406,7 @@
       </c>
       <c r="H630" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I630" t="inlineStr">
@@ -27259,7 +27247,7 @@
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/6，2026/1/15，2026/1/19，2026/3/7</t>
+          <t>2025/09/29，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/6，2026/1/15，2026/1/19，2026/3/7，2026/5/5</t>
         </is>
       </c>
       <c r="F679" t="inlineStr"/>
@@ -27270,7 +27258,7 @@
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I679" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to May 6, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,52 +429,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -1031,7 +1043,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/1/10，2026/1/24，2026/4/9</t>
+          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/1/10，2026/1/24，2026/4/9，2026/5/6</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1042,7 +1054,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1351,7 +1363,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25，2026/4/16</t>
+          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25，2026/4/16，2026/5/6</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1362,7 +1374,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1551,7 +1563,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1562,7 +1574,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2663,7 +2675,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7，2026/3/17，2026/3/21</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/7，2025/12/16，2025/12/28，2026/1/10，2026/1/15，2026/2/19，2026/3/7，2026/3/17，2026/3/21，2026/5/6</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2674,7 +2686,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3699,7 +3711,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/1/1，2026/2/14</t>
+          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/1/1，2026/2/14，2026/5/6</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -3710,7 +3722,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -6651,7 +6663,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8，2026/5/6</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6662,7 +6674,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9615,7 +9627,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/03，2025/05/26，2025/11/9</t>
+          <t>2025/03/28，2025/05/03，2025/05/26，2025/11/9，2026/5/6</t>
         </is>
       </c>
       <c r="F227" t="inlineStr"/>
@@ -9626,7 +9638,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -15591,7 +15603,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/2，2025/12/17</t>
+          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/2，2025/12/17，2026/5/6</t>
         </is>
       </c>
       <c r="F377" t="inlineStr"/>
@@ -15602,7 +15614,7 @@
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
@@ -29675,7 +29687,7 @@
       </c>
       <c r="E743" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1，2026/5/6</t>
         </is>
       </c>
       <c r="F743" t="inlineStr"/>
@@ -29686,7 +29698,7 @@
       </c>
       <c r="H743" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I743" t="inlineStr">
@@ -32155,7 +32167,7 @@
       </c>
       <c r="E806" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2，2026/5/6</t>
         </is>
       </c>
       <c r="F806" t="inlineStr"/>
@@ -32166,7 +32178,7 @@
       </c>
       <c r="H806" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I806" t="inlineStr">
@@ -32963,7 +32975,7 @@
       </c>
       <c r="E826" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20，2026/5/2</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20，2026/5/2，2026/5/6</t>
         </is>
       </c>
       <c r="F826" t="inlineStr"/>
@@ -32974,7 +32986,7 @@
       </c>
       <c r="H826" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to May 7, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -10795,7 +10795,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/9，2025/11/13，2025/12/4，2025/12/13，2026/3/4</t>
+          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/9，2025/11/13，2025/12/4，2025/12/13，2026/3/4，2026/5/7</t>
         </is>
       </c>
       <c r="F317" t="inlineStr"/>
@@ -13230,7 +13230,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -18567,7 +18567,7 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/07/13，2025/10/30，2025/10/31，2025/12/24，2026/1/9，2026/4/9</t>
+          <t>2025/05/19，2025/07/13，2025/10/30，2025/10/31，2025/12/24，2026/1/9，2026/4/9，2026/5/7</t>
         </is>
       </c>
       <c r="F453" t="inlineStr"/>
@@ -18578,7 +18578,7 @@
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I453" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to May 10, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,56 +413,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J859"/>
+  <dimension ref="A1:J860"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -1003,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18，2026/5/10</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1014,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1443,7 +1431,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/1/3，2026/3/25</t>
+          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/1/3，2026/3/25，2026/5/10</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1454,12 +1442,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BV1ssE8zWEaZ</t>
+          <t>BV1cV5s6rEKq，BV1ssE8zWEaZ</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1683,7 +1671,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,7 +1682,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2083,7 +2071,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21，2026/4/26</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21，2026/4/26，2026/5/10</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2094,7 +2082,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2635,7 +2623,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/05/04，2025/05/18，2025/06/09，2025/08/04，2025/08/16，2025/09/18，2025/10/17，2025/11/21，2025/11/28</t>
+          <t>2025/03/07，2025/03/28，2025/05/04，2025/05/18，2025/06/09，2025/08/04，2025/08/16，2025/09/18，2025/10/17，2025/11/21，2025/11/28，2026/5/10</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2646,7 +2634,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3171,7 +3159,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/4/9</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/4/9，2026/5/10</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3182,7 +3170,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3339,7 +3327,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21，2026/4/16</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21，2026/4/16，2026/5/10</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3350,7 +3338,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5619,7 +5607,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5630,7 +5618,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7743,7 +7731,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20，2026/5/10</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7754,7 +7742,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -7903,7 +7891,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22，2026/4/19</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22，2026/4/19，2026/5/10</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7914,7 +7902,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -7983,7 +7971,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/03，2025/04/19，2025/05/26，2025/09/18，2025/10/17，2026/1/1</t>
+          <t>2025/03/22，2025/04/03，2025/04/19，2025/05/26，2025/09/18，2025/10/17，2026/1/1，2026/5/10</t>
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -7994,12 +7982,12 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>BV1EMpQzEEJx，BV18ZiFBgEyW，BV1z4j1zJELw，BV1HvWhzPEe3</t>
+          <t>BV1pu5s65Esw，BV1EMpQzEEJx，BV18ZiFBgEyW，BV1z4j1zJELw，BV1HvWhzPEe3</t>
         </is>
       </c>
       <c r="J186" t="inlineStr"/>
@@ -9115,7 +9103,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25，2026/4/9</t>
+          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25，2026/4/9，2026/5/10</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -9126,12 +9114,12 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>BV142QFBkEXy，BV11GypBUErS，BV1KLVSzYEbC，BV1PFZ3YdENc</t>
+          <t>BV17e5H68EVb，BV142QFBkEXy，BV11GypBUErS，BV1KLVSzYEbC，BV1PFZ3YdENc</t>
         </is>
       </c>
       <c r="J214" t="inlineStr"/>
@@ -9471,7 +9459,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/9，2026/1/9，2026/2/19</t>
+          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/9，2026/1/9，2026/2/19，2026/5/10</t>
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
@@ -9482,12 +9470,12 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>BV14HKhzcET9</t>
+          <t>BV1cV5s6rEVv，BV14HKhzcET9</t>
         </is>
       </c>
       <c r="J223" t="inlineStr"/>
@@ -10795,7 +10783,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7，2026/5/8</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10806,12 +10794,12 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>BV1ocznBSE1q</t>
+          <t>BV1nTR2BiEyK，BV1ocznBSE1q</t>
         </is>
       </c>
       <c r="J256" t="inlineStr"/>
@@ -10875,7 +10863,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/05/10，2025/09/04，2025/09/10，2025/09/28，2025/11/26，2026/1/19</t>
+          <t>2025/04/01，2025/05/10，2025/09/04，2025/09/10，2025/09/28，2025/11/26，2026/1/19，2026/5/10</t>
         </is>
       </c>
       <c r="F258" t="inlineStr"/>
@@ -10886,12 +10874,12 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>BV1iyaUzbE51</t>
+          <t>BV1Jh5H6aEGT，BV1iyaUzbE51</t>
         </is>
       </c>
       <c r="J258" t="inlineStr"/>
@@ -10955,7 +10943,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/1/2，2026/1/5，2026/2/2，2026/2/9，2026/2/19，2026/3/25</t>
+          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/1/2，2026/1/5，2026/2/2，2026/2/9，2026/2/19，2026/3/25，2026/5/10</t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
@@ -10966,12 +10954,12 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>BV1QbqABDEAJ</t>
+          <t>BV17e5H68E9v，BV1QbqABDEAJ</t>
         </is>
       </c>
       <c r="J260" t="inlineStr"/>
@@ -14363,7 +14351,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/1/1，2026/1/9，2026/2/20，2026/4/18</t>
+          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/1/1，2026/1/9，2026/2/20，2026/4/18，2026/5/10</t>
         </is>
       </c>
       <c r="F346" t="inlineStr"/>
@@ -14374,12 +14362,12 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>BV1narMBZEG9，BV1z6fGBSE1m</t>
+          <t>BV1Eh5H6aEdz，BV1narMBZEG9，BV1z6fGBSE1m</t>
         </is>
       </c>
       <c r="J346" t="inlineStr"/>
@@ -18367,7 +18355,7 @@
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/1/2，2026/3/17，2026/4/29</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/1/2，2026/3/17，2026/4/29，2026/5/10</t>
         </is>
       </c>
       <c r="F448" t="inlineStr"/>
@@ -18378,12 +18366,12 @@
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I448" t="inlineStr">
         <is>
-          <t>BV1vgxozAEPC</t>
+          <t>BV1PP5s6mE97，BV1vgxozAEPC</t>
         </is>
       </c>
       <c r="J448" t="inlineStr"/>
@@ -18687,7 +18675,7 @@
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/12，2025/09/02，2025/12/5，2026/4/9</t>
+          <t>2025/05/22，2025/09/12，2025/09/02，2025/12/5，2026/4/9，2026/5/10</t>
         </is>
       </c>
       <c r="F456" t="inlineStr"/>
@@ -18698,12 +18686,12 @@
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I456" t="inlineStr">
         <is>
-          <t>BV1bgAMzbEEW</t>
+          <t>BV1NK5s6jEN9，BV1bgAMzbEEW</t>
         </is>
       </c>
       <c r="J456" t="inlineStr"/>
@@ -18851,7 +18839,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/1/5，2026/2/2，2026/3/17</t>
+          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/1/5，2026/2/2，2026/3/17，2026/5/10</t>
         </is>
       </c>
       <c r="F460" t="inlineStr"/>
@@ -18862,12 +18850,12 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t>BV1RDMVzNEXV</t>
+          <t>BV1sK5s6jE8Y，BV1RDMVzNEXV</t>
         </is>
       </c>
       <c r="J460" t="inlineStr"/>
@@ -21155,7 +21143,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22，2026/5/10</t>
         </is>
       </c>
       <c r="F520" t="inlineStr"/>
@@ -21166,7 +21154,7 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I520" t="inlineStr">
@@ -22203,7 +22191,7 @@
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13，2026/4/12</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13，2026/4/12，2026/5/10</t>
         </is>
       </c>
       <c r="F547" t="inlineStr"/>
@@ -22214,12 +22202,12 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
         <is>
-          <t>BV1iLJdzEEWk</t>
+          <t>BV1fL5s6uEZx，BV1iLJdzEEWk</t>
         </is>
       </c>
       <c r="J547" t="inlineStr">
@@ -22975,7 +22963,7 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9，2026/3/28</t>
+          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9，2026/3/28，2026/5/10</t>
         </is>
       </c>
       <c r="F567" t="inlineStr"/>
@@ -22986,7 +22974,7 @@
       </c>
       <c r="H567" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I567" t="inlineStr">
@@ -28715,7 +28703,7 @@
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>2025/10/28，2025/11/1，2025/11/12，2025/12/19，2026/2/8，2026/2/10</t>
+          <t>2025/10/28，2025/11/1，2025/11/12，2025/12/19，2026/2/8，2026/2/10，2026/5/10</t>
         </is>
       </c>
       <c r="F717" t="inlineStr"/>
@@ -28726,12 +28714,12 @@
       </c>
       <c r="H717" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I717" t="inlineStr">
         <is>
-          <t>BV1bscPz1EEj</t>
+          <t>BV1bscPz1EEj，BV16h5H6aEFe</t>
         </is>
       </c>
       <c r="J717" t="inlineStr"/>
@@ -30483,7 +30471,7 @@
       </c>
       <c r="E764" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10</t>
         </is>
       </c>
       <c r="F764" t="inlineStr"/>
@@ -30494,7 +30482,7 @@
       </c>
       <c r="H764" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I764" t="inlineStr">
@@ -31067,7 +31055,7 @@
       </c>
       <c r="E779" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18，2026/5/10</t>
         </is>
       </c>
       <c r="F779" t="inlineStr"/>
@@ -31078,7 +31066,7 @@
       </c>
       <c r="H779" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I779" t="inlineStr">
@@ -33107,7 +33095,7 @@
       </c>
       <c r="E829" t="inlineStr">
         <is>
-          <t>2026/3/28，2026/4/14</t>
+          <t>2026/3/28，2026/4/14，2026/5/10</t>
         </is>
       </c>
       <c r="F829" t="inlineStr"/>
@@ -33118,7 +33106,7 @@
       </c>
       <c r="H829" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I829" t="inlineStr">
@@ -34351,6 +34339,46 @@
           <t>动漫</t>
         </is>
       </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>859</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>咖喱咖喱</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr"/>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>牛奶咖啡</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>2026/5/10</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr"/>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>BV1WK5s6jEUw</t>
+        </is>
+      </c>
+      <c r="J860" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to May 16, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J860"/>
+  <dimension ref="A1:J861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -703,7 +703,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1，2026/4/20</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1，2026/4/20，2026/5/15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -714,12 +714,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BV1K5d6BhEPj，BV1df7RzGEDY</t>
+          <t>BV1dn5i6vEDX，BV1K5d6BhEPj，BV1df7RzGEDY</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15，2026/5/1</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15，2026/5/1，2026/5/16</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1122,12 +1122,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BV13mfTYcEWn</t>
+          <t>BV13mfTYcEWn，BV1zsL56jEgn</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6，2026/5/16</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1562,12 +1562,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BV1aWPiz7EvJ，BV1W4jbzLEbu</t>
+          <t>BV1aWPiz7EvJ，BV1W4jbzLEbu，BV1BsL56jEft</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2962,12 +2962,12 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>BV1wCoeB3EVt，BV1C9Q3BiE8m，BV1BFXUBwEDj，BV191NVzoEZ7，BV1TzrrBAEpz，BV1L5fUB5Ebn，BV1g9M3zsE7c</t>
+          <t>BV16L5B62E2x，BV1wCoeB3EVt，BV1C9Q3BiE8m，BV1BFXUBwEDj，BV191NVzoEZ7，BV1TzrrBAEpz，BV1L5fUB5Ebn，BV1g9M3zsE7c</t>
         </is>
       </c>
       <c r="J62" t="inlineStr"/>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29，2026/5/15</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3922,12 +3922,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>BV1VC9jBiEcL，BV133Vdz8Eyi</t>
+          <t>BV1sm5B6REWc，BV1VC9jBiEcL，BV133Vdz8Eyi</t>
         </is>
       </c>
       <c r="J85" t="inlineStr"/>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/13，2025/04/19，2025/05/06，2025/06/03，2025/08/28，2025/09/17，2025/10/10，2025/11/17，2025/11/22，2025/12/24，2026/1/15，2026/1/29，2026/3/19</t>
+          <t>2025/03/13，2025/04/13，2025/04/19，2025/05/06，2025/06/03，2025/08/28，2025/09/17，2025/10/10，2025/11/17，2025/11/22，2025/12/24，2026/1/15，2026/1/29，2026/3/19，2026/5/15</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4326,12 +4326,12 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>BV1iRhUzZECK</t>
+          <t>BV1Q85i6bEDR，BV1iRhUzZECK</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -9179,7 +9179,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29，2026/5/15</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9190,12 +9190,12 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>BV1rEdLBDEFV，BV1yYMVz2E5E</t>
+          <t>BV1r55B67EtQ，BV1rEdLBDEFV，BV1yYMVz2E5E</t>
         </is>
       </c>
       <c r="J216" t="inlineStr"/>
@@ -9855,7 +9855,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7，2026/3/28，2026/4/19</t>
+          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/8，2025/12/12，2026/1/28，2026/3/7，2026/3/28，2026/4/19，2026/5/15</t>
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
@@ -9866,12 +9866,12 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>BV1JHdfBBEgk，BV1tzXLB4EDj，BV1r3NAzgErm，BV1crarzEEsn</t>
+          <t>BV1e85B6TEwr，BV1JHdfBBEgk，BV1tzXLB4EDj，BV1r3NAzgErm，BV1crarzEEsn</t>
         </is>
       </c>
       <c r="J233" t="inlineStr"/>
@@ -16795,7 +16795,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/11/18，2026/2/14，2026/4/9</t>
+          <t>2025/04/28，2025/11/18，2026/2/14，2026/4/9，2026/5/16</t>
         </is>
       </c>
       <c r="F408" t="inlineStr"/>
@@ -16806,12 +16806,12 @@
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
         <is>
-          <t>BV125yVBxER9</t>
+          <t>BV125yVBxER9，BV1zsL56jEVx</t>
         </is>
       </c>
       <c r="J408" t="inlineStr"/>
@@ -20303,7 +20303,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5，2026/3/17，2026/4/24</t>
+          <t>2025/06/01，2026/1/23，2026/2/2，2026/2/23，2026/3/5，2026/3/17，2026/4/24，2026/5/16</t>
         </is>
       </c>
       <c r="F498" t="inlineStr"/>
@@ -20314,12 +20314,12 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
         <is>
-          <t>BV1w2fzBhEHL，BV1VuzuB1EQf</t>
+          <t>BV1w2fzBhEHL，BV1VuzuB1EQf，BV1fsL56jEsC</t>
         </is>
       </c>
       <c r="J498" t="inlineStr"/>
@@ -21129,7 +21129,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I519" t="inlineStr"/>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>BV1SxMBztEM2</t>
+        </is>
+      </c>
       <c r="J519" t="inlineStr"/>
     </row>
     <row r="520">
@@ -21151,7 +21155,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22，2026/5/10</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22，2026/5/10，2026/5/15</t>
         </is>
       </c>
       <c r="F520" t="inlineStr"/>
@@ -21162,12 +21166,12 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I520" t="inlineStr">
         <is>
-          <t>BV1g9ojB6Esh，BV1dgmMBeEF4</t>
+          <t>BV1Yh5B6iEN6，BV1g9ojB6Esh，BV1dgmMBeEF4</t>
         </is>
       </c>
       <c r="J520" t="inlineStr"/>
@@ -21815,7 +21819,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24，2026/5/15</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -21826,12 +21830,12 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
         <is>
-          <t>BV1zodeBqEhq，BV1MosGzFEMe</t>
+          <t>BV1CX5B6HE3A，BV1zodeBqEhq，BV1MosGzFEMe</t>
         </is>
       </c>
       <c r="J537" t="inlineStr"/>
@@ -24743,7 +24747,7 @@
       </c>
       <c r="E613" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1，2026/4/8</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1，2026/4/8，2026/5/15</t>
         </is>
       </c>
       <c r="F613" t="inlineStr"/>
@@ -24754,12 +24758,12 @@
       </c>
       <c r="H613" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I613" t="inlineStr">
         <is>
-          <t>BV1SNDEBbEXQ，BV1u4bwzyEez</t>
+          <t>BV1kG5B6UEGv，BV1SNDEBbEXQ，BV1u4bwzyEez</t>
         </is>
       </c>
       <c r="J613" t="inlineStr"/>
@@ -30047,7 +30051,7 @@
       </c>
       <c r="I752" t="inlineStr">
         <is>
-          <t>BV1SLRLBfECg，BV1cWmnB5Etm</t>
+          <t>BV1emR7B1Edj，BV1cWmnB5Etm</t>
         </is>
       </c>
       <c r="J752" t="inlineStr"/>
@@ -30559,7 +30563,7 @@
       </c>
       <c r="E766" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11，2026/4/20</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11，2026/4/20，2026/5/15</t>
         </is>
       </c>
       <c r="F766" t="inlineStr"/>
@@ -30570,12 +30574,12 @@
       </c>
       <c r="H766" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I766" t="inlineStr">
         <is>
-          <t>BV1UodkBzEgD，BV1pfzcBgERV，BV1aff2BvEZF</t>
+          <t>BV1C35B6JEMN，BV1UodkBzEgD，BV1pfzcBgERV，BV1aff2BvEZF</t>
         </is>
       </c>
       <c r="J766" t="inlineStr">
@@ -33827,7 +33831,7 @@
       </c>
       <c r="E847" t="inlineStr">
         <is>
-          <t>2026/4/16，2026/4/29</t>
+          <t>2026/4/16，2026/4/29，2026/5/15</t>
         </is>
       </c>
       <c r="F847" t="inlineStr"/>
@@ -33838,12 +33842,12 @@
       </c>
       <c r="H847" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I847" t="inlineStr">
         <is>
-          <t>BV1XsdaBDEAD</t>
+          <t>BV1qJ5i6KEKZ，BV1XsdaBDEAD</t>
         </is>
       </c>
       <c r="J847" t="inlineStr"/>
@@ -34387,6 +34391,50 @@
         </is>
       </c>
       <c r="J860" t="inlineStr"/>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>860</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t xml:space="preserve">빌런 </t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>反派/Villain</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Stella Jang</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>2026/5/15</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr"/>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>韩语</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>BV1k35B6JED4</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to May 19, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,52 +429,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -6771,7 +6783,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/22，2025/05/29，2025/06/03，2025/08/28，2025/09/11，2025/10/18，2025/10/30，2025/11/28，2025/12/28，2026/3/15</t>
+          <t>2025/03/20，2025/05/22，2025/05/29，2025/06/03，2025/08/28，2025/09/11，2025/10/18，2025/10/30，2025/11/28，2025/12/28，2026/3/15，2026/5/19</t>
         </is>
       </c>
       <c r="F156" t="inlineStr"/>
@@ -6782,12 +6794,12 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>BV1MXvYBfENe</t>
+          <t>BV1i8L26AEz7，BV1MXvYBfENe</t>
         </is>
       </c>
       <c r="J156" t="inlineStr"/>
@@ -9179,7 +9191,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29，2026/5/15</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29，2026/5/15，2026/5/19</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9190,12 +9202,12 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>BV1r55B67EtQ，BV1rEdLBDEFV，BV1yYMVz2E5E</t>
+          <t>BV1r55B67EtQ，BV1i8L26AEZG，BV1rEdLBDEFV，BV1yYMVz2E5E</t>
         </is>
       </c>
       <c r="J216" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: Update song list to May 21, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/17，2025/06/02，2025/07/07，2025/07/14，2025/08/07，2025/09/04，2025/09/29，2025/11/7，2025/12/5</t>
+          <t>2025/03/03，2025/04/17，2025/06/02，2025/07/07，2025/07/14，2025/08/07，2025/09/04，2025/09/29，2025/11/7，2025/12/5，2026/5/21</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -890,12 +890,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>BV11D7SzVE7W</t>
+          <t>BV1rSLh6PER7，BV11D7SzVE7W</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/1/10，2026/1/24，2026/4/9</t>
+          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/1/10，2026/1/24，2026/4/9，2026/5/21</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25，2026/4/16，2026/5/6</t>
+          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/9，2025/11/12，2025/11/27，2025/12/4，2025/12/28，2026/1/22，2026/2/2，2026/2/23，2026/3/25，2026/4/16，2026/5/6，2026/5/21</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6，2026/5/16</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6，2026/5/16，2026/5/20</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BV1aWPiz7EvJ，BV1W4jbzLEbu，BV1BsL56jEft</t>
+          <t>BV1cMLb6sEzs，BV1aWPiz7EvJ，BV1W4jbzLEbu，BV1BsL56jEft</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/7，2025/12/24，2026/1/1，2026/1/16，2026/3/14，2026/5/1</t>
+          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/7，2025/12/24，2026/1/1，2026/1/16，2026/3/14，2026/5/1，2026/5/20</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1734,12 +1734,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BV1LCQrYjECx</t>
+          <t>BV1iaLU6zEFq，BV1LCQrYjECx</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/21，2025/04/05，2025/04/14，2025/04/24，2025/05/20，2025/06/05，2025/06/17，2025/06/23，2025/06/26，2025/08/12，2025/08/21，2025/09/14，2025/09/24，2025/10/16，2025/10/24，2025/12/17，2026/2/14，2026/3/8，2026/4/25</t>
+          <t>2025/03/04，2025/03/21，2025/04/05，2025/04/14，2025/04/24，2025/05/20，2025/06/05，2025/06/17，2025/06/23，2025/06/26，2025/08/12，2025/08/21，2025/09/14，2025/09/24，2025/10/16，2025/10/24，2025/12/17，2026/2/14，2026/3/8，2026/4/25，2026/5/21</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/1/15，2026/2/14，2026/3/22</t>
+          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/1/15，2026/2/14，2026/3/22，2026/5/20</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2362,12 +2362,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>BV1McbQz1EP2</t>
+          <t>BV1FuLb69EvV，BV1McbQz1EP2</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/3，2025/12/12，2026/2/4，2026/4/18</t>
+          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/3，2025/12/12，2026/2/4，2026/4/18，2026/5/20</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2446,12 +2446,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>BV1wtmoB7ERp</t>
+          <t>BV1cMLb6sEhP，BV1wtmoB7ERp</t>
         </is>
       </c>
       <c r="J49" t="inlineStr"/>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/04，2025/04/11，2025/05/20，2025/06/16，2025/06/24，2025/08/29，2025/09/12，2025/10/12，2026/1/9</t>
+          <t>2025/03/09，2025/04/04，2025/04/11，2025/05/20，2025/06/16，2025/06/24，2025/08/29，2025/09/12，2025/10/12，2026/1/9，2026/5/20</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -3262,12 +3262,12 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>BV1SrNtzdEsW，BV1hPJazzEeo</t>
+          <t>BV1FuLb69EiM，BV1SrNtzdEsW，BV1hPJazzEeo</t>
         </is>
       </c>
       <c r="J69" t="inlineStr"/>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/19，2025/08/16，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/1/14，2026/2/4</t>
+          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/19，2025/08/16，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/1/14，2026/2/4，2026/5/20</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -3978,12 +3978,12 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>BV1EpmjBbEte</t>
+          <t>BV1wMLb6sEw9，BV1EpmjBbEte</t>
         </is>
       </c>
       <c r="J86" t="inlineStr"/>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/30，2025/04/17，2025/04/21，2025/05/05，2025/05/13，2025/05/20，2025/06/06，2025/06/20，2025/06/27，2025/07/05，2025/07/31，2025/08/24，2025/08/29，2025/09/20，2025/09/30，2025/10/22，2025/11/26，2026/1/15，2026/2/14，2026/4/8</t>
+          <t>2025/03/13，2025/03/30，2025/04/17，2025/04/21，2025/05/05，2025/05/13，2025/05/20，2025/06/06，2025/06/20，2025/06/27，2025/07/05，2025/07/31，2025/08/24，2025/08/29，2025/09/20，2025/09/30，2025/10/22，2025/11/26，2026/1/15，2026/2/14，2026/4/8，2026/5/20</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/2/10，2026/2/24，2026/3/18</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/2/10，2026/2/24，2026/3/18，2026/5/20</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4418,12 +4418,12 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>BV1zdrTBpETM</t>
+          <t>BV1FuLb69EZ9，BV1zdrTBpETM</t>
         </is>
       </c>
       <c r="J97" t="inlineStr"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/9，2025/11/22，2026/3/9，2026/4/14</t>
+          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/9，2025/11/22，2026/3/9，2026/4/14，2026/5/20</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/12，2025/05/23，2025/06/26，2025/07/08，2025/07/31，2025/08/22，2025/09/02，2025/09/15，2025/10/10，2025/11/3，2026/2/2，2026/4/1</t>
+          <t>2025/03/14，2025/04/02，2025/05/12，2025/05/23，2025/06/26，2025/07/08，2025/07/31，2025/08/22，2025/09/02，2025/09/15，2025/10/10，2025/11/3，2026/2/2，2026/4/1，2026/5/20</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -4658,12 +4658,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>BV1KaauzNE4s</t>
+          <t>BV1MeLb6qE99，BV1KaauzNE4s</t>
         </is>
       </c>
       <c r="J103" t="inlineStr"/>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8，2026/5/6</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8，2026/5/6，2026/5/21</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/19，2025/06/08，2025/06/12，2025/07/13，2025/08/28，2025/09/26，2025/10/25，2025/11/19，2025/11/27，2026/1/22，2026/1/25，2026/2/19</t>
+          <t>2025/03/20，2025/04/04，2025/05/19，2025/06/08，2025/06/12，2025/07/13，2025/08/28，2025/09/26，2025/10/25，2025/11/19，2025/11/27，2026/1/22，2026/1/25，2026/2/19，2026/5/20</t>
         </is>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -6714,12 +6714,12 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>BV1WpzNBnEBD</t>
+          <t>BV1cDLb6dEFn，BV1WpzNBnEBD</t>
         </is>
       </c>
       <c r="J154" t="inlineStr"/>
@@ -7943,7 +7943,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/06/24</t>
+          <t>2025/03/22，2025/06/24，2026/5/20</t>
         </is>
       </c>
       <c r="F185" t="inlineStr"/>
@@ -7954,12 +7954,12 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>BV11GKVzVEfL</t>
+          <t>BV1BdLb6HELG，BV11GKVzVEfL</t>
         </is>
       </c>
       <c r="J185" t="inlineStr"/>
@@ -8303,7 +8303,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/7，2026/1/17，2026/2/14，2026/4/9</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/7，2026/1/17，2026/2/14，2026/4/9，2026/5/20</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8314,12 +8314,12 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>BV1Gn7XzhEHE</t>
+          <t>BV1RnLb6LEoE，BV1Gn7XzhEHE</t>
         </is>
       </c>
       <c r="J194" t="inlineStr"/>
@@ -8743,7 +8743,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/18，2025/04/24，2025/06/23，2025/09/29，2025/12/17，2026/4/8</t>
+          <t>2025/03/25，2025/04/18，2025/04/24，2025/06/23，2025/09/29，2025/12/17，2026/4/8，2026/5/21</t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
@@ -8754,12 +8754,12 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>BV1wiY1zwEKF，BV18j5EzsEtC</t>
+          <t>BV1A2Lh6TE1D，BV1wiY1zwEKF，BV18j5EzsEtC</t>
         </is>
       </c>
       <c r="J205" t="inlineStr"/>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8，2026/4/24</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8，2026/4/24，2026/5/21</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9962,7 +9962,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -10635,7 +10635,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/2/12，2026/4/16</t>
+          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/2/12，2026/4/16，2026/5/20</t>
         </is>
       </c>
       <c r="F252" t="inlineStr"/>
@@ -10646,7 +10646,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -10915,7 +10915,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17，2026/5/5</t>
+          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17，2026/5/5，2026/5/21</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
@@ -10926,12 +10926,12 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>BV1mRvYBtECy</t>
+          <t>BV1pmLh6iEsu，BV1mRvYBtECy</t>
         </is>
       </c>
       <c r="J259" t="inlineStr"/>
@@ -10955,7 +10955,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/1/2，2026/1/5，2026/2/2，2026/2/9，2026/2/19，2026/3/25，2026/5/10</t>
+          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/1/2，2026/1/5，2026/2/2，2026/2/9，2026/2/19，2026/3/25，2026/5/10，2026/5/21</t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
@@ -10966,12 +10966,12 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>BV17e5H68E9v，BV1QbqABDEAJ</t>
+          <t>BV1HMLb6sEgU，BV17e5H68E9v，BV1QbqABDEAJ</t>
         </is>
       </c>
       <c r="J260" t="inlineStr"/>
@@ -11395,7 +11395,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/09，2025/05/20，2025/06/26，2025/07/15，2025/12/5</t>
+          <t>2025/04/02，2025/05/09，2025/05/20，2025/06/26，2025/07/15，2025/12/5，2026/5/20</t>
         </is>
       </c>
       <c r="F271" t="inlineStr"/>
@@ -11406,12 +11406,12 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>BV1LYKfz4EUD，BV1Bp29BFEMn</t>
+          <t>BV17LLb6SEJ9，BV1LYKfz4EUD，BV1Bp29BFEMn</t>
         </is>
       </c>
       <c r="J271" t="inlineStr"/>
@@ -12307,7 +12307,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/2/14，2026/3/5，2026/4/2</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/2/14，2026/3/5，2026/4/2，2026/5/20</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -12318,7 +12318,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/1/3，2026/1/22，2026/2/14</t>
+          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/1/3，2026/1/22，2026/2/14，2026/5/20</t>
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
@@ -12838,12 +12838,12 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>BV1RukTBmEWQ</t>
+          <t>BV1RukTBmEWQ，BV1cuLb69ETt</t>
         </is>
       </c>
       <c r="J307" t="inlineStr"/>
@@ -13451,7 +13451,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24，2026/4/19</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24，2026/4/19，2026/5/21</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -13462,7 +13462,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -13951,7 +13951,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1，2026/5/21</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13962,7 +13962,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19，2026/5/1</t>
+          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19，2026/5/1，2026/5/21</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -14054,12 +14054,12 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>BV1YBKmzWEb2</t>
+          <t>BV1uSLt6qEwz，BV1YBKmzWEb2</t>
         </is>
       </c>
       <c r="J338" t="inlineStr">
@@ -14811,7 +14811,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/2/18</t>
+          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/2/18，2026/5/20</t>
         </is>
       </c>
       <c r="F357" t="inlineStr"/>
@@ -14822,12 +14822,12 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>BV1c5hRznES3</t>
+          <t>BV1LELb6mERb，BV1c5hRznES3</t>
         </is>
       </c>
       <c r="J357" t="inlineStr"/>
@@ -15403,7 +15403,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/9，2025/11/26，2025/12/5，2025/12/6，2026/1/1，2026/1/29，2026/3/1，2026/4/9</t>
+          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/9，2025/11/26，2025/12/5，2025/12/6，2026/1/1，2026/1/29，2026/3/1，2026/4/9，2026/5/20</t>
         </is>
       </c>
       <c r="F372" t="inlineStr"/>
@@ -15414,12 +15414,12 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>BV1NDerzFEoM</t>
+          <t>BV1i7Lb6jEhg，BV1NDerzFEoM</t>
         </is>
       </c>
       <c r="J372" t="inlineStr"/>
@@ -17691,7 +17691,7 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/20，2025/06/24，2025/07/07，2025/09/30</t>
+          <t>2025/05/10，2025/06/20，2025/06/24，2025/07/07，2025/09/30，2026/5/20</t>
         </is>
       </c>
       <c r="F431" t="inlineStr"/>
@@ -17702,12 +17702,12 @@
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>BV12gVfzoEr1，BV1vJM9zmE58</t>
+          <t>BV1B5Lb6EEP5，BV12gVfzoEr1，BV1vJM9zmE58</t>
         </is>
       </c>
       <c r="J431" t="inlineStr"/>
@@ -22351,7 +22351,7 @@
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/07/21，2025/08/18，2025/08/21，2025/09/17，2025/09/22，2025/10/16，2025/11/26，2026/1/19</t>
+          <t>2025/06/27，2025/07/21，2025/08/18，2025/08/21，2025/09/17，2025/09/22，2025/10/16，2025/11/26，2026/1/19，2026/5/20</t>
         </is>
       </c>
       <c r="F550" t="inlineStr"/>
@@ -22362,12 +22362,12 @@
       </c>
       <c r="H550" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I550" t="inlineStr">
         <is>
-          <t>BV1YzYxztEuV</t>
+          <t>BV1i7Lb6jETN，BV1YzYxztEuV</t>
         </is>
       </c>
       <c r="J550" t="inlineStr"/>
@@ -24491,7 +24491,7 @@
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8，2026/4/19</t>
+          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8，2026/4/19，2026/5/20</t>
         </is>
       </c>
       <c r="F606" t="inlineStr"/>
@@ -24502,7 +24502,7 @@
       </c>
       <c r="H606" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I606" t="inlineStr">
@@ -26385,7 +26385,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I655" t="inlineStr"/>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>BV1CyWNzcEb6</t>
+        </is>
+      </c>
       <c r="J655" t="inlineStr"/>
     </row>
     <row r="656">
@@ -26461,7 +26465,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I657" t="inlineStr"/>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>BV1hAWVzwEnG</t>
+        </is>
+      </c>
       <c r="J657" t="inlineStr"/>
     </row>
     <row r="658">
@@ -26533,7 +26541,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I659" t="inlineStr"/>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>BV1gKWVzFEN1</t>
+        </is>
+      </c>
       <c r="J659" t="inlineStr"/>
     </row>
     <row r="660">
@@ -26555,7 +26567,7 @@
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/1，2025/12/6，2025/12/12，2026/1/19，2026/4/8</t>
+          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/1，2025/12/6，2025/12/12，2026/1/19，2026/4/8，2026/5/20</t>
         </is>
       </c>
       <c r="F660" t="inlineStr"/>
@@ -26566,12 +26578,12 @@
       </c>
       <c r="H660" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I660" t="inlineStr">
         <is>
-          <t>BV19wxTzsEnU</t>
+          <t>BV1dnLb6LEcT，BV19wxTzsEnU</t>
         </is>
       </c>
       <c r="J660" t="inlineStr"/>
@@ -26595,7 +26607,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1，2026/5/20</t>
         </is>
       </c>
       <c r="F661" t="inlineStr"/>
@@ -26606,7 +26618,7 @@
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
@@ -31563,7 +31575,7 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20，2026/5/2</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20，2026/5/2，2026/5/21</t>
         </is>
       </c>
       <c r="F791" t="inlineStr"/>
@@ -31574,7 +31586,7 @@
       </c>
       <c r="H791" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I791" t="inlineStr">
@@ -32179,7 +32191,7 @@
       </c>
       <c r="E806" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2，2026/5/6</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2，2026/5/6，2026/5/21</t>
         </is>
       </c>
       <c r="F806" t="inlineStr"/>
@@ -32190,7 +32202,7 @@
       </c>
       <c r="H806" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I806" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to May 23, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -759,7 +759,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17，2026/4/19</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17，2026/4/19，2026/5/23</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -770,7 +770,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15，2026/5/1，2026/5/16</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/1/9，2026/2/12，2026/3/9，2026/3/15，2026/5/1，2026/5/16，2026/5/23</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1134,12 +1134,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BV1vhcGzCEKZ，BV1zsL56jEgn</t>
+          <t>BV1qAGL6zEY5，BV1vhcGzCEKZ，BV1zsL56jEgn</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/3/9，2026/4/18</t>
+          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/3/9，2026/4/18，2026/5/23</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1254,12 +1254,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BV1Ur57zEEs2</t>
+          <t>BV1h7GL6FEjR，BV1Ur57zEEs2</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14，2026/5/6</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14，2026/5/6，2026/5/23</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10，2026/5/23</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,12 +1694,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BV1hYobBkEum，BV1wUojYeEon</t>
+          <t>BV18EGL6bEnV，BV1hYobBkEum，BV1wUojYeEon</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13，2026/4/10</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13，2026/4/10，2026/5/23</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2766,12 +2766,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>BV17uQABvEkz，BV1N8UvB8ExW</t>
+          <t>BV1a7GL6FEv4，BV17uQABvEkz，BV1N8UvB8ExW</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19，2026/5/1</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19，2026/5/1，2026/5/23</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14，2026/5/4</t>
+          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14，2026/5/4，2026/5/23</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2894,12 +2894,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>BV19DUYBTErV</t>
+          <t>BV1Q7GL6FEm3，BV19DUYBTErV</t>
         </is>
       </c>
       <c r="J60" t="inlineStr"/>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/8，2026/1/12，2026/1/30，2026/2/7，2026/4/18</t>
+          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/8，2026/1/12，2026/1/30，2026/2/7，2026/4/18，2026/5/23</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3102,12 +3102,12 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>BV1MQKPzdEA5，BV1fJGqz7E78，BV1icEuzEE86，BV1UhzsB1EwS</t>
+          <t>BV1d5G66ME8p，BV1MQKPzdEA5，BV1fJGqz7E78，BV1icEuzEE86，BV1UhzsB1EwS</t>
         </is>
       </c>
       <c r="J65" t="inlineStr"/>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/1/1，2026/2/14，2026/5/6</t>
+          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/1/1，2026/2/14，2026/5/6，2026/5/23</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -3722,12 +3722,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>BV1A6rxBjE4F</t>
+          <t>BV1h7GL6FEFX，BV1A6rxBjE4F</t>
         </is>
       </c>
       <c r="J80" t="inlineStr"/>
@@ -5139,7 +5139,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/1/19，2026/4/18，2026/5/1</t>
+          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/1/19，2026/4/18，2026/5/1，2026/5/23</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9，2026/4/14，2026/4/24</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/3，2025/11/24，2026/4/9，2026/4/14，2026/4/24，2026/5/23</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5270,12 +5270,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>BV1jPoEBQEPw，BV1DrQ3ByECZ，BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
+          <t>BV1C6G66nEga，BV1jPoEBQEPw，BV1DrQ3ByECZ，BV1CVQFBNEYU，BV1vUUYBzEnY，BV1wDY9z9EYs，BV1DCj3z6Ec7，BV1fLQ6Y1ETv</t>
         </is>
       </c>
       <c r="J118" t="inlineStr"/>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10，2026/5/23</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5630,7 +5630,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11，2026/4/14，2026/4/29</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/7，2025/12/23，2026/1/5，2026/1/21，2026/1/29，2026/2/9，2026/2/20，2026/2/23，2026/3/4，2026/3/6，2026/3/7，2026/4/11，2026/4/14，2026/4/29，2026/5/23</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5750,12 +5750,12 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>BV1pXD2BcECv，BV1A1fzBwEjQ，BV19KmPBDERd，BV1B1fGBjEtL</t>
+          <t>BV1iKGL6qEH3，BV1pXD2BcECv，BV1A1fzBwEjQ，BV19KmPBDERd，BV1B1fGBjEtL</t>
         </is>
       </c>
       <c r="J130" t="inlineStr"/>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25，2026/4/24</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25，2026/4/24，2026/5/23</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/04/11，2025/05/19，2025/05/23，2025/06/12，2025/06/23，2025/07/20，2025/08/19，2025/09/21，2025/10/07，2025/10/20，2025/10/28，2025/11/9，2025/11/24，2025/12/16，2025/12/24，2025/12/26</t>
+          <t>2025/03/19，2025/03/28，2025/04/11，2025/05/19，2025/05/23，2025/06/12，2025/06/23，2025/07/20，2025/08/19，2025/09/21，2025/10/07，2025/10/20，2025/10/28，2025/11/9，2025/11/24，2025/12/16，2025/12/24，2025/12/26，2026/5/23</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -6390,7 +6390,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26，2026/5/5</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26，2026/5/5，2026/5/23</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7223,7 +7223,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/19，2025/06/13，2025/07/22，2025/07/23，2025/08/25，2025/09/12，2025/10/26，2025/12/17，2026/2/9，2026/3/4，2026/3/25，2026/3/29</t>
+          <t>2025/03/21，2025/05/19，2025/06/13，2025/07/22，2025/07/23，2025/08/25，2025/09/12，2025/10/26，2025/12/17，2026/2/9，2026/3/4，2026/3/25，2026/3/29，2026/5/23</t>
         </is>
       </c>
       <c r="F167" t="inlineStr"/>
@@ -7234,7 +7234,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/24，2025/06/05，2025/07/26，2025/09/21，2025/10/16，2025/10/30，2025/11/9，2026/1/9，2026/4/24</t>
+          <t>2025/03/21，2025/04/24，2025/06/05，2025/07/26，2025/09/21，2025/10/16，2025/10/30，2025/11/9，2026/1/9，2026/4/24，2026/5/23</t>
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24，2026/4/26，2026/5/4</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/6，2026/2/7，2026/3/24，2026/4/26，2026/5/4，2026/5/23</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7354,12 +7354,12 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>BV1FU1uBzEst</t>
+          <t>BV174Gz63E6w，BV1FU1uBzEst</t>
         </is>
       </c>
       <c r="J170" t="inlineStr"/>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15，2026/4/2，2026/5/1</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/3，2025/11/22，2026/1/22，2026/2/19，2026/3/15，2026/4/2，2026/5/1，2026/5/23</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7550,12 +7550,12 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>BV1wB9PBHEQp，BV1Rqw3zCEFo，BV1v84TzcEMv</t>
+          <t>BV1G7GL6cEBd，BV1wB9PBHEQp，BV1Rqw3zCEFo，BV1v84TzcEMv</t>
         </is>
       </c>
       <c r="J175" t="inlineStr"/>
@@ -8063,7 +8063,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25，2026/4/19</t>
+          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25，2026/4/19，2026/5/23</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -8074,12 +8074,12 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>BV1JwoFB3E6c，BV1Q6E2zjE2b</t>
+          <t>BV1j8Gz6uELh，BV1JwoFB3E6c，BV1Q6E2zjE2b</t>
         </is>
       </c>
       <c r="J188" t="inlineStr"/>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/18，2025/06/02，2026/2/19</t>
+          <t>2025/03/25，2025/04/18，2025/06/02，2026/2/19，2026/5/23</t>
         </is>
       </c>
       <c r="F203" t="inlineStr"/>
@@ -8674,12 +8674,12 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>BV1oK5EzwExE</t>
+          <t>BV18EGL6bEEd，BV1oK5EzwExE</t>
         </is>
       </c>
       <c r="J203" t="inlineStr"/>
@@ -10239,7 +10239,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/1/16，2026/3/25</t>
+          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/1/16，2026/3/25，2026/5/23</t>
         </is>
       </c>
       <c r="F242" t="inlineStr"/>
@@ -10250,12 +10250,12 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>BV1GPM8zrE7N，BV1VKUhB8EUR，BV1mpjQzjE5U</t>
+          <t>BV1a7GL6FE7h，BV1GPM8zrE7N，BV1VKUhB8EUR，BV1mpjQzjE5U</t>
         </is>
       </c>
       <c r="J242" t="inlineStr"/>
@@ -10359,7 +10359,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/1/9，2026/3/7，2026/4/19</t>
+          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/1/9，2026/3/7，2026/4/19，2026/5/23</t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
@@ -10370,7 +10370,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7，2026/5/8</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7，2026/5/8，2026/5/23</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10806,12 +10806,12 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>BV1nTR2BiEyK，BV1ocznBSE1q</t>
+          <t>BV1a7GL6FE1f，BV1nTR2BiEyK，BV1ocznBSE1q</t>
         </is>
       </c>
       <c r="J256" t="inlineStr"/>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25，2026/4/24</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25，2026/4/24，2026/5/23</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11690,7 +11690,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25，2026/4/8</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25，2026/4/8，2026/5/23</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12918,12 +12918,12 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>BV1aXvxB1EKh，BV1uNSgBeEKj，BV1YBVfzBEpm</t>
+          <t>BV1a7GL6FEYG，BV1aXvxB1EKh，BV1uNSgBeEKj，BV1YBVfzBEpm</t>
         </is>
       </c>
       <c r="J309" t="inlineStr"/>
@@ -13375,7 +13375,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/9，2025/12/8，2026/1/5，2026/2/14</t>
+          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/9，2025/12/8，2026/1/5，2026/2/14，2026/5/23</t>
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
@@ -13386,12 +13386,12 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>BV1YwdXYmEsm</t>
+          <t>BV18EGL6bEST，BV1YwdXYmEsm</t>
         </is>
       </c>
       <c r="J321" t="inlineStr"/>
@@ -14225,7 +14225,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I342" t="inlineStr"/>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>BV1SjyQBBEtG</t>
+        </is>
+      </c>
       <c r="J342" t="inlineStr"/>
     </row>
     <row r="343">
@@ -14341,7 +14345,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I345" t="inlineStr"/>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>BV1PFGczxEpG</t>
+        </is>
+      </c>
       <c r="J345" t="inlineStr"/>
     </row>
     <row r="346">
@@ -14403,7 +14411,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/1/16，2026/3/25，2026/4/24</t>
+          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/1/16，2026/3/25，2026/4/24，2026/5/23</t>
         </is>
       </c>
       <c r="F347" t="inlineStr"/>
@@ -14414,12 +14422,12 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>BV1b1NzzXEMp，BV1MRETzeETU</t>
+          <t>BV1a7GL6FE1G，BV1b1NzzXEMp，BV1MRETzeETU</t>
         </is>
       </c>
       <c r="J347" t="inlineStr"/>
@@ -16331,7 +16339,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/3，2025/12/30，2026/1/9，2026/4/1</t>
+          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/3，2025/12/30，2026/1/9，2026/4/1，2026/5/23</t>
         </is>
       </c>
       <c r="F396" t="inlineStr"/>
@@ -16342,12 +16350,12 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>BV1r9NZzFErx，BV1gLtdzZEHp</t>
+          <t>BV1ArG66DEsf，BV1r9NZzFErx，BV1gLtdzZEHp</t>
         </is>
       </c>
       <c r="J396" t="inlineStr"/>
@@ -17285,7 +17293,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I420" t="inlineStr"/>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>BV1gTuwzfEvi</t>
+        </is>
+      </c>
       <c r="J420" t="inlineStr"/>
     </row>
     <row r="421">
@@ -17321,7 +17333,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I421" t="inlineStr"/>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>BV1h2GRzXEUQ</t>
+        </is>
+      </c>
       <c r="J421" t="inlineStr"/>
     </row>
     <row r="422">
@@ -17357,7 +17373,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I422" t="inlineStr"/>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>BV1aCGRzREQd</t>
+        </is>
+      </c>
       <c r="J422" t="inlineStr"/>
     </row>
     <row r="423">
@@ -17499,7 +17519,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/4/20</t>
+          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/4/20，2026/5/23</t>
         </is>
       </c>
       <c r="F426" t="inlineStr"/>
@@ -17510,12 +17530,12 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t>BV1GJdUBFEgM，BV1oUSuB5EpY</t>
+          <t>BV1P6G66HETG，BV1GJdUBFEgM，BV1oUSuB5EpY</t>
         </is>
       </c>
       <c r="J426" t="inlineStr"/>
@@ -17931,7 +17951,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>2025/05/12，2025/05/22，2025/05/25，2025/07/20，2025/09/12，2026/1/15，2026/1/24，2026/1/30，2026/4/8，2026/5/4</t>
+          <t>2025/05/12，2025/05/22，2025/05/25，2025/07/20，2025/09/12，2026/1/15，2026/1/24，2026/1/30，2026/4/8，2026/5/4，2026/5/23</t>
         </is>
       </c>
       <c r="F437" t="inlineStr"/>
@@ -17942,12 +17962,12 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>BV12U6zBWEfw</t>
+          <t>BV1VTRBBeEYs，BV12U6zBWEfw</t>
         </is>
       </c>
       <c r="J437" t="inlineStr"/>
@@ -18487,7 +18507,7 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/07/13，2025/08/21，2025/12/17</t>
+          <t>2025/05/19，2025/07/13，2025/08/21，2025/12/17，2026/5/23</t>
         </is>
       </c>
       <c r="F451" t="inlineStr"/>
@@ -18498,7 +18518,7 @@
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I451" t="inlineStr">
@@ -18825,7 +18845,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I459" t="inlineStr"/>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>BV1rFJJzXEBq</t>
+        </is>
+      </c>
       <c r="J459" t="inlineStr"/>
     </row>
     <row r="460">
@@ -18975,7 +18999,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>2025/05/23，2025/05/29，2025/09/17，2025/09/02，2025/09/26，2025/10/09，2025/10/24，2026/4/29</t>
+          <t>2025/05/23，2025/05/29，2025/09/17，2025/09/02，2025/09/26，2025/10/09，2025/10/24，2026/4/29，2026/5/23</t>
         </is>
       </c>
       <c r="F463" t="inlineStr"/>
@@ -18986,12 +19010,12 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
         <is>
-          <t>BV1ULsWzoEEy，BV1qCjJzkEGz</t>
+          <t>BV1D7GL6FE8o，BV1ULsWzoEEy，BV1qCjJzkEGz</t>
         </is>
       </c>
       <c r="J463" t="inlineStr"/>
@@ -19141,7 +19165,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I467" t="inlineStr"/>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>BV1D2JRzMEhk</t>
+        </is>
+      </c>
       <c r="J467" t="inlineStr"/>
     </row>
     <row r="468">
@@ -19217,7 +19245,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I469" t="inlineStr"/>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>BV1EKjGzRE5R</t>
+        </is>
+      </c>
       <c r="J469" t="inlineStr"/>
     </row>
     <row r="470">
@@ -19253,7 +19285,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I470" t="inlineStr"/>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>BV15LjGzUEf3</t>
+        </is>
+      </c>
       <c r="J470" t="inlineStr"/>
     </row>
     <row r="471">
@@ -19347,7 +19383,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4，2026/5/23</t>
         </is>
       </c>
       <c r="F473" t="inlineStr"/>
@@ -19358,12 +19394,12 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>BV1ZcdWBNE5r，BV1oQBjBKExX</t>
+          <t>BV1ZcdWBNE5r，BV1oQBjBKExX，BV1e5GL6wEx6</t>
         </is>
       </c>
       <c r="J473" t="inlineStr"/>
@@ -19513,7 +19549,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I477" t="inlineStr"/>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>BV17P7xztEAZ</t>
+        </is>
+      </c>
       <c r="J477" t="inlineStr"/>
     </row>
     <row r="478">
@@ -21831,7 +21871,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24，2026/5/15</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24，2026/5/15，2026/5/23</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -21842,7 +21882,7 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
@@ -22259,7 +22299,7 @@
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/3/8，2026/5/1</t>
+          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/3/8，2026/5/1，2026/5/23</t>
         </is>
       </c>
       <c r="F548" t="inlineStr"/>
@@ -22270,7 +22310,7 @@
       </c>
       <c r="H548" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I548" t="inlineStr">
@@ -23887,7 +23927,7 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24，2026/5/22</t>
         </is>
       </c>
       <c r="F590" t="inlineStr"/>
@@ -23898,12 +23938,12 @@
       </c>
       <c r="H590" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I590" t="inlineStr">
         <is>
-          <t>BV1xxoEBqE8N，BV19UbDzXE7H</t>
+          <t>BV1xxoEBqE8N，BV19UbDzXE7H，BV1eZGb6gEJq</t>
         </is>
       </c>
       <c r="J590" t="inlineStr"/>
@@ -24879,7 +24919,7 @@
       </c>
       <c r="E616" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10，2026/4/23</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10，2026/4/23，2026/5/23</t>
         </is>
       </c>
       <c r="F616" t="inlineStr"/>
@@ -24890,12 +24930,12 @@
       </c>
       <c r="H616" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I616" t="inlineStr">
         <is>
-          <t>BV1NNo7BAEid，BV1RUSTBiEa5</t>
+          <t>BV1Q7GL6FEoT，BV1NNo7BAEid，BV1RUSTBiEa5</t>
         </is>
       </c>
       <c r="J616" t="inlineStr"/>
@@ -25013,7 +25053,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I619" t="inlineStr"/>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>BV1QaezzYE68</t>
+        </is>
+      </c>
       <c r="J619" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -25357,7 +25401,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I628" t="inlineStr"/>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>BV1HkYKz9Ey7</t>
+        </is>
+      </c>
       <c r="J628" t="inlineStr"/>
     </row>
     <row r="629">
@@ -25419,7 +25467,7 @@
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>2025/09/10，2025/09/22，2025/09/24，2025/10/23，2025/12/6，2026/1/24，2026/2/5，2026/2/23，2026/5/5</t>
+          <t>2025/09/10，2025/09/22，2025/09/24，2025/10/23，2025/12/6，2026/1/24，2026/2/5，2026/2/23，2026/5/5，2026/5/23</t>
         </is>
       </c>
       <c r="F630" t="inlineStr"/>
@@ -25430,12 +25478,12 @@
       </c>
       <c r="H630" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I630" t="inlineStr">
         <is>
-          <t>BV1aXvxB1EWN</t>
+          <t>BV1h7GL6FEYH，BV1aXvxB1EWN</t>
         </is>
       </c>
       <c r="J630" t="inlineStr"/>
@@ -25513,7 +25561,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I632" t="inlineStr"/>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>BV1wiHrzxEsm</t>
+        </is>
+      </c>
       <c r="J632" t="inlineStr"/>
     </row>
     <row r="633">
@@ -25845,7 +25897,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I641" t="inlineStr"/>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>BV1iJpgzfEpA</t>
+        </is>
+      </c>
       <c r="J641" t="inlineStr"/>
     </row>
     <row r="642">
@@ -25961,7 +26017,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I644" t="inlineStr"/>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>BV187pVzZE89</t>
+        </is>
+      </c>
       <c r="J644" t="inlineStr"/>
     </row>
     <row r="645">
@@ -26139,7 +26199,7 @@
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/2/23，2026/3/17，2026/3/25</t>
+          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/2/23，2026/3/17，2026/3/25，2026/5/23</t>
         </is>
       </c>
       <c r="F649" t="inlineStr"/>
@@ -26150,12 +26210,12 @@
       </c>
       <c r="H649" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I649" t="inlineStr">
         <is>
-          <t>BV1aZWyzREbb，BV1mLf6B6EYy</t>
+          <t>BV18EGL6bEip，BV1aZWyzREbb，BV1mLf6B6EYy</t>
         </is>
       </c>
       <c r="J649" t="inlineStr"/>
@@ -29711,7 +29771,7 @@
       </c>
       <c r="E743" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1，2026/5/6</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1，2026/5/6，2026/5/23</t>
         </is>
       </c>
       <c r="F743" t="inlineStr"/>
@@ -29722,12 +29782,12 @@
       </c>
       <c r="H743" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I743" t="inlineStr">
         <is>
-          <t>BV181SyBPERE</t>
+          <t>BV1Q7GL6FEwd，BV181SyBPERE</t>
         </is>
       </c>
       <c r="J743" t="inlineStr"/>
@@ -31091,7 +31151,7 @@
       </c>
       <c r="E779" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18，2026/5/10</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18，2026/5/10，2026/5/23</t>
         </is>
       </c>
       <c r="F779" t="inlineStr"/>
@@ -31102,12 +31162,12 @@
       </c>
       <c r="H779" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I779" t="inlineStr">
         <is>
-          <t>BV1mE9nBuEk1，BV1V89GBfE6h，BV1sEzxBCEua</t>
+          <t>BV1mE9nBuEk1，BV1V89GBfE6h，BV1sEzxBCEua，BV18EGL6bEhr</t>
         </is>
       </c>
       <c r="J779" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: Update song list to May 25, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J861"/>
+  <dimension ref="A1:J863"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/19，2025/06/02，2025/06/17，2025/06/23，2025/07/20，2025/09/24，2025/10/09，2026/2/17，2026/3/7</t>
+          <t>2025/03/07，2025/04/04，2025/04/19，2025/06/02，2025/06/17，2025/06/23，2025/07/20，2025/09/24，2025/10/09，2026/2/17，2026/3/7，2026/5/24</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15，2026/5/25</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>65</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6499,7 +6499,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20，2026/5/25</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/06/08，2025/07/13，2025/07/21，2025/07/24，2025/07/28，2025/08/01，2025/08/16，2025/09/26，2025/10/28，2025/11/10，2025/11/17，2025/12/23，2026/4/17</t>
+          <t>2025/03/27，2025/06/08，2025/07/13，2025/07/21，2025/07/24，2025/07/28，2025/08/01，2025/08/16，2025/09/26，2025/10/28，2025/11/10，2025/11/17，2025/12/23，2026/4/17，2026/5/25</t>
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -15251,7 +15251,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/22，2026/4/24</t>
+          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/22，2026/4/24，2026/5/25</t>
         </is>
       </c>
       <c r="F368" t="inlineStr"/>
@@ -15262,7 +15262,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -18151,7 +18151,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12，2026/4/5，2026/5/3</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/1/1，2026/2/10，2026/2/22，2026/3/12，2026/4/5，2026/5/3，2026/5/24</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -18162,7 +18162,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -21667,7 +21667,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1，2026/5/4</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1，2026/5/4，2026/5/25</t>
         </is>
       </c>
       <c r="F532" t="inlineStr"/>
@@ -21678,7 +21678,7 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
@@ -27303,7 +27303,7 @@
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22，2026/4/27</t>
+          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22，2026/4/27，2026/5/25</t>
         </is>
       </c>
       <c r="F678" t="inlineStr"/>
@@ -27314,7 +27314,7 @@
       </c>
       <c r="H678" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I678" t="inlineStr">
@@ -30491,7 +30491,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/19，2026/2/8，2026/5/1</t>
+          <t>2025/12/19，2026/2/8，2026/5/1，2026/5/25</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30502,7 +30502,7 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -31595,7 +31595,7 @@
       </c>
       <c r="E790" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/14，2026/2/20，2026/2/28</t>
+          <t>2026/2/8，2026/2/9，2026/2/14，2026/2/20，2026/2/28，2026/5/25</t>
         </is>
       </c>
       <c r="F790" t="inlineStr"/>
@@ -31606,7 +31606,7 @@
       </c>
       <c r="H790" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I790" t="inlineStr">
@@ -31679,7 +31679,7 @@
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>2026/2/9，2026/2/27，2026/3/9，2026/4/14</t>
+          <t>2026/2/9，2026/2/27，2026/3/9，2026/4/14，2026/5/25</t>
         </is>
       </c>
       <c r="F792" t="inlineStr"/>
@@ -31690,7 +31690,7 @@
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
@@ -32711,7 +32711,7 @@
       </c>
       <c r="E817" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/14，2026/3/28，2026/4/29</t>
+          <t>2026/3/13，2026/3/14，2026/3/28，2026/4/29，2026/5/25</t>
         </is>
       </c>
       <c r="F817" t="inlineStr"/>
@@ -32722,7 +32722,7 @@
       </c>
       <c r="H817" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I817" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="E828" t="inlineStr">
         <is>
-          <t>2026/3/25，2026/4/14</t>
+          <t>2026/3/25，2026/4/14，2026/5/25，2026/5/25</t>
         </is>
       </c>
       <c r="F828" t="inlineStr"/>
@@ -33162,7 +33162,7 @@
       </c>
       <c r="H828" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I828" t="inlineStr">
@@ -33915,7 +33915,7 @@
       </c>
       <c r="E847" t="inlineStr">
         <is>
-          <t>2026/4/16，2026/4/29，2026/5/15</t>
+          <t>2026/4/16，2026/4/29，2026/5/15，2026/5/25</t>
         </is>
       </c>
       <c r="F847" t="inlineStr"/>
@@ -33926,7 +33926,7 @@
       </c>
       <c r="H847" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I847" t="inlineStr">
@@ -33955,7 +33955,7 @@
       </c>
       <c r="E848" t="inlineStr">
         <is>
-          <t>2026/4/17</t>
+          <t>2026/4/17，2026/5/25，2026/5/25</t>
         </is>
       </c>
       <c r="F848" t="inlineStr"/>
@@ -33966,7 +33966,7 @@
       </c>
       <c r="H848" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I848" t="inlineStr">
@@ -34519,6 +34519,90 @@
         </is>
       </c>
       <c r="J861" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>861</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>天ノ弱</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>天之弱</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Akie秋绘</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>2026/5/25，2026/5/25，2026/5/25</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr"/>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>BV1DPVw6sEPJ</t>
+        </is>
+      </c>
+      <c r="J862" t="inlineStr"/>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>862</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>空心吉他</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr"/>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>张玉华</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>2026/5/25</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr"/>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>BV1SNVw69EEk</t>
+        </is>
+      </c>
+      <c r="J863" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: 1.Update song list to Jun.6,2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J860"/>
+  <dimension ref="A1:J862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,7 +571,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7，2026/3/15</t>
+          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7，2026/3/15，2026/6/6</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -582,12 +582,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BV1V7KUzoE22</t>
+          <t>BV1NKEJ61EZ2，BV1V7KUzoE22</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16</t>
+          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16，2026/6/6</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -630,12 +630,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BV1o7daBxEbp，BV1EVGdzNEe7</t>
+          <t>BV14KEJ61EVw，BV1o7daBxEbp，BV1EVGdzNEe7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18，2026/5/10</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18，2026/5/10，2026/6/6</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14，2026/5/6，2026/5/23</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14，2026/5/6，2026/5/23，2026/6/6</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18</t>
+          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18，2026/6/6</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2306,12 +2306,12 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>BV1MYGdzHEtD</t>
+          <t>BV12KEJ61Ea6，BV1MYGdzHEtD</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7，2026/3/14</t>
+          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7，2026/3/14，2026/6/6</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3874,12 +3874,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>BV1nvkjBQEGm，BV1teQ6YYEfw，BV1gD7YzuE2d</t>
+          <t>BV1Pn7Q6aEcn，BV1nvkjBQEGm，BV1teQ6YYEfw，BV1gD7YzuE2d</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/12，2025/05/19，2025/05/25，2025/07/05，2025/08/12，2025/09/03，2025/09/10，2025/11/14，2025/12/31，2026/2/18</t>
+          <t>2025/03/13，2025/04/12，2025/05/19，2025/05/25，2025/07/05，2025/08/12，2025/09/03，2025/09/10，2025/11/14，2025/12/31，2026/2/18，2026/6/6</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4086,12 +4086,12 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>BV1d33ozhE7x</t>
+          <t>BV1n47Q6tE8q，BV1d33ozhE7x</t>
         </is>
       </c>
       <c r="J89" t="inlineStr"/>
@@ -5607,7 +5607,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10，2026/5/23</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10，2026/5/23，2026/6/6</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5，2026/4/9</t>
+          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5，2026/4/9，2026/6/6</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -6218,12 +6218,12 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>BV1tnmmBcEEy</t>
+          <t>BV1HC7D6oEyY，BV1tnmmBcEEy</t>
         </is>
       </c>
       <c r="J142" t="inlineStr"/>
@@ -8091,7 +8091,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/17，2025/05/25，2025/12/2，2026/1/14</t>
+          <t>2025/03/23，2025/04/17，2025/05/25，2025/12/2，2026/1/14，2026/6/6</t>
         </is>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -8102,12 +8102,12 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>BV1CDSbByE47，BV1PKLczAEhW，BV1rEj3zoEfG</t>
+          <t>BV1hT7Q63Ezk，BV1CDSbByE47，BV1PKLczAEhW，BV1rEj3zoEfG</t>
         </is>
       </c>
       <c r="J189" t="inlineStr"/>
@@ -8531,7 +8531,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/07/24，2025/07/29，2025/07/31，2025/09/04，2025/09/24，2025/10/03，2025/10/16，2025/11/18，2025/11/21，2026/3/5</t>
+          <t>2025/03/25，2025/07/24，2025/07/29，2025/07/31，2025/09/04，2025/09/24，2025/10/03，2025/10/16，2025/11/18，2025/11/21，2026/3/5，2026/6/6</t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
@@ -8542,12 +8542,12 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>BV1qgb1z5EKh，BV1ieP2znEAT</t>
+          <t>BV1Yn7D6kEcn，BV1qgb1z5EKh，BV1ieP2znEAT</t>
         </is>
       </c>
       <c r="J200" t="inlineStr"/>
@@ -9259,7 +9259,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/1/16</t>
+          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/1/16，2026/6/6</t>
         </is>
       </c>
       <c r="F218" t="inlineStr"/>
@@ -9270,12 +9270,12 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>BV1bwoRYJEXg，BV1NVahzoELQ</t>
+          <t>BV1M37Q6BE6E，BV1bwoRYJEXg，BV1NVahzoELQ</t>
         </is>
       </c>
       <c r="J218" t="inlineStr"/>
@@ -9315,7 +9315,7 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>BV1gEGSzqEtk</t>
+          <t>BV1gEGSzqEtk，BV1fUD6BzEBW</t>
         </is>
       </c>
       <c r="J219" t="inlineStr"/>
@@ -9979,7 +9979,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15，2026/4/24</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15，2026/4/24，2026/6/6</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/9，2025/12/5，2025/12/19，2025/12/26，2026/1/10，2026/1/19，2026/2/10，2026/3/24，2026/4/18</t>
+          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/9，2025/12/5，2025/12/19，2025/12/26，2026/1/10，2026/1/19，2026/2/10，2026/3/24，2026/4/18，2026/6/6</t>
         </is>
       </c>
       <c r="F313" t="inlineStr"/>
@@ -13062,12 +13062,12 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>BV1nvkjBQE9e</t>
+          <t>BV1vj7D6LEGd，BV1nvkjBQE9e</t>
         </is>
       </c>
       <c r="J313" t="inlineStr"/>
@@ -15283,7 +15283,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/04/25，2025/05/22，2025/07/03，2025/07/11，2025/07/26，2025/09/08，2025/10/03，2025/12/2，2026/1/25</t>
+          <t>2025/04/19，2025/04/25，2025/05/22，2025/07/03，2025/07/11，2025/07/26，2025/09/08，2025/10/03，2025/12/2，2026/1/25，2026/6/6</t>
         </is>
       </c>
       <c r="F369" t="inlineStr"/>
@@ -15294,12 +15294,12 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I369" t="inlineStr">
         <is>
-          <t>BV19FzxBdEQb</t>
+          <t>BV1pW7Q68Epu，BV19FzxBdEQb</t>
         </is>
       </c>
       <c r="J369" t="inlineStr"/>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31，2026/4/24</t>
+          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31，2026/4/24，2026/6/6</t>
         </is>
       </c>
       <c r="F389" t="inlineStr"/>
@@ -16082,7 +16082,7 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I389" t="inlineStr">
@@ -22951,7 +22951,7 @@
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9，2026/3/28，2026/5/10</t>
+          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/9，2026/1/9，2026/1/23，2026/2/12，2026/2/25，2026/3/9，2026/3/28，2026/5/10，2026/6/6</t>
         </is>
       </c>
       <c r="F565" t="inlineStr"/>
@@ -22962,7 +22962,7 @@
       </c>
       <c r="H565" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I565" t="inlineStr">
@@ -23735,7 +23735,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/3，2025/11/22，2026/1/5，2026/2/18，2026/2/23，2026/4/19</t>
+          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/3，2025/11/22，2026/1/5，2026/2/18，2026/2/23，2026/4/19，2026/6/6</t>
         </is>
       </c>
       <c r="F585" t="inlineStr"/>
@@ -23746,7 +23746,7 @@
       </c>
       <c r="H585" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
@@ -24455,7 +24455,7 @@
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8，2026/4/19，2026/5/20</t>
+          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/1/19，2026/2/12，2026/2/14，2026/4/8，2026/4/19，2026/5/20，2026/6/6</t>
         </is>
       </c>
       <c r="F604" t="inlineStr"/>
@@ -24466,7 +24466,7 @@
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I604" t="inlineStr">
@@ -26007,7 +26007,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/3，2025/11/13，2025/11/24，2025/12/5，2025/12/12，2025/12/17，2026/1/6，2026/1/15，2026/1/24，2026/2/27，2026/4/19</t>
+          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/3，2025/11/13，2025/11/24，2025/12/5，2025/12/12，2025/12/17，2026/1/6，2026/1/15，2026/1/24，2026/2/27，2026/4/19，2026/6/6</t>
         </is>
       </c>
       <c r="F644" t="inlineStr"/>
@@ -26018,7 +26018,7 @@
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I644" t="inlineStr">
@@ -26551,7 +26551,7 @@
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/1，2025/12/6，2025/12/12，2026/1/19，2026/4/8，2026/5/20</t>
+          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/1，2025/12/6，2025/12/12，2026/1/19，2026/4/8，2026/5/20，2026/6/6</t>
         </is>
       </c>
       <c r="F658" t="inlineStr"/>
@@ -26562,7 +26562,7 @@
       </c>
       <c r="H658" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I658" t="inlineStr">
@@ -30483,7 +30483,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10，2026/6/6</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30494,7 +30494,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30523,7 +30523,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/1/2，2026/1/10，2026/3/13</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/1/2，2026/1/10，2026/3/13，2026/6/6</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30534,12 +30534,12 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
         <is>
-          <t>BV1GiicB5EFK</t>
+          <t>BV1XC7Q61EDC，BV1GiicB5EFK</t>
         </is>
       </c>
       <c r="J762" t="inlineStr"/>
@@ -34527,6 +34527,86 @@
         </is>
       </c>
       <c r="J860" t="inlineStr"/>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>861</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>世纪末游戏</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr"/>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>VirtuaReal</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>2026/6/6</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr"/>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>BV1KKEJ61EsR</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>862</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Rendezvous</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr"/>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>VirtuaReal</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>2026/6/6</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr"/>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>BV1KKEJ61EBD</t>
+        </is>
+      </c>
+      <c r="J862" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Jun.12, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J862"/>
+  <dimension ref="A1:J863"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,7 +527,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1，2026/4/14，2026/4/24</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/9，2025/11/14，2025/12/24，2025/12/26，2026/1/16，2026/1/24，2026/1/28，2026/1/30，2026/2/10，2026/2/14，2026/3/9，2026/3/27，2026/4/1，2026/4/14，2026/4/24，2026/6/12</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -538,7 +538,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1，2026/4/20，2026/5/15</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/1，2025/11/17，2025/12/2，2025/12/31，2026/2/2，2026/2/14，2026/3/6，2026/4/1，2026/4/20，2026/5/15，2026/6/10</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -714,7 +714,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/4，2026/1/24，2026/1/24，2026/2/19，2026/2/25，2026/3/13，2026/4/8</t>
+          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/4，2026/1/24，2026/1/24，2026/2/19，2026/2/25，2026/3/13，2026/4/8，2026/6/10</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6，2026/5/16，2026/5/20</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/1，2025/11/9，2025/11/21，2025/12/8，2026/1/15，2026/1/24，2026/3/4，2026/3/14，2026/5/6，2026/5/16，2026/5/20，2026/6/12</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10，2026/5/23</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10，2026/5/23，2026/6/10</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17，2026/5/1</t>
+          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17，2026/5/1，2026/6/10</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/05/25</t>
+          <t>2025/03/07，2025/05/25，2026/6/10</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15，2026/5/25</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15，2026/5/25，2026/6/12</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/4/9，2026/5/10</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/4/9，2026/5/10，2026/6/12</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/2/2，2026/2/12，2026/4/14，2026/4/22</t>
+          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/2/2，2026/2/12，2026/4/14，2026/4/22，2026/6/10</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/2/19，2026/4/14</t>
+          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/2/19，2026/4/14，2026/6/12</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29，2026/5/15</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29，2026/5/15，2026/6/12</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/15，2025/06/30，2025/08/13，2025/10/25，2026/3/13</t>
+          <t>2025/03/14，2025/05/15，2025/06/30，2025/08/13，2025/10/25，2026/3/13，2026/6/12</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -4886,12 +4886,12 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>BV1RmEnz1ETY</t>
+          <t>BV1znJ569EPZ，BV1RmEnz1ETY</t>
         </is>
       </c>
       <c r="J109" t="inlineStr"/>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/06/06，2025/06/27，2025/08/01，2025/11/9，2025/11/14</t>
+          <t>2025/03/14，2025/06/06，2025/06/27，2025/08/01，2025/11/9，2025/11/14，2026/6/12</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -4974,12 +4974,12 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>BV1uLQrYvEXC，BV1ZRCMBfEPY，BV1QtgozdEWF</t>
+          <t>BV1RLE16eED7，BV1uLQrYvEXC，BV1ZRCMBfEPY，BV1QtgozdEWF</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14，2026/4/22</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14，2026/4/22，2026/6/10</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/05/18，2025/06/13，2025/09/12，2025/10/01，2026/4/20</t>
+          <t>2025/03/19，2025/04/07，2025/05/18，2025/06/13，2025/09/12，2025/10/01，2026/4/20，2026/6/10</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20，2026/5/25</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20，2026/5/25，2026/6/10</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/06/26，2026/4/14</t>
+          <t>2025/03/20，2025/06/26，2026/4/14，2026/6/10</t>
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26，2026/5/5，2026/5/23</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/8，2025/12/26，2026/1/5，2026/1/24，2026/2/5，2026/2/14，2026/3/9，2026/3/28，2026/4/26，2026/5/5，2026/5/23，2026/6/12</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>2025/3/21</t>
+          <t>2025/3/21，2026/6/12</t>
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -7146,12 +7146,12 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>BV1iuXkYHEUG</t>
+          <t>BV1PoJE61EM6，BV1iuXkYHEUG</t>
         </is>
       </c>
       <c r="J165" t="inlineStr"/>
@@ -7891,7 +7891,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22，2026/4/19，2026/5/10</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/2，2025/12/5，2025/12/30，2026/1/23，2026/1/29，2026/2/23，2026/3/17，2026/3/22，2026/4/19，2026/5/10，2026/6/12</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -8051,7 +8051,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25，2026/4/19，2026/5/23</t>
+          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/1/29，2026/2/9，2026/3/25，2026/4/19，2026/5/23，2026/6/12</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/05，2025/06/23，2025/09/15，2025/12/7</t>
+          <t>2025/03/25，2025/05/05，2025/06/23，2025/09/15，2025/12/7，2026/6/12</t>
         </is>
       </c>
       <c r="F198" t="inlineStr"/>
@@ -8462,12 +8462,12 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>BV19MmPBJEoW，BV1Jg37zfEct</t>
+          <t>BV1EnJ569Ez5，BV19MmPBJEoW，BV1Jg37zfEct</t>
         </is>
       </c>
       <c r="J198" t="inlineStr"/>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/09/24，2025/11/27，2026/4/14</t>
+          <t>2025/03/25，2025/09/24，2025/11/27，2026/4/14，2026/6/10</t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -9103,7 +9103,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25，2026/4/9，2026/5/10</t>
+          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/3/25，2026/4/9，2026/5/10，2026/6/10</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -9179,7 +9179,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29，2026/5/15，2026/5/19</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/1/16，2026/2/2，2026/2/7，2026/3/31，2026/4/17，2026/4/29，2026/5/15，2026/5/19，2026/6/12</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9190,7 +9190,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12，2026/4/1，2026/5/1</t>
+          <t>2025/03/28，2025/04/29，2025/06/09，2025/07/24，2025/08/01，2025/08/03，2025/08/16，2025/09/08，2025/09/12，2025/10/03，2025/10/30，2026/1/10，2026/3/1，2026/3/12，2026/4/1，2026/5/1，2026/6/10</t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -9310,7 +9310,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/03，2025/05/26，2025/11/9，2026/5/6</t>
+          <t>2025/03/28，2025/05/03，2025/05/26，2025/11/9，2026/5/6，2026/6/10</t>
         </is>
       </c>
       <c r="F227" t="inlineStr"/>
@@ -9626,7 +9626,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8，2026/4/24，2026/5/21</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/3，2025/11/9，2025/12/23，2026/4/8，2026/4/24，2026/5/21，2026/6/10</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9950,7 +9950,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8，2026/5/1</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8，2026/5/1，2026/6/10</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10834,7 +10834,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/1/23，2026/2/18，2026/3/12</t>
+          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/1/23，2026/2/18，2026/3/12，2026/6/10</t>
         </is>
       </c>
       <c r="F272" t="inlineStr"/>
@@ -11434,7 +11434,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -13011,7 +13011,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/2/23，2026/3/6，2026/4/22</t>
+          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/2/23，2026/3/6，2026/4/22，2026/6/10</t>
         </is>
       </c>
       <c r="F312" t="inlineStr"/>
@@ -13022,7 +13022,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1，2026/5/21</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1，2026/5/21，2026/6/10</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13950,7 +13950,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -15803,7 +15803,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>2025/04/24，2025/09/22，2026/3/29</t>
+          <t>2025/04/24，2025/09/22，2026/3/29，2026/6/10</t>
         </is>
       </c>
       <c r="F382" t="inlineStr"/>
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
@@ -17671,7 +17671,7 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/20，2025/06/24，2025/07/07，2025/09/30，2026/5/20</t>
+          <t>2025/05/10，2025/06/20，2025/06/24，2025/07/07，2025/09/30，2026/5/20，2026/6/12</t>
         </is>
       </c>
       <c r="F430" t="inlineStr"/>
@@ -17682,7 +17682,7 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
@@ -18151,7 +18151,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/27，2025/07/10，2026/3/9，2026/4/9</t>
+          <t>2025/05/18，2025/06/27，2025/07/10，2026/3/9，2026/4/9，2026/6/10</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -18162,7 +18162,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -21519,7 +21519,7 @@
       </c>
       <c r="E528" t="inlineStr">
         <is>
-          <t>2025/6/19</t>
+          <t>2025/6/19，2026/6/10</t>
         </is>
       </c>
       <c r="F528" t="inlineStr"/>
@@ -21530,10 +21530,14 @@
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I528" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>BV11rNdz8EhY</t>
+        </is>
+      </c>
       <c r="J528" t="inlineStr"/>
     </row>
     <row r="529">
@@ -21795,7 +21799,7 @@
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24，2026/5/15，2026/5/23</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/2/18，2026/3/9，2026/4/16，2026/4/24，2026/5/15，2026/5/23，2026/6/12</t>
         </is>
       </c>
       <c r="F535" t="inlineStr"/>
@@ -21806,7 +21810,7 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
@@ -23851,7 +23855,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24，2026/5/22</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24，2026/5/22，2026/6/12</t>
         </is>
       </c>
       <c r="F588" t="inlineStr"/>
@@ -23862,7 +23866,7 @@
       </c>
       <c r="H588" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I588" t="inlineStr">
@@ -24307,7 +24311,7 @@
       </c>
       <c r="E600" t="inlineStr">
         <is>
-          <t>2025/07/26，2025/09/24，2025/10/28，2025/11/12，2025/12/16，2026/1/14，2026/1/30</t>
+          <t>2025/07/26，2025/09/24，2025/10/28，2025/11/12，2025/12/16，2026/1/14，2026/1/30，2026/6/10</t>
         </is>
       </c>
       <c r="F600" t="inlineStr"/>
@@ -24318,7 +24322,7 @@
       </c>
       <c r="H600" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I600" t="inlineStr">
@@ -24723,7 +24727,7 @@
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1，2026/4/8，2026/5/15</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/2，2025/12/17，2026/1/14，2026/2/2，2026/3/22，2026/4/1，2026/4/8，2026/5/15，2026/6/10</t>
         </is>
       </c>
       <c r="F611" t="inlineStr"/>
@@ -24734,7 +24738,7 @@
       </c>
       <c r="H611" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I611" t="inlineStr">
@@ -26395,7 +26399,7 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>2025/09/19，2025/09/26，2025/10/16，2025/11/26，2026/2/12，2026/4/10</t>
+          <t>2025/09/19，2025/09/26，2025/10/16，2025/11/26，2026/2/12，2026/4/10，2026/6/12</t>
         </is>
       </c>
       <c r="F654" t="inlineStr"/>
@@ -26406,12 +26410,12 @@
       </c>
       <c r="H654" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I654" t="inlineStr">
         <is>
-          <t>BV1B4cqzWEhs</t>
+          <t>BV19EE16aEbA，BV1B4cqzWEhs</t>
         </is>
       </c>
       <c r="J654" t="inlineStr"/>
@@ -26591,7 +26595,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1，2026/5/20</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1，2026/5/20，2026/6/10</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -26602,7 +26606,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -26851,7 +26855,7 @@
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/7，2025/11/26，2025/12/6，2025/12/12，2025/12/24，2026/1/5，2026/1/19，2026/2/18，2026/3/14，2026/3/24</t>
+          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/7，2025/11/26，2025/12/6，2025/12/12，2025/12/24，2026/1/5，2026/1/19，2026/2/18，2026/3/14，2026/3/24，2026/6/10</t>
         </is>
       </c>
       <c r="F666" t="inlineStr"/>
@@ -26862,7 +26866,7 @@
       </c>
       <c r="H666" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I666" t="inlineStr">
@@ -31067,7 +31071,7 @@
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18，2026/5/10，2026/5/23</t>
+          <t>2026/1/24，2026/1/25，2026/1/26，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/3/4，2026/3/12，2026/3/31，2026/4/1，2026/4/14，2026/4/18，2026/5/10，2026/5/23，2026/6/12</t>
         </is>
       </c>
       <c r="F776" t="inlineStr"/>
@@ -31078,7 +31082,7 @@
       </c>
       <c r="H776" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I776" t="inlineStr">
@@ -33111,7 +33115,7 @@
       </c>
       <c r="E826" t="inlineStr">
         <is>
-          <t>2026/3/28，2026/4/14，2026/5/10</t>
+          <t>2026/3/28，2026/4/14，2026/5/10，2026/6/12</t>
         </is>
       </c>
       <c r="F826" t="inlineStr"/>
@@ -33122,7 +33126,7 @@
       </c>
       <c r="H826" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">
@@ -33231,7 +33235,7 @@
       </c>
       <c r="E829" t="inlineStr">
         <is>
-          <t>2026/4/1</t>
+          <t>2026/4/1，2026/6/10</t>
         </is>
       </c>
       <c r="F829" t="inlineStr"/>
@@ -33242,7 +33246,7 @@
       </c>
       <c r="H829" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I829" t="inlineStr">
@@ -34607,6 +34611,46 @@
         </is>
       </c>
       <c r="J862" t="inlineStr"/>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>863</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>DAY BY DAY</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr"/>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>T-ara</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>2026/6/10</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr"/>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>韩语</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>BV119Ed6EEBS</t>
+        </is>
+      </c>
+      <c r="J863" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Jun.13, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -10467,7 +10467,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/1/1，2026/1/25，2026/3/8，2026/4/27</t>
+          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/1/1，2026/1/25，2026/3/8，2026/4/27，2026/6/13</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7，2026/5/8，2026/5/23</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/1/21，2026/2/25，2026/2/27，2026/3/1，2026/3/8，2026/3/13，2026/3/25，2026/4/1，2026/5/1，2026/5/7，2026/5/8，2026/5/23，2026/6/13</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -11183,7 +11183,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/04，2025/05/20，2025/06/23，2025/07/24，2025/09/12，2025/10/17，2025/12/9，2026/2/14，2026/3/25</t>
+          <t>2025/04/02，2025/05/04，2025/05/20，2025/06/23，2025/07/24，2025/09/12，2025/10/17，2025/12/9，2026/2/14，2026/3/25，2026/6/13</t>
         </is>
       </c>
       <c r="F266" t="inlineStr"/>
@@ -11194,7 +11194,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/19，2025/05/20，2025/07/11，2025/09/12，2025/12/9，2025/12/16，2026/2/27</t>
+          <t>2025/04/05，2025/04/19，2025/05/20，2025/07/11，2025/09/12，2025/12/9，2025/12/16，2026/2/27，2026/6/13</t>
         </is>
       </c>
       <c r="F295" t="inlineStr"/>
@@ -12346,12 +12346,12 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>BV16NAXz6EZ7</t>
+          <t>BV1xWJs6aEga，BV16NAXz6EZ7</t>
         </is>
       </c>
       <c r="J295" t="inlineStr"/>
@@ -12855,7 +12855,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/2/4，2026/2/14，2026/4/15</t>
+          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/2/4，2026/2/14，2026/4/15，2026/6/13</t>
         </is>
       </c>
       <c r="F308" t="inlineStr"/>
@@ -12866,7 +12866,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -28550,12 +28550,12 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>NF</t>
+          <t>Dawid Podsiadlo</t>
         </is>
       </c>
       <c r="E710" t="inlineStr">
         <is>
-          <t>2025/10/23，2025/10/28，2026/4/2</t>
+          <t>2025/10/23，2025/10/28，2026/4/2，2026/6/13</t>
         </is>
       </c>
       <c r="F710" t="inlineStr"/>
@@ -28566,12 +28566,12 @@
       </c>
       <c r="H710" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I710" t="inlineStr">
         <is>
-          <t>BV1ax9KBMERF</t>
+          <t>BV1eNJs6yEUY，BV1ax9KBMERF</t>
         </is>
       </c>
       <c r="J710" t="inlineStr"/>
@@ -31515,7 +31515,7 @@
       </c>
       <c r="E787" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/14，2026/2/20，2026/2/28，2026/5/25</t>
+          <t>2026/2/8，2026/2/9，2026/2/14，2026/2/20，2026/2/28，2026/5/25，2026/6/13</t>
         </is>
       </c>
       <c r="F787" t="inlineStr"/>
@@ -31526,12 +31526,12 @@
       </c>
       <c r="H787" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I787" t="inlineStr">
         <is>
-          <t>BV1JncczQEuJ，BV1c6fGBDEG1</t>
+          <t>BV17kJs6JEcm，BV1JncczQEuJ，BV1c6fGBDEG1</t>
         </is>
       </c>
       <c r="J787" t="inlineStr"/>
@@ -32631,7 +32631,7 @@
       </c>
       <c r="E814" t="inlineStr">
         <is>
-          <t>2026/3/13，2026/3/14，2026/3/28，2026/4/29，2026/5/25，2026/6/3</t>
+          <t>2026/3/13，2026/3/14，2026/3/28，2026/4/29，2026/5/25，2026/6/3，2026/6/13</t>
         </is>
       </c>
       <c r="F814" t="inlineStr"/>
@@ -32642,7 +32642,7 @@
       </c>
       <c r="H814" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I814" t="inlineStr">

</xml_diff>

<commit_message>
chore: Update song list to Jun.15, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J863"/>
+  <dimension ref="A1:J867"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11，2026/4/16，2026/4/23</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/9，2025/12/30，2026/2/20，2026/2/23，2026/3/4，2026/4/11，2026/4/16，2026/4/23，2026/6/14</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10，2026/5/23，2026/6/10</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/1，2025/11/28，2025/12/12，2026/1/5，2026/1/22，2026/3/4，2026/3/8，2026/3/22，2026/4/22，2026/4/24，2026/5/10，2026/5/23，2026/6/10，2026/6/15</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1682,12 +1682,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BV18EGL6bEnV，BV1hYobBkEum，BV1wUojYeEon</t>
+          <t>BV1hYobBkEum，BV18EGL6bEnV，BV1wUojYeEon</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17，2026/5/1，2026/6/10</t>
+          <t>2025/03/04，2025/04/24，2025/05/25，2025/06/19，2025/06/20，2025/07/14，2026/4/17，2026/5/1，2026/6/10，2026/6/15</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14，2026/5/4，2026/5/23</t>
+          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/4，2025/12/24，2026/1/15，2026/2/23，2026/3/8，2026/4/14，2026/5/4，2026/5/23，2026/6/14</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2882,12 +2882,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>BV1Q7GL6FEm3，BV19DUYBTErV</t>
+          <t>BV1tyJA6zEgJ，BV1Q7GL6FEm3，BV19DUYBTErV</t>
         </is>
       </c>
       <c r="J60" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/2/19，2026/4/14，2026/6/12</t>
+          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/2/19，2026/4/14，2026/6/12，2026/6/14</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21，2026/4/16，2026/5/10</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/1，2026/1/16，2026/2/2，2026/2/23，2026/3/8，2026/3/19，2026/3/21，2026/4/16，2026/5/10，2026/6/14</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/9，2026/1/23，2026/2/18，2026/4/9</t>
+          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/9，2026/1/23，2026/2/18，2026/4/9，2026/6/15</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/9，2026/3/25，2026/4/26</t>
+          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/9，2026/3/25，2026/4/26，2026/6/15</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4606,12 +4606,12 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>BV1ujQuYyEDq，BV11WjQz1Etp</t>
+          <t>BV1MojP6BERK，BV1ujQuYyEDq，BV11WjQz1Etp</t>
         </is>
       </c>
       <c r="J102" t="inlineStr"/>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/21</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/21，2026/6/14</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/05/22，2025/06/10，2025/11/9，2025/11/14，2026/3/19</t>
+          <t>2025/03/15，2025/05/22，2025/06/10，2025/11/9，2025/11/14，2026/3/19，2026/6/15</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -5578,12 +5578,12 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>BV1zTJHzdEvq，BV1ubQSYZEco</t>
+          <t>BV1EjJG6UEhu，BV1zTJHzdEvq，BV1ubQSYZEco</t>
         </is>
       </c>
       <c r="J126" t="inlineStr"/>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/9，2025/12/4，2026/1/1，2026/1/29，2026/4/9</t>
+          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/9，2025/12/4，2026/1/1，2026/1/29，2026/4/9，2026/6/15</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -6058,12 +6058,12 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>BV1CF2LBhEi1</t>
+          <t>BV1g2QwBnEJV，BV1CF2LBhEi1</t>
         </is>
       </c>
       <c r="J138" t="inlineStr"/>
@@ -6611,7 +6611,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/8，2025/12/24，2026/1/28，2026/4/22，2026/5/5</t>
+          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/8，2025/12/24，2026/1/28，2026/4/22，2026/5/5，2026/6/14</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/06/17，2025/09/28，2025/10/20，2025/10/31，2026/1/16</t>
+          <t>2025/03/30，2025/06/17，2025/09/28，2025/10/20，2025/10/31，2026/1/16，2026/6/14</t>
         </is>
       </c>
       <c r="F241" t="inlineStr"/>
@@ -10198,12 +10198,12 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>BV1SfNizjEvd，BV1GYyXB2Ez5</t>
+          <t>BV1U3Ju6sEkB，BV1SfNizjEvd，BV1GYyXB2Ez5</t>
         </is>
       </c>
       <c r="J241" t="inlineStr"/>
@@ -11143,7 +11143,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/27，2025/07/24，2026/1/1</t>
+          <t>2025/04/02，2025/05/27，2025/07/24，2026/1/1，2026/6/14</t>
         </is>
       </c>
       <c r="F265" t="inlineStr"/>
@@ -11154,12 +11154,12 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>BV1w1jZzdEMn</t>
+          <t>BV1tyJN6jEzQ，BV1w1jZzdEMn</t>
         </is>
       </c>
       <c r="J265" t="inlineStr"/>
@@ -11667,7 +11667,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25，2026/4/24，2026/5/23</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/6，2026/1/9，2026/1/29，2026/3/25，2026/4/24，2026/5/23，2026/6/15</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11678,7 +11678,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>2025/4/4</t>
+          <t>2025/4/4，2026/6/15</t>
         </is>
       </c>
       <c r="F292" t="inlineStr"/>
@@ -12230,10 +12230,14 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I292" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>BV1WmJG6tEQf</t>
+        </is>
+      </c>
       <c r="J292" t="inlineStr"/>
     </row>
     <row r="293">
@@ -12935,7 +12939,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/9，2026/1/24，2026/3/31，2026/4/2</t>
+          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/9，2026/1/24，2026/3/31，2026/4/2，2026/6/15</t>
         </is>
       </c>
       <c r="F310" t="inlineStr"/>
@@ -12946,12 +12950,12 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>BV1BfsmzyE4u</t>
+          <t>BV1wgJG69EET，BV1BfsmzyE4u</t>
         </is>
       </c>
       <c r="J310" t="inlineStr"/>
@@ -13439,7 +13443,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24，2026/4/19，2026/5/21</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/1/29，2026/2/10，2026/3/9，2026/3/24，2026/4/19，2026/5/21，2026/6/15</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -13450,7 +13454,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -14031,7 +14035,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19，2026/5/1，2026/5/21</t>
+          <t>2025/04/13，2025/04/15，2025/04/27，2025/05/22，2025/05/29，2025/06/03，2025/06/13，2025/06/28，2025/08/22，2025/09/19，2025/10/12，2025/12/5，2025/12/9，2026/1/15，2026/1/24，2026/3/19，2026/5/1，2026/5/21，2026/6/15</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -14042,7 +14046,7 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -16071,7 +16075,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31，2026/4/24，2026/6/6</t>
+          <t>2025/04/25，2025/09/08，2025/09/15，2025/12/30，2026/3/31，2026/4/24，2026/6/6，2026/6/14</t>
         </is>
       </c>
       <c r="F389" t="inlineStr"/>
@@ -16082,7 +16086,7 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I389" t="inlineStr">
@@ -16775,7 +16779,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/11/18，2026/2/14，2026/4/9，2026/5/16</t>
+          <t>2025/04/28，2025/11/18，2026/2/14，2026/4/9，2026/5/16，2026/6/14</t>
         </is>
       </c>
       <c r="F407" t="inlineStr"/>
@@ -16786,12 +16790,12 @@
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>BV125yVBxER9，BV1zsL56jEVx</t>
+          <t>BV1M3Ju6xEZ6，BV125yVBxER9，BV1zsL56jEVx</t>
         </is>
       </c>
       <c r="J407" t="inlineStr"/>
@@ -18835,7 +18839,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/1/5，2026/2/2，2026/3/17，2026/5/10</t>
+          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/1/5，2026/2/2，2026/3/17，2026/5/10，2026/6/14，2026/6/15</t>
         </is>
       </c>
       <c r="F459" t="inlineStr"/>
@@ -18846,7 +18850,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -19343,7 +19347,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4，2026/5/23</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4，2026/5/23，2026/6/14</t>
         </is>
       </c>
       <c r="F472" t="inlineStr"/>
@@ -19354,7 +19358,7 @@
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
@@ -20967,7 +20971,7 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>2025/06/12，2025/07/13，2025/07/18，2025/09/28，2025/10/20，2026/1/19，2026/4/17</t>
+          <t>2025/06/12，2025/07/13，2025/07/18，2025/09/28，2025/10/20，2026/1/19，2026/4/17，2026/6/15</t>
         </is>
       </c>
       <c r="F514" t="inlineStr"/>
@@ -20978,12 +20982,12 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
         <is>
-          <t>BV1rEdLBDEsD，BV1ySRJYkEK1</t>
+          <t>BV1uojP6BEHc，BV1rEdLBDEsD，BV1ySRJYkEK1</t>
         </is>
       </c>
       <c r="J514" t="inlineStr">
@@ -23467,7 +23471,7 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/1/9，2026/3/7，2026/3/8</t>
+          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/1/9，2026/3/7，2026/3/8，2026/6/14</t>
         </is>
       </c>
       <c r="F578" t="inlineStr"/>
@@ -23478,12 +23482,12 @@
       </c>
       <c r="H578" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I578" t="inlineStr">
         <is>
-          <t>BV1PNNAzLEvL，BV1bRNVzDETM</t>
+          <t>BV1ixJN6bEmS，BV1PNNAzLEvL，BV1bRNVzDETM</t>
         </is>
       </c>
       <c r="J578" t="inlineStr"/>
@@ -23931,7 +23935,7 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6，2026/3/28，2026/4/19</t>
+          <t>2025/07/17，2025/07/24，2025/07/28，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/26，2025/08/29，2025/09/19，2025/09/29，2025/10/11，2025/10/22，2025/10/28，2025/11/10，2025/11/28，2025/12/16，2026/2/19，2026/3/6，2026/3/28，2026/4/19，2026/6/14</t>
         </is>
       </c>
       <c r="F590" t="inlineStr"/>
@@ -23942,7 +23946,7 @@
       </c>
       <c r="H590" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I590" t="inlineStr">
@@ -24887,7 +24891,7 @@
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>2025/08/21，2026/1/16，2026/2/2，2026/3/17，2026/4/8</t>
+          <t>2025/08/21，2026/1/16，2026/2/2，2026/3/17，2026/4/8，2026/6/14</t>
         </is>
       </c>
       <c r="F615" t="inlineStr"/>
@@ -24898,7 +24902,7 @@
       </c>
       <c r="H615" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I615" t="inlineStr">
@@ -25127,7 +25131,7 @@
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>2025/08/29，2025/09/08，2025/11/24</t>
+          <t>2025/08/29，2025/09/08，2025/11/24，2026/6/14</t>
         </is>
       </c>
       <c r="F621" t="inlineStr"/>
@@ -25138,10 +25142,14 @@
       </c>
       <c r="H621" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I621" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>BV1xaJK65Erp</t>
+        </is>
+      </c>
       <c r="J621" t="inlineStr"/>
     </row>
     <row r="622">
@@ -26439,7 +26447,7 @@
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>2025/9/19</t>
+          <t>2025/9/19，2026/6/14</t>
         </is>
       </c>
       <c r="F655" t="inlineStr"/>
@@ -26450,12 +26458,12 @@
       </c>
       <c r="H655" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I655" t="inlineStr">
         <is>
-          <t>BV1hAWVzwEnG</t>
+          <t>BV1U3Ju6sEB7，BV1hAWVzwEnG</t>
         </is>
       </c>
       <c r="J655" t="inlineStr"/>
@@ -30487,7 +30495,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10，2026/6/6</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10，2026/6/6，2026/6/14</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30498,7 +30506,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30651,7 +30659,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27，2026/4/24，2026/5/1</t>
+          <t>2025/12/26，2026/1/10，2026/1/22，2026/1/23，2026/1/31，2026/2/10，2026/2/23，2026/3/9，2026/3/12，2026/3/14，2026/3/17，2026/3/27，2026/4/24，2026/5/1，2026/6/14</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -30662,7 +30670,7 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -32171,7 +32179,7 @@
       </c>
       <c r="E803" t="inlineStr">
         <is>
-          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2，2026/5/6，2026/5/21，2026/5/26</t>
+          <t>2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/1，2026/3/4，2026/3/5，2026/3/5，2026/3/6，2026/3/12，2026/3/21，2026/3/31，2026/4/20，2026/5/2，2026/5/6，2026/5/21，2026/5/26，2026/6/14</t>
         </is>
       </c>
       <c r="F803" t="inlineStr"/>
@@ -32182,7 +32190,7 @@
       </c>
       <c r="H803" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I803" t="inlineStr">
@@ -32979,7 +32987,7 @@
       </c>
       <c r="E823" t="inlineStr">
         <is>
-          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20，2026/5/2，2026/5/6，2026/5/26</t>
+          <t>2026/3/17，2026/3/17，2026/3/25，2026/3/27，2026/3/29，2026/4/2，2026/4/8，2026/4/16，2026/4/20，2026/5/2，2026/5/6，2026/5/26，2026/6/14</t>
         </is>
       </c>
       <c r="F823" t="inlineStr"/>
@@ -32990,7 +32998,7 @@
       </c>
       <c r="H823" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I823" t="inlineStr">
@@ -33683,7 +33691,7 @@
       </c>
       <c r="E840" t="inlineStr">
         <is>
-          <t>2026/4/14</t>
+          <t>2026/4/14，2026/6/14</t>
         </is>
       </c>
       <c r="F840" t="inlineStr"/>
@@ -33694,7 +33702,7 @@
       </c>
       <c r="H840" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I840" t="inlineStr">
@@ -34511,7 +34519,7 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>2026/5/25，2026/5/26</t>
+          <t>2026/5/25，2026/5/26，2026/6/15</t>
         </is>
       </c>
       <c r="F860" t="inlineStr"/>
@@ -34522,7 +34530,7 @@
       </c>
       <c r="H860" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -34651,6 +34659,170 @@
         </is>
       </c>
       <c r="J863" t="inlineStr"/>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>七色回响</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr"/>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>VirtuaReal</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>2026/6/14，2026/6/14</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr"/>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>BV1U3Ju6sEsm</t>
+        </is>
+      </c>
+      <c r="J864" t="inlineStr"/>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>865</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>天灰</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr"/>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>S.H.E</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>2026/6/14</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr"/>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>BV1U3Ju6sEn7</t>
+        </is>
+      </c>
+      <c r="J865" t="inlineStr"/>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>866</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>愿戴荣光坠入天渊</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr"/>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>鸣潮先约电台/jixwang/VISION SOUND</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>2026/6/14，2026/6/14</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr"/>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>BV1u3Ju6xEAo</t>
+        </is>
+      </c>
+      <c r="J866" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>867</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>耳语</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr"/>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>锦零</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>2026/6/15</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr"/>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>BV1GhJG6uEjo</t>
+        </is>
+      </c>
+      <c r="J867" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Jun.17, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J867"/>
+  <dimension ref="A1:J868"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/07，2025/05/29，2025/06/06，2025/06/19，2025/06/26，2025/07/10，2025/07/11，2025/07/14，2025/08/02，2025/09/03，2025/09/26，2025/10/03，2025/11/9，2025/11/24，2025/11/26，2026/1/5，2026/1/30，2026/3/4</t>
+          <t>2025/03/04，2025/04/07，2025/05/29，2025/06/06，2025/06/19，2025/06/26，2025/07/10，2025/07/11，2025/07/14，2025/08/02，2025/09/03，2025/09/26，2025/10/03，2025/11/9，2025/11/24，2025/11/26，2026/1/5，2026/1/30，2026/3/4，2026/6/17</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -1482,12 +1482,12 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BV11K7LzLErv</t>
+          <t>BV13GLR6mEjV，BV11K7LzLErv</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/13，2025/05/06，2025/05/15，2025/05/25，2025/06/06，2025/06/23，2025/07/15，2025/07/26，2025/09/15，2025/09/24，2025/10/03，2025/11/26，2025/12/26，2026/1/10，2026/3/22</t>
+          <t>2025/03/04，2025/04/13，2025/05/06，2025/05/15，2025/05/25，2025/06/06，2025/06/23，2025/07/15，2025/07/26，2025/09/15，2025/09/24，2025/10/03，2025/11/26，2025/12/26，2026/1/10，2026/3/22，2026/6/17</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -1602,12 +1602,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>BV13HjGzyEv6</t>
+          <t>BV1DLLR6yE6W，BV13HjGzyEv6</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/1/14，2026/2/19，2026/3/14，2026/4/16</t>
+          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/1/14，2026/2/19，2026/3/14，2026/4/16，2026/6/17</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18，2026/6/6</t>
+          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18，2026/6/6，2026/6/16，2026/6/17</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2306,12 +2306,12 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>BV12KEJ61Ea6，BV1MYGdzHEtD</t>
+          <t>BV1Kdj36pEvY，BV12KEJ61Ea6，BV1MYGdzHEtD</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/21，2026/6/14</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/9，2026/1/15，2026/2/19，2026/3/13，2026/3/15，2026/3/21，2026/6/14，2026/6/17</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25，2026/4/24，2026/5/23</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/2，2025/12/17，2026/1/9，2026/1/15，2026/2/2，2026/2/14，2026/3/13，2026/3/25，2026/4/24，2026/5/23，2026/6/17</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6098,12 +6098,12 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>BV1qKrGBwEpo</t>
+          <t>BV1TWLR6gEQV，BV1qKrGBwEpo</t>
         </is>
       </c>
       <c r="J139" t="inlineStr"/>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13，2026/3/22，2026/4/14</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/4，2026/1/3，2026/2/10，2026/3/13，2026/3/22，2026/4/14，2026/6/17</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/06/17，2025/09/28，2025/10/20，2025/10/31，2026/1/16，2026/6/14</t>
+          <t>2025/03/30，2025/06/17，2025/09/28，2025/10/20，2025/10/31，2026/1/16，2026/6/14，2026/6/17</t>
         </is>
       </c>
       <c r="F241" t="inlineStr"/>
@@ -10198,7 +10198,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -19075,7 +19075,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>2025/05/23，2025/06/26，2025/07/21，2025/08/12，2025/09/10，2025/09/19，2025/11/1，2025/12/9，2025/12/13，2026/2/14，2026/4/24</t>
+          <t>2025/05/23，2025/06/26，2025/07/21，2025/08/12，2025/09/10，2025/09/19，2025/11/1，2025/12/9，2025/12/13，2026/2/14，2026/4/24，2026/6/16</t>
         </is>
       </c>
       <c r="F465" t="inlineStr"/>
@@ -19086,7 +19086,7 @@
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I465" t="inlineStr">
@@ -21443,7 +21443,7 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/09/05，2025/11/17，2026/1/9，2026/3/1</t>
+          <t>2025/06/19，2025/09/05，2025/11/17，2026/1/9，2026/3/1，2026/6/17</t>
         </is>
       </c>
       <c r="F526" t="inlineStr"/>
@@ -21454,12 +21454,12 @@
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I526" t="inlineStr">
         <is>
-          <t>BV19MPuzkEZX</t>
+          <t>BV1a9LR6UEjB，BV19MPuzkEZX</t>
         </is>
       </c>
       <c r="J526" t="inlineStr"/>
@@ -21483,7 +21483,7 @@
       </c>
       <c r="E527" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/09/02，2026/3/8，2026/3/17，2026/4/14</t>
+          <t>2025/06/19，2025/09/02，2026/3/8，2026/3/17，2026/4/14，2026/6/17</t>
         </is>
       </c>
       <c r="F527" t="inlineStr"/>
@@ -21494,12 +21494,12 @@
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I527" t="inlineStr">
         <is>
-          <t>BV1eyNVztEz8</t>
+          <t>BV1hoLR62Ej2，BV1eyNVztEz8</t>
         </is>
       </c>
       <c r="J527" t="inlineStr"/>
@@ -22187,7 +22187,7 @@
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13，2026/4/12，2026/5/10</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/1/14，2026/1/22，2026/2/19，2026/3/13，2026/4/12，2026/5/10，2026/6/17</t>
         </is>
       </c>
       <c r="F545" t="inlineStr"/>
@@ -22198,7 +22198,7 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
@@ -23859,7 +23859,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24，2026/5/22，2026/6/12</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/1/9，2026/4/2，2026/4/24，2026/5/22，2026/6/12，2026/6/17</t>
         </is>
       </c>
       <c r="F588" t="inlineStr"/>
@@ -23870,7 +23870,7 @@
       </c>
       <c r="H588" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I588" t="inlineStr">
@@ -28195,7 +28195,7 @@
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>2025/10/19，2025/10/20，2025/11/18，2025/12/8，2025/12/16，2026/1/10</t>
+          <t>2025/10/19，2025/10/20，2025/11/18，2025/12/8，2025/12/16，2026/1/10，2026/6/17</t>
         </is>
       </c>
       <c r="F700" t="inlineStr"/>
@@ -28206,12 +28206,12 @@
       </c>
       <c r="H700" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I700" t="inlineStr">
         <is>
-          <t>BV1FozJBWE2P</t>
+          <t>BV1XGLR62EWo，BV1FozJBWE2P</t>
         </is>
       </c>
       <c r="J700" t="inlineStr"/>
@@ -29139,7 +29139,7 @@
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9，2026/3/25，2026/5/1</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/6，2025/12/12，2025/12/26，2026/1/5，2026/1/30，2026/2/9，2026/3/25，2026/5/1，2026/6/17</t>
         </is>
       </c>
       <c r="F725" t="inlineStr"/>
@@ -29150,12 +29150,12 @@
       </c>
       <c r="H725" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I725" t="inlineStr">
         <is>
-          <t>BV1i1C3BYEKh</t>
+          <t>BV1cfLd6NEQX，BV1i1C3BYEKh</t>
         </is>
       </c>
       <c r="J725" t="inlineStr"/>
@@ -30047,7 +30047,7 @@
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25，2026/4/8，2026/5/1</t>
+          <t>2025/12/9，2025/12/17，2026/1/14，2026/1/23，2026/2/5，2026/2/10，2026/2/25，2026/4/8，2026/5/1，2026/6/16</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
@@ -30058,7 +30058,7 @@
       </c>
       <c r="H749" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I749" t="inlineStr">
@@ -31971,7 +31971,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25，2026/3/14，2026/4/20</t>
+          <t>2026/2/22，2026/2/23，2026/2/24，2026/2/25，2026/3/14，2026/4/20，2026/6/16</t>
         </is>
       </c>
       <c r="F798" t="inlineStr"/>
@@ -31982,12 +31982,12 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
         <is>
-          <t>BV1modkBzEQ9，BV1K7f6BgE9r</t>
+          <t>BV1asjG6aEzV，BV1modkBzEQ9，BV1K7f6BgE9r</t>
         </is>
       </c>
       <c r="J798" t="inlineStr">
@@ -32911,7 +32911,7 @@
       </c>
       <c r="E821" t="inlineStr">
         <is>
-          <t>2026/3/17</t>
+          <t>2026/3/17，2026/6/17</t>
         </is>
       </c>
       <c r="F821" t="inlineStr"/>
@@ -32922,10 +32922,14 @@
       </c>
       <c r="H821" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I821" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>BV1frLR6oEwn</t>
+        </is>
+      </c>
       <c r="J821" t="inlineStr"/>
     </row>
     <row r="822">
@@ -34823,6 +34827,46 @@
         </is>
       </c>
       <c r="J867" t="inlineStr"/>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>868</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>My Jealousy</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr"/>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>3rd Coast</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>2026/6/16，2026/6/17</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr"/>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>BV1DzjT62EHE，BV1bHLR6rEFz</t>
+        </is>
+      </c>
+      <c r="J868" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Jun.20, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J868"/>
+  <dimension ref="A1:J872"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,7 +619,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16，2026/6/6</t>
+          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16，2026/6/6，2026/6/18</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17，2026/4/19，2026/5/23</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/9，2025/11/19，2025/12/16，2026/1/16，2026/1/28，2026/2/7，2026/2/10，2026/3/17，2026/4/19，2026/5/23，2026/6/19</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -758,7 +758,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27，2026/5/1，2026/6/3</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27，2026/5/1，2026/6/3，2026/6/18</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -918,7 +918,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/1/3，2026/3/25，2026/5/10</t>
+          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/1/3，2026/3/25，2026/5/10，2026/6/20</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/3，2025/12/12，2026/2/4，2026/4/18，2026/5/20</t>
+          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/3，2025/12/12，2026/2/4，2026/4/18，2026/5/20，2026/6/20</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/27，2025/04/07，2025/04/12，2025/04/22，2025/04/26，2025/05/05，2025/05/19，2025/06/03，2025/06/09，2025/07/18，2025/07/22，2025/09/10，2025/09/19，2025/10/16，2025/12/24</t>
+          <t>2025/03/07，2025/03/27，2025/04/07，2025/04/12，2025/04/22，2025/04/26，2025/05/05，2025/05/19，2025/06/03，2025/06/09，2025/07/18，2025/07/22，2025/09/10，2025/09/19，2025/10/16，2025/12/24，2026/6/20</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13，2026/4/10，2026/5/23</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/7，2025/11/19，2025/11/26，2025/12/30，2026/1/28，2026/2/14，2026/3/13，2026/4/10，2026/5/23，2026/6/18</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/9，2026/1/1</t>
+          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/9，2026/1/1，2026/6/20</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3422,12 +3422,12 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>BV1WmT4zDE9V，BV11PLczYEDi</t>
+          <t>BV1WmT4zDE9V，BV1eqjn6xEEo，BV11PLczYEDi</t>
         </is>
       </c>
       <c r="J73" t="inlineStr"/>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7，2026/3/14，2026/6/6</t>
+          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/4，2025/11/7，2025/11/9，2025/12/4，2026/1/9，2026/1/19，2026/1/21，2026/1/25，2026/3/4，2026/3/7，2026/3/14，2026/6/6，2026/6/19</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/03，2025/05/26，2025/06/01，2025/06/06，2025/09/08，2025/09/12，2026/4/9</t>
+          <t>2025/03/13，2025/04/03，2025/05/26，2025/06/01，2025/06/06，2025/09/08，2025/09/12，2026/4/9，2026/6/20</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/2/10，2026/2/24，2026/3/18，2026/5/20</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/2/10，2026/2/24，2026/3/18，2026/5/20，2026/6/19</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14，2026/4/22，2026/6/10</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/2/27，2026/4/9，2026/4/14，2026/4/22，2026/6/10，2026/6/19</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/7，2026/3/6，2026/4/2</t>
+          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/7，2026/3/6，2026/4/2，2026/6/20</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -5778,12 +5778,12 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>BV1fgP4zNEYf</t>
+          <t>BV13sjW6wEUF，BV1fgP4zNEYf</t>
         </is>
       </c>
       <c r="J131" t="inlineStr"/>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31，2026/4/20，2026/5/1</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/1/3，2026/1/5，2026/1/30，2026/3/14，2026/3/31，2026/4/20，2026/5/1，2026/6/19</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5，2026/4/9，2026/6/6</t>
+          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/1/2，2026/1/15，2026/1/28，2026/2/19，2026/3/5，2026/4/9，2026/6/6，2026/6/20</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20，2026/5/25，2026/6/10</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/1/1，2026/1/9，2026/3/22，2026/4/9，2026/4/20，2026/5/25，2026/6/10，2026/6/19</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6527,7 +6527,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/4/26</t>
+          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/4/26，2026/6/19，2026/6/20</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -6538,12 +6538,12 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>BV1aApuzQEXg，BV136QZYpEx3</t>
+          <t>BV1bfjB6NEqL，BV1aApuzQEXg，BV136QZYpEx3</t>
         </is>
       </c>
       <c r="J150" t="inlineStr"/>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28，2026/3/29，2026/4/27，2026/5/2</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/8，2026/1/23，2026/1/26，2026/2/7，2026/2/10，2026/2/23，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/13，2026/3/24，2026/3/28，2026/3/29，2026/4/27，2026/5/2，2026/6/18</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -6895,7 +6895,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/13，2025/05/30，2025/06/06，2025/07/08，2025/08/07，2025/08/22，2025/09/30，2025/11/9，2025/11/13，2025/12/31，2026/4/16</t>
+          <t>2025/03/20，2025/04/17，2025/05/13，2025/05/30，2025/06/06，2025/07/08，2025/08/07，2025/08/22，2025/09/30，2025/11/9，2025/11/13，2025/12/31，2026/4/16，2026/6/20</t>
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -6906,7 +6906,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/24，2025/06/05，2025/07/26，2025/09/21，2025/10/16，2025/10/30，2025/11/9，2026/1/9，2026/4/24，2026/5/23</t>
+          <t>2025/03/21，2025/04/24，2025/06/05，2025/07/26，2025/09/21，2025/10/16，2025/10/30，2025/11/9，2026/1/9，2026/4/24，2026/5/23，2026/6/20</t>
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20，2026/5/10</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20，2026/5/10，2026/6/19</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7742,7 +7742,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/7，2026/1/17，2026/2/14，2026/4/9，2026/5/20</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/7，2026/1/17，2026/2/14，2026/4/9，2026/5/20，2026/6/19</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -9063,7 +9063,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/15，2025/05/08，2025/06/10，2025/07/07，2025/08/04，2025/09/04，2025/10/01，2025/11/26，2026/1/10，2026/3/22</t>
+          <t>2025/03/27，2025/04/15，2025/05/08，2025/06/10，2025/07/07，2025/08/04，2025/09/04，2025/10/01，2025/11/26，2026/1/10，2026/3/22，2026/6/20</t>
         </is>
       </c>
       <c r="F213" t="inlineStr"/>
@@ -9074,12 +9074,12 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>BV1pbVgznEsP，BV1rNZ3YHEFy，BV1o1STBBEJK</t>
+          <t>BV1pfjn63E6p，BV1pbVgznEsP，BV1rNZ3YHEFy，BV1o1STBBEJK</t>
         </is>
       </c>
       <c r="J213" t="inlineStr"/>
@@ -9655,7 +9655,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/7，2025/11/24，2025/12/5，2026/1/23，2026/3/9，2026/3/25</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/7，2025/11/24，2025/12/5，2026/1/23，2026/3/9，2026/3/25，2026/6/20</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9666,7 +9666,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -10107,7 +10107,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/08/12，2025/10/20，2025/11/14，2025/12/2，2026/1/10，2026/2/9，2026/4/18</t>
+          <t>2025/03/29，2025/08/12，2025/10/20，2025/11/14，2025/12/2，2026/1/10，2026/2/9，2026/4/18，2026/6/20</t>
         </is>
       </c>
       <c r="F239" t="inlineStr"/>
@@ -10118,12 +10118,12 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>BV1KVWmzpEhZ</t>
+          <t>BV1VGjb61EnZ，BV1KVWmzpEhZ</t>
         </is>
       </c>
       <c r="J239" t="inlineStr"/>
@@ -10623,7 +10623,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/2/12，2026/4/16，2026/5/20</t>
+          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/2/12，2026/4/16，2026/5/20，2026/6/20</t>
         </is>
       </c>
       <c r="F252" t="inlineStr"/>
@@ -10634,7 +10634,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8，2026/5/1，2026/6/10</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/2，2026/4/8，2026/5/1，2026/6/10，2026/6/20</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10834,12 +10834,12 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>BV1ET4gzkEE4</t>
+          <t>BV1atjW6FEji，BV1ET4gzkEE4</t>
         </is>
       </c>
       <c r="J257" t="inlineStr"/>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/1/25，2026/2/14，2026/4/9</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/1/25，2026/2/14，2026/4/9，2026/6/20</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11474,7 +11474,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -11507,7 +11507,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13，2026/3/17，2026/5/1</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/3/9，2026/3/13，2026/3/17，2026/5/1，2026/6/18</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11518,7 +11518,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25，2026/4/8，2026/5/23</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/3，2025/11/9，2025/11/26，2025/12/9，2026/1/23，2026/3/13，2026/3/25，2026/4/8，2026/5/23，2026/6/20</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12910,12 +12910,12 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>BV1a7GL6FEYG，BV1aXvxB1EKh，BV1uNSgBeEKj，BV1YBVfzBEpm</t>
+          <t>BV1MajW64EPT，BV1a7GL6FEYG，BV1aXvxB1EKh，BV1uNSgBeEKj，BV1YBVfzBEpm</t>
         </is>
       </c>
       <c r="J309" t="inlineStr"/>
@@ -13211,7 +13211,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/9，2025/11/13，2025/12/4，2025/12/13，2026/3/4，2026/5/7</t>
+          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/9，2025/11/13，2025/12/4，2025/12/13，2026/3/4，2026/5/7，2026/6/20</t>
         </is>
       </c>
       <c r="F317" t="inlineStr"/>
@@ -13222,12 +13222,12 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
         <is>
-          <t>BV1Aw2LBcE8d</t>
+          <t>BV1LLjH68Ejj，BV1Aw2LBcE8d</t>
         </is>
       </c>
       <c r="J317" t="inlineStr"/>
@@ -13367,7 +13367,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/9，2025/12/8，2026/1/5，2026/2/14，2026/5/23</t>
+          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/9，2025/12/8，2026/1/5，2026/2/14，2026/5/23，2026/6/20</t>
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
@@ -13378,7 +13378,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/1/14，2026/1/23，2026/2/12，2026/3/31</t>
+          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/1/14，2026/1/23，2026/2/12，2026/3/31，2026/6/18</t>
         </is>
       </c>
       <c r="F337" t="inlineStr"/>
@@ -13998,7 +13998,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -14283,7 +14283,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>2025/04/14，2025/05/24，2025/06/15，2025/06/19，2025/07/21，2025/08/22，2025/09/20，2025/10/09，2025/10/28，2025/12/22</t>
+          <t>2025/04/14，2025/05/24，2025/06/15，2025/06/19，2025/07/21，2025/08/22，2025/09/20，2025/10/09，2025/10/28，2025/12/22，2026/6/20</t>
         </is>
       </c>
       <c r="F344" t="inlineStr"/>
@@ -14294,12 +14294,12 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>BV18JjhzZEVj，BV1zzoJYTEka</t>
+          <t>BV1MajW64EZ1，BV18JjhzZEVj，BV1zzoJYTEka</t>
         </is>
       </c>
       <c r="J344" t="inlineStr"/>
@@ -15615,7 +15615,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/19，2025/07/25，2025/08/07，2025/09/15，2025/09/29，2026/1/5，2026/2/14，2026/4/9</t>
+          <t>2025/04/21，2025/05/19，2025/07/25，2025/08/07，2025/09/15，2025/09/29，2026/1/5，2026/2/14，2026/4/9，2026/6/20</t>
         </is>
       </c>
       <c r="F377" t="inlineStr"/>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
@@ -17007,7 +17007,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>2025/05/01，2025/08/12，2025/08/26，2025/11/24</t>
+          <t>2025/05/01，2025/08/12，2025/08/26，2025/11/24，2026/6/20</t>
         </is>
       </c>
       <c r="F413" t="inlineStr"/>
@@ -17018,12 +17018,12 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t>BV1S6GzzrExR</t>
+          <t>BV1PkjW6SETh，BV1S6GzzrExR</t>
         </is>
       </c>
       <c r="J413" t="inlineStr"/>
@@ -18755,7 +18755,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/07/21，2026/4/14</t>
+          <t>2025/05/22，2025/07/21，2026/4/14，2026/6/19</t>
         </is>
       </c>
       <c r="F457" t="inlineStr"/>
@@ -18766,7 +18766,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
@@ -18879,7 +18879,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/12，2025/10/03，2025/10/11，2026/1/15，2026/4/29</t>
+          <t>2025/05/22，2025/09/12，2025/10/03，2025/10/11，2026/1/15，2026/4/29，2026/6/18</t>
         </is>
       </c>
       <c r="F460" t="inlineStr"/>
@@ -18890,7 +18890,7 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
@@ -19347,7 +19347,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4，2026/5/23，2026/6/14</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/7，2025/12/7，2025/12/23，2026/1/9，2026/1/24，2026/2/9，2026/2/25，2026/3/13，2026/3/21，2026/4/18，2026/5/4，2026/5/23，2026/6/14，2026/6/19</t>
         </is>
       </c>
       <c r="F472" t="inlineStr"/>
@@ -19358,7 +19358,7 @@
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
@@ -21135,7 +21135,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22，2026/5/10，2026/5/15</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/2，2025/12/9，2025/12/16，2025/12/26，2026/1/5，2026/1/15，2026/1/28，2026/3/6，2026/4/22，2026/5/10，2026/5/15，2026/6/19</t>
         </is>
       </c>
       <c r="F518" t="inlineStr"/>
@@ -21146,7 +21146,7 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I518" t="inlineStr">
@@ -21599,7 +21599,7 @@
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1，2026/5/4，2026/5/25</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/7，2025/11/21，2025/12/2，2025/12/17，2026/1/1，2026/1/5，2026/1/14，2026/1/22，2026/1/24，2026/2/2，2026/3/5，2026/3/15，2026/4/1，2026/5/4，2026/5/25，2026/6/20</t>
         </is>
       </c>
       <c r="F530" t="inlineStr"/>
@@ -21610,12 +21610,12 @@
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>BV126rrBhEvE</t>
+          <t>BV1TYjW6dEV3，BV126rrBhEvE</t>
         </is>
       </c>
       <c r="J530" t="inlineStr"/>
@@ -22271,7 +22271,7 @@
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22，2026/4/11，2026/4/30，2026/5/26</t>
+          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/1/24，2026/2/9，2026/3/6，2026/3/22，2026/4/11，2026/4/30，2026/5/26，2026/6/18</t>
         </is>
       </c>
       <c r="F547" t="inlineStr">
@@ -22286,7 +22286,7 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -23743,7 +23743,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/3，2025/11/22，2026/1/5，2026/2/18，2026/2/23，2026/4/19，2026/6/6</t>
+          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/3，2025/11/22，2026/1/5，2026/2/18，2026/2/23，2026/4/19，2026/6/6，2026/6/19</t>
         </is>
       </c>
       <c r="F585" t="inlineStr"/>
@@ -23754,7 +23754,7 @@
       </c>
       <c r="H585" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
@@ -24851,7 +24851,7 @@
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10，2026/4/23，2026/5/23</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/1，2025/11/26，2025/12/30，2026/1/10，2026/2/18，2026/4/10，2026/4/23，2026/5/23，2026/6/18</t>
         </is>
       </c>
       <c r="F614" t="inlineStr"/>
@@ -24862,7 +24862,7 @@
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I614" t="inlineStr">
@@ -27247,7 +27247,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22，2026/4/27，2026/5/25</t>
+          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/2，2025/12/11，2026/1/9，2026/1/14，2026/2/7，2026/3/22，2026/4/27，2026/5/25，2026/6/20</t>
         </is>
       </c>
       <c r="F676" t="inlineStr"/>
@@ -27258,7 +27258,7 @@
       </c>
       <c r="H676" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I676" t="inlineStr">
@@ -29699,7 +29699,7 @@
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1，2026/5/6，2026/5/23</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/6，2025/12/13，2026/1/10，2026/1/24，2026/2/14，2026/3/14，2026/4/1，2026/4/8，2026/5/1，2026/5/6，2026/5/23，2026/6/20</t>
         </is>
       </c>
       <c r="F740" t="inlineStr"/>
@@ -29710,7 +29710,7 @@
       </c>
       <c r="H740" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I740" t="inlineStr">
@@ -30379,7 +30379,7 @@
       </c>
       <c r="E758" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29，2026/3/22，2026/4/29</t>
+          <t>2025/12/19，2025/12/24，2025/12/26，2026/1/2，2026/1/9，2026/1/23，2026/1/29，2026/3/22，2026/4/29，2026/6/20</t>
         </is>
       </c>
       <c r="F758" t="inlineStr"/>
@@ -30390,7 +30390,7 @@
       </c>
       <c r="H758" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I758" t="inlineStr">
@@ -30495,7 +30495,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10，2026/6/6，2026/6/14</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/1/2，2026/1/5，2026/1/11，2026/1/25，2026/2/9，2026/2/23，2026/3/20，2026/4/2，2026/4/16，2026/4/29，2026/5/10，2026/6/6，2026/6/14，2026/6/20</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30506,7 +30506,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30575,7 +30575,7 @@
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11，2026/4/20，2026/5/15</t>
+          <t>2025/12/26，2026/1/5，2026/1/19，2026/1/21，2026/1/22，2026/1/24，2026/2/7，2026/2/19，2026/2/24，2026/2/24，2026/2/25，2026/3/6，2026/3/25，2026/4/11，2026/4/20，2026/5/15，2026/6/19</t>
         </is>
       </c>
       <c r="F763" t="inlineStr"/>
@@ -30586,7 +30586,7 @@
       </c>
       <c r="H763" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I763" t="inlineStr">
@@ -31119,7 +31119,7 @@
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>2026/1/24，2026/2/8</t>
+          <t>2026/1/24，2026/2/8，2026/6/20</t>
         </is>
       </c>
       <c r="F777" t="inlineStr"/>
@@ -31130,7 +31130,7 @@
       </c>
       <c r="H777" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I777" t="inlineStr">
@@ -31563,7 +31563,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20，2026/5/2，2026/5/21</t>
+          <t>2026/2/8，2026/2/9，2026/2/12，2026/2/14，2026/2/19，2026/2/23，2026/2/24，2026/2/25，2026/3/1，2026/3/5，2026/3/12，2026/3/17，2026/3/19，2026/3/31，2026/4/20，2026/5/2，2026/5/21，2026/6/20</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
@@ -31574,7 +31574,7 @@
       </c>
       <c r="H788" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I788" t="inlineStr">
@@ -31691,7 +31691,7 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>2026/2/14，2026/2/24，2026/3/7，2026/3/13，2026/5/26</t>
+          <t>2026/2/14，2026/2/24，2026/3/7，2026/3/13，2026/5/26，2026/6/19</t>
         </is>
       </c>
       <c r="F791" t="inlineStr"/>
@@ -31702,7 +31702,7 @@
       </c>
       <c r="H791" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I791" t="inlineStr">
@@ -33535,7 +33535,7 @@
       </c>
       <c r="E836" t="inlineStr">
         <is>
-          <t>2026/4/9</t>
+          <t>2026/4/9，2026/6/20</t>
         </is>
       </c>
       <c r="F836" t="inlineStr"/>
@@ -33546,7 +33546,7 @@
       </c>
       <c r="H836" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I836" t="inlineStr">
@@ -34867,6 +34867,166 @@
         </is>
       </c>
       <c r="J868" t="inlineStr"/>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>869</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>明年今日</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr"/>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>陈奕迅</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>2026/6/18</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr"/>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>粤语</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>BV1r4jw6nEZE</t>
+        </is>
+      </c>
+      <c r="J869" t="inlineStr"/>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>870</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>City Hunter 〜愛よ消えないで〜</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr"/>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>小比類巻かほる</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>2026/6/20</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr"/>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>BV19Gjb6yEgK</t>
+        </is>
+      </c>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>动漫</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>871</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>关键词</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr"/>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>林俊杰</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>2026/6/20</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr"/>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr"/>
+      <c r="J871" t="inlineStr"/>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>872</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>三人游</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr"/>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>方大同</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>2026/6/20</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr"/>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>BV1QLjb6kEJz</t>
+        </is>
+      </c>
+      <c r="J872" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Jun.27, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,56 +425,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J872"/>
+  <dimension ref="A1:J874"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -571,7 +583,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7，2026/3/15，2026/6/6</t>
+          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/7，2026/1/14，2026/1/24，2026/2/19，2026/3/7，2026/3/15，2026/6/6，2026/6/23</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -582,7 +594,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -619,7 +631,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16，2026/6/6，2026/6/18</t>
+          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/1/19，2026/1/21，2026/3/4，2026/4/16，2026/6/6，2026/6/18，2026/6/23</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -630,7 +642,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -787,7 +799,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/20，2025/06/16，2025/06/27，2025/07/31，2025/10/05，2025/11/7，2025/12/4，2026/1/28，2026/4/29</t>
+          <t>2025/03/03，2025/04/20，2025/06/16，2025/06/27，2025/07/31，2025/10/05，2025/11/7，2025/12/4，2026/1/28，2026/4/29，2026/6/25</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -798,7 +810,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -907,7 +919,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27，2026/5/1，2026/6/3，2026/6/18</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/7，2025/12/31，2026/1/14，2026/1/19，2026/3/29，2026/4/12，2026/4/27，2026/5/1，2026/6/3，2026/6/18，2026/6/25</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -918,7 +930,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -991,7 +1003,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18，2026/5/10，2026/6/6</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/7，2025/12/17，2026/1/19，2026/1/29，2026/2/10，2026/2/12，2026/3/22，2026/4/18，2026/5/10，2026/6/6，2026/6/25</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1002,7 +1014,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1631,7 +1643,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14，2026/5/6，2026/5/23，2026/6/6</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/5，2025/11/14，2025/11/21，2025/11/28，2025/12/8，2025/12/17，2026/1/10，2026/1/22，2026/2/10，2026/2/14，2026/2/14，2026/2/27，2026/3/28，2026/4/9，2026/4/14，2026/5/6，2026/5/23，2026/6/6，2026/6/25</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1642,7 +1654,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1751,7 +1763,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/3/15</t>
+          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/3/15，2026/6/23</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -1762,7 +1774,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2071,7 +2083,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21，2026/4/26，2026/5/10</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/1/9，2026/1/28，2026/2/25，2026/3/12，2026/3/21，2026/4/26，2026/5/10，2026/6/26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2082,7 +2094,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2243,7 +2255,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/7，2025/11/9，2025/12/2，2026/1/21，2026/3/5，2026/4/16</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/7，2025/11/9，2025/12/2，2026/1/21，2026/3/5，2026/4/16，2026/6/23</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2254,7 +2266,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2291,7 +2303,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18，2026/6/6，2026/6/16，2026/6/17</t>
+          <t>2025/03/06，2025/03/28，2025/04/19，2025/04/24，2025/05/03，2025/05/15，2025/05/16，2025/05/22，2025/05/30，2025/06/14，2025/06/19，2025/06/26，2025/07/18，2025/08/04，2025/09/10，2025/09/18，2025/10/03，2026/2/7，2026/2/9，2026/2/27，2026/4/18，2026/6/6，2026/6/16，2026/6/17，2026/6/23</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2306,7 +2318,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2783,7 +2795,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19，2026/5/1，2026/5/23</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/1，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/1/9，2026/1/22，2026/2/14，2026/3/22，2026/4/19，2026/5/1，2026/5/23，2026/6/25</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2794,7 +2806,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2951,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15，2026/5/25，2026/6/12</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/1，2025/11/9，2025/12/4，2025/12/16，2025/12/31，2026/1/9，2026/1/15，2026/1/21，2026/1/23，2026/1/29，2026/2/2，2026/2/7，2026/2/10，2026/2/14，2026/2/19，2026/2/24，2026/2/25，2026/2/27，2026/3/1，2026/3/4，2026/3/5，2026/3/7，2026/3/8，2026/3/9，2026/3/12，2026/3/13，2026/3/14，2026/3/15，2026/3/17，2026/3/18，2026/3/19，2026/3/22，2026/3/24，2026/3/27，2026/3/28，2026/3/31，2026/4/8，2026/4/14，2026/4/18，2026/4/25，2026/5/1，2026/5/15，2026/5/25，2026/6/12，2026/6/23，2026/6/26</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2962,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3531,7 +3543,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/3/27，2026/4/1</t>
+          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/3/27，2026/4/1，2026/6/23</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3542,12 +3554,12 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>BV1fsnmzPEoD，BV1DDVQzjEMa，BV1rzXTBWEux</t>
+          <t>BV1smjU6pENa，BV1fsnmzPEoD，BV1DDVQzjEMa，BV1rzXTBWEux</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3659,7 +3671,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/05/03，2025/06/19，2026/1/19</t>
+          <t>2025/03/12，2025/05/03，2025/06/19，2026/1/19，2026/6/23</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -3670,12 +3682,12 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>BV19PGozFEg3，BV1GrkgBWEEt</t>
+          <t>BV1WmjU6WEHm，BV19PGozFEg3，BV1GrkgBWEEt</t>
         </is>
       </c>
       <c r="J79" t="inlineStr"/>
@@ -3911,7 +3923,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29，2026/5/15，2026/6/12</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/3，2025/12/2，2025/12/4，2025/12/12，2026/1/5，2026/1/14，2026/2/19，2026/3/4，2026/3/31，2026/4/12，2026/4/29，2026/5/15，2026/6/12，2026/6/23</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3922,7 +3934,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4755,7 +4767,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/1/12，2026/2/7，2026/3/15，2026/4/19</t>
+          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/1/12，2026/2/7，2026/3/15，2026/4/19，2026/6/26</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -4766,7 +4778,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5607,7 +5619,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10，2026/5/23，2026/6/6</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/8，2025/12/12，2026/2/14，2026/3/12，2026/4/9，2026/5/10，2026/5/23，2026/6/6，2026/6/25</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5618,7 +5630,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5687,7 +5699,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/2/7</t>
+          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/2/7，2026/6/23</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -5698,7 +5710,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -6651,7 +6663,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8，2026/5/6，2026/5/21</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/2，2026/1/16，2026/2/2，2026/2/23，2026/2/25，2026/3/17，2026/4/8，2026/5/6，2026/5/21，2026/6/25</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6662,7 +6674,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7731,7 +7743,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20，2026/5/10，2026/6/19</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/1/19，2026/3/9，2026/4/18，2026/4/20，2026/5/10，2026/6/19，2026/6/26</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7742,7 +7754,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -8411,7 +8423,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/9，2026/1/1，2026/2/7，2026/3/25，2026/4/26</t>
+          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/9，2026/1/1，2026/2/7，2026/3/25，2026/4/26，2026/6/23</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -8422,7 +8434,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -8571,7 +8583,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/3/25</t>
+          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/3/25，2026/6/23</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -8582,7 +8594,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -8691,7 +8703,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/20，2025/06/01，2025/07/15，2025/09/27，2025/10/03，2026/3/9</t>
+          <t>2025/03/25，2025/05/20，2025/06/01，2025/07/15，2025/09/27，2025/10/03，2026/3/9，2026/6/26</t>
         </is>
       </c>
       <c r="F204" t="inlineStr"/>
@@ -8702,7 +8714,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -8979,7 +8991,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/06/08，2025/07/13，2025/07/21，2025/07/24，2025/07/28，2025/08/01，2025/08/16，2025/09/26，2025/10/28，2025/11/10，2025/11/17，2025/12/23，2026/4/17，2026/5/25</t>
+          <t>2025/03/27，2025/06/08，2025/07/13，2025/07/21，2025/07/24，2025/07/28，2025/08/01，2025/08/16，2025/09/26，2025/10/28，2025/11/10，2025/11/17，2025/12/23，2026/4/17，2026/5/25，2026/6/26</t>
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
@@ -8990,7 +9002,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -9575,7 +9587,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/08/28，2025/09/18，2025/11/21，2025/12/4，2026/3/21</t>
+          <t>2025/03/28，2025/04/04，2025/08/28，2025/09/18，2025/11/21，2025/12/4，2026/3/21，2026/6/27</t>
         </is>
       </c>
       <c r="F226" t="inlineStr"/>
@@ -9586,12 +9598,12 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>BV19Lh2zmEUD，BV13hZoYwEet，BV161UjBiEza</t>
+          <t>BV1SsTT69ESD，BV19Lh2zmEUD，BV13hZoYwEet，BV161UjBiEza</t>
         </is>
       </c>
       <c r="J226" t="inlineStr"/>
@@ -9979,7 +9991,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15，2026/4/24，2026/6/6</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/7，2025/11/13，2025/12/2，2026/1/14，2026/1/24，2026/3/7，2026/3/15，2026/4/24，2026/6/6，2026/6/23</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -9990,7 +10002,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -10903,7 +10915,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17，2026/5/5，2026/5/21</t>
+          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/2/8，2026/3/17，2026/5/5，2026/5/21，2026/6/25</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
@@ -10914,7 +10926,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -11103,7 +11115,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/22，2025/08/22，2025/09/12，2026/4/20</t>
+          <t>2025/04/02，2025/05/22，2025/08/22，2025/09/12，2026/4/20，2026/6/26</t>
         </is>
       </c>
       <c r="F264" t="inlineStr"/>
@@ -11114,7 +11126,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -13943,7 +13955,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1，2026/5/21，2026/6/10</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/1/9，2026/2/8，2026/3/1，2026/3/9，2026/3/24，2026/4/17，2026/5/1，2026/5/21，2026/6/10，2026/6/25</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13954,7 +13966,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -16615,7 +16627,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/05/29，2025/06/17，2025/07/11，2025/08/03，2025/09/22，2026/4/9</t>
+          <t>2025/04/27，2025/05/29，2025/06/17，2025/07/11，2025/08/03，2025/09/22，2026/4/9，2026/6/23</t>
         </is>
       </c>
       <c r="F403" t="inlineStr"/>
@@ -16626,7 +16638,7 @@
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I403" t="inlineStr">
@@ -17243,7 +17255,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/07/13，2025/10/23</t>
+          <t>2025/05/03，2025/07/13，2025/10/23，2026/6/23</t>
         </is>
       </c>
       <c r="F419" t="inlineStr"/>
@@ -17254,7 +17266,7 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
@@ -18923,7 +18935,7 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/06/17，2025/07/21，2025/08/16，2025/10/16，2025/12/2，2026/4/22</t>
+          <t>2025/05/22，2025/06/17，2025/07/21，2025/08/16，2025/10/16，2025/12/2，2026/4/22，2026/6/23</t>
         </is>
       </c>
       <c r="F461" t="inlineStr"/>
@@ -18934,7 +18946,7 @@
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I461" t="inlineStr">
@@ -21251,7 +21263,7 @@
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>2025/6/17</t>
+          <t>2025/6/17，2026/6/26</t>
         </is>
       </c>
       <c r="F521" t="inlineStr"/>
@@ -21262,10 +21274,14 @@
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I521" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>BV1Aj7L6bEYM</t>
+        </is>
+      </c>
       <c r="J521" t="inlineStr"/>
     </row>
     <row r="522">
@@ -23155,7 +23171,7 @@
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>2025/07/07，2025/09/30，2026/4/9</t>
+          <t>2025/07/07，2025/09/30，2026/4/9，2026/6/26</t>
         </is>
       </c>
       <c r="F570" t="inlineStr"/>
@@ -23166,7 +23182,7 @@
       </c>
       <c r="H570" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I570" t="inlineStr">
@@ -23819,7 +23835,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>2025/07/15，2026/1/5，2026/1/10，2026/1/25，2026/2/10，2026/2/27，2026/3/7，2026/3/15，2026/3/29</t>
+          <t>2025/07/15，2026/1/5，2026/1/10，2026/1/25，2026/2/10，2026/2/27，2026/3/7，2026/3/15，2026/3/29，2026/6/23</t>
         </is>
       </c>
       <c r="F587" t="inlineStr"/>
@@ -23830,7 +23846,7 @@
       </c>
       <c r="H587" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I587" t="inlineStr">
@@ -26095,7 +26111,7 @@
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/09/15，2025/09/22，2025/09/29，2025/09/29，2025/10/10，2025/10/28，2025/12/2，2026/1/5，2026/3/13</t>
+          <t>2025/09/17，2025/09/15，2025/09/22，2025/09/29，2025/09/29，2025/10/10，2025/10/28，2025/12/2，2026/1/5，2026/3/13，2026/6/23</t>
         </is>
       </c>
       <c r="F646" t="inlineStr"/>
@@ -26106,7 +26122,7 @@
       </c>
       <c r="H646" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I646" t="inlineStr">
@@ -26603,7 +26619,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1，2026/5/20，2026/6/10</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/1，2025/11/9，2025/11/19，2025/11/22，2025/11/28，2025/12/8，2025/12/22，2026/1/5，2026/1/14，2026/1/22，2026/2/7，2026/2/10，2026/3/8，2026/3/22，2026/4/18，2026/5/1，2026/5/20，2026/6/10，2026/6/25</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -26614,7 +26630,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -27827,7 +27843,7 @@
       </c>
       <c r="E691" t="inlineStr">
         <is>
-          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25，2026/4/1，2026/4/25</t>
+          <t>2025/10/13，2026/3/4，2026/3/24，2026/3/25，2026/4/1，2026/4/25，2026/6/23</t>
         </is>
       </c>
       <c r="F691" t="inlineStr">
@@ -27842,7 +27858,7 @@
       </c>
       <c r="H691" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I691" t="inlineStr">
@@ -31243,7 +31259,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28，2026/4/12，2026/4/20</t>
+          <t>2026/1/25，2026/1/30，2026/2/2，2026/2/8，2026/2/19，2026/2/23，2026/2/25，2026/3/12，2026/3/28，2026/4/12，2026/4/20，2026/6/26</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -31254,7 +31270,7 @@
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I780" t="inlineStr">
@@ -33087,7 +33103,7 @@
       </c>
       <c r="E825" t="inlineStr">
         <is>
-          <t>2026/3/25，2026/4/14，2026/5/25，2026/5/25</t>
+          <t>2026/3/25，2026/4/14，2026/5/25，2026/5/25，2026/6/25，2026/6/25，2026/6/25，2026/6/26</t>
         </is>
       </c>
       <c r="F825" t="inlineStr"/>
@@ -33098,12 +33114,12 @@
       </c>
       <c r="H825" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I825" t="inlineStr">
         <is>
-          <t>BV1XYX7BMEZn</t>
+          <t>BV1Hw7j6ZELx，BV1XYX7BMEZn</t>
         </is>
       </c>
       <c r="J825" t="inlineStr"/>
@@ -34479,7 +34495,7 @@
       </c>
       <c r="E859" t="inlineStr">
         <is>
-          <t>2026/5/25，2026/5/25，2026/5/25，2026/5/26，2026/5/26</t>
+          <t>2026/5/25，2026/5/25，2026/5/25，2026/5/26，2026/5/26，2026/6/25，2026/6/26</t>
         </is>
       </c>
       <c r="F859" t="inlineStr"/>
@@ -34490,7 +34506,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -34847,7 +34863,7 @@
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>2026/6/16，2026/6/17</t>
+          <t>2026/6/16，2026/6/17，2026/6/25</t>
         </is>
       </c>
       <c r="F868" t="inlineStr"/>
@@ -34858,7 +34874,7 @@
       </c>
       <c r="H868" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I868" t="inlineStr">
@@ -35027,6 +35043,86 @@
         </is>
       </c>
       <c r="J872" t="inlineStr"/>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>873</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>想自由</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr"/>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>林宥嘉</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>2026/6/25</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr"/>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>BV1qq7h6FEBT</t>
+        </is>
+      </c>
+      <c r="J873" t="inlineStr"/>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>874</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>小小虫</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr"/>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>方大同</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>2026/6/25</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr"/>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>BV1Z9786bEfa</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>